<commit_message>
v7: add Colab, Fractal, Kinebot, Jovens Genios; fix Aprova Digital investors; 4 new aportes
</commit_message>
<xml_diff>
--- a/Radar_GovTechs_Brasil_2026.xlsx
+++ b/Radar_GovTechs_Brasil_2026.xlsx
@@ -147,7 +147,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="30">
+  <cellXfs count="29">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center"/>
@@ -225,9 +225,6 @@
       <alignment vertical="top" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="12" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment vertical="top" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="5" fillId="12" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment vertical="top" wrapText="1"/>
     </xf>
   </cellXfs>
@@ -605,7 +602,7 @@
     <row r="1" ht="32" customHeight="1">
       <c r="A1" s="1" t="inlineStr">
         <is>
-          <t>🇧🇷 Radar GovTech Brasil 2025/2026 — DLG · Maio 2026 · v6</t>
+          <t>🇧🇷 Radar GovTech Brasil 2025/2026 — DLG · Maio 2026 · v7</t>
         </is>
       </c>
     </row>
@@ -628,7 +625,7 @@
         </is>
       </c>
       <c r="B4" s="4" t="n">
-        <v>17</v>
+        <v>19</v>
       </c>
     </row>
     <row r="5">
@@ -648,7 +645,7 @@
         </is>
       </c>
       <c r="B6" s="4" t="n">
-        <v>7</v>
+        <v>8</v>
       </c>
     </row>
     <row r="7">
@@ -658,7 +655,7 @@
         </is>
       </c>
       <c r="B7" s="4" t="n">
-        <v>10</v>
+        <v>11</v>
       </c>
     </row>
     <row r="8">
@@ -688,7 +685,7 @@
         </is>
       </c>
       <c r="B10" s="6" t="n">
-        <v>54</v>
+        <v>58</v>
       </c>
     </row>
     <row r="11">
@@ -698,7 +695,7 @@
         </is>
       </c>
       <c r="B11" s="8" t="n">
-        <v>52</v>
+        <v>56</v>
       </c>
     </row>
     <row r="13">
@@ -708,7 +705,7 @@
         </is>
       </c>
       <c r="B13" s="9" t="n">
-        <v>6</v>
+        <v>9</v>
       </c>
     </row>
   </sheetData>
@@ -725,7 +722,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:J19"/>
+  <dimension ref="A1:J21"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="28" customWidth="1" min="1" max="1"/>
@@ -832,12 +829,12 @@
       </c>
       <c r="G3" s="13" t="inlineStr">
         <is>
-          <t>R$ 22,5M aporte</t>
+          <t>R$ 22,5M (Astella+BB)</t>
         </is>
       </c>
       <c r="H3" s="13" t="inlineStr">
         <is>
-          <t>Maior aporte da história das GovTechs da AL. 120+ cidades. TOP Open Startups 2024.</t>
+          <t>Aporte Seed de R$22,5M (US$4M) liderado por Astella e VOX Capital (CVC do Banco do Brasil), com CAF e Endeavor. 120+ cidades. TOP Open Startups 2024. Maior aporte da história das GovTechs da AL.</t>
         </is>
       </c>
       <c r="I3" s="13" t="inlineStr"/>
@@ -1582,6 +1579,110 @@
         </is>
       </c>
       <c r="J19" s="18" t="inlineStr">
+        <is>
+          <t>✓</t>
+        </is>
+      </c>
+    </row>
+    <row r="20" ht="48" customHeight="1">
+      <c r="A20" s="14" t="inlineStr">
+        <is>
+          <t>Colab</t>
+        </is>
+      </c>
+      <c r="B20" s="15" t="inlineStr">
+        <is>
+          <t>Participação Cidadã / Gestão Pública</t>
+        </is>
+      </c>
+      <c r="C20" s="15" t="inlineStr">
+        <is>
+          <t>Scale-up</t>
+        </is>
+      </c>
+      <c r="D20" s="15" t="inlineStr">
+        <is>
+          <t>Brasil</t>
+        </is>
+      </c>
+      <c r="E20" s="15" t="inlineStr">
+        <is>
+          <t>2013</t>
+        </is>
+      </c>
+      <c r="F20" s="15" t="inlineStr">
+        <is>
+          <t>20M+ pessoas impactadas</t>
+        </is>
+      </c>
+      <c r="G20" s="15" t="inlineStr">
+        <is>
+          <t>R$3-7M (Fundo GovTech)</t>
+        </is>
+      </c>
+      <c r="H20" s="15" t="inlineStr">
+        <is>
+          <t>Plataforma de gestão pública e participação cidadã: zeladoria urbana, CRM prefeitura-cidadão e marketplace de serviços públicos digitais. 1º investimento da KPTL em 2014. Follow-on pelo Fundo GovTech (KPTL+Cedro) em 2023. Co-invest EDP.</t>
+        </is>
+      </c>
+      <c r="I20" s="16" t="inlineStr">
+        <is>
+          <t>Portfólio KPTL+Cedro</t>
+        </is>
+      </c>
+      <c r="J20" s="19" t="inlineStr">
+        <is>
+          <t>✓</t>
+        </is>
+      </c>
+    </row>
+    <row r="21" ht="48" customHeight="1">
+      <c r="A21" s="12" t="inlineStr">
+        <is>
+          <t>Fractal</t>
+        </is>
+      </c>
+      <c r="B21" s="13" t="inlineStr">
+        <is>
+          <t>Gestão Hídrica / Infraestrutura</t>
+        </is>
+      </c>
+      <c r="C21" s="13" t="inlineStr">
+        <is>
+          <t>Startup / Scale-up</t>
+        </is>
+      </c>
+      <c r="D21" s="13" t="inlineStr">
+        <is>
+          <t>Brasil</t>
+        </is>
+      </c>
+      <c r="E21" s="13" t="inlineStr">
+        <is>
+          <t>2010</t>
+        </is>
+      </c>
+      <c r="F21" s="13" t="inlineStr">
+        <is>
+          <t>Setor elétrico + agro</t>
+        </is>
+      </c>
+      <c r="G21" s="13" t="inlineStr">
+        <is>
+          <t>N/D (KPTL 2019)</t>
+        </is>
+      </c>
+      <c r="H21" s="13" t="inlineStr">
+        <is>
+          <t>SaaS hidrológico integrado: previsão de fluxo de água e gestão de bacias hidrográficas. 80 anos de dados históricos. Clientes: CPFL, Statkraft. Aplicações em energia, agronegócio e seguros. Investimento KPTL 2019 (pré-Fundo GovTech).</t>
+        </is>
+      </c>
+      <c r="I21" s="17" t="inlineStr">
+        <is>
+          <t>Portfólio KPTL</t>
+        </is>
+      </c>
+      <c r="J21" s="18" t="inlineStr">
         <is>
           <t>✓</t>
         </is>
@@ -2061,7 +2162,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:J9"/>
+  <dimension ref="A1:J10"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="28" customWidth="1" min="1" max="1"/>
@@ -2451,6 +2552,58 @@
       </c>
       <c r="J9" s="13" t="inlineStr"/>
     </row>
+    <row r="10" ht="48" customHeight="1">
+      <c r="A10" s="14" t="inlineStr">
+        <is>
+          <t>Jovens Gênios</t>
+        </is>
+      </c>
+      <c r="B10" s="15" t="inlineStr">
+        <is>
+          <t>EdTech Gamificada / IA Educacional</t>
+        </is>
+      </c>
+      <c r="C10" s="15" t="inlineStr">
+        <is>
+          <t>Startup</t>
+        </is>
+      </c>
+      <c r="D10" s="15" t="inlineStr">
+        <is>
+          <t>Rio de Janeiro - RJ</t>
+        </is>
+      </c>
+      <c r="E10" s="15" t="inlineStr">
+        <is>
+          <t>N/D</t>
+        </is>
+      </c>
+      <c r="F10" s="15" t="inlineStr">
+        <is>
+          <t>50+ municípios | est. SP</t>
+        </is>
+      </c>
+      <c r="G10" s="15" t="inlineStr">
+        <is>
+          <t>R$11,8M (Fundo GovTech)</t>
+        </is>
+      </c>
+      <c r="H10" s="15" t="inlineStr">
+        <is>
+          <t>Plataforma adaptativa de aprendizagem e avaliação gamificada. 90% dos alunos em escolas públicas. 83% dos usuários em rede pública. Meta: 10M alunos até 2030. Rodada seed R$11,8M liderada pelo Fundo GovTech (KPTL+Cedro) com DOMO.VC, Criabiz Ventures e Rosey Ventures (Grupo Marista). Mar/2026.</t>
+        </is>
+      </c>
+      <c r="I10" s="16" t="inlineStr">
+        <is>
+          <t>Portfólio KPTL+Cedro</t>
+        </is>
+      </c>
+      <c r="J10" s="19" t="inlineStr">
+        <is>
+          <t>✓</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <mergeCells count="1">
     <mergeCell ref="A1:J1"/>
@@ -2465,7 +2618,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:J12"/>
+  <dimension ref="A1:J13"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="28" customWidth="1" min="1" max="1"/>
@@ -3002,6 +3155,58 @@
         </is>
       </c>
       <c r="J12" s="19" t="inlineStr">
+        <is>
+          <t>✓</t>
+        </is>
+      </c>
+    </row>
+    <row r="13" ht="48" customHeight="1">
+      <c r="A13" s="12" t="inlineStr">
+        <is>
+          <t>Kinebot</t>
+        </is>
+      </c>
+      <c r="B13" s="13" t="inlineStr">
+        <is>
+          <t>IA Ergonomia / Saúde do Trabalhador</t>
+        </is>
+      </c>
+      <c r="C13" s="13" t="inlineStr">
+        <is>
+          <t>Startup</t>
+        </is>
+      </c>
+      <c r="D13" s="13" t="inlineStr">
+        <is>
+          <t>Curitiba - PR</t>
+        </is>
+      </c>
+      <c r="E13" s="13" t="inlineStr">
+        <is>
+          <t>N/D</t>
+        </is>
+      </c>
+      <c r="F13" s="13" t="inlineStr">
+        <is>
+          <t>Indústria + gov</t>
+        </is>
+      </c>
+      <c r="G13" s="13" t="inlineStr">
+        <is>
+          <t>R$3M (Fundo GovTech)</t>
+        </is>
+      </c>
+      <c r="H13" s="13" t="inlineStr">
+        <is>
+          <t>IA para análises ergonômicas e psicossociais via visão computacional. Clientes: Marfrig, P&amp;G, Electrolux. 8º investimento do Fundo GovTech (KPTL+Cedro), R$3M em fev/2026. Foco em saúde do trabalhador para setor público e privado. Expansão global planejada.</t>
+        </is>
+      </c>
+      <c r="I13" s="17" t="inlineStr">
+        <is>
+          <t>Portfólio KPTL+Cedro</t>
+        </is>
+      </c>
+      <c r="J13" s="18" t="inlineStr">
         <is>
           <t>✓</t>
         </is>
@@ -3753,7 +3958,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:F8"/>
+  <dimension ref="A1:F11"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="32" customWidth="1" min="1" max="1"/>
@@ -3838,49 +4043,49 @@
     <row r="4" ht="48" customHeight="1">
       <c r="A4" s="27" t="inlineStr">
         <is>
-          <t>Portabilis — Yunus Negócios Sociais</t>
+          <t>Aprova Digital — Astella + BB/VOX</t>
         </is>
       </c>
       <c r="B4" s="28" t="inlineStr">
         <is>
-          <t>Aporte de impacto</t>
+          <t>Aporte Seed</t>
         </is>
       </c>
       <c r="C4" s="28" t="inlineStr">
         <is>
-          <t>Até R$ 2M</t>
+          <t>R$ 22,5M</t>
         </is>
       </c>
       <c r="D4" s="28" t="inlineStr">
         <is>
-          <t>2023</t>
+          <t>2022</t>
         </is>
       </c>
       <c r="E4" s="28" t="inlineStr">
         <is>
-          <t>Educação Pública</t>
+          <t>Gestão Pública Municipal</t>
         </is>
       </c>
       <c r="F4" s="28" t="inlineStr">
         <is>
-          <t>R$800k já desembolsados. Valida modelo de negócio social. Meta: 1,5M alunos até 2027.</t>
+          <t>Rodada liderada por Astella e VOX Capital (CVC do Banco do Brasil), com CAF e Endeavor. Maior aporte da história das GovTechs da América Latina na época. 120+ cidades, 21M de brasileiros impactados.</t>
         </is>
       </c>
     </row>
     <row r="5" ht="48" customHeight="1">
       <c r="A5" s="12" t="inlineStr">
         <is>
-          <t>ImpulsoGov — Mulago Foundation</t>
+          <t>Portabilis — Yunus Negócios Sociais</t>
         </is>
       </c>
       <c r="B5" s="13" t="inlineStr">
         <is>
-          <t>Aporte seed</t>
+          <t>Aporte de impacto</t>
         </is>
       </c>
       <c r="C5" s="13" t="inlineStr">
         <is>
-          <t>US$ 100k</t>
+          <t>Até R$ 2M</t>
         </is>
       </c>
       <c r="D5" s="13" t="inlineStr">
@@ -3890,61 +4095,61 @@
       </c>
       <c r="E5" s="13" t="inlineStr">
         <is>
-          <t>Saúde — Analytics / APS</t>
+          <t>Educação Pública</t>
         </is>
       </c>
       <c r="F5" s="13" t="inlineStr">
         <is>
-          <t>Capital de impacto para BI de atenção básica preventiva. Cofundada por ex-Harvard Kennedy School.</t>
+          <t>R$800k já desembolsados. Valida modelo de negócio social. Meta: 1,5M alunos até 2027.</t>
         </is>
       </c>
     </row>
     <row r="6" ht="48" customHeight="1">
       <c r="A6" s="27" t="inlineStr">
         <is>
-          <t>GovTools — Ventiur + DOMO.VC</t>
+          <t>ImpulsoGov — Mulago Foundation</t>
         </is>
       </c>
       <c r="B6" s="28" t="inlineStr">
         <is>
-          <t>Aporte early-stage</t>
+          <t>Aporte seed</t>
         </is>
       </c>
       <c r="C6" s="28" t="inlineStr">
         <is>
-          <t>N/D</t>
+          <t>US$ 100k</t>
         </is>
       </c>
       <c r="D6" s="28" t="inlineStr">
         <is>
-          <t>2024</t>
+          <t>2023</t>
         </is>
       </c>
       <c r="E6" s="28" t="inlineStr">
         <is>
-          <t>IA Operacional Gov</t>
+          <t>Saúde — Analytics / APS</t>
         </is>
       </c>
       <c r="F6" s="28" t="inlineStr">
         <is>
-          <t>200+ municípios em menos de 12 meses. Modelo viral via WhatsApp. Potencial alvo de aquisição.</t>
+          <t>Capital de impacto para BI de atenção básica preventiva. Cofundada por ex-Harvard Kennedy School.</t>
         </is>
       </c>
     </row>
     <row r="7" ht="48" customHeight="1">
       <c r="A7" s="12" t="inlineStr">
         <is>
-          <t>i4Sea — Fundo GovTech KPTL</t>
+          <t>GovTools — Ventiur + DOMO.VC</t>
         </is>
       </c>
       <c r="B7" s="13" t="inlineStr">
         <is>
-          <t>Aporte</t>
+          <t>Aporte early-stage</t>
         </is>
       </c>
       <c r="C7" s="13" t="inlineStr">
         <is>
-          <t>R$ 7,5M</t>
+          <t>N/D</t>
         </is>
       </c>
       <c r="D7" s="13" t="inlineStr">
@@ -3954,44 +4159,140 @@
       </c>
       <c r="E7" s="13" t="inlineStr">
         <is>
-          <t>Infraestrutura / Clima</t>
+          <t>IA Operacional Gov</t>
         </is>
       </c>
       <c r="F7" s="13" t="inlineStr">
         <is>
-          <t>Previsões microclimáticas para portos e setor elétrico. Portfólio Fundo GovTech KPTL.</t>
+          <t>200+ municípios em menos de 12 meses. Modelo viral via WhatsApp. Potencial alvo de aquisição.</t>
         </is>
       </c>
     </row>
     <row r="8" ht="48" customHeight="1">
       <c r="A8" s="27" t="inlineStr">
         <is>
+          <t>i4Sea — Fundo GovTech KPTL</t>
+        </is>
+      </c>
+      <c r="B8" s="28" t="inlineStr">
+        <is>
+          <t>Aporte</t>
+        </is>
+      </c>
+      <c r="C8" s="28" t="inlineStr">
+        <is>
+          <t>R$ 7,5M</t>
+        </is>
+      </c>
+      <c r="D8" s="28" t="inlineStr">
+        <is>
+          <t>2024</t>
+        </is>
+      </c>
+      <c r="E8" s="28" t="inlineStr">
+        <is>
+          <t>Infraestrutura / Clima</t>
+        </is>
+      </c>
+      <c r="F8" s="28" t="inlineStr">
+        <is>
+          <t>Previsões microclimáticas para portos e setor elétrico. Portfólio Fundo GovTech KPTL.</t>
+        </is>
+      </c>
+    </row>
+    <row r="9" ht="48" customHeight="1">
+      <c r="A9" s="12" t="inlineStr">
+        <is>
           <t>Augen — Biosolvit (exit)</t>
         </is>
       </c>
-      <c r="B8" s="29" t="inlineStr">
+      <c r="B9" s="17" t="inlineStr">
         <is>
           <t>Exit estratégico</t>
         </is>
       </c>
-      <c r="C8" s="28" t="inlineStr">
+      <c r="C9" s="13" t="inlineStr">
         <is>
           <t>R$ 36–48M</t>
         </is>
       </c>
-      <c r="D8" s="28" t="inlineStr">
+      <c r="D9" s="13" t="inlineStr">
         <is>
           <t>out/2024</t>
         </is>
       </c>
-      <c r="E8" s="28" t="inlineStr">
+      <c r="E9" s="13" t="inlineStr">
         <is>
           <t>Infraestrutura / Água</t>
         </is>
       </c>
-      <c r="F8" s="28" t="inlineStr">
+      <c r="F9" s="13" t="inlineStr">
         <is>
           <t>1º exit do Fundo GovTech KPTL. Automação de tratamento de água. Earn-out 3 anos. Comprador: Biosolvit (Laércio Cosentino). Badesul apoiou.</t>
+        </is>
+      </c>
+    </row>
+    <row r="10" ht="48" customHeight="1">
+      <c r="A10" s="27" t="inlineStr">
+        <is>
+          <t>Kinebot — Fundo GovTech (KPTL+Cedro)</t>
+        </is>
+      </c>
+      <c r="B10" s="28" t="inlineStr">
+        <is>
+          <t>Aporte</t>
+        </is>
+      </c>
+      <c r="C10" s="28" t="inlineStr">
+        <is>
+          <t>R$ 3M</t>
+        </is>
+      </c>
+      <c r="D10" s="28" t="inlineStr">
+        <is>
+          <t>fev/2026</t>
+        </is>
+      </c>
+      <c r="E10" s="28" t="inlineStr">
+        <is>
+          <t>IA Ergonomia / Saúde Gov</t>
+        </is>
+      </c>
+      <c r="F10" s="28" t="inlineStr">
+        <is>
+          <t>8º investimento do Fundo GovTech. IA para análises ergonômicas e psicossociais. Clientes: Marfrig, P&amp;G, Electrolux. Expansão global planejada para 2026.</t>
+        </is>
+      </c>
+    </row>
+    <row r="11" ht="48" customHeight="1">
+      <c r="A11" s="12" t="inlineStr">
+        <is>
+          <t>Jovens Gênios — Fundo GovTech+DOMO</t>
+        </is>
+      </c>
+      <c r="B11" s="13" t="inlineStr">
+        <is>
+          <t>Aporte Seed</t>
+        </is>
+      </c>
+      <c r="C11" s="13" t="inlineStr">
+        <is>
+          <t>R$ 11,8M</t>
+        </is>
+      </c>
+      <c r="D11" s="13" t="inlineStr">
+        <is>
+          <t>mar/2026</t>
+        </is>
+      </c>
+      <c r="E11" s="13" t="inlineStr">
+        <is>
+          <t>Educação Pública</t>
+        </is>
+      </c>
+      <c r="F11" s="13" t="inlineStr">
+        <is>
+          <t>Rodada seed liderada pelo Fundo GovTech (KPTL+Cedro), com DOMO.VC, Criabiz Ventures e Rosey Ventures (Grupo Marista). 90% dos alunos em escolas públicas. Meta: 10M alunos até 2030.</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
v9: M&A Volaris/Softplan adicionados; changelog simplificado
- 5 aquisições adicionadas à lista de investimentos:
  Equiplano, GOVBR, IDS, Nydus Systems (Volaris Group) e 1Doc (Softplan)
- Changelog do usuário simplificado: mantidos apenas os 2 últimos meses (v9 + v8)
- Versão atualizada para v9

Co-Authored-By: Claude Sonnet 4.6 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/Radar_GovTechs_Brasil_2026.xlsx
+++ b/Radar_GovTechs_Brasil_2026.xlsx
@@ -14,7 +14,10 @@
     <sheet name="🤖 IA para Governo" sheetId="5" state="visible" r:id="rId5"/>
     <sheet name="⚖️ Procuradorias (PGM-PGE-MP" sheetId="6" state="visible" r:id="rId6"/>
     <sheet name="📋 Licitações &amp; Compras Públ" sheetId="7" state="visible" r:id="rId7"/>
-    <sheet name="💰 Aportes &amp; Investimentos" sheetId="8" state="visible" r:id="rId8"/>
+    <sheet name="🏘️ Habitação &amp; Regularização" sheetId="8" state="visible" r:id="rId8"/>
+    <sheet name="🌿 Meio Ambiente &amp; Licenciam" sheetId="9" state="visible" r:id="rId9"/>
+    <sheet name="🏙️ Smart Cities &amp; Mobilidade" sheetId="10" state="visible" r:id="rId10"/>
+    <sheet name="💰 Aportes &amp; Investimentos" sheetId="11" state="visible" r:id="rId11"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
@@ -58,7 +61,7 @@
       <color rgb="001A7A72"/>
     </font>
   </fonts>
-  <fills count="13">
+  <fills count="16">
     <fill>
       <patternFill/>
     </fill>
@@ -112,6 +115,21 @@
     </fill>
     <fill>
       <patternFill patternType="solid">
+        <fgColor rgb="004E342E"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="001B5E20"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="00283593"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
         <fgColor rgb="00E65100"/>
       </patternFill>
     </fill>
@@ -147,7 +165,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="29">
+  <cellXfs count="32">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center"/>
@@ -218,13 +236,22 @@
     <xf numFmtId="0" fontId="4" fillId="11" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="2" fillId="11" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="0" fontId="4" fillId="12" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="13" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="14" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="14" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center"/>
     </xf>
-    <xf numFmtId="0" fontId="3" fillId="12" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="0" fontId="3" fillId="15" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment vertical="top" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="12" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="0" fontId="0" fillId="15" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment vertical="top" wrapText="1"/>
     </xf>
   </cellXfs>
@@ -592,7 +619,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:B13"/>
+  <dimension ref="A1:B16"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="32" customWidth="1" min="1" max="1"/>
@@ -602,7 +629,7 @@
     <row r="1" ht="32" customHeight="1">
       <c r="A1" s="1" t="inlineStr">
         <is>
-          <t>🇧🇷 Radar GovTech Brasil 2025/2026 — DLG · Maio 2026 · v7</t>
+          <t>🇧🇷 Radar GovTech Brasil 2025/2026 — DLG · Maio 2026 · v9</t>
         </is>
       </c>
     </row>
@@ -625,7 +652,7 @@
         </is>
       </c>
       <c r="B4" s="4" t="n">
-        <v>19</v>
+        <v>20</v>
       </c>
     </row>
     <row r="5">
@@ -655,7 +682,7 @@
         </is>
       </c>
       <c r="B7" s="4" t="n">
-        <v>11</v>
+        <v>12</v>
       </c>
     </row>
     <row r="8">
@@ -679,38 +706,772 @@
       </c>
     </row>
     <row r="10">
-      <c r="A10" s="5" t="inlineStr">
+      <c r="A10" s="3" t="inlineStr">
+        <is>
+          <t>🏘️ Habitação &amp; Regularização Fundiária</t>
+        </is>
+      </c>
+      <c r="B10" s="4" t="n">
+        <v>4</v>
+      </c>
+    </row>
+    <row r="11">
+      <c r="A11" s="3" t="inlineStr">
+        <is>
+          <t>🌿 Meio Ambiente &amp; Licenciamento</t>
+        </is>
+      </c>
+      <c r="B11" s="4" t="n">
+        <v>3</v>
+      </c>
+    </row>
+    <row r="12">
+      <c r="A12" s="3" t="inlineStr">
+        <is>
+          <t>🏙️ Smart Cities &amp; Mobilidade</t>
+        </is>
+      </c>
+      <c r="B12" s="4" t="n">
+        <v>2</v>
+      </c>
+    </row>
+    <row r="13">
+      <c r="A13" s="5" t="inlineStr">
         <is>
           <t>TOTAL (incluindo aparições em múltiplos segs)</t>
         </is>
       </c>
-      <c r="B10" s="6" t="n">
-        <v>58</v>
-      </c>
-    </row>
-    <row r="11">
-      <c r="A11" s="7" t="inlineStr">
+      <c r="B13" s="6" t="n">
+        <v>69</v>
+      </c>
+    </row>
+    <row r="14">
+      <c r="A14" s="7" t="inlineStr">
         <is>
           <t>Empresas únicas mapeadas</t>
         </is>
       </c>
-      <c r="B11" s="8" t="n">
-        <v>56</v>
-      </c>
-    </row>
-    <row r="13">
-      <c r="A13" t="inlineStr">
+      <c r="B14" s="8" t="n">
+        <v>67</v>
+      </c>
+    </row>
+    <row r="16">
+      <c r="A16" t="inlineStr">
         <is>
           <t>Aportes &amp; Investimentos registrados</t>
         </is>
       </c>
-      <c r="B13" s="9" t="n">
-        <v>9</v>
+      <c r="B16" s="9" t="n">
+        <v>14</v>
       </c>
     </row>
   </sheetData>
   <mergeCells count="1">
     <mergeCell ref="A1:B1"/>
+  </mergeCells>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet10.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="A1:J4"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <cols>
+    <col width="28" customWidth="1" min="1" max="1"/>
+    <col width="32" customWidth="1" min="2" max="2"/>
+    <col width="20" customWidth="1" min="3" max="3"/>
+    <col width="24" customWidth="1" min="4" max="4"/>
+    <col width="10" customWidth="1" min="5" max="5"/>
+    <col width="28" customWidth="1" min="6" max="6"/>
+    <col width="20" customWidth="1" min="7" max="7"/>
+    <col width="60" customWidth="1" min="8" max="8"/>
+    <col width="28" customWidth="1" min="9" max="9"/>
+    <col width="6" customWidth="1" min="10" max="10"/>
+  </cols>
+  <sheetData>
+    <row r="1" ht="28" customHeight="1">
+      <c r="A1" s="27" t="inlineStr">
+        <is>
+          <t>🏙️ Smart Cities &amp; Mobilidade — Radar GovTech Brasil 2025/2026</t>
+        </is>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" s="11" t="inlineStr">
+        <is>
+          <t>Nome</t>
+        </is>
+      </c>
+      <c r="B2" s="11" t="inlineStr">
+        <is>
+          <t>Subsegmento</t>
+        </is>
+      </c>
+      <c r="C2" s="11" t="inlineStr">
+        <is>
+          <t>Porte</t>
+        </is>
+      </c>
+      <c r="D2" s="11" t="inlineStr">
+        <is>
+          <t>Localização</t>
+        </is>
+      </c>
+      <c r="E2" s="11" t="inlineStr">
+        <is>
+          <t>Fundação</t>
+        </is>
+      </c>
+      <c r="F2" s="11" t="inlineStr">
+        <is>
+          <t>Presença</t>
+        </is>
+      </c>
+      <c r="G2" s="11" t="inlineStr">
+        <is>
+          <t>Capital / Receita</t>
+        </is>
+      </c>
+      <c r="H2" s="11" t="inlineStr">
+        <is>
+          <t>Análise / Nota</t>
+        </is>
+      </c>
+      <c r="I2" s="11" t="inlineStr">
+        <is>
+          <t>Alerta M&amp;A</t>
+        </is>
+      </c>
+      <c r="J2" s="11" t="inlineStr">
+        <is>
+          <t>Novo</t>
+        </is>
+      </c>
+    </row>
+    <row r="3" ht="48" customHeight="1">
+      <c r="A3" s="12" t="inlineStr">
+        <is>
+          <t>SmartCityTec</t>
+        </is>
+      </c>
+      <c r="B3" s="13" t="inlineStr">
+        <is>
+          <t>Plataforma FIWARE / Interoperabilidade Municipal</t>
+        </is>
+      </c>
+      <c r="C3" s="13" t="inlineStr">
+        <is>
+          <t>Startup</t>
+        </is>
+      </c>
+      <c r="D3" s="13" t="inlineStr">
+        <is>
+          <t>Santa Catarina</t>
+        </is>
+      </c>
+      <c r="E3" s="13" t="inlineStr">
+        <is>
+          <t>~2022</t>
+        </is>
+      </c>
+      <c r="F3" s="13" t="inlineStr">
+        <is>
+          <t>Smart Mafra + Amurel Conectada (18 mun.)</t>
+        </is>
+      </c>
+      <c r="G3" s="13" t="inlineStr">
+        <is>
+          <t>N/D</t>
+        </is>
+      </c>
+      <c r="H3" s="13" t="inlineStr">
+        <is>
+          <t>Plataforma open-source baseada em FIWARE para cidades inteligentes: data spaces, IoT, mobilidade, segurança e clima. Smart Mafra: 1ª cidade BR com lei municipal baseada em FIWARE (centraliza tributação, alvarás e serviços públicos). Amurel Conectada: integra 18 municípios da Região de Laguna/SC. SC aprovou Lei 19.494 adotando FIWARE como padrão estadual. Prêmio GovTech Summit 2025. Smart City Expo Barcelona 2025.</t>
+        </is>
+      </c>
+      <c r="I3" s="17" t="inlineStr">
+        <is>
+          <t>Watch — padrão FIWARE em SC</t>
+        </is>
+      </c>
+      <c r="J3" s="18" t="inlineStr">
+        <is>
+          <t>✓</t>
+        </is>
+      </c>
+    </row>
+    <row r="4" ht="48" customHeight="1">
+      <c r="A4" s="14" t="inlineStr">
+        <is>
+          <t>Iguata</t>
+        </is>
+      </c>
+      <c r="B4" s="15" t="inlineStr">
+        <is>
+          <t>IA para Mobilidade Urbana / Transporte Público</t>
+        </is>
+      </c>
+      <c r="C4" s="15" t="inlineStr">
+        <is>
+          <t>Startup early-stage</t>
+        </is>
+      </c>
+      <c r="D4" s="15" t="inlineStr">
+        <is>
+          <t>Porto Alegre - RS</t>
+        </is>
+      </c>
+      <c r="E4" s="15" t="inlineStr">
+        <is>
+          <t>N/D</t>
+        </is>
+      </c>
+      <c r="F4" s="15" t="inlineStr">
+        <is>
+          <t>N/D (early-stage)</t>
+        </is>
+      </c>
+      <c r="G4" s="15" t="inlineStr">
+        <is>
+          <t>N/D</t>
+        </is>
+      </c>
+      <c r="H4" s="15" t="inlineStr">
+        <is>
+          <t>Plataforma de IA para otimização de redes de transporte público: roteirização dinâmica, previsão de demanda, priorização semafórica e inteligência geoespacial. Resultados declarados: -14% no tempo de viagem (ônibus+IA), -18% custo logístico, +21% satisfação em eventos. Arquitetura modular com API aberta. Early-stage — contratos públicos não confirmados.</t>
+        </is>
+      </c>
+      <c r="I4" s="16" t="inlineStr">
+        <is>
+          <t>Watch — mobilidade pública IA</t>
+        </is>
+      </c>
+      <c r="J4" s="19" t="inlineStr">
+        <is>
+          <t>✓</t>
+        </is>
+      </c>
+    </row>
+  </sheetData>
+  <mergeCells count="1">
+    <mergeCell ref="A1:J1"/>
+  </mergeCells>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet11.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="A1:F16"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <cols>
+    <col width="32" customWidth="1" min="1" max="1"/>
+    <col width="20" customWidth="1" min="2" max="2"/>
+    <col width="14" customWidth="1" min="3" max="3"/>
+    <col width="12" customWidth="1" min="4" max="4"/>
+    <col width="24" customWidth="1" min="5" max="5"/>
+    <col width="60" customWidth="1" min="6" max="6"/>
+  </cols>
+  <sheetData>
+    <row r="1" ht="28" customHeight="1">
+      <c r="A1" s="28" t="inlineStr">
+        <is>
+          <t>💰 Aportes &amp; Investimentos — Radar GovTech Brasil 2025/2026</t>
+        </is>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" s="29" t="inlineStr">
+        <is>
+          <t>Empresa / Investidor</t>
+        </is>
+      </c>
+      <c r="B2" s="29" t="inlineStr">
+        <is>
+          <t>Tipo</t>
+        </is>
+      </c>
+      <c r="C2" s="29" t="inlineStr">
+        <is>
+          <t>Valor</t>
+        </is>
+      </c>
+      <c r="D2" s="29" t="inlineStr">
+        <is>
+          <t>Data</t>
+        </is>
+      </c>
+      <c r="E2" s="29" t="inlineStr">
+        <is>
+          <t>Segmento</t>
+        </is>
+      </c>
+      <c r="F2" s="29" t="inlineStr">
+        <is>
+          <t>Descrição</t>
+        </is>
+      </c>
+    </row>
+    <row r="3" ht="48" customHeight="1">
+      <c r="A3" s="12" t="inlineStr">
+        <is>
+          <t>Gove — Astella</t>
+        </is>
+      </c>
+      <c r="B3" s="13" t="inlineStr">
+        <is>
+          <t>Aporte Series A</t>
+        </is>
+      </c>
+      <c r="C3" s="13" t="inlineStr">
+        <is>
+          <t>R$ 8M</t>
+        </is>
+      </c>
+      <c r="D3" s="13" t="inlineStr">
+        <is>
+          <t>2020</t>
+        </is>
+      </c>
+      <c r="E3" s="13" t="inlineStr">
+        <is>
+          <t>IA Analytics Financeiro</t>
+        </is>
+      </c>
+      <c r="F3" s="13" t="inlineStr">
+        <is>
+          <t>Maior aporte em govtech na época. Plataforma analytics financeiro para prefeituras. Expansão geográfica em curso.</t>
+        </is>
+      </c>
+    </row>
+    <row r="4" ht="48" customHeight="1">
+      <c r="A4" s="30" t="inlineStr">
+        <is>
+          <t>Aprova Digital — Astella + BB/VOX</t>
+        </is>
+      </c>
+      <c r="B4" s="31" t="inlineStr">
+        <is>
+          <t>Aporte Seed</t>
+        </is>
+      </c>
+      <c r="C4" s="31" t="inlineStr">
+        <is>
+          <t>R$ 22,5M</t>
+        </is>
+      </c>
+      <c r="D4" s="31" t="inlineStr">
+        <is>
+          <t>2022</t>
+        </is>
+      </c>
+      <c r="E4" s="31" t="inlineStr">
+        <is>
+          <t>Gestão Pública Municipal</t>
+        </is>
+      </c>
+      <c r="F4" s="31" t="inlineStr">
+        <is>
+          <t>Rodada liderada por Astella e VOX Capital (CVC do Banco do Brasil), com CAF e Endeavor. Maior aporte da história das GovTechs da América Latina na época. 120+ cidades, 21M de brasileiros impactados.</t>
+        </is>
+      </c>
+    </row>
+    <row r="5" ht="48" customHeight="1">
+      <c r="A5" s="12" t="inlineStr">
+        <is>
+          <t>Equiplano — Volaris Group (Constellation Software)</t>
+        </is>
+      </c>
+      <c r="B5" s="13" t="inlineStr">
+        <is>
+          <t>Aquisição (M&amp;A)</t>
+        </is>
+      </c>
+      <c r="C5" s="13" t="inlineStr">
+        <is>
+          <t>N/D</t>
+        </is>
+      </c>
+      <c r="D5" s="13" t="inlineStr">
+        <is>
+          <t>nov/2022</t>
+        </is>
+      </c>
+      <c r="E5" s="13" t="inlineStr">
+        <is>
+          <t>Gestão Pública Municipal</t>
+        </is>
+      </c>
+      <c r="F5" s="13" t="inlineStr">
+        <is>
+          <t>Volaris adquire a Equiplano, ERP municipal líder no Paraná (≈1/3 do mercado estadual). Fundada em 1974, módulos: contabilidade pública, tributos, RH, compras, frotas. 70 funcionários. Opera de forma independente dentro do portfólio Volaris Latam &amp; Ibéria.</t>
+        </is>
+      </c>
+    </row>
+    <row r="6" ht="48" customHeight="1">
+      <c r="A6" s="30" t="inlineStr">
+        <is>
+          <t>Portabilis — Yunus Negócios Sociais</t>
+        </is>
+      </c>
+      <c r="B6" s="31" t="inlineStr">
+        <is>
+          <t>Aporte de impacto</t>
+        </is>
+      </c>
+      <c r="C6" s="31" t="inlineStr">
+        <is>
+          <t>Até R$ 2M</t>
+        </is>
+      </c>
+      <c r="D6" s="31" t="inlineStr">
+        <is>
+          <t>2023</t>
+        </is>
+      </c>
+      <c r="E6" s="31" t="inlineStr">
+        <is>
+          <t>Educação Pública</t>
+        </is>
+      </c>
+      <c r="F6" s="31" t="inlineStr">
+        <is>
+          <t>R$800k já desembolsados. Valida modelo de negócio social. Meta: 1,5M alunos até 2027.</t>
+        </is>
+      </c>
+    </row>
+    <row r="7" ht="48" customHeight="1">
+      <c r="A7" s="12" t="inlineStr">
+        <is>
+          <t>ImpulsoGov — Mulago Foundation</t>
+        </is>
+      </c>
+      <c r="B7" s="13" t="inlineStr">
+        <is>
+          <t>Aporte seed</t>
+        </is>
+      </c>
+      <c r="C7" s="13" t="inlineStr">
+        <is>
+          <t>US$ 100k</t>
+        </is>
+      </c>
+      <c r="D7" s="13" t="inlineStr">
+        <is>
+          <t>2023</t>
+        </is>
+      </c>
+      <c r="E7" s="13" t="inlineStr">
+        <is>
+          <t>Saúde — Analytics / APS</t>
+        </is>
+      </c>
+      <c r="F7" s="13" t="inlineStr">
+        <is>
+          <t>Capital de impacto para BI de atenção básica preventiva. Cofundada por ex-Harvard Kennedy School.</t>
+        </is>
+      </c>
+    </row>
+    <row r="8" ht="48" customHeight="1">
+      <c r="A8" s="30" t="inlineStr">
+        <is>
+          <t>GOVBR — Volaris Group (Constellation Software)</t>
+        </is>
+      </c>
+      <c r="B8" s="31" t="inlineStr">
+        <is>
+          <t>Aquisição (M&amp;A)</t>
+        </is>
+      </c>
+      <c r="C8" s="31" t="inlineStr">
+        <is>
+          <t>N/D</t>
+        </is>
+      </c>
+      <c r="D8" s="31" t="inlineStr">
+        <is>
+          <t>mai/2023</t>
+        </is>
+      </c>
+      <c r="E8" s="31" t="inlineStr">
+        <is>
+          <t>Gestão Pública Municipal</t>
+        </is>
+      </c>
+      <c r="F8" s="31" t="inlineStr">
+        <is>
+          <t>Volaris adquire a GovernançaBrasil (GOVBR), ERP municipal com 35 anos de atuação. Fundador: Roberto Coelho. Plataforma Cidade 360, 24 módulos. Presença em RS, SC, SP, PR, RJ, ES, MG, MS, PE. Descrita como 'aquisição de grande porte' pela Volaris.</t>
+        </is>
+      </c>
+    </row>
+    <row r="9" ht="48" customHeight="1">
+      <c r="A9" s="12" t="inlineStr">
+        <is>
+          <t>GovTools — Ventiur + DOMO.VC</t>
+        </is>
+      </c>
+      <c r="B9" s="13" t="inlineStr">
+        <is>
+          <t>Aporte early-stage</t>
+        </is>
+      </c>
+      <c r="C9" s="13" t="inlineStr">
+        <is>
+          <t>N/D</t>
+        </is>
+      </c>
+      <c r="D9" s="13" t="inlineStr">
+        <is>
+          <t>2024</t>
+        </is>
+      </c>
+      <c r="E9" s="13" t="inlineStr">
+        <is>
+          <t>IA Operacional Gov</t>
+        </is>
+      </c>
+      <c r="F9" s="13" t="inlineStr">
+        <is>
+          <t>200+ municípios em menos de 12 meses. Modelo viral via WhatsApp. Potencial alvo de aquisição.</t>
+        </is>
+      </c>
+    </row>
+    <row r="10" ht="48" customHeight="1">
+      <c r="A10" s="30" t="inlineStr">
+        <is>
+          <t>i4Sea — Fundo GovTech KPTL</t>
+        </is>
+      </c>
+      <c r="B10" s="31" t="inlineStr">
+        <is>
+          <t>Aporte</t>
+        </is>
+      </c>
+      <c r="C10" s="31" t="inlineStr">
+        <is>
+          <t>R$ 7,5M</t>
+        </is>
+      </c>
+      <c r="D10" s="31" t="inlineStr">
+        <is>
+          <t>2024</t>
+        </is>
+      </c>
+      <c r="E10" s="31" t="inlineStr">
+        <is>
+          <t>Infraestrutura / Clima</t>
+        </is>
+      </c>
+      <c r="F10" s="31" t="inlineStr">
+        <is>
+          <t>Previsões microclimáticas para portos e setor elétrico. Portfólio Fundo GovTech KPTL.</t>
+        </is>
+      </c>
+    </row>
+    <row r="11" ht="48" customHeight="1">
+      <c r="A11" s="12" t="inlineStr">
+        <is>
+          <t>Augen — Biosolvit (exit)</t>
+        </is>
+      </c>
+      <c r="B11" s="17" t="inlineStr">
+        <is>
+          <t>Exit estratégico</t>
+        </is>
+      </c>
+      <c r="C11" s="13" t="inlineStr">
+        <is>
+          <t>R$ 36–48M</t>
+        </is>
+      </c>
+      <c r="D11" s="13" t="inlineStr">
+        <is>
+          <t>out/2024</t>
+        </is>
+      </c>
+      <c r="E11" s="13" t="inlineStr">
+        <is>
+          <t>Infraestrutura / Água</t>
+        </is>
+      </c>
+      <c r="F11" s="13" t="inlineStr">
+        <is>
+          <t>1º exit do Fundo GovTech KPTL. Automação de tratamento de água. Earn-out 3 anos. Comprador: Biosolvit (Laércio Cosentino). Badesul apoiou.</t>
+        </is>
+      </c>
+    </row>
+    <row r="12" ht="48" customHeight="1">
+      <c r="A12" s="30" t="inlineStr">
+        <is>
+          <t>IDS — Volaris Group (Constellation Software)</t>
+        </is>
+      </c>
+      <c r="B12" s="31" t="inlineStr">
+        <is>
+          <t>Aquisição (M&amp;A)</t>
+        </is>
+      </c>
+      <c r="C12" s="31" t="inlineStr">
+        <is>
+          <t>N/D</t>
+        </is>
+      </c>
+      <c r="D12" s="31" t="inlineStr">
+        <is>
+          <t>ago/2024</t>
+        </is>
+      </c>
+      <c r="E12" s="31" t="inlineStr">
+        <is>
+          <t>Saúde / Educação / Assistência Social</t>
+        </is>
+      </c>
+      <c r="F12" s="31" t="inlineStr">
+        <is>
+          <t>Volaris adquire a IDS (Pato Branco, PR), fornecedora de software para municípios nas áreas de saúde, assistência social, educação e cidadão. Fundada em 2003, 112 funcionários. CEO: Mauri Dengo. Opera de forma independente dentro do portfólio Volaris Latam &amp; Ibéria.</t>
+        </is>
+      </c>
+    </row>
+    <row r="13" ht="48" customHeight="1">
+      <c r="A13" s="12" t="inlineStr">
+        <is>
+          <t>Nydus Systems — Volaris Group (Constellation Software)</t>
+        </is>
+      </c>
+      <c r="B13" s="13" t="inlineStr">
+        <is>
+          <t>Aquisição (M&amp;A)</t>
+        </is>
+      </c>
+      <c r="C13" s="13" t="inlineStr">
+        <is>
+          <t>N/D</t>
+        </is>
+      </c>
+      <c r="D13" s="13" t="inlineStr">
+        <is>
+          <t>mar/2025</t>
+        </is>
+      </c>
+      <c r="E13" s="13" t="inlineStr">
+        <is>
+          <t>RH / Folha de Pagamento Gov</t>
+        </is>
+      </c>
+      <c r="F13" s="13" t="inlineStr">
+        <is>
+          <t>Volaris adquire a Nydus Systems Informatica (São Paulo), fornecedora de HR/payroll para PMEs no Brasil. CEO: Adalberto Argente. Expansão do portfólio Volaris em RH/folha de pagamento no mercado brasileiro.</t>
+        </is>
+      </c>
+    </row>
+    <row r="14" ht="48" customHeight="1">
+      <c r="A14" s="30" t="inlineStr">
+        <is>
+          <t>1Doc — Softplan (100%)</t>
+        </is>
+      </c>
+      <c r="B14" s="31" t="inlineStr">
+        <is>
+          <t>Aquisição (M&amp;A)</t>
+        </is>
+      </c>
+      <c r="C14" s="31" t="inlineStr">
+        <is>
+          <t>N/D</t>
+        </is>
+      </c>
+      <c r="D14" s="31" t="inlineStr">
+        <is>
+          <t>abr/2025</t>
+        </is>
+      </c>
+      <c r="E14" s="31" t="inlineStr">
+        <is>
+          <t>Digitalização / Gestão Municipal</t>
+        </is>
+      </c>
+      <c r="F14" s="31" t="inlineStr">
+        <is>
+          <t>Softplan adquire 100% da 1Doc, govtech de digitalização de processos e atendimento ao cidadão em prefeituras. Jornada: aporte 2017 → maioria 2019 → 100% abr/2025. CAGR de 75% (2019–2025). Fundada 2014, 1.000 entidades públicas, 22M brasileiros impactados, 141 colaboradores.</t>
+        </is>
+      </c>
+    </row>
+    <row r="15" ht="48" customHeight="1">
+      <c r="A15" s="12" t="inlineStr">
+        <is>
+          <t>Kinebot — Fundo GovTech (KPTL+Cedro)</t>
+        </is>
+      </c>
+      <c r="B15" s="13" t="inlineStr">
+        <is>
+          <t>Aporte</t>
+        </is>
+      </c>
+      <c r="C15" s="13" t="inlineStr">
+        <is>
+          <t>R$ 3M</t>
+        </is>
+      </c>
+      <c r="D15" s="13" t="inlineStr">
+        <is>
+          <t>fev/2026</t>
+        </is>
+      </c>
+      <c r="E15" s="13" t="inlineStr">
+        <is>
+          <t>IA Ergonomia / Saúde Gov</t>
+        </is>
+      </c>
+      <c r="F15" s="13" t="inlineStr">
+        <is>
+          <t>8º investimento do Fundo GovTech. IA para análises ergonômicas e psicossociais. Clientes: Marfrig, P&amp;G, Electrolux. Expansão global planejada para 2026.</t>
+        </is>
+      </c>
+    </row>
+    <row r="16" ht="48" customHeight="1">
+      <c r="A16" s="30" t="inlineStr">
+        <is>
+          <t>Jovens Gênios — Fundo GovTech+DOMO</t>
+        </is>
+      </c>
+      <c r="B16" s="31" t="inlineStr">
+        <is>
+          <t>Aporte Seed</t>
+        </is>
+      </c>
+      <c r="C16" s="31" t="inlineStr">
+        <is>
+          <t>R$ 11,8M</t>
+        </is>
+      </c>
+      <c r="D16" s="31" t="inlineStr">
+        <is>
+          <t>mar/2026</t>
+        </is>
+      </c>
+      <c r="E16" s="31" t="inlineStr">
+        <is>
+          <t>Educação Pública</t>
+        </is>
+      </c>
+      <c r="F16" s="31" t="inlineStr">
+        <is>
+          <t>Rodada seed liderada pelo Fundo GovTech (KPTL+Cedro), com DOMO.VC, Criabiz Ventures e Rosey Ventures (Grupo Marista). 90% dos alunos em escolas públicas. Meta: 10M alunos até 2030.</t>
+        </is>
+      </c>
+    </row>
+  </sheetData>
+  <mergeCells count="1">
+    <mergeCell ref="A1:F1"/>
   </mergeCells>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
@@ -722,7 +1483,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:J21"/>
+  <dimension ref="A1:J22"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="28" customWidth="1" min="1" max="1"/>
@@ -1683,6 +2444,58 @@
         </is>
       </c>
       <c r="J21" s="18" t="inlineStr">
+        <is>
+          <t>✓</t>
+        </is>
+      </c>
+    </row>
+    <row r="22" ht="48" customHeight="1">
+      <c r="A22" s="14" t="inlineStr">
+        <is>
+          <t>PLACE</t>
+        </is>
+      </c>
+      <c r="B22" s="15" t="inlineStr">
+        <is>
+          <t>Planejamento Urbano / GeoInteligência</t>
+        </is>
+      </c>
+      <c r="C22" s="15" t="inlineStr">
+        <is>
+          <t>Startup</t>
+        </is>
+      </c>
+      <c r="D22" s="15" t="inlineStr">
+        <is>
+          <t>Brasil</t>
+        </is>
+      </c>
+      <c r="E22" s="15" t="inlineStr">
+        <is>
+          <t>N/D</t>
+        </is>
+      </c>
+      <c r="F22" s="15" t="inlineStr">
+        <is>
+          <t>Municípios</t>
+        </is>
+      </c>
+      <c r="G22" s="15" t="inlineStr">
+        <is>
+          <t>N/D</t>
+        </is>
+      </c>
+      <c r="H22" s="15" t="inlineStr">
+        <is>
+          <t>Plataforma que integra dados de mercado imobiliário, urbanismo e legislação municipal em interface intuitiva para gestores públicos. Certificada BrazilLAB. Suporte a decisões de planejamento territorial e uso do solo.</t>
+        </is>
+      </c>
+      <c r="I22" s="16" t="inlineStr">
+        <is>
+          <t>Watch — urbanismo digital</t>
+        </is>
+      </c>
+      <c r="J22" s="19" t="inlineStr">
         <is>
           <t>✓</t>
         </is>
@@ -2618,7 +3431,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:J13"/>
+  <dimension ref="A1:J14"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="28" customWidth="1" min="1" max="1"/>
@@ -3111,32 +3924,32 @@
     <row r="12" ht="48" customHeight="1">
       <c r="A12" s="14" t="inlineStr">
         <is>
-          <t>Hub Esfera</t>
+          <t>Inteligov</t>
         </is>
       </c>
       <c r="B12" s="15" t="inlineStr">
         <is>
-          <t>IA Analytics / Gestão</t>
+          <t>Monitoramento Legislativo / Inteligência Regulatória</t>
         </is>
       </c>
       <c r="C12" s="15" t="inlineStr">
         <is>
-          <t>Startup</t>
+          <t>Startup / Scale-up</t>
         </is>
       </c>
       <c r="D12" s="15" t="inlineStr">
         <is>
-          <t>N/D (Brasil)</t>
+          <t>São Paulo - SP</t>
         </is>
       </c>
       <c r="E12" s="15" t="inlineStr">
         <is>
-          <t>N/D</t>
+          <t>2014</t>
         </is>
       </c>
       <c r="F12" s="15" t="inlineStr">
         <is>
-          <t>N/D</t>
+          <t>100+ clientes | 27 estados + 1k+ mun.</t>
         </is>
       </c>
       <c r="G12" s="15" t="inlineStr">
@@ -3146,12 +3959,12 @@
       </c>
       <c r="H12" s="15" t="inlineStr">
         <is>
-          <t>Plataforma IA para gestão municipal: analytics preditivo + preventivo + prescritivo. Integra dados orçamentários, operacionais e sociais para apoio à decisão do gestor público.</t>
+          <t>Pioneira em monitoramento automatizado de dados governamentais (Legislativo, Executivo, Judiciário). 4M+ proposições monitoradas. ~890 fontes de Diários Oficiais. IA com termômetro de aprovação de PLs (&gt;98% acurácia). Única com 100% de cobertura das Assembleias Estaduais. Ranking 100 Open Startups, Mapa GovTech. Cubo Itaú, Inovabra, Distrito.</t>
         </is>
       </c>
       <c r="I12" s="16" t="inlineStr">
         <is>
-          <t>Watch</t>
+          <t>Watch — inteligência regulatória</t>
         </is>
       </c>
       <c r="J12" s="19" t="inlineStr">
@@ -3163,50 +3976,102 @@
     <row r="13" ht="48" customHeight="1">
       <c r="A13" s="12" t="inlineStr">
         <is>
+          <t>Hub Esfera</t>
+        </is>
+      </c>
+      <c r="B13" s="13" t="inlineStr">
+        <is>
+          <t>IA Analytics / Gestão</t>
+        </is>
+      </c>
+      <c r="C13" s="13" t="inlineStr">
+        <is>
+          <t>Startup</t>
+        </is>
+      </c>
+      <c r="D13" s="13" t="inlineStr">
+        <is>
+          <t>N/D (Brasil)</t>
+        </is>
+      </c>
+      <c r="E13" s="13" t="inlineStr">
+        <is>
+          <t>N/D</t>
+        </is>
+      </c>
+      <c r="F13" s="13" t="inlineStr">
+        <is>
+          <t>N/D</t>
+        </is>
+      </c>
+      <c r="G13" s="13" t="inlineStr">
+        <is>
+          <t>N/D</t>
+        </is>
+      </c>
+      <c r="H13" s="13" t="inlineStr">
+        <is>
+          <t>Plataforma IA para gestão municipal: analytics preditivo + preventivo + prescritivo. Integra dados orçamentários, operacionais e sociais para apoio à decisão do gestor público.</t>
+        </is>
+      </c>
+      <c r="I13" s="17" t="inlineStr">
+        <is>
+          <t>Watch</t>
+        </is>
+      </c>
+      <c r="J13" s="18" t="inlineStr">
+        <is>
+          <t>✓</t>
+        </is>
+      </c>
+    </row>
+    <row r="14" ht="48" customHeight="1">
+      <c r="A14" s="14" t="inlineStr">
+        <is>
           <t>Kinebot</t>
         </is>
       </c>
-      <c r="B13" s="13" t="inlineStr">
+      <c r="B14" s="15" t="inlineStr">
         <is>
           <t>IA Ergonomia / Saúde do Trabalhador</t>
         </is>
       </c>
-      <c r="C13" s="13" t="inlineStr">
+      <c r="C14" s="15" t="inlineStr">
         <is>
           <t>Startup</t>
         </is>
       </c>
-      <c r="D13" s="13" t="inlineStr">
+      <c r="D14" s="15" t="inlineStr">
         <is>
           <t>Curitiba - PR</t>
         </is>
       </c>
-      <c r="E13" s="13" t="inlineStr">
-        <is>
-          <t>N/D</t>
-        </is>
-      </c>
-      <c r="F13" s="13" t="inlineStr">
+      <c r="E14" s="15" t="inlineStr">
+        <is>
+          <t>N/D</t>
+        </is>
+      </c>
+      <c r="F14" s="15" t="inlineStr">
         <is>
           <t>Indústria + gov</t>
         </is>
       </c>
-      <c r="G13" s="13" t="inlineStr">
+      <c r="G14" s="15" t="inlineStr">
         <is>
           <t>R$3M (Fundo GovTech)</t>
         </is>
       </c>
-      <c r="H13" s="13" t="inlineStr">
+      <c r="H14" s="15" t="inlineStr">
         <is>
           <t>IA para análises ergonômicas e psicossociais via visão computacional. Clientes: Marfrig, P&amp;G, Electrolux. 8º investimento do Fundo GovTech (KPTL+Cedro), R$3M em fev/2026. Foco em saúde do trabalhador para setor público e privado. Expansão global planejada.</t>
         </is>
       </c>
-      <c r="I13" s="17" t="inlineStr">
+      <c r="I14" s="16" t="inlineStr">
         <is>
           <t>Portfólio KPTL+Cedro</t>
         </is>
       </c>
-      <c r="J13" s="18" t="inlineStr">
+      <c r="J14" s="19" t="inlineStr">
         <is>
           <t>✓</t>
         </is>
@@ -3958,347 +4823,535 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:F11"/>
+  <dimension ref="A1:J6"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
-    <col width="32" customWidth="1" min="1" max="1"/>
-    <col width="20" customWidth="1" min="2" max="2"/>
-    <col width="14" customWidth="1" min="3" max="3"/>
-    <col width="12" customWidth="1" min="4" max="4"/>
-    <col width="24" customWidth="1" min="5" max="5"/>
-    <col width="60" customWidth="1" min="6" max="6"/>
+    <col width="28" customWidth="1" min="1" max="1"/>
+    <col width="32" customWidth="1" min="2" max="2"/>
+    <col width="20" customWidth="1" min="3" max="3"/>
+    <col width="24" customWidth="1" min="4" max="4"/>
+    <col width="10" customWidth="1" min="5" max="5"/>
+    <col width="28" customWidth="1" min="6" max="6"/>
+    <col width="20" customWidth="1" min="7" max="7"/>
+    <col width="60" customWidth="1" min="8" max="8"/>
+    <col width="28" customWidth="1" min="9" max="9"/>
+    <col width="6" customWidth="1" min="10" max="10"/>
   </cols>
   <sheetData>
     <row r="1" ht="28" customHeight="1">
       <c r="A1" s="25" t="inlineStr">
         <is>
-          <t>💰 Aportes &amp; Investimentos — Radar GovTech Brasil 2025/2026</t>
+          <t>🏘️ Habitação &amp; Regularização Fundiária — Radar GovTech Brasil 2025/2026</t>
         </is>
       </c>
     </row>
     <row r="2">
-      <c r="A2" s="26" t="inlineStr">
-        <is>
-          <t>Empresa / Investidor</t>
-        </is>
-      </c>
-      <c r="B2" s="26" t="inlineStr">
-        <is>
-          <t>Tipo</t>
-        </is>
-      </c>
-      <c r="C2" s="26" t="inlineStr">
-        <is>
-          <t>Valor</t>
-        </is>
-      </c>
-      <c r="D2" s="26" t="inlineStr">
-        <is>
-          <t>Data</t>
-        </is>
-      </c>
-      <c r="E2" s="26" t="inlineStr">
-        <is>
-          <t>Segmento</t>
-        </is>
-      </c>
-      <c r="F2" s="26" t="inlineStr">
-        <is>
-          <t>Descrição</t>
+      <c r="A2" s="11" t="inlineStr">
+        <is>
+          <t>Nome</t>
+        </is>
+      </c>
+      <c r="B2" s="11" t="inlineStr">
+        <is>
+          <t>Subsegmento</t>
+        </is>
+      </c>
+      <c r="C2" s="11" t="inlineStr">
+        <is>
+          <t>Porte</t>
+        </is>
+      </c>
+      <c r="D2" s="11" t="inlineStr">
+        <is>
+          <t>Localização</t>
+        </is>
+      </c>
+      <c r="E2" s="11" t="inlineStr">
+        <is>
+          <t>Fundação</t>
+        </is>
+      </c>
+      <c r="F2" s="11" t="inlineStr">
+        <is>
+          <t>Presença</t>
+        </is>
+      </c>
+      <c r="G2" s="11" t="inlineStr">
+        <is>
+          <t>Capital / Receita</t>
+        </is>
+      </c>
+      <c r="H2" s="11" t="inlineStr">
+        <is>
+          <t>Análise / Nota</t>
+        </is>
+      </c>
+      <c r="I2" s="11" t="inlineStr">
+        <is>
+          <t>Alerta M&amp;A</t>
+        </is>
+      </c>
+      <c r="J2" s="11" t="inlineStr">
+        <is>
+          <t>Novo</t>
         </is>
       </c>
     </row>
     <row r="3" ht="48" customHeight="1">
       <c r="A3" s="12" t="inlineStr">
         <is>
-          <t>Gove — Astella</t>
+          <t>ReurBR</t>
         </is>
       </c>
       <c r="B3" s="13" t="inlineStr">
         <is>
-          <t>Aporte Series A</t>
+          <t>SaaS Regularização Fundiária (REURB)</t>
         </is>
       </c>
       <c r="C3" s="13" t="inlineStr">
         <is>
-          <t>R$ 8M</t>
+          <t>Startup</t>
         </is>
       </c>
       <c r="D3" s="13" t="inlineStr">
         <is>
-          <t>2020</t>
+          <t>Brasil (ES, BA, RN)</t>
         </is>
       </c>
       <c r="E3" s="13" t="inlineStr">
         <is>
-          <t>IA Analytics Financeiro</t>
+          <t>N/D</t>
         </is>
       </c>
       <c r="F3" s="13" t="inlineStr">
         <is>
-          <t>Maior aporte em govtech na época. Plataforma analytics financeiro para prefeituras. Expansão geográfica em curso.</t>
+          <t>14 municípios | 17k+ un.</t>
+        </is>
+      </c>
+      <c r="G3" s="13" t="inlineStr">
+        <is>
+          <t>N/D</t>
+        </is>
+      </c>
+      <c r="H3" s="13" t="inlineStr">
+        <is>
+          <t>Plataforma SaaS para regularização fundiária urbana (REURB) de ponta a ponta. App offline para agentes de campo. Emissão automática de CRF, títulos de legitimação e relatórios técnicos. Integração com cartórios. 17k+ unidades habitacionais regularizadas.</t>
+        </is>
+      </c>
+      <c r="I3" s="17" t="inlineStr">
+        <is>
+          <t>Watch — REURB nicho virgem</t>
+        </is>
+      </c>
+      <c r="J3" s="18" t="inlineStr">
+        <is>
+          <t>✓</t>
         </is>
       </c>
     </row>
     <row r="4" ht="48" customHeight="1">
-      <c r="A4" s="27" t="inlineStr">
-        <is>
-          <t>Aprova Digital — Astella + BB/VOX</t>
-        </is>
-      </c>
-      <c r="B4" s="28" t="inlineStr">
-        <is>
-          <t>Aporte Seed</t>
-        </is>
-      </c>
-      <c r="C4" s="28" t="inlineStr">
-        <is>
-          <t>R$ 22,5M</t>
-        </is>
-      </c>
-      <c r="D4" s="28" t="inlineStr">
-        <is>
-          <t>2022</t>
-        </is>
-      </c>
-      <c r="E4" s="28" t="inlineStr">
-        <is>
-          <t>Gestão Pública Municipal</t>
-        </is>
-      </c>
-      <c r="F4" s="28" t="inlineStr">
-        <is>
-          <t>Rodada liderada por Astella e VOX Capital (CVC do Banco do Brasil), com CAF e Endeavor. Maior aporte da história das GovTechs da América Latina na época. 120+ cidades, 21M de brasileiros impactados.</t>
+      <c r="A4" s="14" t="inlineStr">
+        <is>
+          <t>sisHABI</t>
+        </is>
+      </c>
+      <c r="B4" s="15" t="inlineStr">
+        <is>
+          <t>Gestão Habitacional + REURB Municipal</t>
+        </is>
+      </c>
+      <c r="C4" s="15" t="inlineStr">
+        <is>
+          <t>PME</t>
+        </is>
+      </c>
+      <c r="D4" s="15" t="inlineStr">
+        <is>
+          <t>Chapecó - SC</t>
+        </is>
+      </c>
+      <c r="E4" s="15" t="inlineStr">
+        <is>
+          <t>2005</t>
+        </is>
+      </c>
+      <c r="F4" s="15" t="inlineStr">
+        <is>
+          <t>16 estados brasileiros</t>
+        </is>
+      </c>
+      <c r="G4" s="15" t="inlineStr">
+        <is>
+          <t>N/D</t>
+        </is>
+      </c>
+      <c r="H4" s="15" t="inlineStr">
+        <is>
+          <t>Software especialista em habitação de interesse social e regularização fundiária. 18 anos de atuação. Clientes: Governo de Roraima, programas MCMV e Casa Verde Amarela. Gestão de sorteios, hierarquizações e entregas habitacionais para prefeituras.</t>
+        </is>
+      </c>
+      <c r="I4" s="16" t="inlineStr">
+        <is>
+          <t>Target roll-up</t>
+        </is>
+      </c>
+      <c r="J4" s="19" t="inlineStr">
+        <is>
+          <t>✓</t>
         </is>
       </c>
     </row>
     <row r="5" ht="48" customHeight="1">
       <c r="A5" s="12" t="inlineStr">
         <is>
-          <t>Portabilis — Yunus Negócios Sociais</t>
+          <t>CERURB</t>
         </is>
       </c>
       <c r="B5" s="13" t="inlineStr">
         <is>
-          <t>Aporte de impacto</t>
+          <t>REURB Digital com IA</t>
         </is>
       </c>
       <c r="C5" s="13" t="inlineStr">
         <is>
-          <t>Até R$ 2M</t>
+          <t>Startup</t>
         </is>
       </c>
       <c r="D5" s="13" t="inlineStr">
         <is>
-          <t>2023</t>
+          <t>Brasil</t>
         </is>
       </c>
       <c r="E5" s="13" t="inlineStr">
         <is>
-          <t>Educação Pública</t>
+          <t>N/D</t>
         </is>
       </c>
       <c r="F5" s="13" t="inlineStr">
         <is>
-          <t>R$800k já desembolsados. Valida modelo de negócio social. Meta: 1,5M alunos até 2027.</t>
+          <t>Municípios + TJ Piauí</t>
+        </is>
+      </c>
+      <c r="G5" s="13" t="inlineStr">
+        <is>
+          <t>N/D</t>
+        </is>
+      </c>
+      <c r="H5" s="13" t="inlineStr">
+        <is>
+          <t>Plataforma corporativa para REURB: diagnóstico, mapeamento geoespacial, emissão automática de CRF e integração com cartórios. 30k+ matrículas abertas em 12 meses. Contratos com Governo do Piauí (PROURBE) e Tribunal de Justiça.</t>
+        </is>
+      </c>
+      <c r="I5" s="17" t="inlineStr">
+        <is>
+          <t>Watch — tração judicial</t>
+        </is>
+      </c>
+      <c r="J5" s="18" t="inlineStr">
+        <is>
+          <t>✓</t>
         </is>
       </c>
     </row>
     <row r="6" ht="48" customHeight="1">
-      <c r="A6" s="27" t="inlineStr">
-        <is>
-          <t>ImpulsoGov — Mulago Foundation</t>
-        </is>
-      </c>
-      <c r="B6" s="28" t="inlineStr">
-        <is>
-          <t>Aporte seed</t>
-        </is>
-      </c>
-      <c r="C6" s="28" t="inlineStr">
-        <is>
-          <t>US$ 100k</t>
-        </is>
-      </c>
-      <c r="D6" s="28" t="inlineStr">
-        <is>
-          <t>2023</t>
-        </is>
-      </c>
-      <c r="E6" s="28" t="inlineStr">
-        <is>
-          <t>Saúde — Analytics / APS</t>
-        </is>
-      </c>
-      <c r="F6" s="28" t="inlineStr">
-        <is>
-          <t>Capital de impacto para BI de atenção básica preventiva. Cofundada por ex-Harvard Kennedy School.</t>
-        </is>
-      </c>
-    </row>
-    <row r="7" ht="48" customHeight="1">
-      <c r="A7" s="12" t="inlineStr">
-        <is>
-          <t>GovTools — Ventiur + DOMO.VC</t>
-        </is>
-      </c>
-      <c r="B7" s="13" t="inlineStr">
-        <is>
-          <t>Aporte early-stage</t>
-        </is>
-      </c>
-      <c r="C7" s="13" t="inlineStr">
-        <is>
-          <t>N/D</t>
-        </is>
-      </c>
-      <c r="D7" s="13" t="inlineStr">
-        <is>
-          <t>2024</t>
-        </is>
-      </c>
-      <c r="E7" s="13" t="inlineStr">
-        <is>
-          <t>IA Operacional Gov</t>
-        </is>
-      </c>
-      <c r="F7" s="13" t="inlineStr">
-        <is>
-          <t>200+ municípios em menos de 12 meses. Modelo viral via WhatsApp. Potencial alvo de aquisição.</t>
-        </is>
-      </c>
-    </row>
-    <row r="8" ht="48" customHeight="1">
-      <c r="A8" s="27" t="inlineStr">
-        <is>
-          <t>i4Sea — Fundo GovTech KPTL</t>
-        </is>
-      </c>
-      <c r="B8" s="28" t="inlineStr">
-        <is>
-          <t>Aporte</t>
-        </is>
-      </c>
-      <c r="C8" s="28" t="inlineStr">
-        <is>
-          <t>R$ 7,5M</t>
-        </is>
-      </c>
-      <c r="D8" s="28" t="inlineStr">
-        <is>
-          <t>2024</t>
-        </is>
-      </c>
-      <c r="E8" s="28" t="inlineStr">
-        <is>
-          <t>Infraestrutura / Clima</t>
-        </is>
-      </c>
-      <c r="F8" s="28" t="inlineStr">
-        <is>
-          <t>Previsões microclimáticas para portos e setor elétrico. Portfólio Fundo GovTech KPTL.</t>
-        </is>
-      </c>
-    </row>
-    <row r="9" ht="48" customHeight="1">
-      <c r="A9" s="12" t="inlineStr">
-        <is>
-          <t>Augen — Biosolvit (exit)</t>
-        </is>
-      </c>
-      <c r="B9" s="17" t="inlineStr">
-        <is>
-          <t>Exit estratégico</t>
-        </is>
-      </c>
-      <c r="C9" s="13" t="inlineStr">
-        <is>
-          <t>R$ 36–48M</t>
-        </is>
-      </c>
-      <c r="D9" s="13" t="inlineStr">
-        <is>
-          <t>out/2024</t>
-        </is>
-      </c>
-      <c r="E9" s="13" t="inlineStr">
-        <is>
-          <t>Infraestrutura / Água</t>
-        </is>
-      </c>
-      <c r="F9" s="13" t="inlineStr">
-        <is>
-          <t>1º exit do Fundo GovTech KPTL. Automação de tratamento de água. Earn-out 3 anos. Comprador: Biosolvit (Laércio Cosentino). Badesul apoiou.</t>
-        </is>
-      </c>
-    </row>
-    <row r="10" ht="48" customHeight="1">
-      <c r="A10" s="27" t="inlineStr">
-        <is>
-          <t>Kinebot — Fundo GovTech (KPTL+Cedro)</t>
-        </is>
-      </c>
-      <c r="B10" s="28" t="inlineStr">
-        <is>
-          <t>Aporte</t>
-        </is>
-      </c>
-      <c r="C10" s="28" t="inlineStr">
-        <is>
-          <t>R$ 3M</t>
-        </is>
-      </c>
-      <c r="D10" s="28" t="inlineStr">
-        <is>
-          <t>fev/2026</t>
-        </is>
-      </c>
-      <c r="E10" s="28" t="inlineStr">
-        <is>
-          <t>IA Ergonomia / Saúde Gov</t>
-        </is>
-      </c>
-      <c r="F10" s="28" t="inlineStr">
-        <is>
-          <t>8º investimento do Fundo GovTech. IA para análises ergonômicas e psicossociais. Clientes: Marfrig, P&amp;G, Electrolux. Expansão global planejada para 2026.</t>
-        </is>
-      </c>
-    </row>
-    <row r="11" ht="48" customHeight="1">
-      <c r="A11" s="12" t="inlineStr">
-        <is>
-          <t>Jovens Gênios — Fundo GovTech+DOMO</t>
-        </is>
-      </c>
-      <c r="B11" s="13" t="inlineStr">
-        <is>
-          <t>Aporte Seed</t>
-        </is>
-      </c>
-      <c r="C11" s="13" t="inlineStr">
-        <is>
-          <t>R$ 11,8M</t>
-        </is>
-      </c>
-      <c r="D11" s="13" t="inlineStr">
-        <is>
-          <t>mar/2026</t>
-        </is>
-      </c>
-      <c r="E11" s="13" t="inlineStr">
-        <is>
-          <t>Educação Pública</t>
-        </is>
-      </c>
-      <c r="F11" s="13" t="inlineStr">
-        <is>
-          <t>Rodada seed liderada pelo Fundo GovTech (KPTL+Cedro), com DOMO.VC, Criabiz Ventures e Rosey Ventures (Grupo Marista). 90% dos alunos em escolas públicas. Meta: 10M alunos até 2030.</t>
+      <c r="A6" s="14" t="inlineStr">
+        <is>
+          <t>Vivenda</t>
+        </is>
+      </c>
+      <c r="B6" s="15" t="inlineStr">
+        <is>
+          <t>Melhoria Habitacional de Interesse Social</t>
+        </is>
+      </c>
+      <c r="C6" s="15" t="inlineStr">
+        <is>
+          <t>Startup de Impacto</t>
+        </is>
+      </c>
+      <c r="D6" s="15" t="inlineStr">
+        <is>
+          <t>São Paulo - SP</t>
+        </is>
+      </c>
+      <c r="E6" s="15" t="inlineStr">
+        <is>
+          <t>N/D</t>
+        </is>
+      </c>
+      <c r="F6" s="15" t="inlineStr">
+        <is>
+          <t>4.500+ intervenções</t>
+        </is>
+      </c>
+      <c r="G6" s="15" t="inlineStr">
+        <is>
+          <t>N/D</t>
+        </is>
+      </c>
+      <c r="H6" s="15" t="inlineStr">
+        <is>
+          <t>Melhoria habitacional acessível para população de baixa renda. 4.500+ melhorias entregues. Portfólio BrazilLAB. Um dos principais negócios de impacto social do Brasil em habitação.</t>
+        </is>
+      </c>
+      <c r="I6" s="16" t="inlineStr">
+        <is>
+          <t>Impacto social / ESG</t>
+        </is>
+      </c>
+      <c r="J6" s="19" t="inlineStr">
+        <is>
+          <t>✓</t>
         </is>
       </c>
     </row>
   </sheetData>
   <mergeCells count="1">
-    <mergeCell ref="A1:F1"/>
+    <mergeCell ref="A1:J1"/>
+  </mergeCells>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet9.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="A1:J5"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <cols>
+    <col width="28" customWidth="1" min="1" max="1"/>
+    <col width="32" customWidth="1" min="2" max="2"/>
+    <col width="20" customWidth="1" min="3" max="3"/>
+    <col width="24" customWidth="1" min="4" max="4"/>
+    <col width="10" customWidth="1" min="5" max="5"/>
+    <col width="28" customWidth="1" min="6" max="6"/>
+    <col width="20" customWidth="1" min="7" max="7"/>
+    <col width="60" customWidth="1" min="8" max="8"/>
+    <col width="28" customWidth="1" min="9" max="9"/>
+    <col width="6" customWidth="1" min="10" max="10"/>
+  </cols>
+  <sheetData>
+    <row r="1" ht="28" customHeight="1">
+      <c r="A1" s="26" t="inlineStr">
+        <is>
+          <t>🌿 Meio Ambiente &amp; Licenciamento — Radar GovTech Brasil 2025/2026</t>
+        </is>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" s="11" t="inlineStr">
+        <is>
+          <t>Nome</t>
+        </is>
+      </c>
+      <c r="B2" s="11" t="inlineStr">
+        <is>
+          <t>Subsegmento</t>
+        </is>
+      </c>
+      <c r="C2" s="11" t="inlineStr">
+        <is>
+          <t>Porte</t>
+        </is>
+      </c>
+      <c r="D2" s="11" t="inlineStr">
+        <is>
+          <t>Localização</t>
+        </is>
+      </c>
+      <c r="E2" s="11" t="inlineStr">
+        <is>
+          <t>Fundação</t>
+        </is>
+      </c>
+      <c r="F2" s="11" t="inlineStr">
+        <is>
+          <t>Presença</t>
+        </is>
+      </c>
+      <c r="G2" s="11" t="inlineStr">
+        <is>
+          <t>Capital / Receita</t>
+        </is>
+      </c>
+      <c r="H2" s="11" t="inlineStr">
+        <is>
+          <t>Análise / Nota</t>
+        </is>
+      </c>
+      <c r="I2" s="11" t="inlineStr">
+        <is>
+          <t>Alerta M&amp;A</t>
+        </is>
+      </c>
+      <c r="J2" s="11" t="inlineStr">
+        <is>
+          <t>Novo</t>
+        </is>
+      </c>
+    </row>
+    <row r="3" ht="48" customHeight="1">
+      <c r="A3" s="12" t="inlineStr">
+        <is>
+          <t>eGAC</t>
+        </is>
+      </c>
+      <c r="B3" s="13" t="inlineStr">
+        <is>
+          <t>Licenciamento Ambiental Municipal Digital</t>
+        </is>
+      </c>
+      <c r="C3" s="13" t="inlineStr">
+        <is>
+          <t>Startup</t>
+        </is>
+      </c>
+      <c r="D3" s="13" t="inlineStr">
+        <is>
+          <t>Bahia</t>
+        </is>
+      </c>
+      <c r="E3" s="13" t="inlineStr">
+        <is>
+          <t>~2021</t>
+        </is>
+      </c>
+      <c r="F3" s="13" t="inlineStr">
+        <is>
+          <t>Consórcios intermunicipais BA</t>
+        </is>
+      </c>
+      <c r="G3" s="13" t="inlineStr">
+        <is>
+          <t>N/D</t>
+        </is>
+      </c>
+      <c r="H3" s="13" t="inlineStr">
+        <is>
+          <t>SaaS de licenciamento ambiental municipal 100% digital. Integra SINAFLOR, GEOBAHIA, SEMA-BA e CEPRAM. 70% redução de custos declarada, onboarding em 30 dias. Operando via consórcios: CDS Bacia do Paramirim, CONVALE e CONSID Oeste da BA. Conformidade com Resolução CEPRAM 4.327/13.</t>
+        </is>
+      </c>
+      <c r="I3" s="17" t="inlineStr">
+        <is>
+          <t>Watch — lic. ambiental nicho virgem</t>
+        </is>
+      </c>
+      <c r="J3" s="18" t="inlineStr">
+        <is>
+          <t>✓</t>
+        </is>
+      </c>
+    </row>
+    <row r="4" ht="48" customHeight="1">
+      <c r="A4" s="14" t="inlineStr">
+        <is>
+          <t>TUXTU</t>
+        </is>
+      </c>
+      <c r="B4" s="15" t="inlineStr">
+        <is>
+          <t>Licenciamento + Arborização + Crédito de Carbono</t>
+        </is>
+      </c>
+      <c r="C4" s="15" t="inlineStr">
+        <is>
+          <t>Startup</t>
+        </is>
+      </c>
+      <c r="D4" s="15" t="inlineStr">
+        <is>
+          <t>Brasil</t>
+        </is>
+      </c>
+      <c r="E4" s="15" t="inlineStr">
+        <is>
+          <t>~2022</t>
+        </is>
+      </c>
+      <c r="F4" s="15" t="inlineStr">
+        <is>
+          <t>Municípios (via órgãos ambientais)</t>
+        </is>
+      </c>
+      <c r="G4" s="15" t="inlineStr">
+        <is>
+          <t>N/D</t>
+        </is>
+      </c>
+      <c r="H4" s="15" t="inlineStr">
+        <is>
+          <t>3 módulos SaaS para Secretarias de Meio Ambiente: SIBLAM (licenciamento com bio-algoritmo e método Battelle EES — reduz subjetividade do analista), SIGAU (arborização urbana com participação cidadã), SICCA (crédito de carbono). Propõe padronização nacional do licenciamento. CEO: Marcelo Creão. Associada ABES.</t>
+        </is>
+      </c>
+      <c r="I4" s="16" t="inlineStr">
+        <is>
+          <t>Watch — 3 verticais ambientais</t>
+        </is>
+      </c>
+      <c r="J4" s="19" t="inlineStr">
+        <is>
+          <t>✓</t>
+        </is>
+      </c>
+    </row>
+    <row r="5" ht="48" customHeight="1">
+      <c r="A5" s="12" t="inlineStr">
+        <is>
+          <t>Retech Recycle</t>
+        </is>
+      </c>
+      <c r="B5" s="13" t="inlineStr">
+        <is>
+          <t>Gestão de Resíduos Sólidos / Rastreabilidade IoT</t>
+        </is>
+      </c>
+      <c r="C5" s="13" t="inlineStr">
+        <is>
+          <t>Startup early-stage</t>
+        </is>
+      </c>
+      <c r="D5" s="13" t="inlineStr">
+        <is>
+          <t>São José dos Campos - SP</t>
+        </is>
+      </c>
+      <c r="E5" s="13" t="inlineStr">
+        <is>
+          <t>2024</t>
+        </is>
+      </c>
+      <c r="F5" s="13" t="inlineStr">
+        <is>
+          <t>N/D (early-stage)</t>
+        </is>
+      </c>
+      <c r="G5" s="13" t="inlineStr">
+        <is>
+          <t>N/D</t>
+        </is>
+      </c>
+      <c r="H5" s="13" t="inlineStr">
+        <is>
+          <t>Plataforma + hardware IoT proprietário (H-SAT) para rastreabilidade de resíduos sólidos do ponto de coleta ao destino final. Gera documentos auditáveis com fotos georreferenciadas, telemetria e carimbos de tempo. Conformidade PNRS. Modelo híbrido: software + presença onsite. PIT-SJC. Fundada jun/2024.</t>
+        </is>
+      </c>
+      <c r="I5" s="17" t="inlineStr">
+        <is>
+          <t>Watch — PNRS compliance IoT</t>
+        </is>
+      </c>
+      <c r="J5" s="18" t="inlineStr">
+        <is>
+          <t>✓</t>
+        </is>
+      </c>
+    </row>
+  </sheetData>
+  <mergeCells count="1">
+    <mergeCell ref="A1:J1"/>
   </mergeCells>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
v10: reclassificação de segmentos — Gestão e IA divididos
- Novo segmento: Fiscal & Convênios Municipais (Geopixel, Gove, Quasar,
  MuniScore, Qiatech, LICI GovTech, Hub Esfera)
- Novo segmento: Segurança Pública & Infraestrutura (IPQ Tecnologia, Atech,
  Horus, Intelicity, Sipremo, i4Sea, Fractal)
- MinutaIA migrada para Procuradorias & Jurídico
- Gestão passa a 11 empresas (ERP & Suite Municipal)
- IA passa a 6 empresas (horizontal/automação)
- Total: 11 segmentos, 67 empresas

Co-Authored-By: Claude Sonnet 4.6 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/Radar_GovTechs_Brasil_2026.xlsx
+++ b/Radar_GovTechs_Brasil_2026.xlsx
@@ -8,16 +8,18 @@
   </bookViews>
   <sheets>
     <sheet name="Resumo" sheetId="1" state="visible" r:id="rId1"/>
-    <sheet name="🏛️ Gestão Pública Municipal" sheetId="2" state="visible" r:id="rId2"/>
-    <sheet name="🏥 Saúde Pública" sheetId="3" state="visible" r:id="rId3"/>
-    <sheet name="📚 Educação Pública" sheetId="4" state="visible" r:id="rId4"/>
-    <sheet name="🤖 IA para Governo" sheetId="5" state="visible" r:id="rId5"/>
-    <sheet name="⚖️ Procuradorias (PGM-PGE-MP" sheetId="6" state="visible" r:id="rId6"/>
-    <sheet name="📋 Licitações &amp; Compras Públ" sheetId="7" state="visible" r:id="rId7"/>
-    <sheet name="🏘️ Habitação &amp; Regularização" sheetId="8" state="visible" r:id="rId8"/>
-    <sheet name="🌿 Meio Ambiente &amp; Licenciam" sheetId="9" state="visible" r:id="rId9"/>
-    <sheet name="🏙️ Smart Cities &amp; Mobilidade" sheetId="10" state="visible" r:id="rId10"/>
-    <sheet name="💰 Aportes &amp; Investimentos" sheetId="11" state="visible" r:id="rId11"/>
+    <sheet name="🏛️ Gestão &amp; ERP Municipal" sheetId="2" state="visible" r:id="rId2"/>
+    <sheet name="📊 Fiscal &amp; Convênios Munici" sheetId="3" state="visible" r:id="rId3"/>
+    <sheet name="🏥 Saúde Pública" sheetId="4" state="visible" r:id="rId4"/>
+    <sheet name="📚 Educação Pública" sheetId="5" state="visible" r:id="rId5"/>
+    <sheet name="🤖 IA Horizontal &amp; Automação" sheetId="6" state="visible" r:id="rId6"/>
+    <sheet name="⚖️ Procuradorias &amp; Jurídico" sheetId="7" state="visible" r:id="rId7"/>
+    <sheet name="📋 Licitações &amp; Compras Públ" sheetId="8" state="visible" r:id="rId8"/>
+    <sheet name="🏘️ Habitação &amp; Regularização" sheetId="9" state="visible" r:id="rId9"/>
+    <sheet name="🌿 Meio Ambiente &amp; Licenciam" sheetId="10" state="visible" r:id="rId10"/>
+    <sheet name="🏙️ Smart Cities &amp; Mobilidade" sheetId="11" state="visible" r:id="rId11"/>
+    <sheet name="🛡️ Segurança Pública &amp; Infra" sheetId="12" state="visible" r:id="rId12"/>
+    <sheet name="💰 Aportes &amp; Investimentos" sheetId="13" state="visible" r:id="rId13"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
@@ -61,7 +63,7 @@
       <color rgb="001A7A72"/>
     </font>
   </fonts>
-  <fills count="16">
+  <fills count="18">
     <fill>
       <patternFill/>
     </fill>
@@ -91,6 +93,11 @@
     <fill>
       <patternFill patternType="solid">
         <fgColor rgb="00F4F6F9"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="0092400E"/>
       </patternFill>
     </fill>
     <fill>
@@ -130,6 +137,11 @@
     </fill>
     <fill>
       <patternFill patternType="solid">
+        <fgColor rgb="0037474F"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
         <fgColor rgb="00E65100"/>
       </patternFill>
     </fill>
@@ -165,7 +177,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="32">
+  <cellXfs count="34">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center"/>
@@ -221,10 +233,10 @@
     <xf numFmtId="0" fontId="4" fillId="7" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="4" fillId="3" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="0" fontId="4" fillId="8" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="4" fillId="8" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="0" fontId="4" fillId="3" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="4" fillId="9" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
@@ -245,13 +257,19 @@
     <xf numFmtId="0" fontId="4" fillId="14" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="2" fillId="14" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="0" fontId="4" fillId="15" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="16" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="16" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center"/>
     </xf>
-    <xf numFmtId="0" fontId="3" fillId="15" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="0" fontId="3" fillId="17" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment vertical="top" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="15" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="0" fontId="0" fillId="17" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment vertical="top" wrapText="1"/>
     </xf>
   </cellXfs>
@@ -619,7 +637,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:B16"/>
+  <dimension ref="A1:B18"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="32" customWidth="1" min="1" max="1"/>
@@ -629,7 +647,7 @@
     <row r="1" ht="32" customHeight="1">
       <c r="A1" s="1" t="inlineStr">
         <is>
-          <t>🇧🇷 Radar GovTech Brasil 2025/2026 — DLG · Maio 2026 · v9</t>
+          <t>🇧🇷 Radar GovTech Brasil 2025/2026 — DLG · Maio 2026 · v10</t>
         </is>
       </c>
     </row>
@@ -648,27 +666,27 @@
     <row r="4">
       <c r="A4" s="3" t="inlineStr">
         <is>
-          <t>🏛️ Gestão Pública Municipal</t>
+          <t>🏛️ Gestão &amp; ERP Municipal</t>
         </is>
       </c>
       <c r="B4" s="4" t="n">
-        <v>20</v>
+        <v>11</v>
       </c>
     </row>
     <row r="5">
       <c r="A5" s="3" t="inlineStr">
         <is>
-          <t>🏥 Saúde Pública</t>
+          <t>📊 Fiscal &amp; Convênios Municipais</t>
         </is>
       </c>
       <c r="B5" s="4" t="n">
-        <v>8</v>
+        <v>7</v>
       </c>
     </row>
     <row r="6">
       <c r="A6" s="3" t="inlineStr">
         <is>
-          <t>📚 Educação Pública</t>
+          <t>🏥 Saúde Pública</t>
         </is>
       </c>
       <c r="B6" s="4" t="n">
@@ -678,17 +696,17 @@
     <row r="7">
       <c r="A7" s="3" t="inlineStr">
         <is>
-          <t>🤖 IA para Governo</t>
+          <t>📚 Educação Pública</t>
         </is>
       </c>
       <c r="B7" s="4" t="n">
-        <v>12</v>
+        <v>8</v>
       </c>
     </row>
     <row r="8">
       <c r="A8" s="3" t="inlineStr">
         <is>
-          <t>⚖️ Procuradorias (PGM/PGE/MP)</t>
+          <t>🤖 IA Horizontal &amp; Automação</t>
         </is>
       </c>
       <c r="B8" s="4" t="n">
@@ -698,70 +716,90 @@
     <row r="9">
       <c r="A9" s="3" t="inlineStr">
         <is>
-          <t>📋 Licitações &amp; Compras Públicas</t>
+          <t>⚖️ Procuradorias &amp; Jurídico</t>
         </is>
       </c>
       <c r="B9" s="4" t="n">
-        <v>6</v>
+        <v>7</v>
       </c>
     </row>
     <row r="10">
       <c r="A10" s="3" t="inlineStr">
         <is>
-          <t>🏘️ Habitação &amp; Regularização Fundiária</t>
+          <t>📋 Licitações &amp; Compras Públicas</t>
         </is>
       </c>
       <c r="B10" s="4" t="n">
-        <v>4</v>
+        <v>6</v>
       </c>
     </row>
     <row r="11">
       <c r="A11" s="3" t="inlineStr">
         <is>
-          <t>🌿 Meio Ambiente &amp; Licenciamento</t>
+          <t>🏘️ Habitação &amp; Regularização Fundiária</t>
         </is>
       </c>
       <c r="B11" s="4" t="n">
-        <v>3</v>
+        <v>4</v>
       </c>
     </row>
     <row r="12">
       <c r="A12" s="3" t="inlineStr">
         <is>
+          <t>🌿 Meio Ambiente &amp; Licenciamento</t>
+        </is>
+      </c>
+      <c r="B12" s="4" t="n">
+        <v>3</v>
+      </c>
+    </row>
+    <row r="13">
+      <c r="A13" s="3" t="inlineStr">
+        <is>
           <t>🏙️ Smart Cities &amp; Mobilidade</t>
         </is>
       </c>
-      <c r="B12" s="4" t="n">
+      <c r="B13" s="4" t="n">
         <v>2</v>
       </c>
     </row>
-    <row r="13">
-      <c r="A13" s="5" t="inlineStr">
+    <row r="14">
+      <c r="A14" s="3" t="inlineStr">
+        <is>
+          <t>🛡️ Segurança Pública &amp; Infraestrutura</t>
+        </is>
+      </c>
+      <c r="B14" s="4" t="n">
+        <v>7</v>
+      </c>
+    </row>
+    <row r="15">
+      <c r="A15" s="5" t="inlineStr">
         <is>
           <t>TOTAL (incluindo aparições em múltiplos segs)</t>
         </is>
       </c>
-      <c r="B13" s="6" t="n">
+      <c r="B15" s="6" t="n">
         <v>69</v>
       </c>
     </row>
-    <row r="14">
-      <c r="A14" s="7" t="inlineStr">
+    <row r="16">
+      <c r="A16" s="7" t="inlineStr">
         <is>
           <t>Empresas únicas mapeadas</t>
         </is>
       </c>
-      <c r="B14" s="8" t="n">
+      <c r="B16" s="8" t="n">
         <v>67</v>
       </c>
     </row>
-    <row r="16">
-      <c r="A16" t="inlineStr">
+    <row r="18">
+      <c r="A18" t="inlineStr">
         <is>
           <t>Aportes &amp; Investimentos registrados</t>
         </is>
       </c>
-      <c r="B16" s="9" t="n">
+      <c r="B18" s="9" t="n">
         <v>14</v>
       </c>
     </row>
@@ -774,6 +812,250 @@
 </file>
 
 <file path=xl/worksheets/sheet10.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="A1:J5"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <cols>
+    <col width="28" customWidth="1" min="1" max="1"/>
+    <col width="32" customWidth="1" min="2" max="2"/>
+    <col width="20" customWidth="1" min="3" max="3"/>
+    <col width="24" customWidth="1" min="4" max="4"/>
+    <col width="10" customWidth="1" min="5" max="5"/>
+    <col width="28" customWidth="1" min="6" max="6"/>
+    <col width="20" customWidth="1" min="7" max="7"/>
+    <col width="60" customWidth="1" min="8" max="8"/>
+    <col width="28" customWidth="1" min="9" max="9"/>
+    <col width="6" customWidth="1" min="10" max="10"/>
+  </cols>
+  <sheetData>
+    <row r="1" ht="28" customHeight="1">
+      <c r="A1" s="27" t="inlineStr">
+        <is>
+          <t>🌿 Meio Ambiente &amp; Licenciamento — Radar GovTech Brasil 2025/2026</t>
+        </is>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" s="11" t="inlineStr">
+        <is>
+          <t>Nome</t>
+        </is>
+      </c>
+      <c r="B2" s="11" t="inlineStr">
+        <is>
+          <t>Subsegmento</t>
+        </is>
+      </c>
+      <c r="C2" s="11" t="inlineStr">
+        <is>
+          <t>Porte</t>
+        </is>
+      </c>
+      <c r="D2" s="11" t="inlineStr">
+        <is>
+          <t>Localização</t>
+        </is>
+      </c>
+      <c r="E2" s="11" t="inlineStr">
+        <is>
+          <t>Fundação</t>
+        </is>
+      </c>
+      <c r="F2" s="11" t="inlineStr">
+        <is>
+          <t>Presença</t>
+        </is>
+      </c>
+      <c r="G2" s="11" t="inlineStr">
+        <is>
+          <t>Capital / Receita</t>
+        </is>
+      </c>
+      <c r="H2" s="11" t="inlineStr">
+        <is>
+          <t>Análise / Nota</t>
+        </is>
+      </c>
+      <c r="I2" s="11" t="inlineStr">
+        <is>
+          <t>Alerta M&amp;A</t>
+        </is>
+      </c>
+      <c r="J2" s="11" t="inlineStr">
+        <is>
+          <t>Novo</t>
+        </is>
+      </c>
+    </row>
+    <row r="3" ht="48" customHeight="1">
+      <c r="A3" s="12" t="inlineStr">
+        <is>
+          <t>eGAC</t>
+        </is>
+      </c>
+      <c r="B3" s="13" t="inlineStr">
+        <is>
+          <t>Licenciamento Ambiental Municipal Digital</t>
+        </is>
+      </c>
+      <c r="C3" s="13" t="inlineStr">
+        <is>
+          <t>Startup</t>
+        </is>
+      </c>
+      <c r="D3" s="13" t="inlineStr">
+        <is>
+          <t>Bahia</t>
+        </is>
+      </c>
+      <c r="E3" s="13" t="inlineStr">
+        <is>
+          <t>~2021</t>
+        </is>
+      </c>
+      <c r="F3" s="13" t="inlineStr">
+        <is>
+          <t>Consórcios intermunicipais BA</t>
+        </is>
+      </c>
+      <c r="G3" s="13" t="inlineStr">
+        <is>
+          <t>N/D</t>
+        </is>
+      </c>
+      <c r="H3" s="13" t="inlineStr">
+        <is>
+          <t>SaaS de licenciamento ambiental municipal 100% digital. Integra SINAFLOR, GEOBAHIA, SEMA-BA e CEPRAM. 70% redução de custos declarada, onboarding em 30 dias. Operando via consórcios: CDS Bacia do Paramirim, CONVALE e CONSID Oeste da BA. Conformidade com Resolução CEPRAM 4.327/13.</t>
+        </is>
+      </c>
+      <c r="I3" s="17" t="inlineStr">
+        <is>
+          <t>Watch — lic. ambiental nicho virgem</t>
+        </is>
+      </c>
+      <c r="J3" s="18" t="inlineStr">
+        <is>
+          <t>✓</t>
+        </is>
+      </c>
+    </row>
+    <row r="4" ht="48" customHeight="1">
+      <c r="A4" s="14" t="inlineStr">
+        <is>
+          <t>TUXTU</t>
+        </is>
+      </c>
+      <c r="B4" s="15" t="inlineStr">
+        <is>
+          <t>Licenciamento + Arborização + Crédito de Carbono</t>
+        </is>
+      </c>
+      <c r="C4" s="15" t="inlineStr">
+        <is>
+          <t>Startup</t>
+        </is>
+      </c>
+      <c r="D4" s="15" t="inlineStr">
+        <is>
+          <t>Brasil</t>
+        </is>
+      </c>
+      <c r="E4" s="15" t="inlineStr">
+        <is>
+          <t>~2022</t>
+        </is>
+      </c>
+      <c r="F4" s="15" t="inlineStr">
+        <is>
+          <t>Municípios (via órgãos ambientais)</t>
+        </is>
+      </c>
+      <c r="G4" s="15" t="inlineStr">
+        <is>
+          <t>N/D</t>
+        </is>
+      </c>
+      <c r="H4" s="15" t="inlineStr">
+        <is>
+          <t>3 módulos SaaS para Secretarias de Meio Ambiente: SIBLAM (licenciamento com bio-algoritmo e método Battelle EES — reduz subjetividade do analista), SIGAU (arborização urbana com participação cidadã), SICCA (crédito de carbono). Propõe padronização nacional do licenciamento. CEO: Marcelo Creão. Associada ABES.</t>
+        </is>
+      </c>
+      <c r="I4" s="16" t="inlineStr">
+        <is>
+          <t>Watch — 3 verticais ambientais</t>
+        </is>
+      </c>
+      <c r="J4" s="19" t="inlineStr">
+        <is>
+          <t>✓</t>
+        </is>
+      </c>
+    </row>
+    <row r="5" ht="48" customHeight="1">
+      <c r="A5" s="12" t="inlineStr">
+        <is>
+          <t>Retech Recycle</t>
+        </is>
+      </c>
+      <c r="B5" s="13" t="inlineStr">
+        <is>
+          <t>Gestão de Resíduos Sólidos / Rastreabilidade IoT</t>
+        </is>
+      </c>
+      <c r="C5" s="13" t="inlineStr">
+        <is>
+          <t>Startup early-stage</t>
+        </is>
+      </c>
+      <c r="D5" s="13" t="inlineStr">
+        <is>
+          <t>São José dos Campos - SP</t>
+        </is>
+      </c>
+      <c r="E5" s="13" t="inlineStr">
+        <is>
+          <t>2024</t>
+        </is>
+      </c>
+      <c r="F5" s="13" t="inlineStr">
+        <is>
+          <t>N/D (early-stage)</t>
+        </is>
+      </c>
+      <c r="G5" s="13" t="inlineStr">
+        <is>
+          <t>N/D</t>
+        </is>
+      </c>
+      <c r="H5" s="13" t="inlineStr">
+        <is>
+          <t>Plataforma + hardware IoT proprietário (H-SAT) para rastreabilidade de resíduos sólidos do ponto de coleta ao destino final. Gera documentos auditáveis com fotos georreferenciadas, telemetria e carimbos de tempo. Conformidade PNRS. Modelo híbrido: software + presença onsite. PIT-SJC. Fundada jun/2024.</t>
+        </is>
+      </c>
+      <c r="I5" s="17" t="inlineStr">
+        <is>
+          <t>Watch — PNRS compliance IoT</t>
+        </is>
+      </c>
+      <c r="J5" s="18" t="inlineStr">
+        <is>
+          <t>✓</t>
+        </is>
+      </c>
+    </row>
+  </sheetData>
+  <mergeCells count="1">
+    <mergeCell ref="A1:J1"/>
+  </mergeCells>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet11.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <sheetPr>
     <outlinePr summaryBelow="1" summaryRight="1"/>
@@ -795,7 +1077,7 @@
   </cols>
   <sheetData>
     <row r="1" ht="28" customHeight="1">
-      <c r="A1" s="27" t="inlineStr">
+      <c r="A1" s="28" t="inlineStr">
         <is>
           <t>🏙️ Smart Cities &amp; Mobilidade — Radar GovTech Brasil 2025/2026</t>
         </is>
@@ -965,7 +1247,415 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet11.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet12.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="A1:J9"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <cols>
+    <col width="28" customWidth="1" min="1" max="1"/>
+    <col width="32" customWidth="1" min="2" max="2"/>
+    <col width="20" customWidth="1" min="3" max="3"/>
+    <col width="24" customWidth="1" min="4" max="4"/>
+    <col width="10" customWidth="1" min="5" max="5"/>
+    <col width="28" customWidth="1" min="6" max="6"/>
+    <col width="20" customWidth="1" min="7" max="7"/>
+    <col width="60" customWidth="1" min="8" max="8"/>
+    <col width="28" customWidth="1" min="9" max="9"/>
+    <col width="6" customWidth="1" min="10" max="10"/>
+  </cols>
+  <sheetData>
+    <row r="1" ht="28" customHeight="1">
+      <c r="A1" s="29" t="inlineStr">
+        <is>
+          <t>🛡️ Segurança Pública &amp; Infraestrutura — Radar GovTech Brasil 2025/2026</t>
+        </is>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" s="11" t="inlineStr">
+        <is>
+          <t>Nome</t>
+        </is>
+      </c>
+      <c r="B2" s="11" t="inlineStr">
+        <is>
+          <t>Subsegmento</t>
+        </is>
+      </c>
+      <c r="C2" s="11" t="inlineStr">
+        <is>
+          <t>Porte</t>
+        </is>
+      </c>
+      <c r="D2" s="11" t="inlineStr">
+        <is>
+          <t>Localização</t>
+        </is>
+      </c>
+      <c r="E2" s="11" t="inlineStr">
+        <is>
+          <t>Fundação</t>
+        </is>
+      </c>
+      <c r="F2" s="11" t="inlineStr">
+        <is>
+          <t>Presença</t>
+        </is>
+      </c>
+      <c r="G2" s="11" t="inlineStr">
+        <is>
+          <t>Capital / Receita</t>
+        </is>
+      </c>
+      <c r="H2" s="11" t="inlineStr">
+        <is>
+          <t>Análise / Nota</t>
+        </is>
+      </c>
+      <c r="I2" s="11" t="inlineStr">
+        <is>
+          <t>Alerta M&amp;A</t>
+        </is>
+      </c>
+      <c r="J2" s="11" t="inlineStr">
+        <is>
+          <t>Novo</t>
+        </is>
+      </c>
+    </row>
+    <row r="3" ht="48" customHeight="1">
+      <c r="A3" s="12" t="inlineStr">
+        <is>
+          <t>Sipremo</t>
+        </is>
+      </c>
+      <c r="B3" s="13" t="inlineStr">
+        <is>
+          <t>Infraestrutura / Clima</t>
+        </is>
+      </c>
+      <c r="C3" s="13" t="inlineStr">
+        <is>
+          <t>Startup</t>
+        </is>
+      </c>
+      <c r="D3" s="13" t="inlineStr">
+        <is>
+          <t>Ribeirão Preto - SP</t>
+        </is>
+      </c>
+      <c r="E3" s="13" t="inlineStr">
+        <is>
+          <t>~2018</t>
+        </is>
+      </c>
+      <c r="F3" s="13" t="inlineStr">
+        <is>
+          <t>Defesa Civil + seguros</t>
+        </is>
+      </c>
+      <c r="G3" s="13" t="inlineStr">
+        <is>
+          <t>R$200k (2022)</t>
+        </is>
+      </c>
+      <c r="H3" s="13" t="inlineStr">
+        <is>
+          <t>IA para previsão antecipada de desastres naturais. Dados NASA + bases nacionais. Alerta SMS via Defesa Civil. COP26 selecionada.</t>
+        </is>
+      </c>
+      <c r="I3" s="17" t="inlineStr">
+        <is>
+          <t>Watch — clima/risco</t>
+        </is>
+      </c>
+      <c r="J3" s="13" t="inlineStr"/>
+    </row>
+    <row r="4" ht="48" customHeight="1">
+      <c r="A4" s="14" t="inlineStr">
+        <is>
+          <t>i4Sea</t>
+        </is>
+      </c>
+      <c r="B4" s="15" t="inlineStr">
+        <is>
+          <t>Infraestrutura / Clima</t>
+        </is>
+      </c>
+      <c r="C4" s="15" t="inlineStr">
+        <is>
+          <t>Startup</t>
+        </is>
+      </c>
+      <c r="D4" s="15" t="inlineStr">
+        <is>
+          <t>Santos - SP</t>
+        </is>
+      </c>
+      <c r="E4" s="15" t="inlineStr">
+        <is>
+          <t>~2018</t>
+        </is>
+      </c>
+      <c r="F4" s="15" t="inlineStr">
+        <is>
+          <t>N/D</t>
+        </is>
+      </c>
+      <c r="G4" s="15" t="inlineStr">
+        <is>
+          <t>R$ 7,5M aporte</t>
+        </is>
+      </c>
+      <c r="H4" s="15" t="inlineStr">
+        <is>
+          <t>Previsões microclimáticas para portos e setor elétrico. Captou R$7,5M do Fundo GovTech. Resiliência climática.</t>
+        </is>
+      </c>
+      <c r="I4" s="15" t="inlineStr"/>
+      <c r="J4" s="15" t="inlineStr"/>
+    </row>
+    <row r="5" ht="48" customHeight="1">
+      <c r="A5" s="12" t="inlineStr">
+        <is>
+          <t>IPQ Tecnologia</t>
+        </is>
+      </c>
+      <c r="B5" s="13" t="inlineStr">
+        <is>
+          <t>Segurança Pública</t>
+        </is>
+      </c>
+      <c r="C5" s="13" t="inlineStr">
+        <is>
+          <t>PME / Scale-up</t>
+        </is>
+      </c>
+      <c r="D5" s="13" t="inlineStr">
+        <is>
+          <t>Curitiba - PR</t>
+        </is>
+      </c>
+      <c r="E5" s="13" t="inlineStr">
+        <is>
+          <t>~2010</t>
+        </is>
+      </c>
+      <c r="F5" s="13" t="inlineStr">
+        <is>
+          <t>250+ municípios</t>
+        </is>
+      </c>
+      <c r="G5" s="13" t="inlineStr">
+        <is>
+          <t>N/D</t>
+        </is>
+      </c>
+      <c r="H5" s="13" t="inlineStr">
+        <is>
+          <t>Monitoramento e recuperação de veículos. 7.000+ veículos recuperados em 2024. Redução de 15,5% em furtos.</t>
+        </is>
+      </c>
+      <c r="I5" s="13" t="inlineStr"/>
+      <c r="J5" s="13" t="inlineStr"/>
+    </row>
+    <row r="6" ht="48" customHeight="1">
+      <c r="A6" s="14" t="inlineStr">
+        <is>
+          <t>Atech</t>
+        </is>
+      </c>
+      <c r="B6" s="15" t="inlineStr">
+        <is>
+          <t>Segurança Pública / Defesa</t>
+        </is>
+      </c>
+      <c r="C6" s="15" t="inlineStr">
+        <is>
+          <t>Médio Porte</t>
+        </is>
+      </c>
+      <c r="D6" s="15" t="inlineStr">
+        <is>
+          <t>São Paulo - SP</t>
+        </is>
+      </c>
+      <c r="E6" s="15" t="inlineStr">
+        <is>
+          <t>1999</t>
+        </is>
+      </c>
+      <c r="F6" s="15" t="inlineStr">
+        <is>
+          <t>Nacional / Defesa</t>
+        </is>
+      </c>
+      <c r="G6" s="15" t="inlineStr">
+        <is>
+          <t>N/D</t>
+        </is>
+      </c>
+      <c r="H6" s="15" t="inlineStr">
+        <is>
+          <t>Empresa Estratégica de Defesa (MDefesa). Plataformas de Comando &amp; Controle e gestão de crises.</t>
+        </is>
+      </c>
+      <c r="I6" s="15" t="inlineStr"/>
+      <c r="J6" s="15" t="inlineStr"/>
+    </row>
+    <row r="7" ht="48" customHeight="1">
+      <c r="A7" s="12" t="inlineStr">
+        <is>
+          <t>Fractal</t>
+        </is>
+      </c>
+      <c r="B7" s="13" t="inlineStr">
+        <is>
+          <t>Gestão Hídrica / Infraestrutura</t>
+        </is>
+      </c>
+      <c r="C7" s="13" t="inlineStr">
+        <is>
+          <t>Startup / Scale-up</t>
+        </is>
+      </c>
+      <c r="D7" s="13" t="inlineStr">
+        <is>
+          <t>Brasil</t>
+        </is>
+      </c>
+      <c r="E7" s="13" t="inlineStr">
+        <is>
+          <t>2010</t>
+        </is>
+      </c>
+      <c r="F7" s="13" t="inlineStr">
+        <is>
+          <t>Setor elétrico + agro</t>
+        </is>
+      </c>
+      <c r="G7" s="13" t="inlineStr">
+        <is>
+          <t>N/D (KPTL 2019)</t>
+        </is>
+      </c>
+      <c r="H7" s="13" t="inlineStr">
+        <is>
+          <t>SaaS hidrológico integrado: previsão de fluxo de água e gestão de bacias hidrográficas. 80 anos de dados históricos. Clientes: CPFL, Statkraft. Aplicações em energia, agronegócio e seguros. Investimento KPTL 2019 (pré-Fundo GovTech).</t>
+        </is>
+      </c>
+      <c r="I7" s="17" t="inlineStr">
+        <is>
+          <t>Portfólio KPTL</t>
+        </is>
+      </c>
+      <c r="J7" s="18" t="inlineStr">
+        <is>
+          <t>✓</t>
+        </is>
+      </c>
+    </row>
+    <row r="8" ht="48" customHeight="1">
+      <c r="A8" s="14" t="inlineStr">
+        <is>
+          <t>Horus Smart Det.</t>
+        </is>
+      </c>
+      <c r="B8" s="15" t="inlineStr">
+        <is>
+          <t>Fiscalização / Drones / IA</t>
+        </is>
+      </c>
+      <c r="C8" s="15" t="inlineStr">
+        <is>
+          <t>Scale-up</t>
+        </is>
+      </c>
+      <c r="D8" s="15" t="inlineStr">
+        <is>
+          <t>Florianópolis - SC</t>
+        </is>
+      </c>
+      <c r="E8" s="15" t="inlineStr">
+        <is>
+          <t>~2016</t>
+        </is>
+      </c>
+      <c r="F8" s="15" t="inlineStr">
+        <is>
+          <t>100+ gov + privado</t>
+        </is>
+      </c>
+      <c r="G8" s="15" t="inlineStr">
+        <is>
+          <t>N/D</t>
+        </is>
+      </c>
+      <c r="H8" s="15" t="inlineStr">
+        <is>
+          <t>Drones + satélites + visão computacional: obras irregulares, desmatamento, infraestrutura. Cliente: Florianópolis. 9 anos de operação.</t>
+        </is>
+      </c>
+      <c r="I8" s="15" t="inlineStr"/>
+      <c r="J8" s="15" t="inlineStr"/>
+    </row>
+    <row r="9" ht="48" customHeight="1">
+      <c r="A9" s="12" t="inlineStr">
+        <is>
+          <t>Intelicity</t>
+        </is>
+      </c>
+      <c r="B9" s="13" t="inlineStr">
+        <is>
+          <t>IA Infraestrutura Urbana</t>
+        </is>
+      </c>
+      <c r="C9" s="13" t="inlineStr">
+        <is>
+          <t>Startup / Scale-up</t>
+        </is>
+      </c>
+      <c r="D9" s="13" t="inlineStr">
+        <is>
+          <t>São Paulo - SP</t>
+        </is>
+      </c>
+      <c r="E9" s="13" t="inlineStr">
+        <is>
+          <t>~2019</t>
+        </is>
+      </c>
+      <c r="F9" s="13" t="inlineStr">
+        <is>
+          <t>Sabesp + municípios</t>
+        </is>
+      </c>
+      <c r="G9" s="13" t="inlineStr">
+        <is>
+          <t>N/D</t>
+        </is>
+      </c>
+      <c r="H9" s="13" t="inlineStr">
+        <is>
+          <t>Câmeras em veículos + visão computacional: mapeia pavimento, rachaduras. Sabesp: detecção de vazamentos de água.</t>
+        </is>
+      </c>
+      <c r="I9" s="13" t="inlineStr"/>
+      <c r="J9" s="13" t="inlineStr"/>
+    </row>
+  </sheetData>
+  <mergeCells count="1">
+    <mergeCell ref="A1:J1"/>
+  </mergeCells>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet13.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <sheetPr>
     <outlinePr summaryBelow="1" summaryRight="1"/>
@@ -983,39 +1673,39 @@
   </cols>
   <sheetData>
     <row r="1" ht="28" customHeight="1">
-      <c r="A1" s="28" t="inlineStr">
+      <c r="A1" s="30" t="inlineStr">
         <is>
           <t>💰 Aportes &amp; Investimentos — Radar GovTech Brasil 2025/2026</t>
         </is>
       </c>
     </row>
     <row r="2">
-      <c r="A2" s="29" t="inlineStr">
+      <c r="A2" s="31" t="inlineStr">
         <is>
           <t>Empresa / Investidor</t>
         </is>
       </c>
-      <c r="B2" s="29" t="inlineStr">
+      <c r="B2" s="31" t="inlineStr">
         <is>
           <t>Tipo</t>
         </is>
       </c>
-      <c r="C2" s="29" t="inlineStr">
+      <c r="C2" s="31" t="inlineStr">
         <is>
           <t>Valor</t>
         </is>
       </c>
-      <c r="D2" s="29" t="inlineStr">
+      <c r="D2" s="31" t="inlineStr">
         <is>
           <t>Data</t>
         </is>
       </c>
-      <c r="E2" s="29" t="inlineStr">
+      <c r="E2" s="31" t="inlineStr">
         <is>
           <t>Segmento</t>
         </is>
       </c>
-      <c r="F2" s="29" t="inlineStr">
+      <c r="F2" s="31" t="inlineStr">
         <is>
           <t>Descrição</t>
         </is>
@@ -1054,32 +1744,32 @@
       </c>
     </row>
     <row r="4" ht="48" customHeight="1">
-      <c r="A4" s="30" t="inlineStr">
+      <c r="A4" s="32" t="inlineStr">
         <is>
           <t>Aprova Digital — Astella + BB/VOX</t>
         </is>
       </c>
-      <c r="B4" s="31" t="inlineStr">
+      <c r="B4" s="33" t="inlineStr">
         <is>
           <t>Aporte Seed</t>
         </is>
       </c>
-      <c r="C4" s="31" t="inlineStr">
+      <c r="C4" s="33" t="inlineStr">
         <is>
           <t>R$ 22,5M</t>
         </is>
       </c>
-      <c r="D4" s="31" t="inlineStr">
+      <c r="D4" s="33" t="inlineStr">
         <is>
           <t>2022</t>
         </is>
       </c>
-      <c r="E4" s="31" t="inlineStr">
+      <c r="E4" s="33" t="inlineStr">
         <is>
           <t>Gestão Pública Municipal</t>
         </is>
       </c>
-      <c r="F4" s="31" t="inlineStr">
+      <c r="F4" s="33" t="inlineStr">
         <is>
           <t>Rodada liderada por Astella e VOX Capital (CVC do Banco do Brasil), com CAF e Endeavor. Maior aporte da história das GovTechs da América Latina na época. 120+ cidades, 21M de brasileiros impactados.</t>
         </is>
@@ -1118,32 +1808,32 @@
       </c>
     </row>
     <row r="6" ht="48" customHeight="1">
-      <c r="A6" s="30" t="inlineStr">
+      <c r="A6" s="32" t="inlineStr">
         <is>
           <t>Portabilis — Yunus Negócios Sociais</t>
         </is>
       </c>
-      <c r="B6" s="31" t="inlineStr">
+      <c r="B6" s="33" t="inlineStr">
         <is>
           <t>Aporte de impacto</t>
         </is>
       </c>
-      <c r="C6" s="31" t="inlineStr">
+      <c r="C6" s="33" t="inlineStr">
         <is>
           <t>Até R$ 2M</t>
         </is>
       </c>
-      <c r="D6" s="31" t="inlineStr">
+      <c r="D6" s="33" t="inlineStr">
         <is>
           <t>2023</t>
         </is>
       </c>
-      <c r="E6" s="31" t="inlineStr">
+      <c r="E6" s="33" t="inlineStr">
         <is>
           <t>Educação Pública</t>
         </is>
       </c>
-      <c r="F6" s="31" t="inlineStr">
+      <c r="F6" s="33" t="inlineStr">
         <is>
           <t>R$800k já desembolsados. Valida modelo de negócio social. Meta: 1,5M alunos até 2027.</t>
         </is>
@@ -1182,32 +1872,32 @@
       </c>
     </row>
     <row r="8" ht="48" customHeight="1">
-      <c r="A8" s="30" t="inlineStr">
+      <c r="A8" s="32" t="inlineStr">
         <is>
           <t>GOVBR — Volaris Group (Constellation Software)</t>
         </is>
       </c>
-      <c r="B8" s="31" t="inlineStr">
+      <c r="B8" s="33" t="inlineStr">
         <is>
           <t>Aquisição (M&amp;A)</t>
         </is>
       </c>
-      <c r="C8" s="31" t="inlineStr">
-        <is>
-          <t>N/D</t>
-        </is>
-      </c>
-      <c r="D8" s="31" t="inlineStr">
+      <c r="C8" s="33" t="inlineStr">
+        <is>
+          <t>N/D</t>
+        </is>
+      </c>
+      <c r="D8" s="33" t="inlineStr">
         <is>
           <t>mai/2023</t>
         </is>
       </c>
-      <c r="E8" s="31" t="inlineStr">
+      <c r="E8" s="33" t="inlineStr">
         <is>
           <t>Gestão Pública Municipal</t>
         </is>
       </c>
-      <c r="F8" s="31" t="inlineStr">
+      <c r="F8" s="33" t="inlineStr">
         <is>
           <t>Volaris adquire a GovernançaBrasil (GOVBR), ERP municipal com 35 anos de atuação. Fundador: Roberto Coelho. Plataforma Cidade 360, 24 módulos. Presença em RS, SC, SP, PR, RJ, ES, MG, MS, PE. Descrita como 'aquisição de grande porte' pela Volaris.</t>
         </is>
@@ -1246,32 +1936,32 @@
       </c>
     </row>
     <row r="10" ht="48" customHeight="1">
-      <c r="A10" s="30" t="inlineStr">
+      <c r="A10" s="32" t="inlineStr">
         <is>
           <t>i4Sea — Fundo GovTech KPTL</t>
         </is>
       </c>
-      <c r="B10" s="31" t="inlineStr">
+      <c r="B10" s="33" t="inlineStr">
         <is>
           <t>Aporte</t>
         </is>
       </c>
-      <c r="C10" s="31" t="inlineStr">
+      <c r="C10" s="33" t="inlineStr">
         <is>
           <t>R$ 7,5M</t>
         </is>
       </c>
-      <c r="D10" s="31" t="inlineStr">
+      <c r="D10" s="33" t="inlineStr">
         <is>
           <t>2024</t>
         </is>
       </c>
-      <c r="E10" s="31" t="inlineStr">
+      <c r="E10" s="33" t="inlineStr">
         <is>
           <t>Infraestrutura / Clima</t>
         </is>
       </c>
-      <c r="F10" s="31" t="inlineStr">
+      <c r="F10" s="33" t="inlineStr">
         <is>
           <t>Previsões microclimáticas para portos e setor elétrico. Portfólio Fundo GovTech KPTL.</t>
         </is>
@@ -1310,32 +2000,32 @@
       </c>
     </row>
     <row r="12" ht="48" customHeight="1">
-      <c r="A12" s="30" t="inlineStr">
+      <c r="A12" s="32" t="inlineStr">
         <is>
           <t>IDS — Volaris Group (Constellation Software)</t>
         </is>
       </c>
-      <c r="B12" s="31" t="inlineStr">
+      <c r="B12" s="33" t="inlineStr">
         <is>
           <t>Aquisição (M&amp;A)</t>
         </is>
       </c>
-      <c r="C12" s="31" t="inlineStr">
-        <is>
-          <t>N/D</t>
-        </is>
-      </c>
-      <c r="D12" s="31" t="inlineStr">
+      <c r="C12" s="33" t="inlineStr">
+        <is>
+          <t>N/D</t>
+        </is>
+      </c>
+      <c r="D12" s="33" t="inlineStr">
         <is>
           <t>ago/2024</t>
         </is>
       </c>
-      <c r="E12" s="31" t="inlineStr">
+      <c r="E12" s="33" t="inlineStr">
         <is>
           <t>Saúde / Educação / Assistência Social</t>
         </is>
       </c>
-      <c r="F12" s="31" t="inlineStr">
+      <c r="F12" s="33" t="inlineStr">
         <is>
           <t>Volaris adquire a IDS (Pato Branco, PR), fornecedora de software para municípios nas áreas de saúde, assistência social, educação e cidadão. Fundada em 2003, 112 funcionários. CEO: Mauri Dengo. Opera de forma independente dentro do portfólio Volaris Latam &amp; Ibéria.</t>
         </is>
@@ -1374,32 +2064,32 @@
       </c>
     </row>
     <row r="14" ht="48" customHeight="1">
-      <c r="A14" s="30" t="inlineStr">
+      <c r="A14" s="32" t="inlineStr">
         <is>
           <t>1Doc — Softplan (100%)</t>
         </is>
       </c>
-      <c r="B14" s="31" t="inlineStr">
+      <c r="B14" s="33" t="inlineStr">
         <is>
           <t>Aquisição (M&amp;A)</t>
         </is>
       </c>
-      <c r="C14" s="31" t="inlineStr">
-        <is>
-          <t>N/D</t>
-        </is>
-      </c>
-      <c r="D14" s="31" t="inlineStr">
+      <c r="C14" s="33" t="inlineStr">
+        <is>
+          <t>N/D</t>
+        </is>
+      </c>
+      <c r="D14" s="33" t="inlineStr">
         <is>
           <t>abr/2025</t>
         </is>
       </c>
-      <c r="E14" s="31" t="inlineStr">
+      <c r="E14" s="33" t="inlineStr">
         <is>
           <t>Digitalização / Gestão Municipal</t>
         </is>
       </c>
-      <c r="F14" s="31" t="inlineStr">
+      <c r="F14" s="33" t="inlineStr">
         <is>
           <t>Softplan adquire 100% da 1Doc, govtech de digitalização de processos e atendimento ao cidadão em prefeituras. Jornada: aporte 2017 → maioria 2019 → 100% abr/2025. CAGR de 75% (2019–2025). Fundada 2014, 1.000 entidades públicas, 22M brasileiros impactados, 141 colaboradores.</t>
         </is>
@@ -1438,32 +2128,32 @@
       </c>
     </row>
     <row r="16" ht="48" customHeight="1">
-      <c r="A16" s="30" t="inlineStr">
+      <c r="A16" s="32" t="inlineStr">
         <is>
           <t>Jovens Gênios — Fundo GovTech+DOMO</t>
         </is>
       </c>
-      <c r="B16" s="31" t="inlineStr">
+      <c r="B16" s="33" t="inlineStr">
         <is>
           <t>Aporte Seed</t>
         </is>
       </c>
-      <c r="C16" s="31" t="inlineStr">
+      <c r="C16" s="33" t="inlineStr">
         <is>
           <t>R$ 11,8M</t>
         </is>
       </c>
-      <c r="D16" s="31" t="inlineStr">
+      <c r="D16" s="33" t="inlineStr">
         <is>
           <t>mar/2026</t>
         </is>
       </c>
-      <c r="E16" s="31" t="inlineStr">
+      <c r="E16" s="33" t="inlineStr">
         <is>
           <t>Educação Pública</t>
         </is>
       </c>
-      <c r="F16" s="31" t="inlineStr">
+      <c r="F16" s="33" t="inlineStr">
         <is>
           <t>Rodada seed liderada pelo Fundo GovTech (KPTL+Cedro), com DOMO.VC, Criabiz Ventures e Rosey Ventures (Grupo Marista). 90% dos alunos em escolas públicas. Meta: 10M alunos até 2030.</t>
         </is>
@@ -1483,7 +2173,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:J22"/>
+  <dimension ref="A1:J13"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="28" customWidth="1" min="1" max="1"/>
@@ -1501,7 +2191,7 @@
     <row r="1" ht="28" customHeight="1">
       <c r="A1" s="10" t="inlineStr">
         <is>
-          <t>🏛️ Gestão Pública Municipal — Radar GovTech Brasil 2025/2026</t>
+          <t>🏛️ Gestão &amp; ERP Municipal — Radar GovTech Brasil 2025/2026</t>
         </is>
       </c>
     </row>
@@ -1740,32 +2430,32 @@
     <row r="7" ht="48" customHeight="1">
       <c r="A7" s="12" t="inlineStr">
         <is>
-          <t>LICI GovTech</t>
+          <t>GESUAS</t>
         </is>
       </c>
       <c r="B7" s="13" t="inlineStr">
         <is>
-          <t>Smart Cities / Gestão</t>
+          <t>Assistência Social / SUAS</t>
         </is>
       </c>
       <c r="C7" s="13" t="inlineStr">
         <is>
-          <t>Startup</t>
+          <t>Startup / PME</t>
         </is>
       </c>
       <c r="D7" s="13" t="inlineStr">
         <is>
-          <t>Belo Horizonte - MG</t>
+          <t>Viçosa - MG</t>
         </is>
       </c>
       <c r="E7" s="13" t="inlineStr">
         <is>
-          <t>2018</t>
+          <t>~2016</t>
         </is>
       </c>
       <c r="F7" s="13" t="inlineStr">
         <is>
-          <t>Municípios | 2M+ cid.</t>
+          <t>168 mun | 3,5M pessoas</t>
         </is>
       </c>
       <c r="G7" s="13" t="inlineStr">
@@ -1775,21 +2465,25 @@
       </c>
       <c r="H7" s="13" t="inlineStr">
         <is>
-          <t>Plataforma CHESI: 160+ indicadores ODS + fontes de financiamento + governança. Parceria SEDE-MG Cidades do Futuro.</t>
-        </is>
-      </c>
-      <c r="I7" s="13" t="inlineStr"/>
+          <t>Prontuário eletrônico SUAS. 1,2M famílias | 6,5k trabalhadores. Líder IE GovTech 2020. Vertical exclusivo sem concorrente direto.</t>
+        </is>
+      </c>
+      <c r="I7" s="17" t="inlineStr">
+        <is>
+          <t>Vertical exclusivo mapeado</t>
+        </is>
+      </c>
       <c r="J7" s="13" t="inlineStr"/>
     </row>
     <row r="8" ht="48" customHeight="1">
       <c r="A8" s="14" t="inlineStr">
         <is>
-          <t>Quasar</t>
+          <t>Prosas</t>
         </is>
       </c>
       <c r="B8" s="15" t="inlineStr">
         <is>
-          <t>Gestão Municipal / Fiscal</t>
+          <t>Participação Cidadã</t>
         </is>
       </c>
       <c r="C8" s="15" t="inlineStr">
@@ -1799,65 +2493,61 @@
       </c>
       <c r="D8" s="15" t="inlineStr">
         <is>
-          <t>Belo Horizonte - MG</t>
+          <t>São Paulo - SP</t>
         </is>
       </c>
       <c r="E8" s="15" t="inlineStr">
         <is>
-          <t>2019</t>
+          <t>~2016</t>
         </is>
       </c>
       <c r="F8" s="15" t="inlineStr">
         <is>
-          <t>Municípios MG</t>
+          <t>220k+ usuários</t>
         </is>
       </c>
       <c r="G8" s="15" t="inlineStr">
         <is>
-          <t>N/D</t>
+          <t>R$4M (KPTL)</t>
         </is>
       </c>
       <c r="H8" s="15" t="inlineStr">
         <is>
-          <t>Alvarás digitais: reduz 90% do prazo de emissão. 2º DemoDay BrazilLAB 2023. Selecionada PBH Inova (2 desafios).</t>
-        </is>
-      </c>
-      <c r="I8" s="16" t="inlineStr">
-        <is>
-          <t>Watch — fiscal municipal</t>
-        </is>
-      </c>
+          <t>Portfólio Fundo GovTech KPTL. Gestão digital de editais socioculturais e transparência pública.</t>
+        </is>
+      </c>
+      <c r="I8" s="15" t="inlineStr"/>
       <c r="J8" s="15" t="inlineStr"/>
     </row>
     <row r="9" ht="48" customHeight="1">
       <c r="A9" s="12" t="inlineStr">
         <is>
-          <t>GESUAS</t>
+          <t>Lemobs</t>
         </is>
       </c>
       <c r="B9" s="13" t="inlineStr">
         <is>
-          <t>Assistência Social / SUAS</t>
+          <t>Smart Cities / Mobilidade</t>
         </is>
       </c>
       <c r="C9" s="13" t="inlineStr">
         <is>
-          <t>Startup / PME</t>
+          <t>Startup</t>
         </is>
       </c>
       <c r="D9" s="13" t="inlineStr">
         <is>
-          <t>Viçosa - MG</t>
+          <t>Rio de Janeiro - RJ</t>
         </is>
       </c>
       <c r="E9" s="13" t="inlineStr">
         <is>
-          <t>~2016</t>
+          <t>~2015</t>
         </is>
       </c>
       <c r="F9" s="13" t="inlineStr">
         <is>
-          <t>168 mun | 3,5M pessoas</t>
+          <t>N/D</t>
         </is>
       </c>
       <c r="G9" s="13" t="inlineStr">
@@ -1867,25 +2557,21 @@
       </c>
       <c r="H9" s="13" t="inlineStr">
         <is>
-          <t>Prontuário eletrônico SUAS. 1,2M famílias | 6,5k trabalhadores. Líder IE GovTech 2020. Vertical exclusivo sem concorrente direto.</t>
-        </is>
-      </c>
-      <c r="I9" s="17" t="inlineStr">
-        <is>
-          <t>Vertical exclusivo mapeado</t>
-        </is>
-      </c>
+          <t>Origem COPPE/UFRJ. Selo GovTech BrazilLAB. Mobilidade urbana e cidades inteligentes.</t>
+        </is>
+      </c>
+      <c r="I9" s="13" t="inlineStr"/>
       <c r="J9" s="13" t="inlineStr"/>
     </row>
     <row r="10" ht="48" customHeight="1">
       <c r="A10" s="14" t="inlineStr">
         <is>
-          <t>Prosas</t>
+          <t>GRTS Digital</t>
         </is>
       </c>
       <c r="B10" s="15" t="inlineStr">
         <is>
-          <t>Participação Cidadã</t>
+          <t>Relações Trabalhistas</t>
         </is>
       </c>
       <c r="C10" s="15" t="inlineStr">
@@ -1900,22 +2586,22 @@
       </c>
       <c r="E10" s="15" t="inlineStr">
         <is>
-          <t>~2016</t>
+          <t>2019</t>
         </is>
       </c>
       <c r="F10" s="15" t="inlineStr">
         <is>
-          <t>220k+ usuários</t>
+          <t>N/D</t>
         </is>
       </c>
       <c r="G10" s="15" t="inlineStr">
         <is>
-          <t>R$4M (KPTL)</t>
+          <t>R$ 3,4M aporte</t>
         </is>
       </c>
       <c r="H10" s="15" t="inlineStr">
         <is>
-          <t>Portfólio Fundo GovTech KPTL. Gestão digital de editais socioculturais e transparência pública.</t>
+          <t>Digitalização da gestão de relações sindicais. Captou R$3,4M do Fundo GovTech KPTL.</t>
         </is>
       </c>
       <c r="I10" s="15" t="inlineStr"/>
@@ -1924,32 +2610,32 @@
     <row r="11" ht="48" customHeight="1">
       <c r="A11" s="12" t="inlineStr">
         <is>
-          <t>Lemobs</t>
+          <t>Governar</t>
         </is>
       </c>
       <c r="B11" s="13" t="inlineStr">
         <is>
-          <t>Smart Cities / Mobilidade</t>
+          <t>ERP Municipal / SIAFIC</t>
         </is>
       </c>
       <c r="C11" s="13" t="inlineStr">
         <is>
-          <t>Startup</t>
+          <t>Startup / Scale-up</t>
         </is>
       </c>
       <c r="D11" s="13" t="inlineStr">
         <is>
-          <t>Rio de Janeiro - RJ</t>
+          <t>N/D (Brasil)</t>
         </is>
       </c>
       <c r="E11" s="13" t="inlineStr">
         <is>
-          <t>~2015</t>
+          <t>N/D</t>
         </is>
       </c>
       <c r="F11" s="13" t="inlineStr">
         <is>
-          <t>N/D</t>
+          <t>Municípios (SIAFIC)</t>
         </is>
       </c>
       <c r="G11" s="13" t="inlineStr">
@@ -1959,69 +2645,81 @@
       </c>
       <c r="H11" s="13" t="inlineStr">
         <is>
-          <t>Origem COPPE/UFRJ. Selo GovTech BrazilLAB. Mobilidade urbana e cidades inteligentes.</t>
-        </is>
-      </c>
-      <c r="I11" s="13" t="inlineStr"/>
-      <c r="J11" s="13" t="inlineStr"/>
+          <t>ERP municipal integrado 100% cloud: SIAFIC + saúde + educação + assistência social. Conformidade SIAFIC obrigatória impulsiona substituição de legados.</t>
+        </is>
+      </c>
+      <c r="I11" s="17" t="inlineStr">
+        <is>
+          <t>Watch — SIAFIC driver</t>
+        </is>
+      </c>
+      <c r="J11" s="18" t="inlineStr">
+        <is>
+          <t>✓</t>
+        </is>
+      </c>
     </row>
     <row r="12" ht="48" customHeight="1">
       <c r="A12" s="14" t="inlineStr">
         <is>
-          <t>Sipremo</t>
+          <t>Colab</t>
         </is>
       </c>
       <c r="B12" s="15" t="inlineStr">
         <is>
-          <t>Infraestrutura / Clima</t>
+          <t>Participação Cidadã / Gestão Pública</t>
         </is>
       </c>
       <c r="C12" s="15" t="inlineStr">
         <is>
-          <t>Startup</t>
+          <t>Scale-up</t>
         </is>
       </c>
       <c r="D12" s="15" t="inlineStr">
         <is>
-          <t>Ribeirão Preto - SP</t>
+          <t>Brasil</t>
         </is>
       </c>
       <c r="E12" s="15" t="inlineStr">
         <is>
-          <t>~2018</t>
+          <t>2013</t>
         </is>
       </c>
       <c r="F12" s="15" t="inlineStr">
         <is>
-          <t>Defesa Civil + seguros</t>
+          <t>20M+ pessoas impactadas</t>
         </is>
       </c>
       <c r="G12" s="15" t="inlineStr">
         <is>
-          <t>R$200k (2022)</t>
+          <t>R$3-7M (Fundo GovTech)</t>
         </is>
       </c>
       <c r="H12" s="15" t="inlineStr">
         <is>
-          <t>IA para previsão antecipada de desastres naturais. Dados NASA + bases nacionais. Alerta SMS via Defesa Civil. COP26 selecionada.</t>
+          <t>Plataforma de gestão pública e participação cidadã: zeladoria urbana, CRM prefeitura-cidadão e marketplace de serviços públicos digitais. 1º investimento da KPTL em 2014. Follow-on pelo Fundo GovTech (KPTL+Cedro) em 2023. Co-invest EDP.</t>
         </is>
       </c>
       <c r="I12" s="16" t="inlineStr">
         <is>
-          <t>Watch — clima/risco</t>
-        </is>
-      </c>
-      <c r="J12" s="15" t="inlineStr"/>
+          <t>Portfólio KPTL+Cedro</t>
+        </is>
+      </c>
+      <c r="J12" s="19" t="inlineStr">
+        <is>
+          <t>✓</t>
+        </is>
+      </c>
     </row>
     <row r="13" ht="48" customHeight="1">
       <c r="A13" s="12" t="inlineStr">
         <is>
-          <t>i4Sea</t>
+          <t>PLACE</t>
         </is>
       </c>
       <c r="B13" s="13" t="inlineStr">
         <is>
-          <t>Infraestrutura / Clima</t>
+          <t>Planejamento Urbano / GeoInteligência</t>
         </is>
       </c>
       <c r="C13" s="13" t="inlineStr">
@@ -2031,471 +2729,35 @@
       </c>
       <c r="D13" s="13" t="inlineStr">
         <is>
-          <t>Santos - SP</t>
+          <t>Brasil</t>
         </is>
       </c>
       <c r="E13" s="13" t="inlineStr">
         <is>
-          <t>~2018</t>
+          <t>N/D</t>
         </is>
       </c>
       <c r="F13" s="13" t="inlineStr">
         <is>
-          <t>N/D</t>
+          <t>Municípios</t>
         </is>
       </c>
       <c r="G13" s="13" t="inlineStr">
         <is>
-          <t>R$ 7,5M aporte</t>
+          <t>N/D</t>
         </is>
       </c>
       <c r="H13" s="13" t="inlineStr">
         <is>
-          <t>Previsões microclimáticas para portos e setor elétrico. Captou R$7,5M do Fundo GovTech. Resiliência climática.</t>
-        </is>
-      </c>
-      <c r="I13" s="13" t="inlineStr"/>
-      <c r="J13" s="13" t="inlineStr"/>
-    </row>
-    <row r="14" ht="48" customHeight="1">
-      <c r="A14" s="14" t="inlineStr">
-        <is>
-          <t>GRTS Digital</t>
-        </is>
-      </c>
-      <c r="B14" s="15" t="inlineStr">
-        <is>
-          <t>Relações Trabalhistas</t>
-        </is>
-      </c>
-      <c r="C14" s="15" t="inlineStr">
-        <is>
-          <t>Startup</t>
-        </is>
-      </c>
-      <c r="D14" s="15" t="inlineStr">
-        <is>
-          <t>São Paulo - SP</t>
-        </is>
-      </c>
-      <c r="E14" s="15" t="inlineStr">
-        <is>
-          <t>2019</t>
-        </is>
-      </c>
-      <c r="F14" s="15" t="inlineStr">
-        <is>
-          <t>N/D</t>
-        </is>
-      </c>
-      <c r="G14" s="15" t="inlineStr">
-        <is>
-          <t>R$ 3,4M aporte</t>
-        </is>
-      </c>
-      <c r="H14" s="15" t="inlineStr">
-        <is>
-          <t>Digitalização da gestão de relações sindicais. Captou R$3,4M do Fundo GovTech KPTL.</t>
-        </is>
-      </c>
-      <c r="I14" s="15" t="inlineStr"/>
-      <c r="J14" s="15" t="inlineStr"/>
-    </row>
-    <row r="15" ht="48" customHeight="1">
-      <c r="A15" s="12" t="inlineStr">
-        <is>
-          <t>IPQ Tecnologia</t>
-        </is>
-      </c>
-      <c r="B15" s="13" t="inlineStr">
-        <is>
-          <t>Segurança Pública</t>
-        </is>
-      </c>
-      <c r="C15" s="13" t="inlineStr">
-        <is>
-          <t>PME / Scale-up</t>
-        </is>
-      </c>
-      <c r="D15" s="13" t="inlineStr">
-        <is>
-          <t>Curitiba - PR</t>
-        </is>
-      </c>
-      <c r="E15" s="13" t="inlineStr">
-        <is>
-          <t>~2010</t>
-        </is>
-      </c>
-      <c r="F15" s="13" t="inlineStr">
-        <is>
-          <t>250+ municípios</t>
-        </is>
-      </c>
-      <c r="G15" s="13" t="inlineStr">
-        <is>
-          <t>N/D</t>
-        </is>
-      </c>
-      <c r="H15" s="13" t="inlineStr">
-        <is>
-          <t>Monitoramento e recuperação de veículos. 7.000+ veículos recuperados em 2024. Redução de 15,5% em furtos.</t>
-        </is>
-      </c>
-      <c r="I15" s="13" t="inlineStr"/>
-      <c r="J15" s="13" t="inlineStr"/>
-    </row>
-    <row r="16" ht="48" customHeight="1">
-      <c r="A16" s="14" t="inlineStr">
-        <is>
-          <t>Atech</t>
-        </is>
-      </c>
-      <c r="B16" s="15" t="inlineStr">
-        <is>
-          <t>Segurança Pública / Defesa</t>
-        </is>
-      </c>
-      <c r="C16" s="15" t="inlineStr">
-        <is>
-          <t>Médio Porte</t>
-        </is>
-      </c>
-      <c r="D16" s="15" t="inlineStr">
-        <is>
-          <t>São Paulo - SP</t>
-        </is>
-      </c>
-      <c r="E16" s="15" t="inlineStr">
-        <is>
-          <t>1999</t>
-        </is>
-      </c>
-      <c r="F16" s="15" t="inlineStr">
-        <is>
-          <t>Nacional / Defesa</t>
-        </is>
-      </c>
-      <c r="G16" s="15" t="inlineStr">
-        <is>
-          <t>N/D</t>
-        </is>
-      </c>
-      <c r="H16" s="15" t="inlineStr">
-        <is>
-          <t>Empresa Estratégica de Defesa (MDefesa). Plataformas de Comando &amp; Controle e gestão de crises.</t>
-        </is>
-      </c>
-      <c r="I16" s="15" t="inlineStr"/>
-      <c r="J16" s="15" t="inlineStr"/>
-    </row>
-    <row r="17" ht="48" customHeight="1">
-      <c r="A17" s="12" t="inlineStr">
-        <is>
-          <t>Governar</t>
-        </is>
-      </c>
-      <c r="B17" s="13" t="inlineStr">
-        <is>
-          <t>ERP Municipal / SIAFIC</t>
-        </is>
-      </c>
-      <c r="C17" s="13" t="inlineStr">
-        <is>
-          <t>Startup / Scale-up</t>
-        </is>
-      </c>
-      <c r="D17" s="13" t="inlineStr">
-        <is>
-          <t>N/D (Brasil)</t>
-        </is>
-      </c>
-      <c r="E17" s="13" t="inlineStr">
-        <is>
-          <t>N/D</t>
-        </is>
-      </c>
-      <c r="F17" s="13" t="inlineStr">
-        <is>
-          <t>Municípios (SIAFIC)</t>
-        </is>
-      </c>
-      <c r="G17" s="13" t="inlineStr">
-        <is>
-          <t>N/D</t>
-        </is>
-      </c>
-      <c r="H17" s="13" t="inlineStr">
-        <is>
-          <t>ERP municipal integrado 100% cloud: SIAFIC + saúde + educação + assistência social. Conformidade SIAFIC obrigatória impulsiona substituição de legados.</t>
-        </is>
-      </c>
-      <c r="I17" s="17" t="inlineStr">
-        <is>
-          <t>Watch — SIAFIC driver</t>
-        </is>
-      </c>
-      <c r="J17" s="18" t="inlineStr">
-        <is>
-          <t>✓</t>
-        </is>
-      </c>
-    </row>
-    <row r="18" ht="48" customHeight="1">
-      <c r="A18" s="14" t="inlineStr">
-        <is>
-          <t>Qiatech</t>
-        </is>
-      </c>
-      <c r="B18" s="15" t="inlineStr">
-        <is>
-          <t>Convênios / Transferências</t>
-        </is>
-      </c>
-      <c r="C18" s="15" t="inlineStr">
-        <is>
-          <t>Startup</t>
-        </is>
-      </c>
-      <c r="D18" s="15" t="inlineStr">
-        <is>
-          <t>N/D (Brasil)</t>
-        </is>
-      </c>
-      <c r="E18" s="15" t="inlineStr">
-        <is>
-          <t>N/D</t>
-        </is>
-      </c>
-      <c r="F18" s="15" t="inlineStr">
-        <is>
-          <t>Municípios (convênios)</t>
-        </is>
-      </c>
-      <c r="G18" s="15" t="inlineStr">
-        <is>
-          <t>N/D</t>
-        </is>
-      </c>
-      <c r="H18" s="15" t="inlineStr">
-        <is>
-          <t>Gestão de convênios com IA: integra TransfereGov, Simec, SISMOB, FNS. Vertical exclusivo de captação e gestão de transferências federais para municípios.</t>
-        </is>
-      </c>
-      <c r="I18" s="16" t="inlineStr">
-        <is>
-          <t>Watch — convênios nicho virgem</t>
-        </is>
-      </c>
-      <c r="J18" s="19" t="inlineStr">
-        <is>
-          <t>✓</t>
-        </is>
-      </c>
-    </row>
-    <row r="19" ht="48" customHeight="1">
-      <c r="A19" s="12" t="inlineStr">
-        <is>
-          <t>MuniScore</t>
-        </is>
-      </c>
-      <c r="B19" s="13" t="inlineStr">
-        <is>
-          <t>Inteligência Fiscal</t>
-        </is>
-      </c>
-      <c r="C19" s="13" t="inlineStr">
-        <is>
-          <t>Startup</t>
-        </is>
-      </c>
-      <c r="D19" s="13" t="inlineStr">
-        <is>
-          <t>Belo Horizonte - MG</t>
-        </is>
-      </c>
-      <c r="E19" s="13" t="inlineStr">
-        <is>
-          <t>2026</t>
-        </is>
-      </c>
-      <c r="F19" s="13" t="inlineStr">
-        <is>
-          <t>5.570 municípios (dados)</t>
-        </is>
-      </c>
-      <c r="G19" s="13" t="inlineStr">
-        <is>
-          <t>N/D</t>
-        </is>
-      </c>
-      <c r="H19" s="13" t="inlineStr">
-        <is>
-          <t>Score fiscal para todos os 5.570 municípios brasileiros. Fundada 2026. Plataforma B2B/B2G de avaliação de saúde fiscal e creditícia municipal.</t>
-        </is>
-      </c>
-      <c r="I19" s="17" t="inlineStr">
-        <is>
-          <t>Watch — dado fiscal municipal</t>
-        </is>
-      </c>
-      <c r="J19" s="18" t="inlineStr">
-        <is>
-          <t>✓</t>
-        </is>
-      </c>
-    </row>
-    <row r="20" ht="48" customHeight="1">
-      <c r="A20" s="14" t="inlineStr">
-        <is>
-          <t>Colab</t>
-        </is>
-      </c>
-      <c r="B20" s="15" t="inlineStr">
-        <is>
-          <t>Participação Cidadã / Gestão Pública</t>
-        </is>
-      </c>
-      <c r="C20" s="15" t="inlineStr">
-        <is>
-          <t>Scale-up</t>
-        </is>
-      </c>
-      <c r="D20" s="15" t="inlineStr">
-        <is>
-          <t>Brasil</t>
-        </is>
-      </c>
-      <c r="E20" s="15" t="inlineStr">
-        <is>
-          <t>2013</t>
-        </is>
-      </c>
-      <c r="F20" s="15" t="inlineStr">
-        <is>
-          <t>20M+ pessoas impactadas</t>
-        </is>
-      </c>
-      <c r="G20" s="15" t="inlineStr">
-        <is>
-          <t>R$3-7M (Fundo GovTech)</t>
-        </is>
-      </c>
-      <c r="H20" s="15" t="inlineStr">
-        <is>
-          <t>Plataforma de gestão pública e participação cidadã: zeladoria urbana, CRM prefeitura-cidadão e marketplace de serviços públicos digitais. 1º investimento da KPTL em 2014. Follow-on pelo Fundo GovTech (KPTL+Cedro) em 2023. Co-invest EDP.</t>
-        </is>
-      </c>
-      <c r="I20" s="16" t="inlineStr">
-        <is>
-          <t>Portfólio KPTL+Cedro</t>
-        </is>
-      </c>
-      <c r="J20" s="19" t="inlineStr">
-        <is>
-          <t>✓</t>
-        </is>
-      </c>
-    </row>
-    <row r="21" ht="48" customHeight="1">
-      <c r="A21" s="12" t="inlineStr">
-        <is>
-          <t>Fractal</t>
-        </is>
-      </c>
-      <c r="B21" s="13" t="inlineStr">
-        <is>
-          <t>Gestão Hídrica / Infraestrutura</t>
-        </is>
-      </c>
-      <c r="C21" s="13" t="inlineStr">
-        <is>
-          <t>Startup / Scale-up</t>
-        </is>
-      </c>
-      <c r="D21" s="13" t="inlineStr">
-        <is>
-          <t>Brasil</t>
-        </is>
-      </c>
-      <c r="E21" s="13" t="inlineStr">
-        <is>
-          <t>2010</t>
-        </is>
-      </c>
-      <c r="F21" s="13" t="inlineStr">
-        <is>
-          <t>Setor elétrico + agro</t>
-        </is>
-      </c>
-      <c r="G21" s="13" t="inlineStr">
-        <is>
-          <t>N/D (KPTL 2019)</t>
-        </is>
-      </c>
-      <c r="H21" s="13" t="inlineStr">
-        <is>
-          <t>SaaS hidrológico integrado: previsão de fluxo de água e gestão de bacias hidrográficas. 80 anos de dados históricos. Clientes: CPFL, Statkraft. Aplicações em energia, agronegócio e seguros. Investimento KPTL 2019 (pré-Fundo GovTech).</t>
-        </is>
-      </c>
-      <c r="I21" s="17" t="inlineStr">
-        <is>
-          <t>Portfólio KPTL</t>
-        </is>
-      </c>
-      <c r="J21" s="18" t="inlineStr">
-        <is>
-          <t>✓</t>
-        </is>
-      </c>
-    </row>
-    <row r="22" ht="48" customHeight="1">
-      <c r="A22" s="14" t="inlineStr">
-        <is>
-          <t>PLACE</t>
-        </is>
-      </c>
-      <c r="B22" s="15" t="inlineStr">
-        <is>
-          <t>Planejamento Urbano / GeoInteligência</t>
-        </is>
-      </c>
-      <c r="C22" s="15" t="inlineStr">
-        <is>
-          <t>Startup</t>
-        </is>
-      </c>
-      <c r="D22" s="15" t="inlineStr">
-        <is>
-          <t>Brasil</t>
-        </is>
-      </c>
-      <c r="E22" s="15" t="inlineStr">
-        <is>
-          <t>N/D</t>
-        </is>
-      </c>
-      <c r="F22" s="15" t="inlineStr">
-        <is>
-          <t>Municípios</t>
-        </is>
-      </c>
-      <c r="G22" s="15" t="inlineStr">
-        <is>
-          <t>N/D</t>
-        </is>
-      </c>
-      <c r="H22" s="15" t="inlineStr">
-        <is>
           <t>Plataforma que integra dados de mercado imobiliário, urbanismo e legislação municipal em interface intuitiva para gestores públicos. Certificada BrazilLAB. Suporte a decisões de planejamento territorial e uso do solo.</t>
         </is>
       </c>
-      <c r="I22" s="16" t="inlineStr">
+      <c r="I13" s="17" t="inlineStr">
         <is>
           <t>Watch — urbanismo digital</t>
         </is>
       </c>
-      <c r="J22" s="19" t="inlineStr">
+      <c r="J13" s="18" t="inlineStr">
         <is>
           <t>✓</t>
         </is>
@@ -2515,7 +2777,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:J10"/>
+  <dimension ref="A1:J9"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="28" customWidth="1" min="1" max="1"/>
@@ -2533,7 +2795,7 @@
     <row r="1" ht="28" customHeight="1">
       <c r="A1" s="20" t="inlineStr">
         <is>
-          <t>🏥 Saúde Pública — Radar GovTech Brasil 2025/2026</t>
+          <t>📊 Fiscal &amp; Convênios Municipais — Radar GovTech Brasil 2025/2026</t>
         </is>
       </c>
     </row>
@@ -2592,32 +2854,32 @@
     <row r="3" ht="48" customHeight="1">
       <c r="A3" s="12" t="inlineStr">
         <is>
-          <t>OM30</t>
+          <t>LICI GovTech</t>
         </is>
       </c>
       <c r="B3" s="13" t="inlineStr">
         <is>
-          <t>Atenção Primária / Suite</t>
+          <t>Indicadores ODS / Financiamento Municipal</t>
         </is>
       </c>
       <c r="C3" s="13" t="inlineStr">
         <is>
-          <t>PME Estabelecida</t>
+          <t>Startup</t>
         </is>
       </c>
       <c r="D3" s="13" t="inlineStr">
         <is>
-          <t>São Paulo - SP</t>
+          <t>Belo Horizonte - MG</t>
         </is>
       </c>
       <c r="E3" s="13" t="inlineStr">
         <is>
-          <t>~2005</t>
+          <t>2018</t>
         </is>
       </c>
       <c r="F3" s="13" t="inlineStr">
         <is>
-          <t>Municípios SP</t>
+          <t>Municípios | 2M+ cid.</t>
         </is>
       </c>
       <c r="G3" s="13" t="inlineStr">
@@ -2627,45 +2889,41 @@
       </c>
       <c r="H3" s="13" t="inlineStr">
         <is>
-          <t>Suite municipal: Saúde Simples + Educação + DadosGov + Mobilidade + Doc+. 350 colaboradores. Meta: 2x municípios SP até 2030. IA reduz 40% tempo de consultas SUS.</t>
-        </is>
-      </c>
-      <c r="I3" s="17" t="inlineStr">
-        <is>
-          <t>Target roll-up</t>
-        </is>
-      </c>
+          <t>Plataforma CHESI: 160+ indicadores ODS + fontes de financiamento + governança. Parceria SEDE-MG Cidades do Futuro.</t>
+        </is>
+      </c>
+      <c r="I3" s="13" t="inlineStr"/>
       <c r="J3" s="13" t="inlineStr"/>
     </row>
     <row r="4" ht="48" customHeight="1">
       <c r="A4" s="14" t="inlineStr">
         <is>
-          <t>Olostech</t>
+          <t>Quasar</t>
         </is>
       </c>
       <c r="B4" s="15" t="inlineStr">
         <is>
-          <t>Atenção Primária / APS</t>
+          <t>Fiscal / Alvarás Digitais</t>
         </is>
       </c>
       <c r="C4" s="15" t="inlineStr">
         <is>
-          <t>PME Estabelecida</t>
+          <t>Startup</t>
         </is>
       </c>
       <c r="D4" s="15" t="inlineStr">
         <is>
-          <t>Joinville - SC</t>
+          <t>Belo Horizonte - MG</t>
         </is>
       </c>
       <c r="E4" s="15" t="inlineStr">
         <is>
-          <t>1992</t>
+          <t>2019</t>
         </is>
       </c>
       <c r="F4" s="15" t="inlineStr">
         <is>
-          <t>100+ municípios</t>
+          <t>Municípios MG</t>
         </is>
       </c>
       <c r="G4" s="15" t="inlineStr">
@@ -2675,12 +2933,12 @@
       </c>
       <c r="H4" s="15" t="inlineStr">
         <is>
-          <t>Pioneira SaaS cloud em APS (1998). 91% dos clientes melhoraram indicadores Previne Brasil 2023.</t>
+          <t>Alvarás digitais: reduz 90% do prazo de emissão. 2º DemoDay BrazilLAB 2023. Selecionada PBH Inova (2 desafios).</t>
         </is>
       </c>
       <c r="I4" s="16" t="inlineStr">
         <is>
-          <t>Target roll-up</t>
+          <t>Watch — fiscal municipal</t>
         </is>
       </c>
       <c r="J4" s="15" t="inlineStr"/>
@@ -2688,32 +2946,32 @@
     <row r="5" ht="48" customHeight="1">
       <c r="A5" s="12" t="inlineStr">
         <is>
-          <t>Vivver Sistemas</t>
+          <t>Qiatech</t>
         </is>
       </c>
       <c r="B5" s="13" t="inlineStr">
         <is>
-          <t>APS + Educação Municipal</t>
+          <t>Convênios / Transferências Federais</t>
         </is>
       </c>
       <c r="C5" s="13" t="inlineStr">
         <is>
-          <t>PME Estabelecida</t>
+          <t>Startup</t>
         </is>
       </c>
       <c r="D5" s="13" t="inlineStr">
         <is>
-          <t>Belo Horizonte - MG</t>
+          <t>N/D (Brasil)</t>
         </is>
       </c>
       <c r="E5" s="13" t="inlineStr">
         <is>
-          <t>1999</t>
+          <t>N/D</t>
         </is>
       </c>
       <c r="F5" s="13" t="inlineStr">
         <is>
-          <t>Municípios MG + NE</t>
+          <t>Municípios (convênios)</t>
         </is>
       </c>
       <c r="G5" s="13" t="inlineStr">
@@ -2723,45 +2981,49 @@
       </c>
       <c r="H5" s="13" t="inlineStr">
         <is>
-          <t>26 anos de operação. Selos Ouro/Prata Bora Vacinar (mar/2025). Filiais SP e PB. Foco saúde pública + educação municipal integradas.</t>
+          <t>Gestão de convênios com IA: integra TransfereGov, Simec, SISMOB, FNS. Vertical exclusivo de captação e gestão de transferências federais para municípios.</t>
         </is>
       </c>
       <c r="I5" s="17" t="inlineStr">
         <is>
-          <t>Target roll-up</t>
-        </is>
-      </c>
-      <c r="J5" s="13" t="inlineStr"/>
+          <t>Watch — convênios nicho virgem</t>
+        </is>
+      </c>
+      <c r="J5" s="18" t="inlineStr">
+        <is>
+          <t>✓</t>
+        </is>
+      </c>
     </row>
     <row r="6" ht="48" customHeight="1">
       <c r="A6" s="14" t="inlineStr">
         <is>
-          <t>Pública Tecnologia</t>
+          <t>MuniScore</t>
         </is>
       </c>
       <c r="B6" s="15" t="inlineStr">
         <is>
-          <t>Prontuário Eletrônico APS</t>
+          <t>Inteligência Fiscal Municipal</t>
         </is>
       </c>
       <c r="C6" s="15" t="inlineStr">
         <is>
-          <t>PME</t>
+          <t>Startup</t>
         </is>
       </c>
       <c r="D6" s="15" t="inlineStr">
         <is>
-          <t>N/D</t>
+          <t>Belo Horizonte - MG</t>
         </is>
       </c>
       <c r="E6" s="15" t="inlineStr">
         <is>
-          <t>N/D</t>
+          <t>2026</t>
         </is>
       </c>
       <c r="F6" s="15" t="inlineStr">
         <is>
-          <t>Municípios</t>
+          <t>5.570 municípios (dados)</t>
         </is>
       </c>
       <c r="G6" s="15" t="inlineStr">
@@ -2771,70 +3033,82 @@
       </c>
       <c r="H6" s="15" t="inlineStr">
         <is>
-          <t>Prontuário eletrônico certificado SBIS/CFM. Assinatura ICP-Brasil. Integração e-SUS.</t>
-        </is>
-      </c>
-      <c r="I6" s="15" t="inlineStr"/>
-      <c r="J6" s="15" t="inlineStr"/>
+          <t>Score fiscal para todos os 5.570 municípios brasileiros. Fundada 2026. Plataforma B2B/B2G de avaliação de saúde fiscal e creditícia municipal.</t>
+        </is>
+      </c>
+      <c r="I6" s="16" t="inlineStr">
+        <is>
+          <t>Watch — dado fiscal municipal</t>
+        </is>
+      </c>
+      <c r="J6" s="19" t="inlineStr">
+        <is>
+          <t>✓</t>
+        </is>
+      </c>
     </row>
     <row r="7" ht="48" customHeight="1">
       <c r="A7" s="12" t="inlineStr">
         <is>
-          <t>ImpulsoGov</t>
+          <t>Geopixel</t>
         </is>
       </c>
       <c r="B7" s="13" t="inlineStr">
         <is>
-          <t>Analytics / BI para APS</t>
+          <t>GeoInteligência Fiscal</t>
         </is>
       </c>
       <c r="C7" s="13" t="inlineStr">
         <is>
-          <t>Startup early-stage</t>
+          <t>PME</t>
         </is>
       </c>
       <c r="D7" s="13" t="inlineStr">
         <is>
-          <t>São Paulo - SP</t>
+          <t>Curitiba - PR</t>
         </is>
       </c>
       <c r="E7" s="13" t="inlineStr">
         <is>
-          <t>~2020</t>
+          <t>~2010</t>
         </is>
       </c>
       <c r="F7" s="13" t="inlineStr">
         <is>
-          <t>Municípios via SUS</t>
+          <t>100+ municípios</t>
         </is>
       </c>
       <c r="G7" s="13" t="inlineStr">
         <is>
-          <t>US$ 100k</t>
+          <t>N/D</t>
         </is>
       </c>
       <c r="H7" s="13" t="inlineStr">
         <is>
-          <t>BI para gaps de atenção básica preventiva. Cofundada por ex-Harvard Kennedy School. Reconhecida pela CGU. Impulso Previne.</t>
-        </is>
-      </c>
-      <c r="I7" s="13" t="inlineStr"/>
+          <t>Geoprocessamento + IA para IPTU, ITBI, ISS. Reforma Tributária (LC 214/2025) cria janela de demanda direta e imediata.</t>
+        </is>
+      </c>
+      <c r="I7" s="17" t="inlineStr">
+        <is>
+          <t>Oportunidade fiscal 2025</t>
+        </is>
+      </c>
       <c r="J7" s="13" t="inlineStr"/>
     </row>
     <row r="8" ht="48" customHeight="1">
       <c r="A8" s="14" t="inlineStr">
         <is>
-          <t>UpCities</t>
+          <t>Gove</t>
         </is>
       </c>
       <c r="B8" s="15" t="inlineStr">
         <is>
-          <t>Integração e-SUS / Telecare</t>
+          <t>Analytics Financeiro Municipal</t>
         </is>
       </c>
       <c r="C8" s="15" t="inlineStr">
         <is>
-          <t>Startup</t>
+          <t>Startup / Scale-up</t>
         </is>
       </c>
       <c r="D8" s="15" t="inlineStr">
@@ -2844,22 +3118,22 @@
       </c>
       <c r="E8" s="15" t="inlineStr">
         <is>
-          <t>~2019</t>
+          <t>2018</t>
         </is>
       </c>
       <c r="F8" s="15" t="inlineStr">
         <is>
-          <t>Municípios (expansão)</t>
+          <t>SP, MG, RS, SC, ES+</t>
         </is>
       </c>
       <c r="G8" s="15" t="inlineStr">
         <is>
-          <t>N/D</t>
+          <t>R$ 8M (Astella)</t>
         </is>
       </c>
       <c r="H8" s="15" t="inlineStr">
         <is>
-          <t>Integradora e-SUS/RNDS. Prontuário unificado, telecare. App offline para agentes comunitários de saúde.</t>
+          <t>Analytics IA para finanças públicas: identifica ineficiências em receitas/despesas municipais. Aporte Astella. BrazilLAB Turma 7.</t>
         </is>
       </c>
       <c r="I8" s="15" t="inlineStr"/>
@@ -2868,12 +3142,12 @@
     <row r="9" ht="48" customHeight="1">
       <c r="A9" s="12" t="inlineStr">
         <is>
-          <t>ToGov</t>
+          <t>Hub Esfera</t>
         </is>
       </c>
       <c r="B9" s="13" t="inlineStr">
         <is>
-          <t>Analytics APS / Educação</t>
+          <t>IA Analytics / Orçamento Municipal</t>
         </is>
       </c>
       <c r="C9" s="13" t="inlineStr">
@@ -2883,17 +3157,17 @@
       </c>
       <c r="D9" s="13" t="inlineStr">
         <is>
-          <t>Santa Luzia - MG</t>
+          <t>N/D (Brasil)</t>
         </is>
       </c>
       <c r="E9" s="13" t="inlineStr">
         <is>
-          <t>2020</t>
+          <t>N/D</t>
         </is>
       </c>
       <c r="F9" s="13" t="inlineStr">
         <is>
-          <t>Municípios MG e outros</t>
+          <t>N/D</t>
         </is>
       </c>
       <c r="G9" s="13" t="inlineStr">
@@ -2903,59 +3177,15 @@
       </c>
       <c r="H9" s="13" t="inlineStr">
         <is>
-          <t>Analytics Previne Brasil: gaps, captação de recursos, indicadores APS. 3ª DemoDay BrazilLAB 2023.</t>
-        </is>
-      </c>
-      <c r="I9" s="13" t="inlineStr"/>
-      <c r="J9" s="13" t="inlineStr"/>
-    </row>
-    <row r="10" ht="48" customHeight="1">
-      <c r="A10" s="14" t="inlineStr">
-        <is>
-          <t>MedBolso</t>
-        </is>
-      </c>
-      <c r="B10" s="15" t="inlineStr">
-        <is>
-          <t>Escalas / Anti-fraude Saúde</t>
-        </is>
-      </c>
-      <c r="C10" s="15" t="inlineStr">
-        <is>
-          <t>Startup</t>
-        </is>
-      </c>
-      <c r="D10" s="15" t="inlineStr">
-        <is>
-          <t>N/D (Brasil)</t>
-        </is>
-      </c>
-      <c r="E10" s="15" t="inlineStr">
-        <is>
-          <t>~2020</t>
-        </is>
-      </c>
-      <c r="F10" s="15" t="inlineStr">
-        <is>
-          <t>UBS / Municípios</t>
-        </is>
-      </c>
-      <c r="G10" s="15" t="inlineStr">
-        <is>
-          <t>N/D</t>
-        </is>
-      </c>
-      <c r="H10" s="15" t="inlineStr">
-        <is>
-          <t>Gestão de escalas e plantões para saúde pública municipal. Anti-fraude em folha de pagamento. Top 30 Sebrae 2024. Acelerada GovTech Pará.</t>
-        </is>
-      </c>
-      <c r="I10" s="16" t="inlineStr">
-        <is>
-          <t>Watch — anti-fraude saúde</t>
-        </is>
-      </c>
-      <c r="J10" s="19" t="inlineStr">
+          <t>Plataforma IA para gestão municipal: analytics preditivo + preventivo + prescritivo. Integra dados orçamentários, operacionais e sociais para apoio à decisão do gestor público.</t>
+        </is>
+      </c>
+      <c r="I9" s="17" t="inlineStr">
+        <is>
+          <t>Watch</t>
+        </is>
+      </c>
+      <c r="J9" s="18" t="inlineStr">
         <is>
           <t>✓</t>
         </is>
@@ -2993,7 +3223,7 @@
     <row r="1" ht="28" customHeight="1">
       <c r="A1" s="21" t="inlineStr">
         <is>
-          <t>📚 Educação Pública — Radar GovTech Brasil 2025/2026</t>
+          <t>🏥 Saúde Pública — Radar GovTech Brasil 2025/2026</t>
         </is>
       </c>
     </row>
@@ -3052,47 +3282,47 @@
     <row r="3" ht="48" customHeight="1">
       <c r="A3" s="12" t="inlineStr">
         <is>
-          <t>Portabilis</t>
+          <t>OM30</t>
         </is>
       </c>
       <c r="B3" s="13" t="inlineStr">
         <is>
-          <t>Gestão Escolar (SIE)</t>
+          <t>Atenção Primária / Suite</t>
         </is>
       </c>
       <c r="C3" s="13" t="inlineStr">
         <is>
-          <t>Scale-up / PME</t>
+          <t>PME Estabelecida</t>
         </is>
       </c>
       <c r="D3" s="13" t="inlineStr">
         <is>
-          <t>Içara - SC</t>
+          <t>São Paulo - SP</t>
         </is>
       </c>
       <c r="E3" s="13" t="inlineStr">
         <is>
-          <t>2009</t>
+          <t>~2005</t>
         </is>
       </c>
       <c r="F3" s="13" t="inlineStr">
         <is>
-          <t>140+ mun | 700k+ alunos</t>
+          <t>Municípios SP</t>
         </is>
       </c>
       <c r="G3" s="13" t="inlineStr">
         <is>
-          <t>Aporte Yunus R$2M</t>
+          <t>N/D</t>
         </is>
       </c>
       <c r="H3" s="13" t="inlineStr">
         <is>
-          <t>Mantenedora i-Educar (software público federal). Parceria MEC e Fundação Lemann. Meta: 1,5M alunos até 2027.</t>
+          <t>Suite municipal: Saúde Simples + Educação + DadosGov + Mobilidade + Doc+. 350 colaboradores. Meta: 2x municípios SP até 2030. IA reduz 40% tempo de consultas SUS.</t>
         </is>
       </c>
       <c r="I3" s="17" t="inlineStr">
         <is>
-          <t>Target / impacto</t>
+          <t>Target roll-up</t>
         </is>
       </c>
       <c r="J3" s="13" t="inlineStr"/>
@@ -3100,12 +3330,12 @@
     <row r="4" ht="48" customHeight="1">
       <c r="A4" s="14" t="inlineStr">
         <is>
-          <t>Vivver Sistemas</t>
+          <t>Olostech</t>
         </is>
       </c>
       <c r="B4" s="15" t="inlineStr">
         <is>
-          <t>Gestão Escolar (SIE)</t>
+          <t>Atenção Primária / APS</t>
         </is>
       </c>
       <c r="C4" s="15" t="inlineStr">
@@ -3115,17 +3345,17 @@
       </c>
       <c r="D4" s="15" t="inlineStr">
         <is>
-          <t>Belo Horizonte - MG</t>
+          <t>Joinville - SC</t>
         </is>
       </c>
       <c r="E4" s="15" t="inlineStr">
         <is>
-          <t>1999</t>
+          <t>1992</t>
         </is>
       </c>
       <c r="F4" s="15" t="inlineStr">
         <is>
-          <t>Municípios MG + NE</t>
+          <t>100+ municípios</t>
         </is>
       </c>
       <c r="G4" s="15" t="inlineStr">
@@ -3135,41 +3365,45 @@
       </c>
       <c r="H4" s="15" t="inlineStr">
         <is>
-          <t>Cliente Sorocaba (SP): avançou C+ → B no IEGM 2025 (Saúde e Educação). 26 anos no segmento.</t>
-        </is>
-      </c>
-      <c r="I4" s="15" t="inlineStr"/>
+          <t>Pioneira SaaS cloud em APS (1998). 91% dos clientes melhoraram indicadores Previne Brasil 2023.</t>
+        </is>
+      </c>
+      <c r="I4" s="16" t="inlineStr">
+        <is>
+          <t>Target roll-up</t>
+        </is>
+      </c>
       <c r="J4" s="15" t="inlineStr"/>
     </row>
     <row r="5" ht="48" customHeight="1">
       <c r="A5" s="12" t="inlineStr">
         <is>
-          <t>Educ21</t>
+          <t>Vivver Sistemas</t>
         </is>
       </c>
       <c r="B5" s="13" t="inlineStr">
         <is>
-          <t>Gestão Escolar com IA</t>
+          <t>APS + Educação Municipal</t>
         </is>
       </c>
       <c r="C5" s="13" t="inlineStr">
         <is>
-          <t>PME / Startup</t>
+          <t>PME Estabelecida</t>
         </is>
       </c>
       <c r="D5" s="13" t="inlineStr">
         <is>
-          <t>N/D</t>
+          <t>Belo Horizonte - MG</t>
         </is>
       </c>
       <c r="E5" s="13" t="inlineStr">
         <is>
-          <t>N/D</t>
+          <t>1999</t>
         </is>
       </c>
       <c r="F5" s="13" t="inlineStr">
         <is>
-          <t>Municípios</t>
+          <t>Municípios MG + NE</t>
         </is>
       </c>
       <c r="G5" s="13" t="inlineStr">
@@ -3179,41 +3413,45 @@
       </c>
       <c r="H5" s="13" t="inlineStr">
         <is>
-          <t>Gestão acadêmica, administrativa e financeira com IA integrada. Dados institucionais limitados — oportunidade de due diligence.</t>
-        </is>
-      </c>
-      <c r="I5" s="13" t="inlineStr"/>
+          <t>26 anos de operação. Selos Ouro/Prata Bora Vacinar (mar/2025). Filiais SP e PB. Foco saúde pública + educação municipal integradas.</t>
+        </is>
+      </c>
+      <c r="I5" s="17" t="inlineStr">
+        <is>
+          <t>Target roll-up</t>
+        </is>
+      </c>
       <c r="J5" s="13" t="inlineStr"/>
     </row>
     <row r="6" ht="48" customHeight="1">
       <c r="A6" s="14" t="inlineStr">
         <is>
-          <t>Geekie</t>
+          <t>Pública Tecnologia</t>
         </is>
       </c>
       <c r="B6" s="15" t="inlineStr">
         <is>
-          <t>Aprendizagem IA / Híbrida</t>
+          <t>Prontuário Eletrônico APS</t>
         </is>
       </c>
       <c r="C6" s="15" t="inlineStr">
         <is>
-          <t>Scale-up</t>
+          <t>PME</t>
         </is>
       </c>
       <c r="D6" s="15" t="inlineStr">
         <is>
-          <t>São Paulo - SP</t>
+          <t>N/D</t>
         </is>
       </c>
       <c r="E6" s="15" t="inlineStr">
         <is>
-          <t>2011</t>
+          <t>N/D</t>
         </is>
       </c>
       <c r="F6" s="15" t="inlineStr">
         <is>
-          <t>5k esc | 12M alunos</t>
+          <t>Municípios</t>
         </is>
       </c>
       <c r="G6" s="15" t="inlineStr">
@@ -3223,7 +3461,7 @@
       </c>
       <c r="H6" s="15" t="inlineStr">
         <is>
-          <t>415k alunos rede estadual SP (gratuito). Parceria MEC desde 2014. IA + ensino híbrido. Potencial alvo M&amp;A.</t>
+          <t>Prontuário eletrônico certificado SBIS/CFM. Assinatura ICP-Brasil. Integração e-SUS.</t>
         </is>
       </c>
       <c r="I6" s="15" t="inlineStr"/>
@@ -3232,42 +3470,42 @@
     <row r="7" ht="48" customHeight="1">
       <c r="A7" s="12" t="inlineStr">
         <is>
-          <t>Educacross</t>
+          <t>ImpulsoGov</t>
         </is>
       </c>
       <c r="B7" s="13" t="inlineStr">
         <is>
-          <t>Gamificação + IA Educacional</t>
+          <t>Analytics / BI para APS</t>
         </is>
       </c>
       <c r="C7" s="13" t="inlineStr">
         <is>
-          <t>Startup</t>
+          <t>Startup early-stage</t>
         </is>
       </c>
       <c r="D7" s="13" t="inlineStr">
         <is>
-          <t>N/D (Brasil)</t>
+          <t>São Paulo - SP</t>
         </is>
       </c>
       <c r="E7" s="13" t="inlineStr">
         <is>
-          <t>N/D</t>
+          <t>~2020</t>
         </is>
       </c>
       <c r="F7" s="13" t="inlineStr">
         <is>
-          <t>Rede estadual GO</t>
+          <t>Municípios via SUS</t>
         </is>
       </c>
       <c r="G7" s="13" t="inlineStr">
         <is>
-          <t>N/D</t>
+          <t>US$ 100k</t>
         </is>
       </c>
       <c r="H7" s="13" t="inlineStr">
         <is>
-          <t>Selecionada Governo de Goiás. Gamificação + IA em Português e Matemática para redes públicas.</t>
+          <t>BI para gaps de atenção básica preventiva. Cofundada por ex-Harvard Kennedy School. Reconhecida pela CGU. Impulso Previne.</t>
         </is>
       </c>
       <c r="I7" s="13" t="inlineStr"/>
@@ -3276,12 +3514,12 @@
     <row r="8" ht="48" customHeight="1">
       <c r="A8" s="14" t="inlineStr">
         <is>
-          <t>ToGov</t>
+          <t>UpCities</t>
         </is>
       </c>
       <c r="B8" s="15" t="inlineStr">
         <is>
-          <t>Analytics Educacionais</t>
+          <t>Integração e-SUS / Telecare</t>
         </is>
       </c>
       <c r="C8" s="15" t="inlineStr">
@@ -3291,17 +3529,17 @@
       </c>
       <c r="D8" s="15" t="inlineStr">
         <is>
-          <t>Santa Luzia - MG</t>
+          <t>São Paulo - SP</t>
         </is>
       </c>
       <c r="E8" s="15" t="inlineStr">
         <is>
-          <t>2020</t>
+          <t>~2019</t>
         </is>
       </c>
       <c r="F8" s="15" t="inlineStr">
         <is>
-          <t>Municípios MG e outros</t>
+          <t>Municípios (expansão)</t>
         </is>
       </c>
       <c r="G8" s="15" t="inlineStr">
@@ -3311,7 +3549,7 @@
       </c>
       <c r="H8" s="15" t="inlineStr">
         <is>
-          <t>Monitoramento IDEB, IEGM, captação de recursos. Camada analítica sobre SIEs existentes. BrazilLAB 2023.</t>
+          <t>Integradora e-SUS/RNDS. Prontuário unificado, telecare. App offline para agentes comunitários de saúde.</t>
         </is>
       </c>
       <c r="I8" s="15" t="inlineStr"/>
@@ -3320,60 +3558,56 @@
     <row r="9" ht="48" customHeight="1">
       <c r="A9" s="12" t="inlineStr">
         <is>
-          <t>i-Educar</t>
+          <t>ToGov</t>
         </is>
       </c>
       <c r="B9" s="13" t="inlineStr">
         <is>
-          <t>Open Source / Software Público</t>
+          <t>Analytics APS / Educação</t>
         </is>
       </c>
       <c r="C9" s="13" t="inlineStr">
         <is>
-          <t>Software Público</t>
+          <t>Startup</t>
         </is>
       </c>
       <c r="D9" s="13" t="inlineStr">
         <is>
-          <t>Itajaí - SC (origem)</t>
+          <t>Santa Luzia - MG</t>
         </is>
       </c>
       <c r="E9" s="13" t="inlineStr">
         <is>
-          <t>2008</t>
+          <t>2020</t>
         </is>
       </c>
       <c r="F9" s="13" t="inlineStr">
         <is>
-          <t>80+ prefeituras ativas</t>
+          <t>Municípios MG e outros</t>
         </is>
       </c>
       <c r="G9" s="13" t="inlineStr">
         <is>
-          <t>Gratuito</t>
+          <t>N/D</t>
         </is>
       </c>
       <c r="H9" s="13" t="inlineStr">
         <is>
-          <t>Software público federal mantido por Portabilis. Monte Alegre (RN) economizou R$2,4M. Parceria MEC + MP.</t>
-        </is>
-      </c>
-      <c r="I9" s="17" t="inlineStr">
-        <is>
-          <t>Referência pública</t>
-        </is>
-      </c>
+          <t>Analytics Previne Brasil: gaps, captação de recursos, indicadores APS. 3ª DemoDay BrazilLAB 2023.</t>
+        </is>
+      </c>
+      <c r="I9" s="13" t="inlineStr"/>
       <c r="J9" s="13" t="inlineStr"/>
     </row>
     <row r="10" ht="48" customHeight="1">
       <c r="A10" s="14" t="inlineStr">
         <is>
-          <t>Jovens Gênios</t>
+          <t>MedBolso</t>
         </is>
       </c>
       <c r="B10" s="15" t="inlineStr">
         <is>
-          <t>EdTech Gamificada / IA Educacional</t>
+          <t>Escalas / Anti-fraude Saúde</t>
         </is>
       </c>
       <c r="C10" s="15" t="inlineStr">
@@ -3383,32 +3617,32 @@
       </c>
       <c r="D10" s="15" t="inlineStr">
         <is>
-          <t>Rio de Janeiro - RJ</t>
+          <t>N/D (Brasil)</t>
         </is>
       </c>
       <c r="E10" s="15" t="inlineStr">
         <is>
-          <t>N/D</t>
+          <t>~2020</t>
         </is>
       </c>
       <c r="F10" s="15" t="inlineStr">
         <is>
-          <t>50+ municípios | est. SP</t>
+          <t>UBS / Municípios</t>
         </is>
       </c>
       <c r="G10" s="15" t="inlineStr">
         <is>
-          <t>R$11,8M (Fundo GovTech)</t>
+          <t>N/D</t>
         </is>
       </c>
       <c r="H10" s="15" t="inlineStr">
         <is>
-          <t>Plataforma adaptativa de aprendizagem e avaliação gamificada. 90% dos alunos em escolas públicas. 83% dos usuários em rede pública. Meta: 10M alunos até 2030. Rodada seed R$11,8M liderada pelo Fundo GovTech (KPTL+Cedro) com DOMO.VC, Criabiz Ventures e Rosey Ventures (Grupo Marista). Mar/2026.</t>
+          <t>Gestão de escalas e plantões para saúde pública municipal. Anti-fraude em folha de pagamento. Top 30 Sebrae 2024. Acelerada GovTech Pará.</t>
         </is>
       </c>
       <c r="I10" s="16" t="inlineStr">
         <is>
-          <t>Portfólio KPTL+Cedro</t>
+          <t>Watch — anti-fraude saúde</t>
         </is>
       </c>
       <c r="J10" s="19" t="inlineStr">
@@ -3431,7 +3665,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:J14"/>
+  <dimension ref="A1:J10"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="28" customWidth="1" min="1" max="1"/>
@@ -3449,7 +3683,7 @@
     <row r="1" ht="28" customHeight="1">
       <c r="A1" s="22" t="inlineStr">
         <is>
-          <t>🤖 IA para Governo — Radar GovTech Brasil 2025/2026</t>
+          <t>📚 Educação Pública — Radar GovTech Brasil 2025/2026</t>
         </is>
       </c>
     </row>
@@ -3508,47 +3742,47 @@
     <row r="3" ht="48" customHeight="1">
       <c r="A3" s="12" t="inlineStr">
         <is>
-          <t>GovTools</t>
+          <t>Portabilis</t>
         </is>
       </c>
       <c r="B3" s="13" t="inlineStr">
         <is>
-          <t>Agentes RPA / WhatsApp</t>
+          <t>Gestão Escolar (SIE)</t>
         </is>
       </c>
       <c r="C3" s="13" t="inlineStr">
         <is>
-          <t>Startup</t>
+          <t>Scale-up / PME</t>
         </is>
       </c>
       <c r="D3" s="13" t="inlineStr">
         <is>
-          <t>Porto Alegre - RS</t>
+          <t>Içara - SC</t>
         </is>
       </c>
       <c r="E3" s="13" t="inlineStr">
         <is>
-          <t>2024</t>
+          <t>2009</t>
         </is>
       </c>
       <c r="F3" s="13" t="inlineStr">
         <is>
-          <t>200+ municípios</t>
+          <t>140+ mun | 700k+ alunos</t>
         </is>
       </c>
       <c r="G3" s="13" t="inlineStr">
         <is>
-          <t>Aporte Ventiur+DOMO</t>
+          <t>Aporte Yunus R$2M</t>
         </is>
       </c>
       <c r="H3" s="13" t="inlineStr">
         <is>
-          <t>Agentes IA via WhatsApp. Opera sistemas municipais sem integração tradicional. 200+ municípios em &lt;12 meses. Modelo viral, alta tração.</t>
+          <t>Mantenedora i-Educar (software público federal). Parceria MEC e Fundação Lemann. Meta: 1,5M alunos até 2027.</t>
         </is>
       </c>
       <c r="I3" s="17" t="inlineStr">
         <is>
-          <t>M&amp;A Watch</t>
+          <t>Target / impacto</t>
         </is>
       </c>
       <c r="J3" s="13" t="inlineStr"/>
@@ -3556,32 +3790,32 @@
     <row r="4" ht="48" customHeight="1">
       <c r="A4" s="14" t="inlineStr">
         <is>
-          <t>Nuveo</t>
+          <t>Vivver Sistemas</t>
         </is>
       </c>
       <c r="B4" s="15" t="inlineStr">
         <is>
-          <t>Document AI / Ultra OCR</t>
+          <t>Gestão Escolar (SIE)</t>
         </is>
       </c>
       <c r="C4" s="15" t="inlineStr">
         <is>
-          <t>Startup</t>
+          <t>PME Estabelecida</t>
         </is>
       </c>
       <c r="D4" s="15" t="inlineStr">
         <is>
-          <t>SP / Campina Grande - PB</t>
+          <t>Belo Horizonte - MG</t>
         </is>
       </c>
       <c r="E4" s="15" t="inlineStr">
         <is>
-          <t>2016</t>
+          <t>1999</t>
         </is>
       </c>
       <c r="F4" s="15" t="inlineStr">
         <is>
-          <t>Setor público e privado</t>
+          <t>Municípios MG + NE</t>
         </is>
       </c>
       <c r="G4" s="15" t="inlineStr">
@@ -3591,7 +3825,7 @@
       </c>
       <c r="H4" s="15" t="inlineStr">
         <is>
-          <t>Ultra OCR®: automação de documentos públicos. Contratos, invoices, documentos de identidade. Gov + corporativo.</t>
+          <t>Cliente Sorocaba (SP): avançou C+ → B no IEGM 2025 (Saúde e Educação). 26 anos no segmento.</t>
         </is>
       </c>
       <c r="I4" s="15" t="inlineStr"/>
@@ -3600,22 +3834,22 @@
     <row r="5" ht="48" customHeight="1">
       <c r="A5" s="12" t="inlineStr">
         <is>
-          <t>CPQD</t>
+          <t>Educ21</t>
         </is>
       </c>
       <c r="B5" s="13" t="inlineStr">
         <is>
-          <t>IA P&amp;D / Gov Digital</t>
+          <t>Gestão Escolar com IA</t>
         </is>
       </c>
       <c r="C5" s="13" t="inlineStr">
         <is>
-          <t>Instituto P&amp;D</t>
+          <t>PME / Startup</t>
         </is>
       </c>
       <c r="D5" s="13" t="inlineStr">
         <is>
-          <t>Campinas - SP</t>
+          <t>N/D</t>
         </is>
       </c>
       <c r="E5" s="13" t="inlineStr">
@@ -3625,35 +3859,31 @@
       </c>
       <c r="F5" s="13" t="inlineStr">
         <is>
-          <t>Governo Federal</t>
+          <t>Municípios</t>
         </is>
       </c>
       <c r="G5" s="13" t="inlineStr">
         <is>
-          <t>R$ 390M contrato</t>
+          <t>N/D</t>
         </is>
       </c>
       <c r="H5" s="13" t="inlineStr">
         <is>
-          <t>Projeto INSPIRE com MGI (R$390M, 4 anos). IA personalizada para serviços de governo digital: chatbots, recomendação, acessibilidade.</t>
-        </is>
-      </c>
-      <c r="I5" s="17" t="inlineStr">
-        <is>
-          <t>Parceria estratégica MGI</t>
-        </is>
-      </c>
+          <t>Gestão acadêmica, administrativa e financeira com IA integrada. Dados institucionais limitados — oportunidade de due diligence.</t>
+        </is>
+      </c>
+      <c r="I5" s="13" t="inlineStr"/>
       <c r="J5" s="13" t="inlineStr"/>
     </row>
     <row r="6" ht="48" customHeight="1">
       <c r="A6" s="14" t="inlineStr">
         <is>
-          <t>Horus Smart Det.</t>
+          <t>Geekie</t>
         </is>
       </c>
       <c r="B6" s="15" t="inlineStr">
         <is>
-          <t>Fiscalização / Drones / IA</t>
+          <t>Aprendizagem IA / Híbrida</t>
         </is>
       </c>
       <c r="C6" s="15" t="inlineStr">
@@ -3663,17 +3893,17 @@
       </c>
       <c r="D6" s="15" t="inlineStr">
         <is>
-          <t>Florianópolis - SC</t>
+          <t>São Paulo - SP</t>
         </is>
       </c>
       <c r="E6" s="15" t="inlineStr">
         <is>
-          <t>~2016</t>
+          <t>2011</t>
         </is>
       </c>
       <c r="F6" s="15" t="inlineStr">
         <is>
-          <t>100+ gov + privado</t>
+          <t>5k esc | 12M alunos</t>
         </is>
       </c>
       <c r="G6" s="15" t="inlineStr">
@@ -3683,7 +3913,7 @@
       </c>
       <c r="H6" s="15" t="inlineStr">
         <is>
-          <t>Drones + satélites + visão computacional: obras irregulares, desmatamento, infraestrutura. Cliente: Florianópolis. 9 anos de operação.</t>
+          <t>415k alunos rede estadual SP (gratuito). Parceria MEC desde 2014. IA + ensino híbrido. Potencial alvo M&amp;A.</t>
         </is>
       </c>
       <c r="I6" s="15" t="inlineStr"/>
@@ -3692,32 +3922,32 @@
     <row r="7" ht="48" customHeight="1">
       <c r="A7" s="12" t="inlineStr">
         <is>
-          <t>Geopixel</t>
+          <t>Educacross</t>
         </is>
       </c>
       <c r="B7" s="13" t="inlineStr">
         <is>
-          <t>GeoInteligência Fiscal</t>
+          <t>Gamificação + IA Educacional</t>
         </is>
       </c>
       <c r="C7" s="13" t="inlineStr">
         <is>
-          <t>PME</t>
+          <t>Startup</t>
         </is>
       </c>
       <c r="D7" s="13" t="inlineStr">
         <is>
-          <t>Curitiba - PR</t>
+          <t>N/D (Brasil)</t>
         </is>
       </c>
       <c r="E7" s="13" t="inlineStr">
         <is>
-          <t>~2010</t>
+          <t>N/D</t>
         </is>
       </c>
       <c r="F7" s="13" t="inlineStr">
         <is>
-          <t>100+ municípios</t>
+          <t>Rede estadual GO</t>
         </is>
       </c>
       <c r="G7" s="13" t="inlineStr">
@@ -3727,45 +3957,41 @@
       </c>
       <c r="H7" s="13" t="inlineStr">
         <is>
-          <t>Geoprocessamento + IA para IPTU, ITBI, ISS. Reforma Tributária (LC 214/2025) cria janela de demanda direta e imediata.</t>
-        </is>
-      </c>
-      <c r="I7" s="17" t="inlineStr">
-        <is>
-          <t>Oportunidade fiscal 2025</t>
-        </is>
-      </c>
+          <t>Selecionada Governo de Goiás. Gamificação + IA em Português e Matemática para redes públicas.</t>
+        </is>
+      </c>
+      <c r="I7" s="13" t="inlineStr"/>
       <c r="J7" s="13" t="inlineStr"/>
     </row>
     <row r="8" ht="48" customHeight="1">
       <c r="A8" s="14" t="inlineStr">
         <is>
-          <t>Intelicity</t>
+          <t>ToGov</t>
         </is>
       </c>
       <c r="B8" s="15" t="inlineStr">
         <is>
-          <t>IA Infraestrutura Urbana</t>
+          <t>Analytics Educacionais</t>
         </is>
       </c>
       <c r="C8" s="15" t="inlineStr">
         <is>
-          <t>Startup / Scale-up</t>
+          <t>Startup</t>
         </is>
       </c>
       <c r="D8" s="15" t="inlineStr">
         <is>
-          <t>São Paulo - SP</t>
+          <t>Santa Luzia - MG</t>
         </is>
       </c>
       <c r="E8" s="15" t="inlineStr">
         <is>
-          <t>~2019</t>
+          <t>2020</t>
         </is>
       </c>
       <c r="F8" s="15" t="inlineStr">
         <is>
-          <t>Sabesp + municípios</t>
+          <t>Municípios MG e outros</t>
         </is>
       </c>
       <c r="G8" s="15" t="inlineStr">
@@ -3775,7 +4001,7 @@
       </c>
       <c r="H8" s="15" t="inlineStr">
         <is>
-          <t>Câmeras em veículos + visão computacional: mapeia pavimento, rachaduras. Sabesp: detecção de vazamentos de água.</t>
+          <t>Monitoramento IDEB, IEGM, captação de recursos. Camada analítica sobre SIEs existentes. BrazilLAB 2023.</t>
         </is>
       </c>
       <c r="I8" s="15" t="inlineStr"/>
@@ -3784,47 +4010,47 @@
     <row r="9" ht="48" customHeight="1">
       <c r="A9" s="12" t="inlineStr">
         <is>
-          <t>MinutaIA (jAI)</t>
+          <t>i-Educar</t>
         </is>
       </c>
       <c r="B9" s="13" t="inlineStr">
         <is>
-          <t>IA Jurídica / Judicial</t>
+          <t>Open Source / Software Público</t>
         </is>
       </c>
       <c r="C9" s="13" t="inlineStr">
         <is>
-          <t>Startup</t>
+          <t>Software Público</t>
         </is>
       </c>
       <c r="D9" s="13" t="inlineStr">
         <is>
-          <t>Belo Horizonte - MG</t>
+          <t>Itajaí - SC (origem)</t>
         </is>
       </c>
       <c r="E9" s="13" t="inlineStr">
         <is>
-          <t>2025</t>
+          <t>2008</t>
         </is>
       </c>
       <c r="F9" s="13" t="inlineStr">
         <is>
-          <t>7 tribunais | 100k+ usr</t>
+          <t>80+ prefeituras ativas</t>
         </is>
       </c>
       <c r="G9" s="13" t="inlineStr">
         <is>
-          <t>N/D</t>
+          <t>Gratuito</t>
         </is>
       </c>
       <c r="H9" s="13" t="inlineStr">
         <is>
-          <t>10M+ minutas geradas. TJRS, STM, TRE-PB/BA, Tocantins. CNJ Resolução 615/2025. Exportou para a Argentina.</t>
+          <t>Software público federal mantido por Portabilis. Monte Alegre (RN) economizou R$2,4M. Parceria MEC + MP.</t>
         </is>
       </c>
       <c r="I9" s="17" t="inlineStr">
         <is>
-          <t>Watch — tração judicial</t>
+          <t>Referência pública</t>
         </is>
       </c>
       <c r="J9" s="13" t="inlineStr"/>
@@ -3832,12 +4058,12 @@
     <row r="10" ht="48" customHeight="1">
       <c r="A10" s="14" t="inlineStr">
         <is>
-          <t>Tolky</t>
+          <t>Jovens Gênios</t>
         </is>
       </c>
       <c r="B10" s="15" t="inlineStr">
         <is>
-          <t>IA Atendimento ao Cidadão</t>
+          <t>EdTech Gamificada / IA Educacional</t>
         </is>
       </c>
       <c r="C10" s="15" t="inlineStr">
@@ -3847,231 +4073,35 @@
       </c>
       <c r="D10" s="15" t="inlineStr">
         <is>
-          <t>N/D (Brasil)</t>
+          <t>Rio de Janeiro - RJ</t>
         </is>
       </c>
       <c r="E10" s="15" t="inlineStr">
         <is>
-          <t>~2023</t>
+          <t>N/D</t>
         </is>
       </c>
       <c r="F10" s="15" t="inlineStr">
         <is>
-          <t>Contratos gov / CNJ</t>
+          <t>50+ municípios | est. SP</t>
         </is>
       </c>
       <c r="G10" s="15" t="inlineStr">
         <is>
-          <t>N/D</t>
+          <t>R$11,8M (Fundo GovTech)</t>
         </is>
       </c>
       <c r="H10" s="15" t="inlineStr">
         <is>
-          <t>Multichannel (WhatsApp, chat, email) + processos end-to-end. ABES CSC 2025. Contrato CPSI CNJ.</t>
+          <t>Plataforma adaptativa de aprendizagem e avaliação gamificada. 90% dos alunos em escolas públicas. 83% dos usuários em rede pública. Meta: 10M alunos até 2030. Rodada seed R$11,8M liderada pelo Fundo GovTech (KPTL+Cedro) com DOMO.VC, Criabiz Ventures e Rosey Ventures (Grupo Marista). Mar/2026.</t>
         </is>
       </c>
       <c r="I10" s="16" t="inlineStr">
         <is>
-          <t>Selecionada CPSI CNJ</t>
-        </is>
-      </c>
-      <c r="J10" s="15" t="inlineStr"/>
-    </row>
-    <row r="11" ht="48" customHeight="1">
-      <c r="A11" s="12" t="inlineStr">
-        <is>
-          <t>Gove</t>
-        </is>
-      </c>
-      <c r="B11" s="13" t="inlineStr">
-        <is>
-          <t>Analytics Financeiro Municipal</t>
-        </is>
-      </c>
-      <c r="C11" s="13" t="inlineStr">
-        <is>
-          <t>Startup / Scale-up</t>
-        </is>
-      </c>
-      <c r="D11" s="13" t="inlineStr">
-        <is>
-          <t>São Paulo - SP</t>
-        </is>
-      </c>
-      <c r="E11" s="13" t="inlineStr">
-        <is>
-          <t>2018</t>
-        </is>
-      </c>
-      <c r="F11" s="13" t="inlineStr">
-        <is>
-          <t>SP, MG, RS, SC, ES+</t>
-        </is>
-      </c>
-      <c r="G11" s="13" t="inlineStr">
-        <is>
-          <t>R$ 8M (Astella)</t>
-        </is>
-      </c>
-      <c r="H11" s="13" t="inlineStr">
-        <is>
-          <t>Analytics IA para finanças públicas: identifica ineficiências em receitas/despesas municipais. Aporte Astella. BrazilLAB Turma 7.</t>
-        </is>
-      </c>
-      <c r="I11" s="13" t="inlineStr"/>
-      <c r="J11" s="13" t="inlineStr"/>
-    </row>
-    <row r="12" ht="48" customHeight="1">
-      <c r="A12" s="14" t="inlineStr">
-        <is>
-          <t>Inteligov</t>
-        </is>
-      </c>
-      <c r="B12" s="15" t="inlineStr">
-        <is>
-          <t>Monitoramento Legislativo / Inteligência Regulatória</t>
-        </is>
-      </c>
-      <c r="C12" s="15" t="inlineStr">
-        <is>
-          <t>Startup / Scale-up</t>
-        </is>
-      </c>
-      <c r="D12" s="15" t="inlineStr">
-        <is>
-          <t>São Paulo - SP</t>
-        </is>
-      </c>
-      <c r="E12" s="15" t="inlineStr">
-        <is>
-          <t>2014</t>
-        </is>
-      </c>
-      <c r="F12" s="15" t="inlineStr">
-        <is>
-          <t>100+ clientes | 27 estados + 1k+ mun.</t>
-        </is>
-      </c>
-      <c r="G12" s="15" t="inlineStr">
-        <is>
-          <t>N/D</t>
-        </is>
-      </c>
-      <c r="H12" s="15" t="inlineStr">
-        <is>
-          <t>Pioneira em monitoramento automatizado de dados governamentais (Legislativo, Executivo, Judiciário). 4M+ proposições monitoradas. ~890 fontes de Diários Oficiais. IA com termômetro de aprovação de PLs (&gt;98% acurácia). Única com 100% de cobertura das Assembleias Estaduais. Ranking 100 Open Startups, Mapa GovTech. Cubo Itaú, Inovabra, Distrito.</t>
-        </is>
-      </c>
-      <c r="I12" s="16" t="inlineStr">
-        <is>
-          <t>Watch — inteligência regulatória</t>
-        </is>
-      </c>
-      <c r="J12" s="19" t="inlineStr">
-        <is>
-          <t>✓</t>
-        </is>
-      </c>
-    </row>
-    <row r="13" ht="48" customHeight="1">
-      <c r="A13" s="12" t="inlineStr">
-        <is>
-          <t>Hub Esfera</t>
-        </is>
-      </c>
-      <c r="B13" s="13" t="inlineStr">
-        <is>
-          <t>IA Analytics / Gestão</t>
-        </is>
-      </c>
-      <c r="C13" s="13" t="inlineStr">
-        <is>
-          <t>Startup</t>
-        </is>
-      </c>
-      <c r="D13" s="13" t="inlineStr">
-        <is>
-          <t>N/D (Brasil)</t>
-        </is>
-      </c>
-      <c r="E13" s="13" t="inlineStr">
-        <is>
-          <t>N/D</t>
-        </is>
-      </c>
-      <c r="F13" s="13" t="inlineStr">
-        <is>
-          <t>N/D</t>
-        </is>
-      </c>
-      <c r="G13" s="13" t="inlineStr">
-        <is>
-          <t>N/D</t>
-        </is>
-      </c>
-      <c r="H13" s="13" t="inlineStr">
-        <is>
-          <t>Plataforma IA para gestão municipal: analytics preditivo + preventivo + prescritivo. Integra dados orçamentários, operacionais e sociais para apoio à decisão do gestor público.</t>
-        </is>
-      </c>
-      <c r="I13" s="17" t="inlineStr">
-        <is>
-          <t>Watch</t>
-        </is>
-      </c>
-      <c r="J13" s="18" t="inlineStr">
-        <is>
-          <t>✓</t>
-        </is>
-      </c>
-    </row>
-    <row r="14" ht="48" customHeight="1">
-      <c r="A14" s="14" t="inlineStr">
-        <is>
-          <t>Kinebot</t>
-        </is>
-      </c>
-      <c r="B14" s="15" t="inlineStr">
-        <is>
-          <t>IA Ergonomia / Saúde do Trabalhador</t>
-        </is>
-      </c>
-      <c r="C14" s="15" t="inlineStr">
-        <is>
-          <t>Startup</t>
-        </is>
-      </c>
-      <c r="D14" s="15" t="inlineStr">
-        <is>
-          <t>Curitiba - PR</t>
-        </is>
-      </c>
-      <c r="E14" s="15" t="inlineStr">
-        <is>
-          <t>N/D</t>
-        </is>
-      </c>
-      <c r="F14" s="15" t="inlineStr">
-        <is>
-          <t>Indústria + gov</t>
-        </is>
-      </c>
-      <c r="G14" s="15" t="inlineStr">
-        <is>
-          <t>R$3M (Fundo GovTech)</t>
-        </is>
-      </c>
-      <c r="H14" s="15" t="inlineStr">
-        <is>
-          <t>IA para análises ergonômicas e psicossociais via visão computacional. Clientes: Marfrig, P&amp;G, Electrolux. 8º investimento do Fundo GovTech (KPTL+Cedro), R$3M em fev/2026. Foco em saúde do trabalhador para setor público e privado. Expansão global planejada.</t>
-        </is>
-      </c>
-      <c r="I14" s="16" t="inlineStr">
-        <is>
           <t>Portfólio KPTL+Cedro</t>
         </is>
       </c>
-      <c r="J14" s="19" t="inlineStr">
+      <c r="J10" s="19" t="inlineStr">
         <is>
           <t>✓</t>
         </is>
@@ -4109,7 +4139,7 @@
     <row r="1" ht="28" customHeight="1">
       <c r="A1" s="23" t="inlineStr">
         <is>
-          <t>⚖️ Procuradorias (PGM/PGE/MP) — Radar GovTech Brasil 2025/2026</t>
+          <t>🤖 IA Horizontal &amp; Automação — Radar GovTech Brasil 2025/2026</t>
         </is>
       </c>
     </row>
@@ -4168,47 +4198,47 @@
     <row r="3" ht="48" customHeight="1">
       <c r="A3" s="12" t="inlineStr">
         <is>
-          <t>Attus Procuradoria Digital</t>
+          <t>GovTools</t>
         </is>
       </c>
       <c r="B3" s="13" t="inlineStr">
         <is>
-          <t>IA Contencioso + Consultivo (PGE/PGM)</t>
+          <t>Agentes RPA / WhatsApp</t>
         </is>
       </c>
       <c r="C3" s="13" t="inlineStr">
         <is>
-          <t>Scale-up</t>
+          <t>Startup</t>
         </is>
       </c>
       <c r="D3" s="13" t="inlineStr">
         <is>
-          <t>São Ludgero, SC (Eloware)</t>
+          <t>Porto Alegre - RS</t>
         </is>
       </c>
       <c r="E3" s="13" t="inlineStr">
         <is>
-          <t>~2018</t>
+          <t>2024</t>
         </is>
       </c>
       <c r="F3" s="13" t="inlineStr">
         <is>
-          <t>PGE-SP, PGE-BA, PGE-PA, PGM-Palmas</t>
+          <t>200+ municípios</t>
         </is>
       </c>
       <c r="G3" s="13" t="inlineStr">
         <is>
-          <t>SaaS Oracle Cloud</t>
+          <t>Aporte Ventiur+DOMO</t>
         </is>
       </c>
       <c r="H3" s="13" t="inlineStr">
         <is>
-          <t>4,3M+ processos analisados. 73% classificados automaticamente (98,5% acurácia). 642k+ peças geradas por IA. Referência nacional pós PGE-SP.</t>
+          <t>Agentes IA via WhatsApp. Opera sistemas municipais sem integração tradicional. 200+ municípios em &lt;12 meses. Modelo viral, alta tração.</t>
         </is>
       </c>
       <c r="I3" s="17" t="inlineStr">
         <is>
-          <t>M&amp;A Watch — líder do segmento</t>
+          <t>M&amp;A Watch</t>
         </is>
       </c>
       <c r="J3" s="13" t="inlineStr"/>
@@ -4216,32 +4246,32 @@
     <row r="4" ht="48" customHeight="1">
       <c r="A4" s="14" t="inlineStr">
         <is>
-          <t>Eicon / Giex</t>
+          <t>Nuveo</t>
         </is>
       </c>
       <c r="B4" s="15" t="inlineStr">
         <is>
-          <t>Dívida Ativa / Execução Fiscal</t>
+          <t>Document AI / Ultra OCR</t>
         </is>
       </c>
       <c r="C4" s="15" t="inlineStr">
         <is>
-          <t>PME</t>
+          <t>Startup</t>
         </is>
       </c>
       <c r="D4" s="15" t="inlineStr">
         <is>
-          <t>N/D (Brasil)</t>
+          <t>SP / Campina Grande - PB</t>
         </is>
       </c>
       <c r="E4" s="15" t="inlineStr">
         <is>
-          <t>N/D</t>
+          <t>2016</t>
         </is>
       </c>
       <c r="F4" s="15" t="inlineStr">
         <is>
-          <t>PGE e PGM — múltiplos estados</t>
+          <t>Setor público e privado</t>
         </is>
       </c>
       <c r="G4" s="15" t="inlineStr">
@@ -4251,7 +4281,7 @@
       </c>
       <c r="H4" s="15" t="inlineStr">
         <is>
-          <t>Giex: perfil completo do devedor. Integração direta com TJs. Automação de CDA, penhoras e prazos. iCad: alvarás e licenças digitais (concorrente da Quasar). +15 produtos para governo.</t>
+          <t>Ultra OCR®: automação de documentos públicos. Contratos, invoices, documentos de identidade. Gov + corporativo.</t>
         </is>
       </c>
       <c r="I4" s="15" t="inlineStr"/>
@@ -4260,22 +4290,22 @@
     <row r="5" ht="48" customHeight="1">
       <c r="A5" s="12" t="inlineStr">
         <is>
-          <t>PGMNET</t>
+          <t>CPQD</t>
         </is>
       </c>
       <c r="B5" s="13" t="inlineStr">
         <is>
-          <t>Gestão Jurídica Municipal + RPA</t>
+          <t>IA P&amp;D / Gov Digital</t>
         </is>
       </c>
       <c r="C5" s="13" t="inlineStr">
         <is>
-          <t>PME</t>
+          <t>Instituto P&amp;D</t>
         </is>
       </c>
       <c r="D5" s="13" t="inlineStr">
         <is>
-          <t>N/D (Brasil)</t>
+          <t>Campinas - SP</t>
         </is>
       </c>
       <c r="E5" s="13" t="inlineStr">
@@ -4285,31 +4315,35 @@
       </c>
       <c r="F5" s="13" t="inlineStr">
         <is>
-          <t>Procuradorias municipais</t>
+          <t>Governo Federal</t>
         </is>
       </c>
       <c r="G5" s="13" t="inlineStr">
         <is>
-          <t>N/D</t>
+          <t>R$ 390M contrato</t>
         </is>
       </c>
       <c r="H5" s="13" t="inlineStr">
         <is>
-          <t>RPA integrado para peticionamento automático em qualquer TJ do país. Interface co-desenvolvida com procuradores municipais.</t>
-        </is>
-      </c>
-      <c r="I5" s="13" t="inlineStr"/>
+          <t>Projeto INSPIRE com MGI (R$390M, 4 anos). IA personalizada para serviços de governo digital: chatbots, recomendação, acessibilidade.</t>
+        </is>
+      </c>
+      <c r="I5" s="17" t="inlineStr">
+        <is>
+          <t>Parceria estratégica MGI</t>
+        </is>
+      </c>
       <c r="J5" s="13" t="inlineStr"/>
     </row>
     <row r="6" ht="48" customHeight="1">
       <c r="A6" s="14" t="inlineStr">
         <is>
-          <t>Aetos Tech</t>
+          <t>Tolky</t>
         </is>
       </c>
       <c r="B6" s="15" t="inlineStr">
         <is>
-          <t>IA Anti-fraude Contratos (Prisma)</t>
+          <t>IA Atendimento ao Cidadão</t>
         </is>
       </c>
       <c r="C6" s="15" t="inlineStr">
@@ -4324,27 +4358,27 @@
       </c>
       <c r="E6" s="15" t="inlineStr">
         <is>
-          <t>N/D</t>
+          <t>~2023</t>
         </is>
       </c>
       <c r="F6" s="15" t="inlineStr">
         <is>
-          <t>MPRJ (CPSI 2024)</t>
+          <t>Contratos gov / CNJ</t>
         </is>
       </c>
       <c r="G6" s="15" t="inlineStr">
         <is>
-          <t>Contrato CPSI</t>
+          <t>N/D</t>
         </is>
       </c>
       <c r="H6" s="15" t="inlineStr">
         <is>
-          <t>Prisma: detecção de irregularidades em contratos públicos e lavagem de dinheiro. Cruzamento de bases abertas por IA. Selecionada CPSI MPRJ.</t>
+          <t>Multichannel (WhatsApp, chat, email) + processos end-to-end. ABES CSC 2025. Contrato CPSI CNJ.</t>
         </is>
       </c>
       <c r="I6" s="16" t="inlineStr">
         <is>
-          <t>Contrato CPSI</t>
+          <t>Selecionada CPSI CNJ</t>
         </is>
       </c>
       <c r="J6" s="15" t="inlineStr"/>
@@ -4352,70 +4386,74 @@
     <row r="7" ht="48" customHeight="1">
       <c r="A7" s="12" t="inlineStr">
         <is>
-          <t>Sumé Tecnologia</t>
+          <t>Inteligov</t>
         </is>
       </c>
       <c r="B7" s="13" t="inlineStr">
         <is>
-          <t>Monitoramento Políticas Públicas (Sonar)</t>
+          <t>Monitoramento Legislativo / Inteligência Regulatória</t>
         </is>
       </c>
       <c r="C7" s="13" t="inlineStr">
         <is>
-          <t>Startup</t>
+          <t>Startup / Scale-up</t>
         </is>
       </c>
       <c r="D7" s="13" t="inlineStr">
         <is>
-          <t>N/D (Brasil)</t>
+          <t>São Paulo - SP</t>
         </is>
       </c>
       <c r="E7" s="13" t="inlineStr">
         <is>
-          <t>N/D</t>
+          <t>2014</t>
         </is>
       </c>
       <c r="F7" s="13" t="inlineStr">
         <is>
-          <t>MPRJ (CPSI 2024)</t>
+          <t>100+ clientes | 27 estados + 1k+ mun.</t>
         </is>
       </c>
       <c r="G7" s="13" t="inlineStr">
         <is>
-          <t>Contrato CPSI</t>
+          <t>N/D</t>
         </is>
       </c>
       <c r="H7" s="13" t="inlineStr">
         <is>
-          <t>Sonar: controle externo automatizado do executivo municipal. Monitora 92 municípios do RJ via MPRJ. Selecionada CPSI MPRJ.</t>
+          <t>Pioneira em monitoramento automatizado de dados governamentais (Legislativo, Executivo, Judiciário). 4M+ proposições monitoradas. ~890 fontes de Diários Oficiais. IA com termômetro de aprovação de PLs (&gt;98% acurácia). Única com 100% de cobertura das Assembleias Estaduais. Ranking 100 Open Startups, Mapa GovTech. Cubo Itaú, Inovabra, Distrito.</t>
         </is>
       </c>
       <c r="I7" s="17" t="inlineStr">
         <is>
-          <t>Contrato CPSI</t>
-        </is>
-      </c>
-      <c r="J7" s="13" t="inlineStr"/>
+          <t>Watch — inteligência regulatória</t>
+        </is>
+      </c>
+      <c r="J7" s="18" t="inlineStr">
+        <is>
+          <t>✓</t>
+        </is>
+      </c>
     </row>
     <row r="8" ht="48" customHeight="1">
       <c r="A8" s="14" t="inlineStr">
         <is>
-          <t>Prodata Gestão Estratégica</t>
+          <t>Kinebot</t>
         </is>
       </c>
       <c r="B8" s="15" t="inlineStr">
         <is>
-          <t>Módulo Procuradoria / ERP Municipal</t>
+          <t>IA Ergonomia / Saúde do Trabalhador</t>
         </is>
       </c>
       <c r="C8" s="15" t="inlineStr">
         <is>
-          <t>PME</t>
+          <t>Startup</t>
         </is>
       </c>
       <c r="D8" s="15" t="inlineStr">
         <is>
-          <t>Goiânia - GO</t>
+          <t>Curitiba - PR</t>
         </is>
       </c>
       <c r="E8" s="15" t="inlineStr">
@@ -4425,21 +4463,29 @@
       </c>
       <c r="F8" s="15" t="inlineStr">
         <is>
-          <t>Municípios Centro-Oeste</t>
+          <t>Indústria + gov</t>
         </is>
       </c>
       <c r="G8" s="15" t="inlineStr">
         <is>
-          <t>N/D</t>
+          <t>R$3M (Fundo GovTech)</t>
         </is>
       </c>
       <c r="H8" s="15" t="inlineStr">
         <is>
-          <t>Módulo procuradoria integrado ao ERP municipal Prodata. Gestão de contencioso, consultivo e execução fiscal para prefeituras de pequeno e médio porte.</t>
-        </is>
-      </c>
-      <c r="I8" s="15" t="inlineStr"/>
-      <c r="J8" s="15" t="inlineStr"/>
+          <t>IA para análises ergonômicas e psicossociais via visão computacional. Clientes: Marfrig, P&amp;G, Electrolux. 8º investimento do Fundo GovTech (KPTL+Cedro), R$3M em fev/2026. Foco em saúde do trabalhador para setor público e privado. Expansão global planejada.</t>
+        </is>
+      </c>
+      <c r="I8" s="16" t="inlineStr">
+        <is>
+          <t>Portfólio KPTL+Cedro</t>
+        </is>
+      </c>
+      <c r="J8" s="19" t="inlineStr">
+        <is>
+          <t>✓</t>
+        </is>
+      </c>
     </row>
   </sheetData>
   <mergeCells count="1">
@@ -4450,6 +4496,418 @@
 </file>
 
 <file path=xl/worksheets/sheet7.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="A1:J9"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <cols>
+    <col width="28" customWidth="1" min="1" max="1"/>
+    <col width="32" customWidth="1" min="2" max="2"/>
+    <col width="20" customWidth="1" min="3" max="3"/>
+    <col width="24" customWidth="1" min="4" max="4"/>
+    <col width="10" customWidth="1" min="5" max="5"/>
+    <col width="28" customWidth="1" min="6" max="6"/>
+    <col width="20" customWidth="1" min="7" max="7"/>
+    <col width="60" customWidth="1" min="8" max="8"/>
+    <col width="28" customWidth="1" min="9" max="9"/>
+    <col width="6" customWidth="1" min="10" max="10"/>
+  </cols>
+  <sheetData>
+    <row r="1" ht="28" customHeight="1">
+      <c r="A1" s="24" t="inlineStr">
+        <is>
+          <t>⚖️ Procuradorias &amp; Jurídico — Radar GovTech Brasil 2025/2026</t>
+        </is>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" s="11" t="inlineStr">
+        <is>
+          <t>Nome</t>
+        </is>
+      </c>
+      <c r="B2" s="11" t="inlineStr">
+        <is>
+          <t>Subsegmento</t>
+        </is>
+      </c>
+      <c r="C2" s="11" t="inlineStr">
+        <is>
+          <t>Porte</t>
+        </is>
+      </c>
+      <c r="D2" s="11" t="inlineStr">
+        <is>
+          <t>Localização</t>
+        </is>
+      </c>
+      <c r="E2" s="11" t="inlineStr">
+        <is>
+          <t>Fundação</t>
+        </is>
+      </c>
+      <c r="F2" s="11" t="inlineStr">
+        <is>
+          <t>Presença</t>
+        </is>
+      </c>
+      <c r="G2" s="11" t="inlineStr">
+        <is>
+          <t>Capital / Receita</t>
+        </is>
+      </c>
+      <c r="H2" s="11" t="inlineStr">
+        <is>
+          <t>Análise / Nota</t>
+        </is>
+      </c>
+      <c r="I2" s="11" t="inlineStr">
+        <is>
+          <t>Alerta M&amp;A</t>
+        </is>
+      </c>
+      <c r="J2" s="11" t="inlineStr">
+        <is>
+          <t>Novo</t>
+        </is>
+      </c>
+    </row>
+    <row r="3" ht="48" customHeight="1">
+      <c r="A3" s="12" t="inlineStr">
+        <is>
+          <t>MinutaIA (jAI)</t>
+        </is>
+      </c>
+      <c r="B3" s="13" t="inlineStr">
+        <is>
+          <t>IA Jurídica / Judicial</t>
+        </is>
+      </c>
+      <c r="C3" s="13" t="inlineStr">
+        <is>
+          <t>Startup</t>
+        </is>
+      </c>
+      <c r="D3" s="13" t="inlineStr">
+        <is>
+          <t>Belo Horizonte - MG</t>
+        </is>
+      </c>
+      <c r="E3" s="13" t="inlineStr">
+        <is>
+          <t>2025</t>
+        </is>
+      </c>
+      <c r="F3" s="13" t="inlineStr">
+        <is>
+          <t>7 tribunais | 100k+ usr</t>
+        </is>
+      </c>
+      <c r="G3" s="13" t="inlineStr">
+        <is>
+          <t>N/D</t>
+        </is>
+      </c>
+      <c r="H3" s="13" t="inlineStr">
+        <is>
+          <t>10M+ minutas geradas. TJRS, STM, TRE-PB/BA, Tocantins. CNJ Resolução 615/2025. Exportou para a Argentina.</t>
+        </is>
+      </c>
+      <c r="I3" s="17" t="inlineStr">
+        <is>
+          <t>Watch — tração judicial</t>
+        </is>
+      </c>
+      <c r="J3" s="13" t="inlineStr"/>
+    </row>
+    <row r="4" ht="48" customHeight="1">
+      <c r="A4" s="14" t="inlineStr">
+        <is>
+          <t>Attus Procuradoria Digital</t>
+        </is>
+      </c>
+      <c r="B4" s="15" t="inlineStr">
+        <is>
+          <t>IA Contencioso + Consultivo (PGE/PGM)</t>
+        </is>
+      </c>
+      <c r="C4" s="15" t="inlineStr">
+        <is>
+          <t>Scale-up</t>
+        </is>
+      </c>
+      <c r="D4" s="15" t="inlineStr">
+        <is>
+          <t>São Ludgero, SC (Eloware)</t>
+        </is>
+      </c>
+      <c r="E4" s="15" t="inlineStr">
+        <is>
+          <t>~2018</t>
+        </is>
+      </c>
+      <c r="F4" s="15" t="inlineStr">
+        <is>
+          <t>PGE-SP, PGE-BA, PGE-PA, PGM-Palmas</t>
+        </is>
+      </c>
+      <c r="G4" s="15" t="inlineStr">
+        <is>
+          <t>SaaS Oracle Cloud</t>
+        </is>
+      </c>
+      <c r="H4" s="15" t="inlineStr">
+        <is>
+          <t>4,3M+ processos analisados. 73% classificados automaticamente (98,5% acurácia). 642k+ peças geradas por IA. Referência nacional pós PGE-SP.</t>
+        </is>
+      </c>
+      <c r="I4" s="16" t="inlineStr">
+        <is>
+          <t>M&amp;A Watch — líder do segmento</t>
+        </is>
+      </c>
+      <c r="J4" s="15" t="inlineStr"/>
+    </row>
+    <row r="5" ht="48" customHeight="1">
+      <c r="A5" s="12" t="inlineStr">
+        <is>
+          <t>Eicon / Giex</t>
+        </is>
+      </c>
+      <c r="B5" s="13" t="inlineStr">
+        <is>
+          <t>Dívida Ativa / Execução Fiscal</t>
+        </is>
+      </c>
+      <c r="C5" s="13" t="inlineStr">
+        <is>
+          <t>PME</t>
+        </is>
+      </c>
+      <c r="D5" s="13" t="inlineStr">
+        <is>
+          <t>N/D (Brasil)</t>
+        </is>
+      </c>
+      <c r="E5" s="13" t="inlineStr">
+        <is>
+          <t>N/D</t>
+        </is>
+      </c>
+      <c r="F5" s="13" t="inlineStr">
+        <is>
+          <t>PGE e PGM — múltiplos estados</t>
+        </is>
+      </c>
+      <c r="G5" s="13" t="inlineStr">
+        <is>
+          <t>N/D</t>
+        </is>
+      </c>
+      <c r="H5" s="13" t="inlineStr">
+        <is>
+          <t>Giex: perfil completo do devedor. Integração direta com TJs. Automação de CDA, penhoras e prazos. iCad: alvarás e licenças digitais (concorrente da Quasar). +15 produtos para governo.</t>
+        </is>
+      </c>
+      <c r="I5" s="13" t="inlineStr"/>
+      <c r="J5" s="13" t="inlineStr"/>
+    </row>
+    <row r="6" ht="48" customHeight="1">
+      <c r="A6" s="14" t="inlineStr">
+        <is>
+          <t>PGMNET</t>
+        </is>
+      </c>
+      <c r="B6" s="15" t="inlineStr">
+        <is>
+          <t>Gestão Jurídica Municipal + RPA</t>
+        </is>
+      </c>
+      <c r="C6" s="15" t="inlineStr">
+        <is>
+          <t>PME</t>
+        </is>
+      </c>
+      <c r="D6" s="15" t="inlineStr">
+        <is>
+          <t>N/D (Brasil)</t>
+        </is>
+      </c>
+      <c r="E6" s="15" t="inlineStr">
+        <is>
+          <t>N/D</t>
+        </is>
+      </c>
+      <c r="F6" s="15" t="inlineStr">
+        <is>
+          <t>Procuradorias municipais</t>
+        </is>
+      </c>
+      <c r="G6" s="15" t="inlineStr">
+        <is>
+          <t>N/D</t>
+        </is>
+      </c>
+      <c r="H6" s="15" t="inlineStr">
+        <is>
+          <t>RPA integrado para peticionamento automático em qualquer TJ do país. Interface co-desenvolvida com procuradores municipais.</t>
+        </is>
+      </c>
+      <c r="I6" s="15" t="inlineStr"/>
+      <c r="J6" s="15" t="inlineStr"/>
+    </row>
+    <row r="7" ht="48" customHeight="1">
+      <c r="A7" s="12" t="inlineStr">
+        <is>
+          <t>Aetos Tech</t>
+        </is>
+      </c>
+      <c r="B7" s="13" t="inlineStr">
+        <is>
+          <t>IA Anti-fraude Contratos (Prisma)</t>
+        </is>
+      </c>
+      <c r="C7" s="13" t="inlineStr">
+        <is>
+          <t>Startup</t>
+        </is>
+      </c>
+      <c r="D7" s="13" t="inlineStr">
+        <is>
+          <t>N/D (Brasil)</t>
+        </is>
+      </c>
+      <c r="E7" s="13" t="inlineStr">
+        <is>
+          <t>N/D</t>
+        </is>
+      </c>
+      <c r="F7" s="13" t="inlineStr">
+        <is>
+          <t>MPRJ (CPSI 2024)</t>
+        </is>
+      </c>
+      <c r="G7" s="13" t="inlineStr">
+        <is>
+          <t>Contrato CPSI</t>
+        </is>
+      </c>
+      <c r="H7" s="13" t="inlineStr">
+        <is>
+          <t>Prisma: detecção de irregularidades em contratos públicos e lavagem de dinheiro. Cruzamento de bases abertas por IA. Selecionada CPSI MPRJ.</t>
+        </is>
+      </c>
+      <c r="I7" s="17" t="inlineStr">
+        <is>
+          <t>Contrato CPSI</t>
+        </is>
+      </c>
+      <c r="J7" s="13" t="inlineStr"/>
+    </row>
+    <row r="8" ht="48" customHeight="1">
+      <c r="A8" s="14" t="inlineStr">
+        <is>
+          <t>Sumé Tecnologia</t>
+        </is>
+      </c>
+      <c r="B8" s="15" t="inlineStr">
+        <is>
+          <t>Monitoramento Políticas Públicas (Sonar)</t>
+        </is>
+      </c>
+      <c r="C8" s="15" t="inlineStr">
+        <is>
+          <t>Startup</t>
+        </is>
+      </c>
+      <c r="D8" s="15" t="inlineStr">
+        <is>
+          <t>N/D (Brasil)</t>
+        </is>
+      </c>
+      <c r="E8" s="15" t="inlineStr">
+        <is>
+          <t>N/D</t>
+        </is>
+      </c>
+      <c r="F8" s="15" t="inlineStr">
+        <is>
+          <t>MPRJ (CPSI 2024)</t>
+        </is>
+      </c>
+      <c r="G8" s="15" t="inlineStr">
+        <is>
+          <t>Contrato CPSI</t>
+        </is>
+      </c>
+      <c r="H8" s="15" t="inlineStr">
+        <is>
+          <t>Sonar: controle externo automatizado do executivo municipal. Monitora 92 municípios do RJ via MPRJ. Selecionada CPSI MPRJ.</t>
+        </is>
+      </c>
+      <c r="I8" s="16" t="inlineStr">
+        <is>
+          <t>Contrato CPSI</t>
+        </is>
+      </c>
+      <c r="J8" s="15" t="inlineStr"/>
+    </row>
+    <row r="9" ht="48" customHeight="1">
+      <c r="A9" s="12" t="inlineStr">
+        <is>
+          <t>Prodata Gestão Estratégica</t>
+        </is>
+      </c>
+      <c r="B9" s="13" t="inlineStr">
+        <is>
+          <t>Módulo Procuradoria / ERP Municipal</t>
+        </is>
+      </c>
+      <c r="C9" s="13" t="inlineStr">
+        <is>
+          <t>PME</t>
+        </is>
+      </c>
+      <c r="D9" s="13" t="inlineStr">
+        <is>
+          <t>Goiânia - GO</t>
+        </is>
+      </c>
+      <c r="E9" s="13" t="inlineStr">
+        <is>
+          <t>N/D</t>
+        </is>
+      </c>
+      <c r="F9" s="13" t="inlineStr">
+        <is>
+          <t>Municípios Centro-Oeste</t>
+        </is>
+      </c>
+      <c r="G9" s="13" t="inlineStr">
+        <is>
+          <t>N/D</t>
+        </is>
+      </c>
+      <c r="H9" s="13" t="inlineStr">
+        <is>
+          <t>Módulo procuradoria integrado ao ERP municipal Prodata. Gestão de contencioso, consultivo e execução fiscal para prefeituras de pequeno e médio porte.</t>
+        </is>
+      </c>
+      <c r="I9" s="13" t="inlineStr"/>
+      <c r="J9" s="13" t="inlineStr"/>
+    </row>
+  </sheetData>
+  <mergeCells count="1">
+    <mergeCell ref="A1:J1"/>
+  </mergeCells>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet8.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <sheetPr>
     <outlinePr summaryBelow="1" summaryRight="1"/>
@@ -4471,7 +4929,7 @@
   </cols>
   <sheetData>
     <row r="1" ht="28" customHeight="1">
-      <c r="A1" s="24" t="inlineStr">
+      <c r="A1" s="25" t="inlineStr">
         <is>
           <t>📋 Licitações &amp; Compras Públicas — Radar GovTech Brasil 2025/2026</t>
         </is>
@@ -4817,7 +5275,7 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet8.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet9.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <sheetPr>
     <outlinePr summaryBelow="1" summaryRight="1"/>
@@ -4839,7 +5297,7 @@
   </cols>
   <sheetData>
     <row r="1" ht="28" customHeight="1">
-      <c r="A1" s="25" t="inlineStr">
+      <c r="A1" s="26" t="inlineStr">
         <is>
           <t>🏘️ Habitação &amp; Regularização Fundiária — Radar GovTech Brasil 2025/2026</t>
         </is>
@@ -5100,250 +5558,6 @@
         </is>
       </c>
       <c r="J6" s="19" t="inlineStr">
-        <is>
-          <t>✓</t>
-        </is>
-      </c>
-    </row>
-  </sheetData>
-  <mergeCells count="1">
-    <mergeCell ref="A1:J1"/>
-  </mergeCells>
-  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
-</worksheet>
-</file>
-
-<file path=xl/worksheets/sheet9.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
-  <sheetPr>
-    <outlinePr summaryBelow="1" summaryRight="1"/>
-    <pageSetUpPr/>
-  </sheetPr>
-  <dimension ref="A1:J5"/>
-  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
-  <cols>
-    <col width="28" customWidth="1" min="1" max="1"/>
-    <col width="32" customWidth="1" min="2" max="2"/>
-    <col width="20" customWidth="1" min="3" max="3"/>
-    <col width="24" customWidth="1" min="4" max="4"/>
-    <col width="10" customWidth="1" min="5" max="5"/>
-    <col width="28" customWidth="1" min="6" max="6"/>
-    <col width="20" customWidth="1" min="7" max="7"/>
-    <col width="60" customWidth="1" min="8" max="8"/>
-    <col width="28" customWidth="1" min="9" max="9"/>
-    <col width="6" customWidth="1" min="10" max="10"/>
-  </cols>
-  <sheetData>
-    <row r="1" ht="28" customHeight="1">
-      <c r="A1" s="26" t="inlineStr">
-        <is>
-          <t>🌿 Meio Ambiente &amp; Licenciamento — Radar GovTech Brasil 2025/2026</t>
-        </is>
-      </c>
-    </row>
-    <row r="2">
-      <c r="A2" s="11" t="inlineStr">
-        <is>
-          <t>Nome</t>
-        </is>
-      </c>
-      <c r="B2" s="11" t="inlineStr">
-        <is>
-          <t>Subsegmento</t>
-        </is>
-      </c>
-      <c r="C2" s="11" t="inlineStr">
-        <is>
-          <t>Porte</t>
-        </is>
-      </c>
-      <c r="D2" s="11" t="inlineStr">
-        <is>
-          <t>Localização</t>
-        </is>
-      </c>
-      <c r="E2" s="11" t="inlineStr">
-        <is>
-          <t>Fundação</t>
-        </is>
-      </c>
-      <c r="F2" s="11" t="inlineStr">
-        <is>
-          <t>Presença</t>
-        </is>
-      </c>
-      <c r="G2" s="11" t="inlineStr">
-        <is>
-          <t>Capital / Receita</t>
-        </is>
-      </c>
-      <c r="H2" s="11" t="inlineStr">
-        <is>
-          <t>Análise / Nota</t>
-        </is>
-      </c>
-      <c r="I2" s="11" t="inlineStr">
-        <is>
-          <t>Alerta M&amp;A</t>
-        </is>
-      </c>
-      <c r="J2" s="11" t="inlineStr">
-        <is>
-          <t>Novo</t>
-        </is>
-      </c>
-    </row>
-    <row r="3" ht="48" customHeight="1">
-      <c r="A3" s="12" t="inlineStr">
-        <is>
-          <t>eGAC</t>
-        </is>
-      </c>
-      <c r="B3" s="13" t="inlineStr">
-        <is>
-          <t>Licenciamento Ambiental Municipal Digital</t>
-        </is>
-      </c>
-      <c r="C3" s="13" t="inlineStr">
-        <is>
-          <t>Startup</t>
-        </is>
-      </c>
-      <c r="D3" s="13" t="inlineStr">
-        <is>
-          <t>Bahia</t>
-        </is>
-      </c>
-      <c r="E3" s="13" t="inlineStr">
-        <is>
-          <t>~2021</t>
-        </is>
-      </c>
-      <c r="F3" s="13" t="inlineStr">
-        <is>
-          <t>Consórcios intermunicipais BA</t>
-        </is>
-      </c>
-      <c r="G3" s="13" t="inlineStr">
-        <is>
-          <t>N/D</t>
-        </is>
-      </c>
-      <c r="H3" s="13" t="inlineStr">
-        <is>
-          <t>SaaS de licenciamento ambiental municipal 100% digital. Integra SINAFLOR, GEOBAHIA, SEMA-BA e CEPRAM. 70% redução de custos declarada, onboarding em 30 dias. Operando via consórcios: CDS Bacia do Paramirim, CONVALE e CONSID Oeste da BA. Conformidade com Resolução CEPRAM 4.327/13.</t>
-        </is>
-      </c>
-      <c r="I3" s="17" t="inlineStr">
-        <is>
-          <t>Watch — lic. ambiental nicho virgem</t>
-        </is>
-      </c>
-      <c r="J3" s="18" t="inlineStr">
-        <is>
-          <t>✓</t>
-        </is>
-      </c>
-    </row>
-    <row r="4" ht="48" customHeight="1">
-      <c r="A4" s="14" t="inlineStr">
-        <is>
-          <t>TUXTU</t>
-        </is>
-      </c>
-      <c r="B4" s="15" t="inlineStr">
-        <is>
-          <t>Licenciamento + Arborização + Crédito de Carbono</t>
-        </is>
-      </c>
-      <c r="C4" s="15" t="inlineStr">
-        <is>
-          <t>Startup</t>
-        </is>
-      </c>
-      <c r="D4" s="15" t="inlineStr">
-        <is>
-          <t>Brasil</t>
-        </is>
-      </c>
-      <c r="E4" s="15" t="inlineStr">
-        <is>
-          <t>~2022</t>
-        </is>
-      </c>
-      <c r="F4" s="15" t="inlineStr">
-        <is>
-          <t>Municípios (via órgãos ambientais)</t>
-        </is>
-      </c>
-      <c r="G4" s="15" t="inlineStr">
-        <is>
-          <t>N/D</t>
-        </is>
-      </c>
-      <c r="H4" s="15" t="inlineStr">
-        <is>
-          <t>3 módulos SaaS para Secretarias de Meio Ambiente: SIBLAM (licenciamento com bio-algoritmo e método Battelle EES — reduz subjetividade do analista), SIGAU (arborização urbana com participação cidadã), SICCA (crédito de carbono). Propõe padronização nacional do licenciamento. CEO: Marcelo Creão. Associada ABES.</t>
-        </is>
-      </c>
-      <c r="I4" s="16" t="inlineStr">
-        <is>
-          <t>Watch — 3 verticais ambientais</t>
-        </is>
-      </c>
-      <c r="J4" s="19" t="inlineStr">
-        <is>
-          <t>✓</t>
-        </is>
-      </c>
-    </row>
-    <row r="5" ht="48" customHeight="1">
-      <c r="A5" s="12" t="inlineStr">
-        <is>
-          <t>Retech Recycle</t>
-        </is>
-      </c>
-      <c r="B5" s="13" t="inlineStr">
-        <is>
-          <t>Gestão de Resíduos Sólidos / Rastreabilidade IoT</t>
-        </is>
-      </c>
-      <c r="C5" s="13" t="inlineStr">
-        <is>
-          <t>Startup early-stage</t>
-        </is>
-      </c>
-      <c r="D5" s="13" t="inlineStr">
-        <is>
-          <t>São José dos Campos - SP</t>
-        </is>
-      </c>
-      <c r="E5" s="13" t="inlineStr">
-        <is>
-          <t>2024</t>
-        </is>
-      </c>
-      <c r="F5" s="13" t="inlineStr">
-        <is>
-          <t>N/D (early-stage)</t>
-        </is>
-      </c>
-      <c r="G5" s="13" t="inlineStr">
-        <is>
-          <t>N/D</t>
-        </is>
-      </c>
-      <c r="H5" s="13" t="inlineStr">
-        <is>
-          <t>Plataforma + hardware IoT proprietário (H-SAT) para rastreabilidade de resíduos sólidos do ponto de coleta ao destino final. Gera documentos auditáveis com fotos georreferenciadas, telemetria e carimbos de tempo. Conformidade PNRS. Modelo híbrido: software + presença onsite. PIT-SJC. Fundada jun/2024.</t>
-        </is>
-      </c>
-      <c r="I5" s="17" t="inlineStr">
-        <is>
-          <t>Watch — PNRS compliance IoT</t>
-        </is>
-      </c>
-      <c r="J5" s="18" t="inlineStr">
         <is>
           <t>✓</t>
         </is>

</xml_diff>

<commit_message>
v11: Datapolicy adicionada; Portal de Compras atualizado
- Datapolicy (Brasília): inteligência regulatória B2B, portfólio Cedro Capital
  FIP VBC, disponível para M&A sem mandatada — adicionada em IA Gov
- Portal de Compras Públicas: confirmado portfólio Cedro Capital (FIP VBC),
  alerta atualizado para M&A Watch

Co-Authored-By: Claude Sonnet 4.6 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/Radar_GovTechs_Brasil_2026.xlsx
+++ b/Radar_GovTechs_Brasil_2026.xlsx
@@ -647,7 +647,7 @@
     <row r="1" ht="32" customHeight="1">
       <c r="A1" s="1" t="inlineStr">
         <is>
-          <t>🇧🇷 Radar GovTech Brasil 2025/2026 — DLG · Maio 2026 · v10</t>
+          <t>🇧🇷 Radar GovTech Brasil 2025/2026 — DLG · Maio 2026 · v11</t>
         </is>
       </c>
     </row>
@@ -710,7 +710,7 @@
         </is>
       </c>
       <c r="B8" s="4" t="n">
-        <v>6</v>
+        <v>7</v>
       </c>
     </row>
     <row r="9">
@@ -780,7 +780,7 @@
         </is>
       </c>
       <c r="B15" s="6" t="n">
-        <v>69</v>
+        <v>70</v>
       </c>
     </row>
     <row r="16">
@@ -790,7 +790,7 @@
         </is>
       </c>
       <c r="B16" s="8" t="n">
-        <v>67</v>
+        <v>68</v>
       </c>
     </row>
     <row r="18">
@@ -4121,7 +4121,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:J8"/>
+  <dimension ref="A1:J9"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="28" customWidth="1" min="1" max="1"/>
@@ -4438,50 +4438,102 @@
     <row r="8" ht="48" customHeight="1">
       <c r="A8" s="14" t="inlineStr">
         <is>
+          <t>Datapolicy</t>
+        </is>
+      </c>
+      <c r="B8" s="15" t="inlineStr">
+        <is>
+          <t>Inteligência Regulatória B2B / RelGov</t>
+        </is>
+      </c>
+      <c r="C8" s="15" t="inlineStr">
+        <is>
+          <t>Startup</t>
+        </is>
+      </c>
+      <c r="D8" s="15" t="inlineStr">
+        <is>
+          <t>Brasília - DF</t>
+        </is>
+      </c>
+      <c r="E8" s="15" t="inlineStr">
+        <is>
+          <t>N/D</t>
+        </is>
+      </c>
+      <c r="F8" s="15" t="inlineStr">
+        <is>
+          <t>+80 clientes | 200+ fontes</t>
+        </is>
+      </c>
+      <c r="G8" s="15" t="inlineStr">
+        <is>
+          <t>N/D</t>
+        </is>
+      </c>
+      <c r="H8" s="15" t="inlineStr">
+        <is>
+          <t>Plataforma de inteligência regulatória voltada para corporações e escritórios de RelGov: monitora PLs, decretos, normas de agências reguladoras e órgãos de controle (federal, estadual, municipal). +16M proposições e atos indexados. Diferente da Inteligov (B2G): Datapolicy é B2B — vende para empresas que monitoram o governo. Portfólio Cedro Capital (FIP VBC) — disponível para M&amp;A, sem mandatada.</t>
+        </is>
+      </c>
+      <c r="I8" s="16" t="inlineStr">
+        <is>
+          <t>M&amp;A Watch — portfólio Cedro</t>
+        </is>
+      </c>
+      <c r="J8" s="19" t="inlineStr">
+        <is>
+          <t>✓</t>
+        </is>
+      </c>
+    </row>
+    <row r="9" ht="48" customHeight="1">
+      <c r="A9" s="12" t="inlineStr">
+        <is>
           <t>Kinebot</t>
         </is>
       </c>
-      <c r="B8" s="15" t="inlineStr">
+      <c r="B9" s="13" t="inlineStr">
         <is>
           <t>IA Ergonomia / Saúde do Trabalhador</t>
         </is>
       </c>
-      <c r="C8" s="15" t="inlineStr">
+      <c r="C9" s="13" t="inlineStr">
         <is>
           <t>Startup</t>
         </is>
       </c>
-      <c r="D8" s="15" t="inlineStr">
+      <c r="D9" s="13" t="inlineStr">
         <is>
           <t>Curitiba - PR</t>
         </is>
       </c>
-      <c r="E8" s="15" t="inlineStr">
-        <is>
-          <t>N/D</t>
-        </is>
-      </c>
-      <c r="F8" s="15" t="inlineStr">
+      <c r="E9" s="13" t="inlineStr">
+        <is>
+          <t>N/D</t>
+        </is>
+      </c>
+      <c r="F9" s="13" t="inlineStr">
         <is>
           <t>Indústria + gov</t>
         </is>
       </c>
-      <c r="G8" s="15" t="inlineStr">
+      <c r="G9" s="13" t="inlineStr">
         <is>
           <t>R$3M (Fundo GovTech)</t>
         </is>
       </c>
-      <c r="H8" s="15" t="inlineStr">
+      <c r="H9" s="13" t="inlineStr">
         <is>
           <t>IA para análises ergonômicas e psicossociais via visão computacional. Clientes: Marfrig, P&amp;G, Electrolux. 8º investimento do Fundo GovTech (KPTL+Cedro), R$3M em fev/2026. Foco em saúde do trabalhador para setor público e privado. Expansão global planejada.</t>
         </is>
       </c>
-      <c r="I8" s="16" t="inlineStr">
+      <c r="I9" s="17" t="inlineStr">
         <is>
           <t>Portfólio KPTL+Cedro</t>
         </is>
       </c>
-      <c r="J8" s="19" t="inlineStr">
+      <c r="J9" s="18" t="inlineStr">
         <is>
           <t>✓</t>
         </is>
@@ -5025,12 +5077,12 @@
       </c>
       <c r="H3" s="13" t="inlineStr">
         <is>
-          <t>40%+ dos municípios brasileiros. Fundadores: Leonardo + Bruno Ladeira (Ecustomize). 35% crescimento anual. Marketplace B2G de referência nacional.</t>
+          <t>40%+ dos municípios brasileiros. Fundadores: Leonardo + Bruno Ladeira (Ecustomize). 35% crescimento anual. Marketplace B2G de referência nacional. Portfólio Cedro Capital (FIP Venture Brasil Central) — disponível para M&amp;A, sem mandatada.</t>
         </is>
       </c>
       <c r="I3" s="17" t="inlineStr">
         <is>
-          <t>Referência nacional</t>
+          <t>M&amp;A Watch — portfólio Cedro</t>
         </is>
       </c>
       <c r="J3" s="13" t="inlineStr"/>

</xml_diff>

<commit_message>
Gove: atualização completa de produto e cases (gove.digital)
- Subseg: Analytics Financeiro → CRM Municipal / Cobrança & Automação via IA
- Produto atual: CRM gov + chatbot WhatsApp verificado + automação IA + enriquecimento cadastral
- Presença ampliada: SP, MG, AM, BA, RJ, TO+
- Cases: Salvador BA (R$29M), Araguaína TO (ROI 32x, 1º CPSI), Areal RJ (+135% DAtiva)
- CEO: Rodolfo Fiori (MIT); CTO: Dayanne Ramos

Co-Authored-By: Claude Sonnet 4.6 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/Radar_GovTechs_Brasil_2026.xlsx
+++ b/Radar_GovTechs_Brasil_2026.xlsx
@@ -3103,7 +3103,7 @@
       </c>
       <c r="B8" s="15" t="inlineStr">
         <is>
-          <t>Analytics Financeiro Municipal</t>
+          <t>CRM Municipal / Cobrança &amp; Automação via IA</t>
         </is>
       </c>
       <c r="C8" s="15" t="inlineStr">
@@ -3123,7 +3123,7 @@
       </c>
       <c r="F8" s="15" t="inlineStr">
         <is>
-          <t>SP, MG, RS, SC, ES+</t>
+          <t>SP, MG, AM, BA, RJ, TO+</t>
         </is>
       </c>
       <c r="G8" s="15" t="inlineStr">
@@ -3133,10 +3133,14 @@
       </c>
       <c r="H8" s="15" t="inlineStr">
         <is>
-          <t>Analytics IA para finanças públicas: identifica ineficiências em receitas/despesas municipais. Aporte Astella. BrazilLAB Turma 7.</t>
-        </is>
-      </c>
-      <c r="I8" s="15" t="inlineStr"/>
+          <t>Único CRM para setor público com chatbot WhatsApp verificado (login Gov.br), automação de serviços via IA e enriquecimento cadastral contínuo. Foco em arrecadação: cobrança ativa por WhatsApp/SMS/email/Domicílio Eletrônico, cruzamento com Receita Federal. CEO: Rodolfo Fiori (MIT). CTO: Dayanne Ramos. Cases: Salvador BA (R$29M recuperação crédito tributário), Araguaína TO (ROI 32x — R$300k→R$9,6M, 1º CPSI do país), Areal RJ (+135% arrecadação dívida ativa), Manaus AM, Pindamonhangaba SP. Prêmio InovaCidade 2023. Aporte Astella Series A (R$8M, 2020). BrazilLAB Turma 7.</t>
+        </is>
+      </c>
+      <c r="I8" s="16" t="inlineStr">
+        <is>
+          <t>M&amp;A Watch — tração comprovada</t>
+        </is>
+      </c>
       <c r="J8" s="15" t="inlineStr"/>
     </row>
     <row r="9" ht="48" customHeight="1">

</xml_diff>

<commit_message>
Badge NOVO: resetado para empresas anteriores, mantido apenas na entrada atual
Co-Authored-By: Claude Sonnet 4.6 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/Radar_GovTechs_Brasil_2026.xlsx
+++ b/Radar_GovTechs_Brasil_2026.xlsx
@@ -177,7 +177,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="34">
+  <cellXfs count="33">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center"/>
@@ -224,12 +224,6 @@
     <xf numFmtId="0" fontId="5" fillId="5" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment vertical="top" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="6" fillId="5" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment vertical="top" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="6" fillId="6" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment vertical="top" wrapText="1"/>
-    </xf>
     <xf numFmtId="0" fontId="4" fillId="7" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center"/>
     </xf>
@@ -241,6 +235,9 @@
     </xf>
     <xf numFmtId="0" fontId="4" fillId="9" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="6" fillId="6" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment vertical="top" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="4" fillId="10" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center"/>
@@ -833,7 +830,7 @@
   </cols>
   <sheetData>
     <row r="1" ht="28" customHeight="1">
-      <c r="A1" s="27" t="inlineStr">
+      <c r="A1" s="26" t="inlineStr">
         <is>
           <t>🌿 Meio Ambiente &amp; Licenciamento — Radar GovTech Brasil 2025/2026</t>
         </is>
@@ -937,11 +934,7 @@
           <t>Watch — lic. ambiental nicho virgem</t>
         </is>
       </c>
-      <c r="J3" s="18" t="inlineStr">
-        <is>
-          <t>✓</t>
-        </is>
-      </c>
+      <c r="J3" s="13" t="inlineStr"/>
     </row>
     <row r="4" ht="48" customHeight="1">
       <c r="A4" s="14" t="inlineStr">
@@ -989,11 +982,7 @@
           <t>Watch — 3 verticais ambientais</t>
         </is>
       </c>
-      <c r="J4" s="19" t="inlineStr">
-        <is>
-          <t>✓</t>
-        </is>
-      </c>
+      <c r="J4" s="15" t="inlineStr"/>
     </row>
     <row r="5" ht="48" customHeight="1">
       <c r="A5" s="12" t="inlineStr">
@@ -1041,11 +1030,7 @@
           <t>Watch — PNRS compliance IoT</t>
         </is>
       </c>
-      <c r="J5" s="18" t="inlineStr">
-        <is>
-          <t>✓</t>
-        </is>
-      </c>
+      <c r="J5" s="13" t="inlineStr"/>
     </row>
   </sheetData>
   <mergeCells count="1">
@@ -1077,7 +1062,7 @@
   </cols>
   <sheetData>
     <row r="1" ht="28" customHeight="1">
-      <c r="A1" s="28" t="inlineStr">
+      <c r="A1" s="27" t="inlineStr">
         <is>
           <t>🏙️ Smart Cities &amp; Mobilidade — Radar GovTech Brasil 2025/2026</t>
         </is>
@@ -1181,11 +1166,7 @@
           <t>Watch — padrão FIWARE em SC</t>
         </is>
       </c>
-      <c r="J3" s="18" t="inlineStr">
-        <is>
-          <t>✓</t>
-        </is>
-      </c>
+      <c r="J3" s="13" t="inlineStr"/>
     </row>
     <row r="4" ht="48" customHeight="1">
       <c r="A4" s="14" t="inlineStr">
@@ -1233,11 +1214,7 @@
           <t>Watch — mobilidade pública IA</t>
         </is>
       </c>
-      <c r="J4" s="19" t="inlineStr">
-        <is>
-          <t>✓</t>
-        </is>
-      </c>
+      <c r="J4" s="15" t="inlineStr"/>
     </row>
   </sheetData>
   <mergeCells count="1">
@@ -1269,7 +1246,7 @@
   </cols>
   <sheetData>
     <row r="1" ht="28" customHeight="1">
-      <c r="A1" s="29" t="inlineStr">
+      <c r="A1" s="28" t="inlineStr">
         <is>
           <t>🛡️ Segurança Pública &amp; Infraestrutura — Radar GovTech Brasil 2025/2026</t>
         </is>
@@ -1553,11 +1530,7 @@
           <t>Portfólio KPTL</t>
         </is>
       </c>
-      <c r="J7" s="18" t="inlineStr">
-        <is>
-          <t>✓</t>
-        </is>
-      </c>
+      <c r="J7" s="13" t="inlineStr"/>
     </row>
     <row r="8" ht="48" customHeight="1">
       <c r="A8" s="14" t="inlineStr">
@@ -1673,39 +1646,39 @@
   </cols>
   <sheetData>
     <row r="1" ht="28" customHeight="1">
-      <c r="A1" s="30" t="inlineStr">
+      <c r="A1" s="29" t="inlineStr">
         <is>
           <t>💰 Aportes &amp; Investimentos — Radar GovTech Brasil 2025/2026</t>
         </is>
       </c>
     </row>
     <row r="2">
-      <c r="A2" s="31" t="inlineStr">
+      <c r="A2" s="30" t="inlineStr">
         <is>
           <t>Empresa / Investidor</t>
         </is>
       </c>
-      <c r="B2" s="31" t="inlineStr">
+      <c r="B2" s="30" t="inlineStr">
         <is>
           <t>Tipo</t>
         </is>
       </c>
-      <c r="C2" s="31" t="inlineStr">
+      <c r="C2" s="30" t="inlineStr">
         <is>
           <t>Valor</t>
         </is>
       </c>
-      <c r="D2" s="31" t="inlineStr">
+      <c r="D2" s="30" t="inlineStr">
         <is>
           <t>Data</t>
         </is>
       </c>
-      <c r="E2" s="31" t="inlineStr">
+      <c r="E2" s="30" t="inlineStr">
         <is>
           <t>Segmento</t>
         </is>
       </c>
-      <c r="F2" s="31" t="inlineStr">
+      <c r="F2" s="30" t="inlineStr">
         <is>
           <t>Descrição</t>
         </is>
@@ -1744,32 +1717,32 @@
       </c>
     </row>
     <row r="4" ht="48" customHeight="1">
-      <c r="A4" s="32" t="inlineStr">
+      <c r="A4" s="31" t="inlineStr">
         <is>
           <t>Aprova Digital — Astella + BB/VOX</t>
         </is>
       </c>
-      <c r="B4" s="33" t="inlineStr">
+      <c r="B4" s="32" t="inlineStr">
         <is>
           <t>Aporte Seed</t>
         </is>
       </c>
-      <c r="C4" s="33" t="inlineStr">
+      <c r="C4" s="32" t="inlineStr">
         <is>
           <t>R$ 22,5M</t>
         </is>
       </c>
-      <c r="D4" s="33" t="inlineStr">
+      <c r="D4" s="32" t="inlineStr">
         <is>
           <t>2022</t>
         </is>
       </c>
-      <c r="E4" s="33" t="inlineStr">
+      <c r="E4" s="32" t="inlineStr">
         <is>
           <t>Gestão Pública Municipal</t>
         </is>
       </c>
-      <c r="F4" s="33" t="inlineStr">
+      <c r="F4" s="32" t="inlineStr">
         <is>
           <t>Rodada liderada por Astella e VOX Capital (CVC do Banco do Brasil), com CAF e Endeavor. Maior aporte da história das GovTechs da América Latina na época. 120+ cidades, 21M de brasileiros impactados.</t>
         </is>
@@ -1808,32 +1781,32 @@
       </c>
     </row>
     <row r="6" ht="48" customHeight="1">
-      <c r="A6" s="32" t="inlineStr">
+      <c r="A6" s="31" t="inlineStr">
         <is>
           <t>Portabilis — Yunus Negócios Sociais</t>
         </is>
       </c>
-      <c r="B6" s="33" t="inlineStr">
+      <c r="B6" s="32" t="inlineStr">
         <is>
           <t>Aporte de impacto</t>
         </is>
       </c>
-      <c r="C6" s="33" t="inlineStr">
+      <c r="C6" s="32" t="inlineStr">
         <is>
           <t>Até R$ 2M</t>
         </is>
       </c>
-      <c r="D6" s="33" t="inlineStr">
+      <c r="D6" s="32" t="inlineStr">
         <is>
           <t>2023</t>
         </is>
       </c>
-      <c r="E6" s="33" t="inlineStr">
+      <c r="E6" s="32" t="inlineStr">
         <is>
           <t>Educação Pública</t>
         </is>
       </c>
-      <c r="F6" s="33" t="inlineStr">
+      <c r="F6" s="32" t="inlineStr">
         <is>
           <t>R$800k já desembolsados. Valida modelo de negócio social. Meta: 1,5M alunos até 2027.</t>
         </is>
@@ -1872,32 +1845,32 @@
       </c>
     </row>
     <row r="8" ht="48" customHeight="1">
-      <c r="A8" s="32" t="inlineStr">
+      <c r="A8" s="31" t="inlineStr">
         <is>
           <t>GOVBR — Volaris Group (Constellation Software)</t>
         </is>
       </c>
-      <c r="B8" s="33" t="inlineStr">
+      <c r="B8" s="32" t="inlineStr">
         <is>
           <t>Aquisição (M&amp;A)</t>
         </is>
       </c>
-      <c r="C8" s="33" t="inlineStr">
-        <is>
-          <t>N/D</t>
-        </is>
-      </c>
-      <c r="D8" s="33" t="inlineStr">
+      <c r="C8" s="32" t="inlineStr">
+        <is>
+          <t>N/D</t>
+        </is>
+      </c>
+      <c r="D8" s="32" t="inlineStr">
         <is>
           <t>mai/2023</t>
         </is>
       </c>
-      <c r="E8" s="33" t="inlineStr">
+      <c r="E8" s="32" t="inlineStr">
         <is>
           <t>Gestão Pública Municipal</t>
         </is>
       </c>
-      <c r="F8" s="33" t="inlineStr">
+      <c r="F8" s="32" t="inlineStr">
         <is>
           <t>Volaris adquire a GovernançaBrasil (GOVBR), ERP municipal com 35 anos de atuação. Fundador: Roberto Coelho. Plataforma Cidade 360, 24 módulos. Presença em RS, SC, SP, PR, RJ, ES, MG, MS, PE. Descrita como 'aquisição de grande porte' pela Volaris.</t>
         </is>
@@ -1936,32 +1909,32 @@
       </c>
     </row>
     <row r="10" ht="48" customHeight="1">
-      <c r="A10" s="32" t="inlineStr">
+      <c r="A10" s="31" t="inlineStr">
         <is>
           <t>i4Sea — Fundo GovTech KPTL</t>
         </is>
       </c>
-      <c r="B10" s="33" t="inlineStr">
+      <c r="B10" s="32" t="inlineStr">
         <is>
           <t>Aporte</t>
         </is>
       </c>
-      <c r="C10" s="33" t="inlineStr">
+      <c r="C10" s="32" t="inlineStr">
         <is>
           <t>R$ 7,5M</t>
         </is>
       </c>
-      <c r="D10" s="33" t="inlineStr">
+      <c r="D10" s="32" t="inlineStr">
         <is>
           <t>2024</t>
         </is>
       </c>
-      <c r="E10" s="33" t="inlineStr">
+      <c r="E10" s="32" t="inlineStr">
         <is>
           <t>Infraestrutura / Clima</t>
         </is>
       </c>
-      <c r="F10" s="33" t="inlineStr">
+      <c r="F10" s="32" t="inlineStr">
         <is>
           <t>Previsões microclimáticas para portos e setor elétrico. Portfólio Fundo GovTech KPTL.</t>
         </is>
@@ -2000,32 +1973,32 @@
       </c>
     </row>
     <row r="12" ht="48" customHeight="1">
-      <c r="A12" s="32" t="inlineStr">
+      <c r="A12" s="31" t="inlineStr">
         <is>
           <t>IDS — Volaris Group (Constellation Software)</t>
         </is>
       </c>
-      <c r="B12" s="33" t="inlineStr">
+      <c r="B12" s="32" t="inlineStr">
         <is>
           <t>Aquisição (M&amp;A)</t>
         </is>
       </c>
-      <c r="C12" s="33" t="inlineStr">
-        <is>
-          <t>N/D</t>
-        </is>
-      </c>
-      <c r="D12" s="33" t="inlineStr">
+      <c r="C12" s="32" t="inlineStr">
+        <is>
+          <t>N/D</t>
+        </is>
+      </c>
+      <c r="D12" s="32" t="inlineStr">
         <is>
           <t>ago/2024</t>
         </is>
       </c>
-      <c r="E12" s="33" t="inlineStr">
+      <c r="E12" s="32" t="inlineStr">
         <is>
           <t>Saúde / Educação / Assistência Social</t>
         </is>
       </c>
-      <c r="F12" s="33" t="inlineStr">
+      <c r="F12" s="32" t="inlineStr">
         <is>
           <t>Volaris adquire a IDS (Pato Branco, PR), fornecedora de software para municípios nas áreas de saúde, assistência social, educação e cidadão. Fundada em 2003, 112 funcionários. CEO: Mauri Dengo. Opera de forma independente dentro do portfólio Volaris Latam &amp; Ibéria.</t>
         </is>
@@ -2064,32 +2037,32 @@
       </c>
     </row>
     <row r="14" ht="48" customHeight="1">
-      <c r="A14" s="32" t="inlineStr">
+      <c r="A14" s="31" t="inlineStr">
         <is>
           <t>1Doc — Softplan (100%)</t>
         </is>
       </c>
-      <c r="B14" s="33" t="inlineStr">
+      <c r="B14" s="32" t="inlineStr">
         <is>
           <t>Aquisição (M&amp;A)</t>
         </is>
       </c>
-      <c r="C14" s="33" t="inlineStr">
-        <is>
-          <t>N/D</t>
-        </is>
-      </c>
-      <c r="D14" s="33" t="inlineStr">
+      <c r="C14" s="32" t="inlineStr">
+        <is>
+          <t>N/D</t>
+        </is>
+      </c>
+      <c r="D14" s="32" t="inlineStr">
         <is>
           <t>abr/2025</t>
         </is>
       </c>
-      <c r="E14" s="33" t="inlineStr">
+      <c r="E14" s="32" t="inlineStr">
         <is>
           <t>Digitalização / Gestão Municipal</t>
         </is>
       </c>
-      <c r="F14" s="33" t="inlineStr">
+      <c r="F14" s="32" t="inlineStr">
         <is>
           <t>Softplan adquire 100% da 1Doc, govtech de digitalização de processos e atendimento ao cidadão em prefeituras. Jornada: aporte 2017 → maioria 2019 → 100% abr/2025. CAGR de 75% (2019–2025). Fundada 2014, 1.000 entidades públicas, 22M brasileiros impactados, 141 colaboradores.</t>
         </is>
@@ -2128,32 +2101,32 @@
       </c>
     </row>
     <row r="16" ht="48" customHeight="1">
-      <c r="A16" s="32" t="inlineStr">
+      <c r="A16" s="31" t="inlineStr">
         <is>
           <t>Jovens Gênios — Fundo GovTech+DOMO</t>
         </is>
       </c>
-      <c r="B16" s="33" t="inlineStr">
+      <c r="B16" s="32" t="inlineStr">
         <is>
           <t>Aporte Seed</t>
         </is>
       </c>
-      <c r="C16" s="33" t="inlineStr">
+      <c r="C16" s="32" t="inlineStr">
         <is>
           <t>R$ 11,8M</t>
         </is>
       </c>
-      <c r="D16" s="33" t="inlineStr">
+      <c r="D16" s="32" t="inlineStr">
         <is>
           <t>mar/2026</t>
         </is>
       </c>
-      <c r="E16" s="33" t="inlineStr">
+      <c r="E16" s="32" t="inlineStr">
         <is>
           <t>Educação Pública</t>
         </is>
       </c>
-      <c r="F16" s="33" t="inlineStr">
+      <c r="F16" s="32" t="inlineStr">
         <is>
           <t>Rodada seed liderada pelo Fundo GovTech (KPTL+Cedro), com DOMO.VC, Criabiz Ventures e Rosey Ventures (Grupo Marista). 90% dos alunos em escolas públicas. Meta: 10M alunos até 2030.</t>
         </is>
@@ -2653,11 +2626,7 @@
           <t>Watch — SIAFIC driver</t>
         </is>
       </c>
-      <c r="J11" s="18" t="inlineStr">
-        <is>
-          <t>✓</t>
-        </is>
-      </c>
+      <c r="J11" s="13" t="inlineStr"/>
     </row>
     <row r="12" ht="48" customHeight="1">
       <c r="A12" s="14" t="inlineStr">
@@ -2705,11 +2674,7 @@
           <t>Portfólio KPTL+Cedro</t>
         </is>
       </c>
-      <c r="J12" s="19" t="inlineStr">
-        <is>
-          <t>✓</t>
-        </is>
-      </c>
+      <c r="J12" s="15" t="inlineStr"/>
     </row>
     <row r="13" ht="48" customHeight="1">
       <c r="A13" s="12" t="inlineStr">
@@ -2757,11 +2722,7 @@
           <t>Watch — urbanismo digital</t>
         </is>
       </c>
-      <c r="J13" s="18" t="inlineStr">
-        <is>
-          <t>✓</t>
-        </is>
-      </c>
+      <c r="J13" s="13" t="inlineStr"/>
     </row>
   </sheetData>
   <mergeCells count="1">
@@ -2793,7 +2754,7 @@
   </cols>
   <sheetData>
     <row r="1" ht="28" customHeight="1">
-      <c r="A1" s="20" t="inlineStr">
+      <c r="A1" s="18" t="inlineStr">
         <is>
           <t>📊 Fiscal &amp; Convênios Municipais — Radar GovTech Brasil 2025/2026</t>
         </is>
@@ -2989,11 +2950,7 @@
           <t>Watch — convênios nicho virgem</t>
         </is>
       </c>
-      <c r="J5" s="18" t="inlineStr">
-        <is>
-          <t>✓</t>
-        </is>
-      </c>
+      <c r="J5" s="13" t="inlineStr"/>
     </row>
     <row r="6" ht="48" customHeight="1">
       <c r="A6" s="14" t="inlineStr">
@@ -3041,11 +2998,7 @@
           <t>Watch — dado fiscal municipal</t>
         </is>
       </c>
-      <c r="J6" s="19" t="inlineStr">
-        <is>
-          <t>✓</t>
-        </is>
-      </c>
+      <c r="J6" s="15" t="inlineStr"/>
     </row>
     <row r="7" ht="48" customHeight="1">
       <c r="A7" s="12" t="inlineStr">
@@ -3189,11 +3142,7 @@
           <t>Watch</t>
         </is>
       </c>
-      <c r="J9" s="18" t="inlineStr">
-        <is>
-          <t>✓</t>
-        </is>
-      </c>
+      <c r="J9" s="13" t="inlineStr"/>
     </row>
   </sheetData>
   <mergeCells count="1">
@@ -3225,7 +3174,7 @@
   </cols>
   <sheetData>
     <row r="1" ht="28" customHeight="1">
-      <c r="A1" s="21" t="inlineStr">
+      <c r="A1" s="19" t="inlineStr">
         <is>
           <t>🏥 Saúde Pública — Radar GovTech Brasil 2025/2026</t>
         </is>
@@ -3649,11 +3598,7 @@
           <t>Watch — anti-fraude saúde</t>
         </is>
       </c>
-      <c r="J10" s="19" t="inlineStr">
-        <is>
-          <t>✓</t>
-        </is>
-      </c>
+      <c r="J10" s="15" t="inlineStr"/>
     </row>
   </sheetData>
   <mergeCells count="1">
@@ -3685,7 +3630,7 @@
   </cols>
   <sheetData>
     <row r="1" ht="28" customHeight="1">
-      <c r="A1" s="22" t="inlineStr">
+      <c r="A1" s="20" t="inlineStr">
         <is>
           <t>📚 Educação Pública — Radar GovTech Brasil 2025/2026</t>
         </is>
@@ -4105,11 +4050,7 @@
           <t>Portfólio KPTL+Cedro</t>
         </is>
       </c>
-      <c r="J10" s="19" t="inlineStr">
-        <is>
-          <t>✓</t>
-        </is>
-      </c>
+      <c r="J10" s="15" t="inlineStr"/>
     </row>
   </sheetData>
   <mergeCells count="1">
@@ -4141,7 +4082,7 @@
   </cols>
   <sheetData>
     <row r="1" ht="28" customHeight="1">
-      <c r="A1" s="23" t="inlineStr">
+      <c r="A1" s="21" t="inlineStr">
         <is>
           <t>🤖 IA Horizontal &amp; Automação — Radar GovTech Brasil 2025/2026</t>
         </is>
@@ -4433,11 +4374,7 @@
           <t>Watch — inteligência regulatória</t>
         </is>
       </c>
-      <c r="J7" s="18" t="inlineStr">
-        <is>
-          <t>✓</t>
-        </is>
-      </c>
+      <c r="J7" s="13" t="inlineStr"/>
     </row>
     <row r="8" ht="48" customHeight="1">
       <c r="A8" s="14" t="inlineStr">
@@ -4485,7 +4422,7 @@
           <t>M&amp;A Watch — portfólio Cedro</t>
         </is>
       </c>
-      <c r="J8" s="19" t="inlineStr">
+      <c r="J8" s="22" t="inlineStr">
         <is>
           <t>✓</t>
         </is>
@@ -4537,11 +4474,7 @@
           <t>Portfólio KPTL+Cedro</t>
         </is>
       </c>
-      <c r="J9" s="18" t="inlineStr">
-        <is>
-          <t>✓</t>
-        </is>
-      </c>
+      <c r="J9" s="13" t="inlineStr"/>
     </row>
   </sheetData>
   <mergeCells count="1">
@@ -4573,7 +4506,7 @@
   </cols>
   <sheetData>
     <row r="1" ht="28" customHeight="1">
-      <c r="A1" s="24" t="inlineStr">
+      <c r="A1" s="23" t="inlineStr">
         <is>
           <t>⚖️ Procuradorias &amp; Jurídico — Radar GovTech Brasil 2025/2026</t>
         </is>
@@ -4985,7 +4918,7 @@
   </cols>
   <sheetData>
     <row r="1" ht="28" customHeight="1">
-      <c r="A1" s="25" t="inlineStr">
+      <c r="A1" s="24" t="inlineStr">
         <is>
           <t>📋 Licitações &amp; Compras Públicas — Radar GovTech Brasil 2025/2026</t>
         </is>
@@ -5317,11 +5250,7 @@
           <t>Watch — buy-side gov</t>
         </is>
       </c>
-      <c r="J8" s="19" t="inlineStr">
-        <is>
-          <t>✓</t>
-        </is>
-      </c>
+      <c r="J8" s="15" t="inlineStr"/>
     </row>
   </sheetData>
   <mergeCells count="1">
@@ -5353,7 +5282,7 @@
   </cols>
   <sheetData>
     <row r="1" ht="28" customHeight="1">
-      <c r="A1" s="26" t="inlineStr">
+      <c r="A1" s="25" t="inlineStr">
         <is>
           <t>🏘️ Habitação &amp; Regularização Fundiária — Radar GovTech Brasil 2025/2026</t>
         </is>
@@ -5457,11 +5386,7 @@
           <t>Watch — REURB nicho virgem</t>
         </is>
       </c>
-      <c r="J3" s="18" t="inlineStr">
-        <is>
-          <t>✓</t>
-        </is>
-      </c>
+      <c r="J3" s="13" t="inlineStr"/>
     </row>
     <row r="4" ht="48" customHeight="1">
       <c r="A4" s="14" t="inlineStr">
@@ -5509,11 +5434,7 @@
           <t>Target roll-up</t>
         </is>
       </c>
-      <c r="J4" s="19" t="inlineStr">
-        <is>
-          <t>✓</t>
-        </is>
-      </c>
+      <c r="J4" s="15" t="inlineStr"/>
     </row>
     <row r="5" ht="48" customHeight="1">
       <c r="A5" s="12" t="inlineStr">
@@ -5561,11 +5482,7 @@
           <t>Watch — tração judicial</t>
         </is>
       </c>
-      <c r="J5" s="18" t="inlineStr">
-        <is>
-          <t>✓</t>
-        </is>
-      </c>
+      <c r="J5" s="13" t="inlineStr"/>
     </row>
     <row r="6" ht="48" customHeight="1">
       <c r="A6" s="14" t="inlineStr">
@@ -5613,11 +5530,7 @@
           <t>Impacto social / ESG</t>
         </is>
       </c>
-      <c r="J6" s="19" t="inlineStr">
-        <is>
-          <t>✓</t>
-        </is>
-      </c>
+      <c r="J6" s="15" t="inlineStr"/>
     </row>
   </sheetData>
   <mergeCells count="1">

</xml_diff>

<commit_message>
Pública Tecnologia: atualização completa e reclassificação
- Migrada de Saúde para Gestão & ERP Municipal (é ERP full suite, não prontuário)
- Subseg: Prontuário APS → ERP Municipal Full Suite (9 áreas)
- Fundação: 1993 | Sede: Blumenau/SC | 98 funcionários | Great Place to Work
- Presença: Brasil + Portugal + Venezuela
- Módulos: Financeira, Tributária, RH, Saúde, Escolar, SUAS, Adm, Cidadão, Gestão

Co-Authored-By: Claude Sonnet 4.6 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/Radar_GovTechs_Brasil_2026.xlsx
+++ b/Radar_GovTechs_Brasil_2026.xlsx
@@ -667,7 +667,7 @@
         </is>
       </c>
       <c r="B4" s="4" t="n">
-        <v>11</v>
+        <v>12</v>
       </c>
     </row>
     <row r="5">
@@ -687,7 +687,7 @@
         </is>
       </c>
       <c r="B6" s="4" t="n">
-        <v>8</v>
+        <v>7</v>
       </c>
     </row>
     <row r="7">
@@ -2146,7 +2146,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:J13"/>
+  <dimension ref="A1:J14"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="28" customWidth="1" min="1" max="1"/>
@@ -2679,50 +2679,98 @@
     <row r="13" ht="48" customHeight="1">
       <c r="A13" s="12" t="inlineStr">
         <is>
+          <t>Pública Tecnologia</t>
+        </is>
+      </c>
+      <c r="B13" s="13" t="inlineStr">
+        <is>
+          <t>ERP Municipal Full Suite</t>
+        </is>
+      </c>
+      <c r="C13" s="13" t="inlineStr">
+        <is>
+          <t>PME Estabelecida</t>
+        </is>
+      </c>
+      <c r="D13" s="13" t="inlineStr">
+        <is>
+          <t>Blumenau - SC</t>
+        </is>
+      </c>
+      <c r="E13" s="13" t="inlineStr">
+        <is>
+          <t>1993</t>
+        </is>
+      </c>
+      <c r="F13" s="13" t="inlineStr">
+        <is>
+          <t>Municípios BR + Portugal + Venezuela</t>
+        </is>
+      </c>
+      <c r="G13" s="13" t="inlineStr">
+        <is>
+          <t>N/D</t>
+        </is>
+      </c>
+      <c r="H13" s="13" t="inlineStr">
+        <is>
+          <t>ERP municipal full suite com 9 áreas: Financeira (contabilidade pública, NF-e), Tributária (ISS, IPTU), Gestão de Pessoas (RH, eSocial, ponto eletrônico), Saúde, Escolar, Assistência Social (SUAS), Administrativa (compras, frotas, patrimônio), Atendimento ao Cidadão (portal transparência, app Cidade Pública) e Gestão (BI, GED, PPA). 33 anos de atuação, 98 funcionários. Great Place to Work. Presença internacional: Portugal e Venezuela. Sede Blumenau/SC.</t>
+        </is>
+      </c>
+      <c r="I13" s="17" t="inlineStr">
+        <is>
+          <t>Target roll-up</t>
+        </is>
+      </c>
+      <c r="J13" s="13" t="inlineStr"/>
+    </row>
+    <row r="14" ht="48" customHeight="1">
+      <c r="A14" s="14" t="inlineStr">
+        <is>
           <t>PLACE</t>
         </is>
       </c>
-      <c r="B13" s="13" t="inlineStr">
+      <c r="B14" s="15" t="inlineStr">
         <is>
           <t>Planejamento Urbano / GeoInteligência</t>
         </is>
       </c>
-      <c r="C13" s="13" t="inlineStr">
+      <c r="C14" s="15" t="inlineStr">
         <is>
           <t>Startup</t>
         </is>
       </c>
-      <c r="D13" s="13" t="inlineStr">
+      <c r="D14" s="15" t="inlineStr">
         <is>
           <t>Brasil</t>
         </is>
       </c>
-      <c r="E13" s="13" t="inlineStr">
-        <is>
-          <t>N/D</t>
-        </is>
-      </c>
-      <c r="F13" s="13" t="inlineStr">
+      <c r="E14" s="15" t="inlineStr">
+        <is>
+          <t>N/D</t>
+        </is>
+      </c>
+      <c r="F14" s="15" t="inlineStr">
         <is>
           <t>Municípios</t>
         </is>
       </c>
-      <c r="G13" s="13" t="inlineStr">
-        <is>
-          <t>N/D</t>
-        </is>
-      </c>
-      <c r="H13" s="13" t="inlineStr">
+      <c r="G14" s="15" t="inlineStr">
+        <is>
+          <t>N/D</t>
+        </is>
+      </c>
+      <c r="H14" s="15" t="inlineStr">
         <is>
           <t>Plataforma que integra dados de mercado imobiliário, urbanismo e legislação municipal em interface intuitiva para gestores públicos. Certificada BrazilLAB. Suporte a decisões de planejamento territorial e uso do solo.</t>
         </is>
       </c>
-      <c r="I13" s="17" t="inlineStr">
+      <c r="I14" s="16" t="inlineStr">
         <is>
           <t>Watch — urbanismo digital</t>
         </is>
       </c>
-      <c r="J13" s="13" t="inlineStr"/>
+      <c r="J14" s="15" t="inlineStr"/>
     </row>
   </sheetData>
   <mergeCells count="1">
@@ -3158,7 +3206,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:J10"/>
+  <dimension ref="A1:J9"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="28" customWidth="1" min="1" max="1"/>
@@ -3379,42 +3427,42 @@
     <row r="6" ht="48" customHeight="1">
       <c r="A6" s="14" t="inlineStr">
         <is>
-          <t>Pública Tecnologia</t>
+          <t>ImpulsoGov</t>
         </is>
       </c>
       <c r="B6" s="15" t="inlineStr">
         <is>
-          <t>Prontuário Eletrônico APS</t>
+          <t>Analytics / BI para APS</t>
         </is>
       </c>
       <c r="C6" s="15" t="inlineStr">
         <is>
-          <t>PME</t>
+          <t>Startup early-stage</t>
         </is>
       </c>
       <c r="D6" s="15" t="inlineStr">
         <is>
-          <t>N/D</t>
+          <t>São Paulo - SP</t>
         </is>
       </c>
       <c r="E6" s="15" t="inlineStr">
         <is>
-          <t>N/D</t>
+          <t>~2020</t>
         </is>
       </c>
       <c r="F6" s="15" t="inlineStr">
         <is>
-          <t>Municípios</t>
+          <t>Municípios via SUS</t>
         </is>
       </c>
       <c r="G6" s="15" t="inlineStr">
         <is>
-          <t>N/D</t>
+          <t>US$ 100k</t>
         </is>
       </c>
       <c r="H6" s="15" t="inlineStr">
         <is>
-          <t>Prontuário eletrônico certificado SBIS/CFM. Assinatura ICP-Brasil. Integração e-SUS.</t>
+          <t>BI para gaps de atenção básica preventiva. Cofundada por ex-Harvard Kennedy School. Reconhecida pela CGU. Impulso Previne.</t>
         </is>
       </c>
       <c r="I6" s="15" t="inlineStr"/>
@@ -3423,17 +3471,17 @@
     <row r="7" ht="48" customHeight="1">
       <c r="A7" s="12" t="inlineStr">
         <is>
-          <t>ImpulsoGov</t>
+          <t>UpCities</t>
         </is>
       </c>
       <c r="B7" s="13" t="inlineStr">
         <is>
-          <t>Analytics / BI para APS</t>
+          <t>Integração e-SUS / Telecare</t>
         </is>
       </c>
       <c r="C7" s="13" t="inlineStr">
         <is>
-          <t>Startup early-stage</t>
+          <t>Startup</t>
         </is>
       </c>
       <c r="D7" s="13" t="inlineStr">
@@ -3443,22 +3491,22 @@
       </c>
       <c r="E7" s="13" t="inlineStr">
         <is>
-          <t>~2020</t>
+          <t>~2019</t>
         </is>
       </c>
       <c r="F7" s="13" t="inlineStr">
         <is>
-          <t>Municípios via SUS</t>
+          <t>Municípios (expansão)</t>
         </is>
       </c>
       <c r="G7" s="13" t="inlineStr">
         <is>
-          <t>US$ 100k</t>
+          <t>N/D</t>
         </is>
       </c>
       <c r="H7" s="13" t="inlineStr">
         <is>
-          <t>BI para gaps de atenção básica preventiva. Cofundada por ex-Harvard Kennedy School. Reconhecida pela CGU. Impulso Previne.</t>
+          <t>Integradora e-SUS/RNDS. Prontuário unificado, telecare. App offline para agentes comunitários de saúde.</t>
         </is>
       </c>
       <c r="I7" s="13" t="inlineStr"/>
@@ -3467,12 +3515,12 @@
     <row r="8" ht="48" customHeight="1">
       <c r="A8" s="14" t="inlineStr">
         <is>
-          <t>UpCities</t>
+          <t>ToGov</t>
         </is>
       </c>
       <c r="B8" s="15" t="inlineStr">
         <is>
-          <t>Integração e-SUS / Telecare</t>
+          <t>Analytics APS / Educação</t>
         </is>
       </c>
       <c r="C8" s="15" t="inlineStr">
@@ -3482,17 +3530,17 @@
       </c>
       <c r="D8" s="15" t="inlineStr">
         <is>
-          <t>São Paulo - SP</t>
+          <t>Santa Luzia - MG</t>
         </is>
       </c>
       <c r="E8" s="15" t="inlineStr">
         <is>
-          <t>~2019</t>
+          <t>2020</t>
         </is>
       </c>
       <c r="F8" s="15" t="inlineStr">
         <is>
-          <t>Municípios (expansão)</t>
+          <t>Municípios MG e outros</t>
         </is>
       </c>
       <c r="G8" s="15" t="inlineStr">
@@ -3502,7 +3550,7 @@
       </c>
       <c r="H8" s="15" t="inlineStr">
         <is>
-          <t>Integradora e-SUS/RNDS. Prontuário unificado, telecare. App offline para agentes comunitários de saúde.</t>
+          <t>Analytics Previne Brasil: gaps, captação de recursos, indicadores APS. 3ª DemoDay BrazilLAB 2023.</t>
         </is>
       </c>
       <c r="I8" s="15" t="inlineStr"/>
@@ -3511,12 +3559,12 @@
     <row r="9" ht="48" customHeight="1">
       <c r="A9" s="12" t="inlineStr">
         <is>
-          <t>ToGov</t>
+          <t>MedBolso</t>
         </is>
       </c>
       <c r="B9" s="13" t="inlineStr">
         <is>
-          <t>Analytics APS / Educação</t>
+          <t>Escalas / Anti-fraude Saúde</t>
         </is>
       </c>
       <c r="C9" s="13" t="inlineStr">
@@ -3526,17 +3574,17 @@
       </c>
       <c r="D9" s="13" t="inlineStr">
         <is>
-          <t>Santa Luzia - MG</t>
+          <t>N/D (Brasil)</t>
         </is>
       </c>
       <c r="E9" s="13" t="inlineStr">
         <is>
-          <t>2020</t>
+          <t>~2020</t>
         </is>
       </c>
       <c r="F9" s="13" t="inlineStr">
         <is>
-          <t>Municípios MG e outros</t>
+          <t>UBS / Municípios</t>
         </is>
       </c>
       <c r="G9" s="13" t="inlineStr">
@@ -3546,59 +3594,15 @@
       </c>
       <c r="H9" s="13" t="inlineStr">
         <is>
-          <t>Analytics Previne Brasil: gaps, captação de recursos, indicadores APS. 3ª DemoDay BrazilLAB 2023.</t>
-        </is>
-      </c>
-      <c r="I9" s="13" t="inlineStr"/>
+          <t>Gestão de escalas e plantões para saúde pública municipal. Anti-fraude em folha de pagamento. Top 30 Sebrae 2024. Acelerada GovTech Pará.</t>
+        </is>
+      </c>
+      <c r="I9" s="17" t="inlineStr">
+        <is>
+          <t>Watch — anti-fraude saúde</t>
+        </is>
+      </c>
       <c r="J9" s="13" t="inlineStr"/>
-    </row>
-    <row r="10" ht="48" customHeight="1">
-      <c r="A10" s="14" t="inlineStr">
-        <is>
-          <t>MedBolso</t>
-        </is>
-      </c>
-      <c r="B10" s="15" t="inlineStr">
-        <is>
-          <t>Escalas / Anti-fraude Saúde</t>
-        </is>
-      </c>
-      <c r="C10" s="15" t="inlineStr">
-        <is>
-          <t>Startup</t>
-        </is>
-      </c>
-      <c r="D10" s="15" t="inlineStr">
-        <is>
-          <t>N/D (Brasil)</t>
-        </is>
-      </c>
-      <c r="E10" s="15" t="inlineStr">
-        <is>
-          <t>~2020</t>
-        </is>
-      </c>
-      <c r="F10" s="15" t="inlineStr">
-        <is>
-          <t>UBS / Municípios</t>
-        </is>
-      </c>
-      <c r="G10" s="15" t="inlineStr">
-        <is>
-          <t>N/D</t>
-        </is>
-      </c>
-      <c r="H10" s="15" t="inlineStr">
-        <is>
-          <t>Gestão de escalas e plantões para saúde pública municipal. Anti-fraude em folha de pagamento. Top 30 Sebrae 2024. Acelerada GovTech Pará.</t>
-        </is>
-      </c>
-      <c r="I10" s="16" t="inlineStr">
-        <is>
-          <t>Watch — anti-fraude saúde</t>
-        </is>
-      </c>
-      <c r="J10" s="15" t="inlineStr"/>
     </row>
   </sheetData>
   <mergeCells count="1">

</xml_diff>

<commit_message>
v12: site oficial (url) adicionado a todas as 68 empresas + atualizações massivas
- Link para site oficial adicionado ao card de cada empresa no radar
- Atuação, segmento e dados revisados com base nos sites oficiais
- Correções factuais: ImpulsoGov (ONG), Attus (rebrand + IA generativa),
  MinutaIA (fund fev/2024), Geopixel (SJC-SP), IPQ (Porto Alegre RS),
  GovTools (Gravataí RS), UpCities (Vitória ES), PGMNET (Campos RJ),
  StartGov (Imperatriz MA), CERURB (Teresina PI), TUXTU (Macapá AP)
- Vivenda: 6.500+ reformas, COHAB-SP parceiro, R$54M+ gerenciados
- SmartCityTec: membro oficial FIWARE Foundation, URL smartcity.tec.br
- Notas atualizadas: OM30, Kinebot (29 países), Qiatech, MuniScore,
  Hub Esfera, Portabilis (SUAS), Geekie, Educacross, ReurBR, sisHABI,
  Portal Compras, StartGi, StartGov, Nuveo, CPQD, Atech (Grupo Embraer)

Co-Authored-By: Claude Sonnet 4.6 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/Radar_GovTechs_Brasil_2026.xlsx
+++ b/Radar_GovTechs_Brasil_2026.xlsx
@@ -644,7 +644,7 @@
     <row r="1" ht="32" customHeight="1">
       <c r="A1" s="1" t="inlineStr">
         <is>
-          <t>🇧🇷 Radar GovTech Brasil 2025/2026 — DLG · Maio 2026 · v11</t>
+          <t>🇧🇷 Radar GovTech Brasil 2025/2026 — DLG · Maio 2026 · v12</t>
         </is>
       </c>
     </row>
@@ -916,7 +916,7 @@
       </c>
       <c r="F3" s="13" t="inlineStr">
         <is>
-          <t>Consórcios intermunicipais BA</t>
+          <t>Consórcios intermunicipais BA | CONSID, CONVALE, CDS Bacia do Paramirim</t>
         </is>
       </c>
       <c r="G3" s="13" t="inlineStr">
@@ -926,7 +926,7 @@
       </c>
       <c r="H3" s="13" t="inlineStr">
         <is>
-          <t>SaaS de licenciamento ambiental municipal 100% digital. Integra SINAFLOR, GEOBAHIA, SEMA-BA e CEPRAM. 70% redução de custos declarada, onboarding em 30 dias. Operando via consórcios: CDS Bacia do Paramirim, CONVALE e CONSID Oeste da BA. Conformidade com Resolução CEPRAM 4.327/13.</t>
+          <t>Sistema de Gestão Ambiental Compartilhada (eGAC): SaaS de licenciamento ambiental municipal 100% digital. Integra SINAFLOR, GEOBAHIA, SEMA-BA e CEPRAM. Cobrança automática de taxa ambiental via Pix/boleto. 70% redução de custos declarada, onboarding em 30 dias. Nasceu da pandemia de 2021 em colaboração com gestores municipais baianos. Conformidade CEPRAM 4.327/13.</t>
         </is>
       </c>
       <c r="I3" s="17" t="inlineStr">
@@ -954,7 +954,7 @@
       </c>
       <c r="D4" s="15" t="inlineStr">
         <is>
-          <t>Brasil</t>
+          <t>Macapá - AP</t>
         </is>
       </c>
       <c r="E4" s="15" t="inlineStr">
@@ -964,7 +964,7 @@
       </c>
       <c r="F4" s="15" t="inlineStr">
         <is>
-          <t>Municípios (via órgãos ambientais)</t>
+          <t>Municípios (via órgãos ambientais) | Associada ABES</t>
         </is>
       </c>
       <c r="G4" s="15" t="inlineStr">
@@ -974,7 +974,7 @@
       </c>
       <c r="H4" s="15" t="inlineStr">
         <is>
-          <t>3 módulos SaaS para Secretarias de Meio Ambiente: SIBLAM (licenciamento com bio-algoritmo e método Battelle EES — reduz subjetividade do analista), SIGAU (arborização urbana com participação cidadã), SICCA (crédito de carbono). Propõe padronização nacional do licenciamento. CEO: Marcelo Creão. Associada ABES.</t>
+          <t>Suite SaaS para Secretarias de Meio Ambiente: SIBLAM (licenciamento com bio-algoritmo e método Battelle EES — reduz subjetividade do analista), SIGAU (arborização urbana com participação cidadã), Sistema de Resíduos Sólidos, Crédito de Carbono (SICCA) e Controle e Fiscalização. Propõe padronização nacional do licenciamento. CEO: Marcelo Creão.</t>
         </is>
       </c>
       <c r="I4" s="16" t="inlineStr">
@@ -1128,7 +1128,7 @@
       </c>
       <c r="B3" s="13" t="inlineStr">
         <is>
-          <t>Plataforma FIWARE / Interoperabilidade Municipal</t>
+          <t>Plataforma FIWARE / Data Spaces Municipais</t>
         </is>
       </c>
       <c r="C3" s="13" t="inlineStr">
@@ -1148,7 +1148,7 @@
       </c>
       <c r="F3" s="13" t="inlineStr">
         <is>
-          <t>Smart Mafra + Amurel Conectada (18 mun.)</t>
+          <t>Smart Mafra + Amurel Conectada (18 mun.) | Membro FIWARE Foundation</t>
         </is>
       </c>
       <c r="G3" s="13" t="inlineStr">
@@ -1158,7 +1158,7 @@
       </c>
       <c r="H3" s="13" t="inlineStr">
         <is>
-          <t>Plataforma open-source baseada em FIWARE para cidades inteligentes: data spaces, IoT, mobilidade, segurança e clima. Smart Mafra: 1ª cidade BR com lei municipal baseada em FIWARE (centraliza tributação, alvarás e serviços públicos). Amurel Conectada: integra 18 municípios da Região de Laguna/SC. SC aprovou Lei 19.494 adotando FIWARE como padrão estadual. Prêmio GovTech Summit 2025. Smart City Expo Barcelona 2025.</t>
+          <t>Plataforma baseada em FIWARE para cidades inteligentes: data spaces interoperáveis, IoT, mobilidade, segurança e clima. Smart Mafra: 1ª cidade BR com lei municipal FIWARE (centraliza tributação, alvarás e todos os serviços públicos em sistema único). Amurel Conectada: integra 18 municípios Região de Laguna/SC — 1º espaço de dados regional BR em operação. SC aprovou Lei 19.494 adotando FIWARE como padrão estadual. CEO: Gilsoni Lunardi Albino. Prêmio Smart City Expo Curitiba 2025 + Barcelona 2025.</t>
         </is>
       </c>
       <c r="I3" s="17" t="inlineStr">
@@ -1312,7 +1312,7 @@
       </c>
       <c r="B3" s="13" t="inlineStr">
         <is>
-          <t>Infraestrutura / Clima</t>
+          <t>Previsão de Desastres / ClimateTech</t>
         </is>
       </c>
       <c r="C3" s="13" t="inlineStr">
@@ -1342,7 +1342,7 @@
       </c>
       <c r="H3" s="13" t="inlineStr">
         <is>
-          <t>IA para previsão antecipada de desastres naturais. Dados NASA + bases nacionais. Alerta SMS via Defesa Civil. COP26 selecionada.</t>
+          <t>IA para previsão antecipada de desastres naturais com dados NASA e bases nacionais. Alerta SMS via Defesa Civil municipal. Selecionada COP26. Foco em mitigação de riscos climáticos e resiliência urbana.</t>
         </is>
       </c>
       <c r="I3" s="17" t="inlineStr">
@@ -1360,7 +1360,7 @@
       </c>
       <c r="B4" s="15" t="inlineStr">
         <is>
-          <t>Infraestrutura / Clima</t>
+          <t>Previsões Microclimáticas / Portos e Energia</t>
         </is>
       </c>
       <c r="C4" s="15" t="inlineStr">
@@ -1380,20 +1380,24 @@
       </c>
       <c r="F4" s="15" t="inlineStr">
         <is>
-          <t>N/D</t>
+          <t>Portos, setor elétrico e renovável | Porto do Açu, Wilson Sons, Santos Brasil</t>
         </is>
       </c>
       <c r="G4" s="15" t="inlineStr">
         <is>
-          <t>R$ 7,5M aporte</t>
+          <t>R$ 7,5M (Fundo GovTech)</t>
         </is>
       </c>
       <c r="H4" s="15" t="inlineStr">
         <is>
-          <t>Previsões microclimáticas para portos e setor elétrico. Captou R$7,5M do Fundo GovTech. Resiliência climática.</t>
-        </is>
-      </c>
-      <c r="I4" s="15" t="inlineStr"/>
+          <t>Plataforma i4cast® de decisão baseada em inteligência climática: previsões hiperlocais de mar e clima para operações portuárias, logística marítima e geração de energia renovável. Precisão 2x superior a previsões genéricas (94% acurácia no Porto do Açu). Captou R$7,5M do Fundo GovTech KPTL.</t>
+        </is>
+      </c>
+      <c r="I4" s="16" t="inlineStr">
+        <is>
+          <t>Portfólio KPTL</t>
+        </is>
+      </c>
       <c r="J4" s="15" t="inlineStr"/>
     </row>
     <row r="5" ht="48" customHeight="1">
@@ -1404,7 +1408,7 @@
       </c>
       <c r="B5" s="13" t="inlineStr">
         <is>
-          <t>Segurança Pública</t>
+          <t>Segurança Pública / TIC para Ambientes Críticos</t>
         </is>
       </c>
       <c r="C5" s="13" t="inlineStr">
@@ -1414,17 +1418,17 @@
       </c>
       <c r="D5" s="13" t="inlineStr">
         <is>
-          <t>Curitiba - PR</t>
+          <t>Porto Alegre - RS</t>
         </is>
       </c>
       <c r="E5" s="13" t="inlineStr">
         <is>
-          <t>~2010</t>
+          <t>~2001</t>
         </is>
       </c>
       <c r="F5" s="13" t="inlineStr">
         <is>
-          <t>250+ municípios</t>
+          <t>Nacional e internacional | órgãos públicos, presídios, hospitais, rodovias</t>
         </is>
       </c>
       <c r="G5" s="13" t="inlineStr">
@@ -1434,7 +1438,7 @@
       </c>
       <c r="H5" s="13" t="inlineStr">
         <is>
-          <t>Monitoramento e recuperação de veículos. 7.000+ veículos recuperados em 2024. Redução de 15,5% em furtos.</t>
+          <t>25+ anos desenvolvendo e integrando soluções de TIC com IA e Analytics para segurança pública e ambientes críticos. Portfólio: videomonitoramento, controle de acesso, redes de dados públicas/privadas, infraestrutura para Defesa e Segurança. Atuação descentralizada com cobertura nacional.</t>
         </is>
       </c>
       <c r="I5" s="13" t="inlineStr"/>
@@ -1448,7 +1452,7 @@
       </c>
       <c r="B6" s="15" t="inlineStr">
         <is>
-          <t>Segurança Pública / Defesa</t>
+          <t>Comando &amp; Controle / Defesa e Segurança Pública</t>
         </is>
       </c>
       <c r="C6" s="15" t="inlineStr">
@@ -1468,7 +1472,7 @@
       </c>
       <c r="F6" s="15" t="inlineStr">
         <is>
-          <t>Nacional / Defesa</t>
+          <t>Nacional / Defesa, ATM, Segurança</t>
         </is>
       </c>
       <c r="G6" s="15" t="inlineStr">
@@ -1478,7 +1482,7 @@
       </c>
       <c r="H6" s="15" t="inlineStr">
         <is>
-          <t>Empresa Estratégica de Defesa (MDefesa). Plataformas de Comando &amp; Controle e gestão de crises.</t>
+          <t>Empresa do Grupo Embraer e Empresa Estratégica de Defesa (EED). Especialista em sistemas de missão crítica: Gerenciamento de Tráfego Aéreo (ATM), Comando &amp; Controle (C4I), Gestão de UTM (drones), Segurança Pública, Sistemas Navais, Cibersegurança e Sistemas Embarcados. Certificações ISO internacionais.</t>
         </is>
       </c>
       <c r="I6" s="15" t="inlineStr"/>
@@ -1492,7 +1496,7 @@
       </c>
       <c r="B7" s="13" t="inlineStr">
         <is>
-          <t>Gestão Hídrica / Infraestrutura</t>
+          <t>Previsão Hidroclimática / ClimateTech</t>
         </is>
       </c>
       <c r="C7" s="13" t="inlineStr">
@@ -1502,7 +1506,7 @@
       </c>
       <c r="D7" s="13" t="inlineStr">
         <is>
-          <t>Brasil</t>
+          <t>Florianópolis - SC</t>
         </is>
       </c>
       <c r="E7" s="13" t="inlineStr">
@@ -1512,7 +1516,7 @@
       </c>
       <c r="F7" s="13" t="inlineStr">
         <is>
-          <t>Setor elétrico + agro</t>
+          <t>Defesa Civil SC | usinas hidrelétricas | Clientes: CPFL, Statkraft</t>
         </is>
       </c>
       <c r="G7" s="13" t="inlineStr">
@@ -1522,7 +1526,7 @@
       </c>
       <c r="H7" s="13" t="inlineStr">
         <is>
-          <t>SaaS hidrológico integrado: previsão de fluxo de água e gestão de bacias hidrográficas. 80 anos de dados históricos. Clientes: CPFL, Statkraft. Aplicações em energia, agronegócio e seguros. Investimento KPTL 2019 (pré-Fundo GovTech).</t>
+          <t>ClimaTech com plataforma SPEHC (SaaS) para previsões hidroclimáticas: antecipação de enchentes, gestão de barragens e operação de usinas. Integra múltiplos modelos, radares e dados em tempo real. Referência nacional na Defesa Civil de SC. Escritório também em Bauru/SP. Portfólio KPTL 2019.</t>
         </is>
       </c>
       <c r="I7" s="17" t="inlineStr">
@@ -1540,7 +1544,7 @@
       </c>
       <c r="B8" s="15" t="inlineStr">
         <is>
-          <t>Fiscalização / Drones / IA</t>
+          <t>Monitoramento Aéreo / Fiscalização com IA</t>
         </is>
       </c>
       <c r="C8" s="15" t="inlineStr">
@@ -1555,12 +1559,12 @@
       </c>
       <c r="E8" s="15" t="inlineStr">
         <is>
-          <t>~2016</t>
+          <t>2014</t>
         </is>
       </c>
       <c r="F8" s="15" t="inlineStr">
         <is>
-          <t>100+ gov + privado</t>
+          <t>100+ clientes gov e privado | Florianópolis (Monitora Floripa), telco, energia</t>
         </is>
       </c>
       <c r="G8" s="15" t="inlineStr">
@@ -1570,7 +1574,7 @@
       </c>
       <c r="H8" s="15" t="inlineStr">
         <is>
-          <t>Drones + satélites + visão computacional: obras irregulares, desmatamento, infraestrutura. Cliente: Florianópolis. 9 anos de operação.</t>
+          <t>Plataforma de análise de imagens com IA para decisões inteligentes: sistema Monitora detecta obras irregulares e desmatamento via satélite + drones (identificação automática, 50% mais eficácia de fiscalização). Prêmio Connected Smart Cities 2021. Também atua em inspeção solar e telecom (Vivo, ENEL). CEO: Fabrício Hertz. Sede Parque Tecnológico ALFA Florianópolis.</t>
         </is>
       </c>
       <c r="I8" s="15" t="inlineStr"/>
@@ -1584,7 +1588,7 @@
       </c>
       <c r="B9" s="13" t="inlineStr">
         <is>
-          <t>IA Infraestrutura Urbana</t>
+          <t>Gestão Urbana Preditiva / Pavimento e Zeladoria com IA</t>
         </is>
       </c>
       <c r="C9" s="13" t="inlineStr">
@@ -1604,7 +1608,7 @@
       </c>
       <c r="F9" s="13" t="inlineStr">
         <is>
-          <t>Sabesp + municípios</t>
+          <t>15M+ cidadãos | 8+ estados | São Paulo, Porto Alegre, Gravatá</t>
         </is>
       </c>
       <c r="G9" s="13" t="inlineStr">
@@ -1614,7 +1618,7 @@
       </c>
       <c r="H9" s="13" t="inlineStr">
         <is>
-          <t>Câmeras em veículos + visão computacional: mapeia pavimento, rachaduras. Sabesp: detecção de vazamentos de água.</t>
+          <t>Plataforma de gestão urbana inteligente com visão computacional embarcada em veículos: mapeia qualidade de pavimento, iluminação, encostas e ativos urbanos georreferenciados. Sistema Gaia (SP) apoia programa de recape. Dashboard preditivo com Machine Learning. Também gerencia zeladoria (OS) e intervenções de concessionárias. Integra portal do cidadão. 40+ tipos de ativos monitorados.</t>
         </is>
       </c>
       <c r="I9" s="13" t="inlineStr"/>
@@ -2228,7 +2232,7 @@
       </c>
       <c r="B3" s="13" t="inlineStr">
         <is>
-          <t>Gestão Pública Municipal</t>
+          <t>Gestão de Processos Administrativos Municipais</t>
         </is>
       </c>
       <c r="C3" s="13" t="inlineStr">
@@ -2238,7 +2242,7 @@
       </c>
       <c r="D3" s="13" t="inlineStr">
         <is>
-          <t>São Paulo - SP</t>
+          <t>Cascavel - PR</t>
         </is>
       </c>
       <c r="E3" s="13" t="inlineStr">
@@ -2248,7 +2252,7 @@
       </c>
       <c r="F3" s="13" t="inlineStr">
         <is>
-          <t>120+ cidades</t>
+          <t>150+ cidades | 23M+ brasileiros</t>
         </is>
       </c>
       <c r="G3" s="13" t="inlineStr">
@@ -2258,7 +2262,7 @@
       </c>
       <c r="H3" s="13" t="inlineStr">
         <is>
-          <t>Aporte Seed de R$22,5M (US$4M) liderado por Astella e VOX Capital (CVC do Banco do Brasil), com CAF e Endeavor. 120+ cidades. TOP Open Startups 2024. Maior aporte da história das GovTechs da AL.</t>
+          <t>Plataforma SaaS de processos eletrônicos para prefeituras: protocolo, assinatura digital ICP-Brasil, tramitação com IA, portal de serviços e arrecadação (Aprova Pay). Cobre obras, meio ambiente, RH e compras. Primeira govtech investida pelo Banco do Brasil. TOP Open Startups 2024.</t>
         </is>
       </c>
       <c r="I3" s="13" t="inlineStr"/>
@@ -2272,7 +2276,7 @@
       </c>
       <c r="B4" s="15" t="inlineStr">
         <is>
-          <t>Gestão Pública Municipal</t>
+          <t>App Municipal SaaS / Relacionamento Cidadão-Governo</t>
         </is>
       </c>
       <c r="C4" s="15" t="inlineStr">
@@ -2292,7 +2296,7 @@
       </c>
       <c r="F4" s="15" t="inlineStr">
         <is>
-          <t>5 estados | 600+ serv.</t>
+          <t>Múltiplos municípios SC e outros estados</t>
         </is>
       </c>
       <c r="G4" s="15" t="inlineStr">
@@ -2302,7 +2306,7 @@
       </c>
       <c r="H4" s="15" t="inlineStr">
         <is>
-          <t>App SaaS municipal customizável. 600+ serviços digitalizados. CEO: Elias Raasch. Expansão nacional sem VC. Referência SC.</t>
+          <t>App oficial white-label de prefeituras reunindo zeladoria, agendamento, formulários online, notícias e comunicação direta cidadão-prefeitura. Integrações com IPTU, protocolo e ouvidoria. CEO: Elias Raasch. Expansão nacional sem VC.</t>
         </is>
       </c>
       <c r="I4" s="16" t="inlineStr">
@@ -2320,7 +2324,7 @@
       </c>
       <c r="B5" s="13" t="inlineStr">
         <is>
-          <t>Gestão Pública Municipal</t>
+          <t>Licenciamento e Tributação Municipal Digital</t>
         </is>
       </c>
       <c r="C5" s="13" t="inlineStr">
@@ -2330,7 +2334,7 @@
       </c>
       <c r="D5" s="13" t="inlineStr">
         <is>
-          <t>Campinas/RJ</t>
+          <t>Campinas - SP</t>
         </is>
       </c>
       <c r="E5" s="13" t="inlineStr">
@@ -2340,7 +2344,7 @@
       </c>
       <c r="F5" s="13" t="inlineStr">
         <is>
-          <t>N/D</t>
+          <t>Municípios Norte e outras regiões | Scale-Up Endeavor 2021</t>
         </is>
       </c>
       <c r="G5" s="13" t="inlineStr">
@@ -2350,7 +2354,7 @@
       </c>
       <c r="H5" s="13" t="inlineStr">
         <is>
-          <t>TOP 2 Ranking 100 Open Startups 2024 (GovTech).</t>
+          <t>Plataforma integrada de licenciamento digital (urbanístico, ambiental, sanitário, obras), abertura/baixa de empresas, IPTU e ISS digitais integrada à REDESIM federal. Foco em desburocratização e aumento de receita própria municipal. TOP2 Open Startups 2024.</t>
         </is>
       </c>
       <c r="I5" s="13" t="inlineStr"/>
@@ -2364,7 +2368,7 @@
       </c>
       <c r="B6" s="15" t="inlineStr">
         <is>
-          <t>Gestão Pública Municipal</t>
+          <t>Capacitação e Consultoria em Gestão Pública</t>
         </is>
       </c>
       <c r="C6" s="15" t="inlineStr">
@@ -2379,12 +2383,12 @@
       </c>
       <c r="E6" s="15" t="inlineStr">
         <is>
-          <t>~2018</t>
+          <t>2014</t>
         </is>
       </c>
       <c r="F6" s="15" t="inlineStr">
         <is>
-          <t>N/D</t>
+          <t>Ecossistema Norte do Brasil</t>
         </is>
       </c>
       <c r="G6" s="15" t="inlineStr">
@@ -2394,10 +2398,14 @@
       </c>
       <c r="H6" s="15" t="inlineStr">
         <is>
-          <t>TOP 3 Open Startups 2024. Representante do ecossistema Norte do Brasil.</t>
-        </is>
-      </c>
-      <c r="I6" s="15" t="inlineStr"/>
+          <t>Empresa de capacitação e consultoria para gestão pública municipal na região Norte. TOP 3 Open Startups 2024. Não foram identificados produtos SaaS com identidade digital clara — oportunidade de due diligence.</t>
+        </is>
+      </c>
+      <c r="I6" s="16" t="inlineStr">
+        <is>
+          <t>Watch — due diligence necessário</t>
+        </is>
+      </c>
       <c r="J6" s="15" t="inlineStr"/>
     </row>
     <row r="7" ht="48" customHeight="1">
@@ -2408,7 +2416,7 @@
       </c>
       <c r="B7" s="13" t="inlineStr">
         <is>
-          <t>Assistência Social / SUAS</t>
+          <t>Gestão do SUAS / Assistência Social</t>
         </is>
       </c>
       <c r="C7" s="13" t="inlineStr">
@@ -2423,12 +2431,12 @@
       </c>
       <c r="E7" s="13" t="inlineStr">
         <is>
-          <t>~2016</t>
+          <t>2008</t>
         </is>
       </c>
       <c r="F7" s="13" t="inlineStr">
         <is>
-          <t>168 mun | 3,5M pessoas</t>
+          <t>Centenas de municípios | CRASs e CREASs</t>
         </is>
       </c>
       <c r="G7" s="13" t="inlineStr">
@@ -2438,7 +2446,7 @@
       </c>
       <c r="H7" s="13" t="inlineStr">
         <is>
-          <t>Prontuário eletrônico SUAS. 1,2M famílias | 6,5k trabalhadores. Líder IE GovTech 2020. Vertical exclusivo sem concorrente direto.</t>
+          <t>SaaS de gestão do SUAS com Prontuário Digital integrado ao CadÚnico, planos PAIF/PAEFI/PIA, vigilância socioassistencial georreferenciada e relatórios MDS. 56 colaboradores. Líder IE GovTech 2020. Vertical exclusivo sem concorrente direto.</t>
         </is>
       </c>
       <c r="I7" s="17" t="inlineStr">
@@ -2456,7 +2464,7 @@
       </c>
       <c r="B8" s="15" t="inlineStr">
         <is>
-          <t>Participação Cidadã</t>
+          <t>Gestão de Editais e Investimento Social</t>
         </is>
       </c>
       <c r="C8" s="15" t="inlineStr">
@@ -2466,17 +2474,17 @@
       </c>
       <c r="D8" s="15" t="inlineStr">
         <is>
-          <t>São Paulo - SP</t>
+          <t>Belo Horizonte - MG</t>
         </is>
       </c>
       <c r="E8" s="15" t="inlineStr">
         <is>
-          <t>~2016</t>
+          <t>2014</t>
         </is>
       </c>
       <c r="F8" s="15" t="inlineStr">
         <is>
-          <t>220k+ usuários</t>
+          <t>13k+ editais | institutos e fundações corporativas</t>
         </is>
       </c>
       <c r="G8" s="15" t="inlineStr">
@@ -2486,10 +2494,14 @@
       </c>
       <c r="H8" s="15" t="inlineStr">
         <is>
-          <t>Portfólio Fundo GovTech KPTL. Gestão digital de editais socioculturais e transparência pública.</t>
-        </is>
-      </c>
-      <c r="I8" s="15" t="inlineStr"/>
+          <t>Maior base de editais do terceiro setor no Brasil. Plataforma para criação de editais, inscrições online, pareceristas e monitoramento de projetos. Venture Round out/2024. Portfólio Fundo GovTech KPTL. 51 funcionários.</t>
+        </is>
+      </c>
+      <c r="I8" s="16" t="inlineStr">
+        <is>
+          <t>Portfólio KPTL</t>
+        </is>
+      </c>
       <c r="J8" s="15" t="inlineStr"/>
     </row>
     <row r="9" ht="48" customHeight="1">
@@ -2500,7 +2512,7 @@
       </c>
       <c r="B9" s="13" t="inlineStr">
         <is>
-          <t>Smart Cities / Mobilidade</t>
+          <t>Gestão Urbana Integrada / Smart Cities</t>
         </is>
       </c>
       <c r="C9" s="13" t="inlineStr">
@@ -2515,12 +2527,12 @@
       </c>
       <c r="E9" s="13" t="inlineStr">
         <is>
-          <t>~2015</t>
+          <t>2015</t>
         </is>
       </c>
       <c r="F9" s="13" t="inlineStr">
         <is>
-          <t>N/D</t>
+          <t>79k+ pontos monitorados | prefeituras e Petrobras</t>
         </is>
       </c>
       <c r="G9" s="13" t="inlineStr">
@@ -2530,7 +2542,7 @@
       </c>
       <c r="H9" s="13" t="inlineStr">
         <is>
-          <t>Origem COPPE/UFRJ. Selo GovTech BrazilLAB. Mobilidade urbana e cidades inteligentes.</t>
+          <t>GovTech de cidades inteligentes com SIGELU (limpeza urbana), fiscalização móvel, gestão nutricional escolar e saúde. Primeiro contrato pelo Marco Legal das Startups. Origem COPPE/UFRJ. Selo GovTech BrazilLAB.</t>
         </is>
       </c>
       <c r="I9" s="13" t="inlineStr"/>
@@ -2544,7 +2556,7 @@
       </c>
       <c r="B10" s="15" t="inlineStr">
         <is>
-          <t>Relações Trabalhistas</t>
+          <t>Gestão de Relações Trabalhistas e Sindicais (RTS)</t>
         </is>
       </c>
       <c r="C10" s="15" t="inlineStr">
@@ -2564,7 +2576,7 @@
       </c>
       <c r="F10" s="15" t="inlineStr">
         <is>
-          <t>N/D</t>
+          <t>Unilever, Coca-Cola, Vivo, Burger King, C&amp;A | 29 colaboradores</t>
         </is>
       </c>
       <c r="G10" s="15" t="inlineStr">
@@ -2574,10 +2586,14 @@
       </c>
       <c r="H10" s="15" t="inlineStr">
         <is>
-          <t>Digitalização da gestão de relações sindicais. Captou R$3,4M do Fundo GovTech KPTL.</t>
-        </is>
-      </c>
-      <c r="I10" s="15" t="inlineStr"/>
+          <t>Ecossistema SaaS de digitalização de RTS: gestão de CCTs, IA 'Norma' para análise de cláusulas, assembleias virtuais e data intelligence. Integração com HCM via parceria LG. Prêmio inovação RH 2025. R$3,4M Fundo GovTech KPTL.</t>
+        </is>
+      </c>
+      <c r="I10" s="16" t="inlineStr">
+        <is>
+          <t>Portfólio KPTL</t>
+        </is>
+      </c>
       <c r="J10" s="15" t="inlineStr"/>
     </row>
     <row r="11" ht="48" customHeight="1">
@@ -2588,7 +2604,7 @@
       </c>
       <c r="B11" s="13" t="inlineStr">
         <is>
-          <t>ERP Municipal / SIAFIC</t>
+          <t>ERP Municipal Integrado / SIAFIC Cloud</t>
         </is>
       </c>
       <c r="C11" s="13" t="inlineStr">
@@ -2598,7 +2614,7 @@
       </c>
       <c r="D11" s="13" t="inlineStr">
         <is>
-          <t>N/D (Brasil)</t>
+          <t>Brasil</t>
         </is>
       </c>
       <c r="E11" s="13" t="inlineStr">
@@ -2608,7 +2624,7 @@
       </c>
       <c r="F11" s="13" t="inlineStr">
         <is>
-          <t>Municípios (SIAFIC)</t>
+          <t>Municípios de qualquer porte | SIAFIC + SIEDUC disponíveis</t>
         </is>
       </c>
       <c r="G11" s="13" t="inlineStr">
@@ -2618,7 +2634,7 @@
       </c>
       <c r="H11" s="13" t="inlineStr">
         <is>
-          <t>ERP municipal integrado 100% cloud: SIAFIC + saúde + educação + assistência social. Conformidade SIAFIC obrigatória impulsiona substituição de legados.</t>
+          <t>Suite ERP municipal integrada em nuvem com base de dados única: SIAFIC (financeiro/tributário), SIEDUC (educação), SISAÚDE e SIASOC. Conformidade SICONFI, SIOPE, e-Social, eSUS. Produto novo no mercado com proposta de stack completo integrado.</t>
         </is>
       </c>
       <c r="I11" s="17" t="inlineStr">
@@ -2636,7 +2652,7 @@
       </c>
       <c r="B12" s="15" t="inlineStr">
         <is>
-          <t>Participação Cidadã / Gestão Pública</t>
+          <t>Participação Cidadã e Serviços Digitais Municipais</t>
         </is>
       </c>
       <c r="C12" s="15" t="inlineStr">
@@ -2646,7 +2662,7 @@
       </c>
       <c r="D12" s="15" t="inlineStr">
         <is>
-          <t>Brasil</t>
+          <t>São Paulo - SP</t>
         </is>
       </c>
       <c r="E12" s="15" t="inlineStr">
@@ -2656,7 +2672,7 @@
       </c>
       <c r="F12" s="15" t="inlineStr">
         <is>
-          <t>20M+ pessoas impactadas</t>
+          <t>5 países | 1M+ cidadãos | Piauí, São Gonçalo, Santo André | Parceiro ONU-Habitat</t>
         </is>
       </c>
       <c r="G12" s="15" t="inlineStr">
@@ -2666,7 +2682,7 @@
       </c>
       <c r="H12" s="15" t="inlineStr">
         <is>
-          <t>Plataforma de gestão pública e participação cidadã: zeladoria urbana, CRM prefeitura-cidadão e marketplace de serviços públicos digitais. 1º investimento da KPTL em 2014. Follow-on pelo Fundo GovTech (KPTL+Cedro) em 2023. Co-invest EDP.</t>
+          <t>Plataforma multicanal (web, app, WhatsApp) de gestão de serviços digitais, participação cidadã e CRM governamental. IA digitaliza qualquer serviço público em minutos. Em 2025 viabilizou OP Digital do Piauí (273k participantes) com validação via Receita Federal e blockchain. Portfólio KPTL+Cedro. Co-invest EDP.</t>
         </is>
       </c>
       <c r="I12" s="16" t="inlineStr">
@@ -2732,7 +2748,7 @@
       </c>
       <c r="B14" s="15" t="inlineStr">
         <is>
-          <t>Planejamento Urbano / GeoInteligência</t>
+          <t>Planejamento Urbano e Geointeligência / Urban Twin</t>
         </is>
       </c>
       <c r="C14" s="15" t="inlineStr">
@@ -2752,7 +2768,7 @@
       </c>
       <c r="F14" s="15" t="inlineStr">
         <is>
-          <t>Municípios</t>
+          <t>Prefeituras e mercado imobiliário privado</t>
         </is>
       </c>
       <c r="G14" s="15" t="inlineStr">
@@ -2762,7 +2778,7 @@
       </c>
       <c r="H14" s="15" t="inlineStr">
         <is>
-          <t>Plataforma que integra dados de mercado imobiliário, urbanismo e legislação municipal em interface intuitiva para gestores públicos. Certificada BrazilLAB. Suporte a decisões de planejamento territorial e uso do solo.</t>
+          <t>Plataforma dual (govtech + proptech) de inteligência territorial com Gêmeo Digital: integra bases públicas, rotinas urbanísticas, pré-aprovação de projetos e visualização 2D/3D com IA aplicada à legislação urbanística. Para o setor privado: viabilidade e gestão de portfólio imobiliário. Certificada BrazilLAB.</t>
         </is>
       </c>
       <c r="I14" s="16" t="inlineStr">
@@ -2868,7 +2884,7 @@
       </c>
       <c r="B3" s="13" t="inlineStr">
         <is>
-          <t>Indicadores ODS / Financiamento Municipal</t>
+          <t>Governança Municipal Baseada em Dados / ODS</t>
         </is>
       </c>
       <c r="C3" s="13" t="inlineStr">
@@ -2888,7 +2904,7 @@
       </c>
       <c r="F3" s="13" t="inlineStr">
         <is>
-          <t>Municípios | 2M+ cid.</t>
+          <t>1.000+ gestores formados | SEDE-MG, FINEP, PNUD, UNESCO, ALMG</t>
         </is>
       </c>
       <c r="G3" s="13" t="inlineStr">
@@ -2898,7 +2914,7 @@
       </c>
       <c r="H3" s="13" t="inlineStr">
         <is>
-          <t>Plataforma CHESI: 160+ indicadores ODS + fontes de financiamento + governança. Parceria SEDE-MG Cidades do Futuro.</t>
+          <t>GovTech de governança orientada a dados com metodologia CHESI (registrada no INPI): 160+ indicadores ODS monitorados em tempo real, conectando projetos a financiamento público. Produz Relatórios Locais Voluntários para Agenda 2030. Coordena GT Cidades Inteligentes da ALMG.</t>
         </is>
       </c>
       <c r="I3" s="13" t="inlineStr"/>
@@ -2912,7 +2928,7 @@
       </c>
       <c r="B4" s="15" t="inlineStr">
         <is>
-          <t>Fiscal / Alvarás Digitais</t>
+          <t>Alvará Digital e Licenciamento de Empresas Municipal</t>
         </is>
       </c>
       <c r="C4" s="15" t="inlineStr">
@@ -2932,7 +2948,7 @@
       </c>
       <c r="F4" s="15" t="inlineStr">
         <is>
-          <t>Municípios MG</t>
+          <t>MG, RO, PE, MT | 480+ municípios via Jucemg/SINAL</t>
         </is>
       </c>
       <c r="G4" s="15" t="inlineStr">
@@ -2942,12 +2958,12 @@
       </c>
       <c r="H4" s="15" t="inlineStr">
         <is>
-          <t>Alvarás digitais: reduz 90% do prazo de emissão. 2º DemoDay BrazilLAB 2023. Selecionada PBH Inova (2 desafios).</t>
+          <t>Sistema de gestão de licenciamento e abertura de empresas, com alvarás digitais via QR Code e integração REDESIM. Parceiro estadual da Jucemg para o sistema SINAL (480+ municípios de MG). Apoio Seed-MG e AWS. Reduz prazo de emissão de alvarás em 90%. BrazilLAB 2023.</t>
         </is>
       </c>
       <c r="I4" s="16" t="inlineStr">
         <is>
-          <t>Watch — fiscal municipal</t>
+          <t>Watch — expansão estadual Jucemg</t>
         </is>
       </c>
       <c r="J4" s="15" t="inlineStr"/>
@@ -2960,7 +2976,7 @@
       </c>
       <c r="B5" s="13" t="inlineStr">
         <is>
-          <t>Convênios / Transferências Federais</t>
+          <t>Gestão de Convênios e Transferências Federais com IA</t>
         </is>
       </c>
       <c r="C5" s="13" t="inlineStr">
@@ -2970,7 +2986,7 @@
       </c>
       <c r="D5" s="13" t="inlineStr">
         <is>
-          <t>N/D (Brasil)</t>
+          <t>Brasil</t>
         </is>
       </c>
       <c r="E5" s="13" t="inlineStr">
@@ -2980,7 +2996,7 @@
       </c>
       <c r="F5" s="13" t="inlineStr">
         <is>
-          <t>Municípios (convênios)</t>
+          <t>Municípios de qualquer porte | integra TransfereGov, Simec, Sismob, FNS, Sigcon</t>
         </is>
       </c>
       <c r="G5" s="13" t="inlineStr">
@@ -2990,7 +3006,7 @@
       </c>
       <c r="H5" s="13" t="inlineStr">
         <is>
-          <t>Gestão de convênios com IA: integra TransfereGov, Simec, SISMOB, FNS. Vertical exclusivo de captação e gestão de transferências federais para municípios.</t>
+          <t>Primeiro sistema inteligente de gestão de convênios para prefeituras: unifica automaticamente TransfereGov, Simec, Sismob, FNS e Sigcon em painel único com IA. Kanban automático de diligências, alertas de prazo, monitoramento de certidões, previsão de repasses e elaboração de propostas com IA baseadas em cotações federais. Diferencial: deixa a IA captar e monitorar enquanto a prefeitura foca na execução.</t>
         </is>
       </c>
       <c r="I5" s="17" t="inlineStr">
@@ -3008,7 +3024,7 @@
       </c>
       <c r="B6" s="15" t="inlineStr">
         <is>
-          <t>Inteligência Fiscal Municipal</t>
+          <t>Score Fiscal e Inteligência de Risco Municipal</t>
         </is>
       </c>
       <c r="C6" s="15" t="inlineStr">
@@ -3028,7 +3044,7 @@
       </c>
       <c r="F6" s="15" t="inlineStr">
         <is>
-          <t>5.570 municípios (dados)</t>
+          <t>100% dos 5.570 municípios brasileiros (dados) | B2B: fornecedores, bancos, seguradoras</t>
         </is>
       </c>
       <c r="G6" s="15" t="inlineStr">
@@ -3038,7 +3054,7 @@
       </c>
       <c r="H6" s="15" t="inlineStr">
         <is>
-          <t>Score fiscal para todos os 5.570 municípios brasileiros. Fundada 2026. Plataforma B2B/B2G de avaliação de saúde fiscal e creditícia municipal.</t>
+          <t>Plataforma SaaS de score fiscal para municípios: nota de 0 a 1000 cruzando receita, despesa, endividamento e CAPAG (STN). Integra PNCP, TransfereGov, emendas parlamentares e PCA para identificar oportunidades de fornecimento. Assistente de IA com 4 perspectivas analíticas. Fundadores: Diego Barros (CEO) e Antonio Firmino (Chairman / Grupo Triasa). Planos a partir de R$97/mês.</t>
         </is>
       </c>
       <c r="I6" s="16" t="inlineStr">
@@ -3056,7 +3072,7 @@
       </c>
       <c r="B7" s="13" t="inlineStr">
         <is>
-          <t>GeoInteligência Fiscal</t>
+          <t>GeoInteligência Fiscal / Cadastro Imobiliário</t>
         </is>
       </c>
       <c r="C7" s="13" t="inlineStr">
@@ -3066,17 +3082,17 @@
       </c>
       <c r="D7" s="13" t="inlineStr">
         <is>
-          <t>Curitiba - PR</t>
+          <t>São José dos Campos - SP</t>
         </is>
       </c>
       <c r="E7" s="13" t="inlineStr">
         <is>
-          <t>~2010</t>
+          <t>~2008</t>
         </is>
       </c>
       <c r="F7" s="13" t="inlineStr">
         <is>
-          <t>100+ municípios</t>
+          <t>100+ municípios | clientes: Amparo SP, Teresópolis RJ, Guaratinguetá SP</t>
         </is>
       </c>
       <c r="G7" s="13" t="inlineStr">
@@ -3086,7 +3102,7 @@
       </c>
       <c r="H7" s="13" t="inlineStr">
         <is>
-          <t>Geoprocessamento + IA para IPTU, ITBI, ISS. Reforma Tributária (LC 214/2025) cria janela de demanda direta e imediata.</t>
+          <t>18 anos como líder em geointeligência para prefeituras. Plataforma Geopixel Cidades integra geoprocessamento com IA para IPTU, ITBI, ISS e alvarás (digital e por QR Code). Módulos: SIG municipal integrado, monitoramento por satélite de alterações, mobilidade de campo e eventos ambientais. Reforma Tributária (LC 214/2025) cria janela de demanda direta e imediata.</t>
         </is>
       </c>
       <c r="I7" s="17" t="inlineStr">
@@ -3152,7 +3168,7 @@
       </c>
       <c r="B9" s="13" t="inlineStr">
         <is>
-          <t>IA Analytics / Orçamento Municipal</t>
+          <t>IA 3P para Gestão Municipal / Dashboard Analítico</t>
         </is>
       </c>
       <c r="C9" s="13" t="inlineStr">
@@ -3162,7 +3178,7 @@
       </c>
       <c r="D9" s="13" t="inlineStr">
         <is>
-          <t>N/D (Brasil)</t>
+          <t>Porto Alegre - RS</t>
         </is>
       </c>
       <c r="E9" s="13" t="inlineStr">
@@ -3172,7 +3188,7 @@
       </c>
       <c r="F9" s="13" t="inlineStr">
         <is>
-          <t>N/D</t>
+          <t>50+ municípios | 8 áreas da gestão pública</t>
         </is>
       </c>
       <c r="G9" s="13" t="inlineStr">
@@ -3182,7 +3198,7 @@
       </c>
       <c r="H9" s="13" t="inlineStr">
         <is>
-          <t>Plataforma IA para gestão municipal: analytics preditivo + preventivo + prescritivo. Integra dados orçamentários, operacionais e sociais para apoio à decisão do gestor público.</t>
+          <t>Plataforma de IA para gestão pública com metodologia exclusiva 3P: Preditiva (projeta receitas, saúde e matrículas), Preventiva (alertas automáticos de anomalias e contratos) e Prescritiva (sugere onde cortar custos, otimizar frota e compras). Dashboards interativos para todas as secretarias. Chat inteligente para consultas sobre dados oficiais da cidade. Marketplace de soluções parceiras integradas nativamente.</t>
         </is>
       </c>
       <c r="I9" s="17" t="inlineStr">
@@ -3288,7 +3304,7 @@
       </c>
       <c r="B3" s="13" t="inlineStr">
         <is>
-          <t>Atenção Primária / Suite</t>
+          <t>Suite de Gestão Pública Municipal (Saúde, Educ, Dados, Frota)</t>
         </is>
       </c>
       <c r="C3" s="13" t="inlineStr">
@@ -3308,7 +3324,7 @@
       </c>
       <c r="F3" s="13" t="inlineStr">
         <is>
-          <t>Municípios SP</t>
+          <t>Municípios SP e outros estados</t>
         </is>
       </c>
       <c r="G3" s="13" t="inlineStr">
@@ -3318,7 +3334,7 @@
       </c>
       <c r="H3" s="13" t="inlineStr">
         <is>
-          <t>Suite municipal: Saúde Simples + Educação + DadosGov + Mobilidade + Doc+. 350 colaboradores. Meta: 2x municípios SP até 2030. IA reduz 40% tempo de consultas SUS.</t>
+          <t>Suite modular de soluções estratégicas para gestão pública: Saúde Simples (prontuário, telemedicina, IA transcrevendo consultas), Educação Simples (gestão escolar), DadosGov Simples (BI exclusivo setor público), Mob Simples (gestão de frotas), Doc+ Simples (gestão documental), Outsourcing Simples (impressão) e Mentor Público (IEG-M com IA). 1º prontuário transcrito por IA da saúde pública do Brasil. Crescimento 40% na pandemia.</t>
         </is>
       </c>
       <c r="I3" s="17" t="inlineStr">
@@ -3404,7 +3420,7 @@
       </c>
       <c r="F5" s="13" t="inlineStr">
         <is>
-          <t>Municípios MG + NE</t>
+          <t>Municípios MG + NE | Filiais SP e PB</t>
         </is>
       </c>
       <c r="G5" s="13" t="inlineStr">
@@ -3414,7 +3430,7 @@
       </c>
       <c r="H5" s="13" t="inlineStr">
         <is>
-          <t>26 anos de operação. Selos Ouro/Prata Bora Vacinar (mar/2025). Filiais SP e PB. Foco saúde pública + educação municipal integradas.</t>
+          <t>26 anos de operação em saúde pública e gestão municipal. Selos Ouro/Prata Bora Vacinar (mar/2025). Cliente Sorocaba SP avançou C+ → B no IEGM 2025. Foco saúde pública + educação municipal integradas.</t>
         </is>
       </c>
       <c r="I5" s="17" t="inlineStr">
@@ -3432,12 +3448,12 @@
       </c>
       <c r="B6" s="15" t="inlineStr">
         <is>
-          <t>Analytics / BI para APS</t>
+          <t>BI Preventivo para APS / Saúde Pública</t>
         </is>
       </c>
       <c r="C6" s="15" t="inlineStr">
         <is>
-          <t>Startup early-stage</t>
+          <t>ONG / Não-lucrativa</t>
         </is>
       </c>
       <c r="D6" s="15" t="inlineStr">
@@ -3452,17 +3468,17 @@
       </c>
       <c r="F6" s="15" t="inlineStr">
         <is>
-          <t>Municípios via SUS</t>
+          <t>410+ municípios | 16M pessoas | 134k+ rotinas preventivas adicionais (2023)</t>
         </is>
       </c>
       <c r="G6" s="15" t="inlineStr">
         <is>
-          <t>US$ 100k</t>
+          <t>US$ 100k (Mulago Foundation)</t>
         </is>
       </c>
       <c r="H6" s="15" t="inlineStr">
         <is>
-          <t>BI para gaps de atenção básica preventiva. Cofundada por ex-Harvard Kennedy School. Reconhecida pela CGU. Impulso Previne.</t>
+          <t>ONG com execução de startup focada em fechar gaps da atenção primária do SUS. Plataforma Impulso Previne: identifica pacientes em atraso em exames, vacinas e pré-natal e direciona agentes comunitários com listas priorizadas + SMS automático para cidadãos. Também atua em saúde mental (capacitação para depressão). Cofundada por ex-Harvard Kennedy School. Reconhecida pela CGU.</t>
         </is>
       </c>
       <c r="I6" s="15" t="inlineStr"/>
@@ -3486,7 +3502,7 @@
       </c>
       <c r="D7" s="13" t="inlineStr">
         <is>
-          <t>São Paulo - SP</t>
+          <t>Vitória - ES</t>
         </is>
       </c>
       <c r="E7" s="13" t="inlineStr">
@@ -3520,7 +3536,7 @@
       </c>
       <c r="B8" s="15" t="inlineStr">
         <is>
-          <t>Analytics APS / Educação</t>
+          <t>Gestão de Saúde e Dados Municipais</t>
         </is>
       </c>
       <c r="C8" s="15" t="inlineStr">
@@ -3540,7 +3556,7 @@
       </c>
       <c r="F8" s="15" t="inlineStr">
         <is>
-          <t>Municípios MG e outros</t>
+          <t>15+ municípios | 5 estados | MG, PR, ES, AL, PA</t>
         </is>
       </c>
       <c r="G8" s="15" t="inlineStr">
@@ -3550,7 +3566,7 @@
       </c>
       <c r="H8" s="15" t="inlineStr">
         <is>
-          <t>Analytics Previne Brasil: gaps, captação de recursos, indicadores APS. 3ª DemoDay BrazilLAB 2023.</t>
+          <t>Soluções integradas para modernização municipal: Módulo Saúde (prontuários, regulação, vigilância sanitária) e Módulo Gestão de Dados (integração e consultoria em BI municipal). 100 Open Startups Top 10, Seed Gov, BrazilLAB, Centelha, Young Founders Program. +R$100M gerenciados em clientes.</t>
         </is>
       </c>
       <c r="I8" s="15" t="inlineStr"/>
@@ -3564,7 +3580,7 @@
       </c>
       <c r="B9" s="13" t="inlineStr">
         <is>
-          <t>Escalas / Anti-fraude Saúde</t>
+          <t>Gestão de Escalas Médicas / Anti-fraude em Saúde</t>
         </is>
       </c>
       <c r="C9" s="13" t="inlineStr">
@@ -3574,7 +3590,7 @@
       </c>
       <c r="D9" s="13" t="inlineStr">
         <is>
-          <t>N/D (Brasil)</t>
+          <t>Brasil</t>
         </is>
       </c>
       <c r="E9" s="13" t="inlineStr">
@@ -3584,7 +3600,7 @@
       </c>
       <c r="F9" s="13" t="inlineStr">
         <is>
-          <t>UBS / Municípios</t>
+          <t>50+ organizações | cooperativas, hospitais e grupos médicos</t>
         </is>
       </c>
       <c r="G9" s="13" t="inlineStr">
@@ -3594,7 +3610,7 @@
       </c>
       <c r="H9" s="13" t="inlineStr">
         <is>
-          <t>Gestão de escalas e plantões para saúde pública municipal. Anti-fraude em folha de pagamento. Top 30 Sebrae 2024. Acelerada GovTech Pará.</t>
+          <t>Aplicativo para gestão de escala médica em um só lugar: elimina planilhas, automatiza escalas de plantão e reduz glosas e fraudes administrativas. 50+ organizações economizando milhões. Top 30 Sebrae 2024. Acelerada GovTech Pará.</t>
         </is>
       </c>
       <c r="I9" s="17" t="inlineStr">
@@ -3700,7 +3716,7 @@
       </c>
       <c r="B3" s="13" t="inlineStr">
         <is>
-          <t>Gestão Escolar (SIE)</t>
+          <t>Gestão Escolar e SUAS (SIE + Software Público)</t>
         </is>
       </c>
       <c r="C3" s="13" t="inlineStr">
@@ -3720,7 +3736,7 @@
       </c>
       <c r="F3" s="13" t="inlineStr">
         <is>
-          <t>140+ mun | 700k+ alunos</t>
+          <t>100+ mun | 700k+ alunos | 200k+ famílias SUAS | 47k+ professores</t>
         </is>
       </c>
       <c r="G3" s="13" t="inlineStr">
@@ -3730,7 +3746,7 @@
       </c>
       <c r="H3" s="13" t="inlineStr">
         <is>
-          <t>Mantenedora i-Educar (software público federal). Parceria MEC e Fundação Lemann. Meta: 1,5M alunos até 2027.</t>
+          <t>Mantenedora do i-Educar (software público federal MEC). Abriu o código-fonte do Pré-Matrícula Digital (PMD) em parceria com MEC, Fundação Lemann e MP-SC. Também atua em assistência social (SUAS): 50+ municípios, 200k+ famílias. Meta: 1,5M alunos até 2027. Parceria Portábilis+Educa Rios expandindo para AM.</t>
         </is>
       </c>
       <c r="I3" s="17" t="inlineStr">
@@ -3802,7 +3818,7 @@
       </c>
       <c r="D5" s="13" t="inlineStr">
         <is>
-          <t>N/D</t>
+          <t>Brasil</t>
         </is>
       </c>
       <c r="E5" s="13" t="inlineStr">
@@ -3836,7 +3852,7 @@
       </c>
       <c r="B6" s="15" t="inlineStr">
         <is>
-          <t>Aprendizagem IA / Híbrida</t>
+          <t>Aprendizagem IA / Ensino Híbrido</t>
         </is>
       </c>
       <c r="C6" s="15" t="inlineStr">
@@ -3856,7 +3872,7 @@
       </c>
       <c r="F6" s="15" t="inlineStr">
         <is>
-          <t>5k esc | 12M alunos</t>
+          <t>5k+ escolas | 12M alunos | parceria MEC + Arco Educação</t>
         </is>
       </c>
       <c r="G6" s="15" t="inlineStr">
@@ -3866,7 +3882,7 @@
       </c>
       <c r="H6" s="15" t="inlineStr">
         <is>
-          <t>415k alunos rede estadual SP (gratuito). Parceria MEC desde 2014. IA + ensino híbrido. Potencial alvo M&amp;A.</t>
+          <t>Plataforma Geekie One: solução completa de aprendizagem personalizada com IA para todos os segmentos (Infantil, Fund., Médio). BNCC-compliant. 415k+ alunos rede estadual SP (gratuito). Parceria MEC desde 2014 e Arco Educação+OpenAI. Brilhando Juntos: programa de marketing e retenção para escolas parceiras.</t>
         </is>
       </c>
       <c r="I6" s="15" t="inlineStr"/>
@@ -3890,17 +3906,17 @@
       </c>
       <c r="D7" s="13" t="inlineStr">
         <is>
-          <t>N/D (Brasil)</t>
+          <t>Ribeirão Preto - SP</t>
         </is>
       </c>
       <c r="E7" s="13" t="inlineStr">
         <is>
-          <t>N/D</t>
+          <t>~2015</t>
         </is>
       </c>
       <c r="F7" s="13" t="inlineStr">
         <is>
-          <t>Rede estadual GO</t>
+          <t>4M+ pessoas | 430M+ exercícios | 100% das redes parceiras melhoraram IDEB</t>
         </is>
       </c>
       <c r="G7" s="13" t="inlineStr">
@@ -3910,7 +3926,7 @@
       </c>
       <c r="H7" s="13" t="inlineStr">
         <is>
-          <t>Selecionada Governo de Goiás. Gamificação + IA em Português e Matemática para redes públicas.</t>
+          <t>10 anos de EdTech gamificada com IA adaptativa: avaliações digitais, jogos adaptativos e leitura Fi.Git.Al (físico+digital+social). Metodologia Flow + BNCC. Clientes: redes estaduais GO e BR, escolas públicas e privadas. 100% das redes parceiras melhoraram seu IDEB. Programas: Liga das Corujinhas, Alfabetização, Expedição, Olimpíadas.</t>
         </is>
       </c>
       <c r="I7" s="13" t="inlineStr"/>
@@ -3988,7 +4004,7 @@
       </c>
       <c r="F9" s="13" t="inlineStr">
         <is>
-          <t>80+ prefeituras ativas</t>
+          <t>80+ prefeituras | 2.050+ escolas | 500k+ alunos</t>
         </is>
       </c>
       <c r="G9" s="13" t="inlineStr">
@@ -3998,7 +4014,7 @@
       </c>
       <c r="H9" s="13" t="inlineStr">
         <is>
-          <t>Software público federal mantido por Portabilis. Monte Alegre (RN) economizou R$2,4M. Parceria MEC + MP.</t>
+          <t>Software público federal mantido pela Portabilis. Pré-Matrícula Digital PMD aberto ao público em 2025 (código no GitHub). Monte Alegre (RN) economizou R$2,4M. Parceria MEC + Fundação Lemann + MP-SC. Canoas RS referência em implementação.</t>
         </is>
       </c>
       <c r="I9" s="17" t="inlineStr">
@@ -4036,7 +4052,7 @@
       </c>
       <c r="F10" s="15" t="inlineStr">
         <is>
-          <t>50+ municípios | est. SP</t>
+          <t>5.000+ instituições | 100M+ questões | 400k+ conteúdos BNCC</t>
         </is>
       </c>
       <c r="G10" s="15" t="inlineStr">
@@ -4046,7 +4062,7 @@
       </c>
       <c r="H10" s="15" t="inlineStr">
         <is>
-          <t>Plataforma adaptativa de aprendizagem e avaliação gamificada. 90% dos alunos em escolas públicas. 83% dos usuários em rede pública. Meta: 10M alunos até 2030. Rodada seed R$11,8M liderada pelo Fundo GovTech (KPTL+Cedro) com DOMO.VC, Criabiz Ventures e Rosey Ventures (Grupo Marista). Mar/2026.</t>
+          <t>Maior plataforma de aprendizagem adaptativa gamificada do Brasil. 90% dos alunos em escolas públicas. +18% ganho de aprendizagem em poucos meses. Meta: 10M alunos até 2030. Rodada seed R$11,8M liderada pelo Fundo GovTech (KPTL+Cedro) com DOMO.VC, Criabiz Ventures e Rosey Ventures (Grupo Marista). Mar/2026. Parceiro Edebê Brasil (escolas Salesianas).</t>
         </is>
       </c>
       <c r="I10" s="16" t="inlineStr">
@@ -4152,7 +4168,7 @@
       </c>
       <c r="B3" s="13" t="inlineStr">
         <is>
-          <t>Agentes RPA / WhatsApp</t>
+          <t>Agentes IA / WhatsApp Municipal</t>
         </is>
       </c>
       <c r="C3" s="13" t="inlineStr">
@@ -4162,7 +4178,7 @@
       </c>
       <c r="D3" s="13" t="inlineStr">
         <is>
-          <t>Porto Alegre - RS</t>
+          <t>Gravataí - RS</t>
         </is>
       </c>
       <c r="E3" s="13" t="inlineStr">
@@ -4182,7 +4198,7 @@
       </c>
       <c r="H3" s="13" t="inlineStr">
         <is>
-          <t>Agentes IA via WhatsApp. Opera sistemas municipais sem integração tradicional. 200+ municípios em &lt;12 meses. Modelo viral, alta tração.</t>
+          <t>Agentes IA via WhatsApp que operam sistemas municipais sem integração tradicional. 200+ municípios em menos de 12 meses. Modelo viral de adoção. Potencial alvo de aquisição.</t>
         </is>
       </c>
       <c r="I3" s="17" t="inlineStr">
@@ -4220,7 +4236,7 @@
       </c>
       <c r="F4" s="15" t="inlineStr">
         <is>
-          <t>Setor público e privado</t>
+          <t>Setor público e privado | financeiro, seguros, utilities, gov</t>
         </is>
       </c>
       <c r="G4" s="15" t="inlineStr">
@@ -4230,7 +4246,7 @@
       </c>
       <c r="H4" s="15" t="inlineStr">
         <is>
-          <t>Ultra OCR®: automação de documentos públicos. Contratos, invoices, documentos de identidade. Gov + corporativo.</t>
+          <t>Ultra OCR®: automação de análise de documentos com IA — classificação, extração de dados, comparação e validação em bases públicas. Gov Hub: onboarding de alunos, profissionais liberais e pessoas jurídicas. Human-in-the-loop para revisão de casos críticos. Presente em grandes empresas financeiras e setor público.</t>
         </is>
       </c>
       <c r="I4" s="15" t="inlineStr"/>
@@ -4264,7 +4280,7 @@
       </c>
       <c r="F5" s="13" t="inlineStr">
         <is>
-          <t>Governo Federal</t>
+          <t>Governo Federal | MGI, telecom, utilities</t>
         </is>
       </c>
       <c r="G5" s="13" t="inlineStr">
@@ -4274,7 +4290,7 @@
       </c>
       <c r="H5" s="13" t="inlineStr">
         <is>
-          <t>Projeto INSPIRE com MGI (R$390M, 4 anos). IA personalizada para serviços de governo digital: chatbots, recomendação, acessibilidade.</t>
+          <t>Instituto de P&amp;D referência em telecomunicações e tecnologias convergentes. Projeto INSPIRE com MGI (R$390M, 4 anos): IA personalizada para serviços de governo digital — assistentes virtuais de voz, recomendação e acessibilidade. Portfólio inclui IoT, Blockchain, IA, Conectividade Inteligente, OSS/BSS. Mais de 30 soluções comerciais.</t>
         </is>
       </c>
       <c r="I5" s="17" t="inlineStr">
@@ -4302,7 +4318,7 @@
       </c>
       <c r="D6" s="15" t="inlineStr">
         <is>
-          <t>N/D (Brasil)</t>
+          <t>Brasil</t>
         </is>
       </c>
       <c r="E6" s="15" t="inlineStr">
@@ -4360,7 +4376,7 @@
       </c>
       <c r="F7" s="13" t="inlineStr">
         <is>
-          <t>100+ clientes | 27 estados + 1k+ mun.</t>
+          <t>100+ clientes | 27 estados + 1k+ mun. | +700 fontes</t>
         </is>
       </c>
       <c r="G7" s="13" t="inlineStr">
@@ -4370,7 +4386,7 @@
       </c>
       <c r="H7" s="13" t="inlineStr">
         <is>
-          <t>Pioneira em monitoramento automatizado de dados governamentais (Legislativo, Executivo, Judiciário). 4M+ proposições monitoradas. ~890 fontes de Diários Oficiais. IA com termômetro de aprovação de PLs (&gt;98% acurácia). Única com 100% de cobertura das Assembleias Estaduais. Ranking 100 Open Startups, Mapa GovTech. Cubo Itaú, Inovabra, Distrito.</t>
+          <t>Pioneira em monitoramento automatizado de dados governamentais (Legislativo, Executivo, Judiciário). 4M+ proposições monitoradas, +700 fontes incluindo Diários Oficiais. IA com termômetro de aprovação de PLs (&gt;98% acurácia). Única com 100% de cobertura das Assembleias Estaduais. Plataforma de Stakeholders para gestão de contatos e RIG. Ranking 100 Open Startups, Mapa GovTech. Cubo Itaú, Inovabra, Distrito.</t>
         </is>
       </c>
       <c r="I7" s="17" t="inlineStr">
@@ -4460,7 +4476,7 @@
       </c>
       <c r="F9" s="13" t="inlineStr">
         <is>
-          <t>Indústria + gov</t>
+          <t>29 países | Indústria + gov | 300k+ trabalhadores monitorados</t>
         </is>
       </c>
       <c r="G9" s="13" t="inlineStr">
@@ -4470,7 +4486,7 @@
       </c>
       <c r="H9" s="13" t="inlineStr">
         <is>
-          <t>IA para análises ergonômicas e psicossociais via visão computacional. Clientes: Marfrig, P&amp;G, Electrolux. 8º investimento do Fundo GovTech (KPTL+Cedro), R$3M em fev/2026. Foco em saúde do trabalhador para setor público e privado. Expansão global planejada.</t>
+          <t>IA + visão computacional para análises ergonômicas e psicossociais automatizadas: reconhecimento de movimentos, quantificação de riscos biomecânicos e cronoanálise (Indústria 4.0). Resultados: -38% FAP, -30% afastamentos por DORT, análises 5x mais rápidas. Clientes: Marfrig, CNH Industrial, P&amp;G, Electrolux, Vibra. 8º investimento Fundo GovTech (KPTL+Cedro), R$3M fev/2026. Campus da Indústria FIEP. 29 países.</t>
         </is>
       </c>
       <c r="I9" s="17" t="inlineStr">
@@ -4591,7 +4607,7 @@
       </c>
       <c r="E3" s="13" t="inlineStr">
         <is>
-          <t>2025</t>
+          <t>fev/2024</t>
         </is>
       </c>
       <c r="F3" s="13" t="inlineStr">
@@ -4619,12 +4635,12 @@
     <row r="4" ht="48" customHeight="1">
       <c r="A4" s="14" t="inlineStr">
         <is>
-          <t>Attus Procuradoria Digital</t>
+          <t>Attus</t>
         </is>
       </c>
       <c r="B4" s="15" t="inlineStr">
         <is>
-          <t>IA Contencioso + Consultivo (PGE/PGM)</t>
+          <t>IA Generativa + Automações para Procuradorias (PGE/PGM)</t>
         </is>
       </c>
       <c r="C4" s="15" t="inlineStr">
@@ -4634,7 +4650,7 @@
       </c>
       <c r="D4" s="15" t="inlineStr">
         <is>
-          <t>São Ludgero, SC (Eloware)</t>
+          <t>São Ludgero - SC (Grupo Eloware)</t>
         </is>
       </c>
       <c r="E4" s="15" t="inlineStr">
@@ -4654,7 +4670,7 @@
       </c>
       <c r="H4" s="15" t="inlineStr">
         <is>
-          <t>4,3M+ processos analisados. 73% classificados automaticamente (98,5% acurácia). 642k+ peças geradas por IA. Referência nacional pós PGE-SP.</t>
+          <t>Rebrand de Attornatus (dez/2023) para Attus. IA generativa treinada exclusivamente na realidade de cada procuradoria: sínteses inteligentes de processos, geração de minutas, agente jurídico interativo. Centenas de automações em bastidores. Recuperação inteligente de Dívida Ativa com enriquecimento cadastral via Receita Federal. 4,3M+ processos analisados. 73% classificados automaticamente (98,5% acurácia). 642k+ peças geradas por IA. Referência nacional pós PGE-SP.</t>
         </is>
       </c>
       <c r="I4" s="16" t="inlineStr">
@@ -4682,7 +4698,7 @@
       </c>
       <c r="D5" s="13" t="inlineStr">
         <is>
-          <t>N/D (Brasil)</t>
+          <t>Brasil</t>
         </is>
       </c>
       <c r="E5" s="13" t="inlineStr">
@@ -4726,7 +4742,7 @@
       </c>
       <c r="D6" s="15" t="inlineStr">
         <is>
-          <t>N/D (Brasil)</t>
+          <t>Campos dos Goytacazes - RJ</t>
         </is>
       </c>
       <c r="E6" s="15" t="inlineStr">
@@ -4736,7 +4752,7 @@
       </c>
       <c r="F6" s="15" t="inlineStr">
         <is>
-          <t>Procuradorias municipais</t>
+          <t>Procuradorias municipais RJ e outros estados</t>
         </is>
       </c>
       <c r="G6" s="15" t="inlineStr">
@@ -4746,7 +4762,7 @@
       </c>
       <c r="H6" s="15" t="inlineStr">
         <is>
-          <t>RPA integrado para peticionamento automático em qualquer TJ do país. Interface co-desenvolvida com procuradores municipais.</t>
+          <t>Software jurídico SaaS para procuradorias municipais com automação RPA: peticionamento automático em qualquer TJ do país, captura de publicações e intimações 24/7, gestão de prazos e processos judiciais e administrativos. IA integrada. Desenvolvido co-criação com procuradores. Cases: PGM Campos dos Goytacazes RJ, São Francisco de Itabopoana RJ, São Pedro da Aldeia RJ, COMSERCAF Cabo Frio RJ.</t>
         </is>
       </c>
       <c r="I6" s="15" t="inlineStr"/>
@@ -4770,7 +4786,7 @@
       </c>
       <c r="D7" s="13" t="inlineStr">
         <is>
-          <t>N/D (Brasil)</t>
+          <t>Brasil</t>
         </is>
       </c>
       <c r="E7" s="13" t="inlineStr">
@@ -4818,7 +4834,7 @@
       </c>
       <c r="D8" s="15" t="inlineStr">
         <is>
-          <t>N/D (Brasil)</t>
+          <t>Brasil</t>
         </is>
       </c>
       <c r="E8" s="15" t="inlineStr">
@@ -5008,7 +5024,7 @@
       </c>
       <c r="F3" s="13" t="inlineStr">
         <is>
-          <t>4.300+ entes | 600k+ forn.</t>
+          <t>4.000+ entes | 634k+ forn. | +R$616M oportunidades/dia | 300+ processos/dia</t>
         </is>
       </c>
       <c r="G3" s="13" t="inlineStr">
@@ -5018,7 +5034,7 @@
       </c>
       <c r="H3" s="13" t="inlineStr">
         <is>
-          <t>40%+ dos municípios brasileiros. Fundadores: Leonardo + Bruno Ladeira (Ecustomize). 35% crescimento anual. Marketplace B2G de referência nacional. Portfólio Cedro Capital (FIP Venture Brasil Central) — disponível para M&amp;A, sem mandatada.</t>
+          <t>Maior marketplace de licitações do Brasil. 40%+ dos municípios. Fundadores: Leonardo + Bruno Ladeira (Ecustomize). Certificações ISO 9001, 27001, 27701, 20000-1. Integrado ao PNCP. 35% crescimento anual. Portfólio Cedro Capital (FIP Venture Brasil Central) — disponível para M&amp;A, sem mandatada.</t>
         </is>
       </c>
       <c r="I3" s="17" t="inlineStr">
@@ -5036,7 +5052,7 @@
       </c>
       <c r="B4" s="15" t="inlineStr">
         <is>
-          <t>SaaS Credenciamento Eletrônico</t>
+          <t>Plataforma Licitações Eletrônicas / Credenciamento</t>
         </is>
       </c>
       <c r="C4" s="15" t="inlineStr">
@@ -5046,7 +5062,7 @@
       </c>
       <c r="D4" s="15" t="inlineStr">
         <is>
-          <t>N/D (Brasil)</t>
+          <t>Sete Lagoas - MG</t>
         </is>
       </c>
       <c r="E4" s="15" t="inlineStr">
@@ -5056,7 +5072,7 @@
       </c>
       <c r="F4" s="15" t="inlineStr">
         <is>
-          <t>90k+ fornecedores</t>
+          <t>90k+ fornecedores | clientes: Recife PE, Sete Lagoas MG, Itabira MG</t>
         </is>
       </c>
       <c r="G4" s="15" t="inlineStr">
@@ -5066,7 +5082,7 @@
       </c>
       <c r="H4" s="15" t="inlineStr">
         <is>
-          <t>Única plataforma de credenciamento eletrônico automatizado do Brasil. CEO: Aniele H. Figueiredo. Diferencial regulatório: elimina burocracia de habilitação presencial.</t>
+          <t>Plataforma completa de compras públicas conectando entes públicos, fornecedores e cidadãos. Diferencial regulatório em credenciamento eletrônico automatizado. Suporte especializado por telefone, WhatsApp e chat. Compatível com Lei 14.133/2021: pregão eletrônico, dispensa, credenciamento e chamamentos. CEO: Aniele H. Figueiredo.</t>
         </is>
       </c>
       <c r="I4" s="15" t="inlineStr"/>
@@ -5080,7 +5096,7 @@
       </c>
       <c r="B5" s="13" t="inlineStr">
         <is>
-          <t>CRM B2G para Fornecedores</t>
+          <t>Suite B2G para Fornecedores / Gestão de Licitações Sell-side</t>
         </is>
       </c>
       <c r="C5" s="13" t="inlineStr">
@@ -5100,7 +5116,7 @@
       </c>
       <c r="F5" s="13" t="inlineStr">
         <is>
-          <t>N/D</t>
+          <t>50M+ licitações monitoradas</t>
         </is>
       </c>
       <c r="G5" s="13" t="inlineStr">
@@ -5110,10 +5126,14 @@
       </c>
       <c r="H5" s="13" t="inlineStr">
         <is>
-          <t>Portfólio Fundo GovTech KPTL. CRM especializado na jornada de vendas B2G. Gestão de oportunidades, propostas e relacionamento com entes públicos.</t>
-        </is>
-      </c>
-      <c r="I5" s="13" t="inlineStr"/>
+          <t>Suite SaaS para fornecedores que vendem para governo: i-Ganhei (captação com IA, workflow, propostas automáticas, gestão de contratos), i-Pesquisei (inteligência de mercado B2G), i-Documentei (gestão de certidões), BPO de Licitações e i-One (projetos IA sob medida). Portfólio Fundo GovTech KPTL. 300% mais eficiência declarada.</t>
+        </is>
+      </c>
+      <c r="I5" s="17" t="inlineStr">
+        <is>
+          <t>Portfólio KPTL</t>
+        </is>
+      </c>
       <c r="J5" s="13" t="inlineStr"/>
     </row>
     <row r="6" ht="48" customHeight="1">
@@ -5168,7 +5188,7 @@
       </c>
       <c r="B7" s="13" t="inlineStr">
         <is>
-          <t>IA Contratos Pós-adjudicação</t>
+          <t>Plataforma SaaS de Cotação e Compras / Compliance Setor Público</t>
         </is>
       </c>
       <c r="C7" s="13" t="inlineStr">
@@ -5178,7 +5198,7 @@
       </c>
       <c r="D7" s="13" t="inlineStr">
         <is>
-          <t>N/D (Brasil)</t>
+          <t>Brasil</t>
         </is>
       </c>
       <c r="E7" s="13" t="inlineStr">
@@ -5188,7 +5208,7 @@
       </c>
       <c r="F7" s="13" t="inlineStr">
         <is>
-          <t>N/D</t>
+          <t>CEB, Onitel e outros | Grupo Squadra</t>
         </is>
       </c>
       <c r="G7" s="13" t="inlineStr">
@@ -5198,12 +5218,12 @@
       </c>
       <c r="H7" s="13" t="inlineStr">
         <is>
-          <t>Gestão do ciclo de vida de contratos públicos com IA: análise de cláusulas, alertas de prazo, auditoria automatizada. Segmento pós-licitação ainda sem líder claro.</t>
+          <t>Plataforma SaaS 100% flexível de gestão de compras corporativas com IA: cotação, disputas (aberta/fechada/leilão reverso), gestão de contratos, portal do fornecedor e BI de saving. Conformidade 14.133, 13.303 e Pregão Eletrônico. IA Pesquisa de Mercado premiada (Desafio TREM). Parte do Grupo Squadra (venture builder + data intelligence + cybersec). Integra Totvs, SAP, Oracle, Dynamics.</t>
         </is>
       </c>
       <c r="I7" s="17" t="inlineStr">
         <is>
-          <t>Watch — nicho virgem</t>
+          <t>Watch — compras gov</t>
         </is>
       </c>
       <c r="J7" s="13" t="inlineStr"/>
@@ -5226,7 +5246,7 @@
       </c>
       <c r="D8" s="15" t="inlineStr">
         <is>
-          <t>N/D (Brasil)</t>
+          <t>Imperatriz - MA</t>
         </is>
       </c>
       <c r="E8" s="15" t="inlineStr">
@@ -5246,7 +5266,7 @@
       </c>
       <c r="H8" s="15" t="inlineStr">
         <is>
-          <t>Plataforma buy-side: gestão de licitações e contratos para entes públicos. 290+ clientes. Lei 14.133/2021 compliance. Distinto do StartGi (B2G para fornecedores privados).</t>
+          <t>Plataforma buy-side para gestão de licitações e contratos de entes públicos. 290+ órgãos atendidos. Módulos: PCA, Planejamento &amp; Licitação (ETP com IA, Mapa de Riscos), Cotação de Preços (IA + PNCP) e Gestão de Contratação. 100% aderente à Lei 14.133/2021. Metodologia em 5 etapas. Diferente do StartGi (B2G para fornecedores).</t>
         </is>
       </c>
       <c r="I8" s="16" t="inlineStr">
@@ -5372,7 +5392,7 @@
       </c>
       <c r="F3" s="13" t="inlineStr">
         <is>
-          <t>14 municípios | 17k+ un.</t>
+          <t>14 municípios | 9.872 títulos emitidos | 17k+ projetos em andamento</t>
         </is>
       </c>
       <c r="G3" s="13" t="inlineStr">
@@ -5382,7 +5402,7 @@
       </c>
       <c r="H3" s="13" t="inlineStr">
         <is>
-          <t>Plataforma SaaS para regularização fundiária urbana (REURB) de ponta a ponta. App offline para agentes de campo. Emissão automática de CRF, títulos de legitimação e relatórios técnicos. Integração com cartórios. 17k+ unidades habitacionais regularizadas.</t>
+          <t>Plataforma SaaS para regularização fundiária urbana (REURB) ponta a ponta. App offline para coleta de campo. Emissão automática de relatórios técnicos, Títulos de Legitimação e Posse (TLP) e CRF. Integração com cartórios. Reduz 180 dias para 60 dias no processo. Municípios atendidos: Vitória ES, Vila Velha ES, Aracruz ES, Itabuna BA, Parnamirim RN, entre outros. ESG: 100% digital, zero papel.</t>
         </is>
       </c>
       <c r="I3" s="17" t="inlineStr">
@@ -5415,12 +5435,12 @@
       </c>
       <c r="E4" s="15" t="inlineStr">
         <is>
-          <t>2005</t>
+          <t>~2007</t>
         </is>
       </c>
       <c r="F4" s="15" t="inlineStr">
         <is>
-          <t>16 estados brasileiros</t>
+          <t>16 estados brasileiros | MCMV, Casa Verde Amarela, REURB</t>
         </is>
       </c>
       <c r="G4" s="15" t="inlineStr">
@@ -5430,7 +5450,7 @@
       </c>
       <c r="H4" s="15" t="inlineStr">
         <is>
-          <t>Software especialista em habitação de interesse social e regularização fundiária. 18 anos de atuação. Clientes: Governo de Roraima, programas MCMV e Casa Verde Amarela. Gestão de sorteios, hierarquizações e entregas habitacionais para prefeituras.</t>
+          <t>17+ anos como especialista em software para habitação de interesse social: cadastro multifinalitário georreferenciado, seleção de famílias (Portaria 2.081/20), sorteios, auxílio aluguel, cheque-reforma e REURB-S/E com emissão de CRF. Aplicativo móvel online/offline. LGPD-compliant. Equipe multidisciplinar (assistente social, arquiteta, contadora). 100% auditável. Cliente referência: Chapecó SC.</t>
         </is>
       </c>
       <c r="I4" s="16" t="inlineStr">
@@ -5458,7 +5478,7 @@
       </c>
       <c r="D5" s="13" t="inlineStr">
         <is>
-          <t>Brasil</t>
+          <t>Teresina - PI</t>
         </is>
       </c>
       <c r="E5" s="13" t="inlineStr">
@@ -5496,7 +5516,7 @@
       </c>
       <c r="B6" s="15" t="inlineStr">
         <is>
-          <t>Melhoria Habitacional de Interesse Social</t>
+          <t>Plataforma Gerenciadora de Reformas Habitacionais Populares</t>
         </is>
       </c>
       <c r="C6" s="15" t="inlineStr">
@@ -5516,7 +5536,7 @@
       </c>
       <c r="F6" s="15" t="inlineStr">
         <is>
-          <t>4.500+ intervenções</t>
+          <t>6.500+ reformas | 40+ cidades | 16 estados | R$54M+ gerenciados</t>
         </is>
       </c>
       <c r="G6" s="15" t="inlineStr">
@@ -5526,7 +5546,7 @@
       </c>
       <c r="H6" s="15" t="inlineStr">
         <is>
-          <t>Melhoria habitacional acessível para população de baixa renda. 4.500+ melhorias entregues. Portfólio BrazilLAB. Um dos principais negócios de impacto social do Brasil em habitação.</t>
+          <t>Primeira plataforma gerenciadora de reformas habitacionais populares do Brasil. Conecta beneficiários, prestadores e assistentes sociais em sistema único. Parceiros: COHAB-SP (Pode Entrar – Melhorias), Gerdau, Instituto BID, Instituto Cyrela. 24k+ pessoas vivendo melhor. Empresa B certificada. BrazilLAB.</t>
         </is>
       </c>
       <c r="I6" s="16" t="inlineStr">

</xml_diff>

<commit_message>
v13: Licitagram, Licitei, Proesc + correções Colab/GRTS + Fundo GovTech R$105,7M + M&A MITRA
- Licitagram adicionada (lic): 1º SO de IA Multi-Agente para Licitações da AL, 200k+ licitações/mês, 14 módulos IA
- Licitei adicionada (lic): sell-side PMEs, R$3,5M aporte Thompson Participações, 4.000+ usuários
- Proesc adicionada (educ): edtech amapaense, Proesc Gov na Prefeitura de Macapá (105 escolas, Alerta Escolar, IA LIA)
- Colab: receita atualizada (~R$25M total), Colab Gov.AI (AWS Bedrock, 94% aceleração), rodada US$10M+, novos clientes TCU
- GRTS Digital: sede corrigida Salvador BA, GRTS Contábil lançada, co-invest Aleve, meta R$25M faturamento 2027
- Fundo GovTech: R$105,7M total (Finep+Fapesp out/2025), meta R$150M, parceria Prodesp For Startups
- M&A: Valid adquire 51% MITRA (gestão municipal integrada, 1,7M+ cidadãos, SP+RJ)

Co-Authored-By: Claude Sonnet 4.6 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/Radar_GovTechs_Brasil_2026.xlsx
+++ b/Radar_GovTechs_Brasil_2026.xlsx
@@ -177,7 +177,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="33">
+  <cellXfs count="34">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center"/>
@@ -232,6 +232,9 @@
     </xf>
     <xf numFmtId="0" fontId="4" fillId="3" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="6" fillId="5" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment vertical="top" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="4" fillId="9" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center"/>
@@ -644,7 +647,7 @@
     <row r="1" ht="32" customHeight="1">
       <c r="A1" s="1" t="inlineStr">
         <is>
-          <t>🇧🇷 Radar GovTech Brasil 2025/2026 — DLG · Maio 2026 · v12</t>
+          <t>🇧🇷 Radar GovTech Brasil 2025/2026 — DLG · Maio 2026 · v13</t>
         </is>
       </c>
     </row>
@@ -697,7 +700,7 @@
         </is>
       </c>
       <c r="B7" s="4" t="n">
-        <v>8</v>
+        <v>9</v>
       </c>
     </row>
     <row r="8">
@@ -727,7 +730,7 @@
         </is>
       </c>
       <c r="B10" s="4" t="n">
-        <v>6</v>
+        <v>8</v>
       </c>
     </row>
     <row r="11">
@@ -777,7 +780,7 @@
         </is>
       </c>
       <c r="B15" s="6" t="n">
-        <v>70</v>
+        <v>73</v>
       </c>
     </row>
     <row r="16">
@@ -787,7 +790,7 @@
         </is>
       </c>
       <c r="B16" s="8" t="n">
-        <v>68</v>
+        <v>71</v>
       </c>
     </row>
     <row r="18">
@@ -797,7 +800,7 @@
         </is>
       </c>
       <c r="B18" s="9" t="n">
-        <v>14</v>
+        <v>16</v>
       </c>
     </row>
   </sheetData>
@@ -830,7 +833,7 @@
   </cols>
   <sheetData>
     <row r="1" ht="28" customHeight="1">
-      <c r="A1" s="26" t="inlineStr">
+      <c r="A1" s="27" t="inlineStr">
         <is>
           <t>🌿 Meio Ambiente &amp; Licenciamento — Radar GovTech Brasil 2025/2026</t>
         </is>
@@ -1062,7 +1065,7 @@
   </cols>
   <sheetData>
     <row r="1" ht="28" customHeight="1">
-      <c r="A1" s="27" t="inlineStr">
+      <c r="A1" s="28" t="inlineStr">
         <is>
           <t>🏙️ Smart Cities &amp; Mobilidade — Radar GovTech Brasil 2025/2026</t>
         </is>
@@ -1246,7 +1249,7 @@
   </cols>
   <sheetData>
     <row r="1" ht="28" customHeight="1">
-      <c r="A1" s="28" t="inlineStr">
+      <c r="A1" s="29" t="inlineStr">
         <is>
           <t>🛡️ Segurança Pública &amp; Infraestrutura — Radar GovTech Brasil 2025/2026</t>
         </is>
@@ -1638,7 +1641,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:F16"/>
+  <dimension ref="A1:F18"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="32" customWidth="1" min="1" max="1"/>
@@ -1650,39 +1653,39 @@
   </cols>
   <sheetData>
     <row r="1" ht="28" customHeight="1">
-      <c r="A1" s="29" t="inlineStr">
+      <c r="A1" s="30" t="inlineStr">
         <is>
           <t>💰 Aportes &amp; Investimentos — Radar GovTech Brasil 2025/2026</t>
         </is>
       </c>
     </row>
     <row r="2">
-      <c r="A2" s="30" t="inlineStr">
+      <c r="A2" s="31" t="inlineStr">
         <is>
           <t>Empresa / Investidor</t>
         </is>
       </c>
-      <c r="B2" s="30" t="inlineStr">
+      <c r="B2" s="31" t="inlineStr">
         <is>
           <t>Tipo</t>
         </is>
       </c>
-      <c r="C2" s="30" t="inlineStr">
+      <c r="C2" s="31" t="inlineStr">
         <is>
           <t>Valor</t>
         </is>
       </c>
-      <c r="D2" s="30" t="inlineStr">
+      <c r="D2" s="31" t="inlineStr">
         <is>
           <t>Data</t>
         </is>
       </c>
-      <c r="E2" s="30" t="inlineStr">
+      <c r="E2" s="31" t="inlineStr">
         <is>
           <t>Segmento</t>
         </is>
       </c>
-      <c r="F2" s="30" t="inlineStr">
+      <c r="F2" s="31" t="inlineStr">
         <is>
           <t>Descrição</t>
         </is>
@@ -1721,32 +1724,32 @@
       </c>
     </row>
     <row r="4" ht="48" customHeight="1">
-      <c r="A4" s="31" t="inlineStr">
+      <c r="A4" s="32" t="inlineStr">
         <is>
           <t>Aprova Digital — Astella + BB/VOX</t>
         </is>
       </c>
-      <c r="B4" s="32" t="inlineStr">
+      <c r="B4" s="33" t="inlineStr">
         <is>
           <t>Aporte Seed</t>
         </is>
       </c>
-      <c r="C4" s="32" t="inlineStr">
+      <c r="C4" s="33" t="inlineStr">
         <is>
           <t>R$ 22,5M</t>
         </is>
       </c>
-      <c r="D4" s="32" t="inlineStr">
+      <c r="D4" s="33" t="inlineStr">
         <is>
           <t>2022</t>
         </is>
       </c>
-      <c r="E4" s="32" t="inlineStr">
+      <c r="E4" s="33" t="inlineStr">
         <is>
           <t>Gestão Pública Municipal</t>
         </is>
       </c>
-      <c r="F4" s="32" t="inlineStr">
+      <c r="F4" s="33" t="inlineStr">
         <is>
           <t>Rodada liderada por Astella e VOX Capital (CVC do Banco do Brasil), com CAF e Endeavor. Maior aporte da história das GovTechs da América Latina na época. 120+ cidades, 21M de brasileiros impactados.</t>
         </is>
@@ -1785,32 +1788,32 @@
       </c>
     </row>
     <row r="6" ht="48" customHeight="1">
-      <c r="A6" s="31" t="inlineStr">
+      <c r="A6" s="32" t="inlineStr">
         <is>
           <t>Portabilis — Yunus Negócios Sociais</t>
         </is>
       </c>
-      <c r="B6" s="32" t="inlineStr">
+      <c r="B6" s="33" t="inlineStr">
         <is>
           <t>Aporte de impacto</t>
         </is>
       </c>
-      <c r="C6" s="32" t="inlineStr">
+      <c r="C6" s="33" t="inlineStr">
         <is>
           <t>Até R$ 2M</t>
         </is>
       </c>
-      <c r="D6" s="32" t="inlineStr">
+      <c r="D6" s="33" t="inlineStr">
         <is>
           <t>2023</t>
         </is>
       </c>
-      <c r="E6" s="32" t="inlineStr">
+      <c r="E6" s="33" t="inlineStr">
         <is>
           <t>Educação Pública</t>
         </is>
       </c>
-      <c r="F6" s="32" t="inlineStr">
+      <c r="F6" s="33" t="inlineStr">
         <is>
           <t>R$800k já desembolsados. Valida modelo de negócio social. Meta: 1,5M alunos até 2027.</t>
         </is>
@@ -1849,32 +1852,32 @@
       </c>
     </row>
     <row r="8" ht="48" customHeight="1">
-      <c r="A8" s="31" t="inlineStr">
+      <c r="A8" s="32" t="inlineStr">
         <is>
           <t>GOVBR — Volaris Group (Constellation Software)</t>
         </is>
       </c>
-      <c r="B8" s="32" t="inlineStr">
+      <c r="B8" s="33" t="inlineStr">
         <is>
           <t>Aquisição (M&amp;A)</t>
         </is>
       </c>
-      <c r="C8" s="32" t="inlineStr">
-        <is>
-          <t>N/D</t>
-        </is>
-      </c>
-      <c r="D8" s="32" t="inlineStr">
+      <c r="C8" s="33" t="inlineStr">
+        <is>
+          <t>N/D</t>
+        </is>
+      </c>
+      <c r="D8" s="33" t="inlineStr">
         <is>
           <t>mai/2023</t>
         </is>
       </c>
-      <c r="E8" s="32" t="inlineStr">
+      <c r="E8" s="33" t="inlineStr">
         <is>
           <t>Gestão Pública Municipal</t>
         </is>
       </c>
-      <c r="F8" s="32" t="inlineStr">
+      <c r="F8" s="33" t="inlineStr">
         <is>
           <t>Volaris adquire a GovernançaBrasil (GOVBR), ERP municipal com 35 anos de atuação. Fundador: Roberto Coelho. Plataforma Cidade 360, 24 módulos. Presença em RS, SC, SP, PR, RJ, ES, MG, MS, PE. Descrita como 'aquisição de grande porte' pela Volaris.</t>
         </is>
@@ -1913,32 +1916,32 @@
       </c>
     </row>
     <row r="10" ht="48" customHeight="1">
-      <c r="A10" s="31" t="inlineStr">
+      <c r="A10" s="32" t="inlineStr">
         <is>
           <t>i4Sea — Fundo GovTech KPTL</t>
         </is>
       </c>
-      <c r="B10" s="32" t="inlineStr">
+      <c r="B10" s="33" t="inlineStr">
         <is>
           <t>Aporte</t>
         </is>
       </c>
-      <c r="C10" s="32" t="inlineStr">
+      <c r="C10" s="33" t="inlineStr">
         <is>
           <t>R$ 7,5M</t>
         </is>
       </c>
-      <c r="D10" s="32" t="inlineStr">
+      <c r="D10" s="33" t="inlineStr">
         <is>
           <t>2024</t>
         </is>
       </c>
-      <c r="E10" s="32" t="inlineStr">
+      <c r="E10" s="33" t="inlineStr">
         <is>
           <t>Infraestrutura / Clima</t>
         </is>
       </c>
-      <c r="F10" s="32" t="inlineStr">
+      <c r="F10" s="33" t="inlineStr">
         <is>
           <t>Previsões microclimáticas para portos e setor elétrico. Portfólio Fundo GovTech KPTL.</t>
         </is>
@@ -1977,32 +1980,32 @@
       </c>
     </row>
     <row r="12" ht="48" customHeight="1">
-      <c r="A12" s="31" t="inlineStr">
+      <c r="A12" s="32" t="inlineStr">
         <is>
           <t>IDS — Volaris Group (Constellation Software)</t>
         </is>
       </c>
-      <c r="B12" s="32" t="inlineStr">
+      <c r="B12" s="33" t="inlineStr">
         <is>
           <t>Aquisição (M&amp;A)</t>
         </is>
       </c>
-      <c r="C12" s="32" t="inlineStr">
-        <is>
-          <t>N/D</t>
-        </is>
-      </c>
-      <c r="D12" s="32" t="inlineStr">
+      <c r="C12" s="33" t="inlineStr">
+        <is>
+          <t>N/D</t>
+        </is>
+      </c>
+      <c r="D12" s="33" t="inlineStr">
         <is>
           <t>ago/2024</t>
         </is>
       </c>
-      <c r="E12" s="32" t="inlineStr">
+      <c r="E12" s="33" t="inlineStr">
         <is>
           <t>Saúde / Educação / Assistência Social</t>
         </is>
       </c>
-      <c r="F12" s="32" t="inlineStr">
+      <c r="F12" s="33" t="inlineStr">
         <is>
           <t>Volaris adquire a IDS (Pato Branco, PR), fornecedora de software para municípios nas áreas de saúde, assistência social, educação e cidadão. Fundada em 2003, 112 funcionários. CEO: Mauri Dengo. Opera de forma independente dentro do portfólio Volaris Latam &amp; Ibéria.</t>
         </is>
@@ -2041,32 +2044,32 @@
       </c>
     </row>
     <row r="14" ht="48" customHeight="1">
-      <c r="A14" s="31" t="inlineStr">
+      <c r="A14" s="32" t="inlineStr">
         <is>
           <t>1Doc — Softplan (100%)</t>
         </is>
       </c>
-      <c r="B14" s="32" t="inlineStr">
+      <c r="B14" s="33" t="inlineStr">
         <is>
           <t>Aquisição (M&amp;A)</t>
         </is>
       </c>
-      <c r="C14" s="32" t="inlineStr">
-        <is>
-          <t>N/D</t>
-        </is>
-      </c>
-      <c r="D14" s="32" t="inlineStr">
+      <c r="C14" s="33" t="inlineStr">
+        <is>
+          <t>N/D</t>
+        </is>
+      </c>
+      <c r="D14" s="33" t="inlineStr">
         <is>
           <t>abr/2025</t>
         </is>
       </c>
-      <c r="E14" s="32" t="inlineStr">
+      <c r="E14" s="33" t="inlineStr">
         <is>
           <t>Digitalização / Gestão Municipal</t>
         </is>
       </c>
-      <c r="F14" s="32" t="inlineStr">
+      <c r="F14" s="33" t="inlineStr">
         <is>
           <t>Softplan adquire 100% da 1Doc, govtech de digitalização de processos e atendimento ao cidadão em prefeituras. Jornada: aporte 2017 → maioria 2019 → 100% abr/2025. CAGR de 75% (2019–2025). Fundada 2014, 1.000 entidades públicas, 22M brasileiros impactados, 141 colaboradores.</t>
         </is>
@@ -2075,62 +2078,126 @@
     <row r="15" ht="48" customHeight="1">
       <c r="A15" s="12" t="inlineStr">
         <is>
+          <t>Fundo GovTech — Finep + Fapesp</t>
+        </is>
+      </c>
+      <c r="B15" s="13" t="inlineStr">
+        <is>
+          <t>Expansão de fundo</t>
+        </is>
+      </c>
+      <c r="C15" s="13" t="inlineStr">
+        <is>
+          <t>R$ 105,7M total</t>
+        </is>
+      </c>
+      <c r="D15" s="13" t="inlineStr">
+        <is>
+          <t>out/2025</t>
+        </is>
+      </c>
+      <c r="E15" s="13" t="inlineStr">
+        <is>
+          <t>Fundo de Investimento GovTech</t>
+        </is>
+      </c>
+      <c r="F15" s="13" t="inlineStr">
+        <is>
+          <t>Fundo GovTech KPTL+Cedro cresce de R$49M para R$105,7M com aportes da Finep (R$40M) e Fapesp (R$30M) em out/2025. Meta para 2026: R$150M. Parceria Prodesp For Startups (SP) para aceleração de startups do portfólio. Portfólio atual: Augen (exit Biosolvit), Prosas, Colab, StartGi, i4Sea, GRTS Digital, Jovens Gênios, Kinebot.</t>
+        </is>
+      </c>
+    </row>
+    <row r="16" ht="48" customHeight="1">
+      <c r="A16" s="32" t="inlineStr">
+        <is>
+          <t>MITRA — Valid (51%)</t>
+        </is>
+      </c>
+      <c r="B16" s="33" t="inlineStr">
+        <is>
+          <t>Aquisição (M&amp;A)</t>
+        </is>
+      </c>
+      <c r="C16" s="33" t="inlineStr">
+        <is>
+          <t>N/D</t>
+        </is>
+      </c>
+      <c r="D16" s="33" t="inlineStr">
+        <is>
+          <t>2025</t>
+        </is>
+      </c>
+      <c r="E16" s="33" t="inlineStr">
+        <is>
+          <t>Gestão Municipal Integrada</t>
+        </is>
+      </c>
+      <c r="F16" s="33" t="inlineStr">
+        <is>
+          <t>Valid adquire 51% da MITRA, plataforma de gestão municipal integrada com proposta 'Governo Único para um Cidadão Único'. Cidades atendidas: São Caetano do Sul SP, Santo André SP, Vinhedo SP, Araraquara SP, Campos dos Goytacazes RJ. 1,7M+ cidadãos impactados.</t>
+        </is>
+      </c>
+    </row>
+    <row r="17" ht="48" customHeight="1">
+      <c r="A17" s="12" t="inlineStr">
+        <is>
           <t>Kinebot — Fundo GovTech (KPTL+Cedro)</t>
         </is>
       </c>
-      <c r="B15" s="13" t="inlineStr">
+      <c r="B17" s="13" t="inlineStr">
         <is>
           <t>Aporte</t>
         </is>
       </c>
-      <c r="C15" s="13" t="inlineStr">
+      <c r="C17" s="13" t="inlineStr">
         <is>
           <t>R$ 3M</t>
         </is>
       </c>
-      <c r="D15" s="13" t="inlineStr">
+      <c r="D17" s="13" t="inlineStr">
         <is>
           <t>fev/2026</t>
         </is>
       </c>
-      <c r="E15" s="13" t="inlineStr">
+      <c r="E17" s="13" t="inlineStr">
         <is>
           <t>IA Ergonomia / Saúde Gov</t>
         </is>
       </c>
-      <c r="F15" s="13" t="inlineStr">
+      <c r="F17" s="13" t="inlineStr">
         <is>
           <t>8º investimento do Fundo GovTech. IA para análises ergonômicas e psicossociais. Clientes: Marfrig, P&amp;G, Electrolux. Expansão global planejada para 2026.</t>
         </is>
       </c>
     </row>
-    <row r="16" ht="48" customHeight="1">
-      <c r="A16" s="31" t="inlineStr">
+    <row r="18" ht="48" customHeight="1">
+      <c r="A18" s="32" t="inlineStr">
         <is>
           <t>Jovens Gênios — Fundo GovTech+DOMO</t>
         </is>
       </c>
-      <c r="B16" s="32" t="inlineStr">
+      <c r="B18" s="33" t="inlineStr">
         <is>
           <t>Aporte Seed</t>
         </is>
       </c>
-      <c r="C16" s="32" t="inlineStr">
+      <c r="C18" s="33" t="inlineStr">
         <is>
           <t>R$ 11,8M</t>
         </is>
       </c>
-      <c r="D16" s="32" t="inlineStr">
+      <c r="D18" s="33" t="inlineStr">
         <is>
           <t>mar/2026</t>
         </is>
       </c>
-      <c r="E16" s="32" t="inlineStr">
+      <c r="E18" s="33" t="inlineStr">
         <is>
           <t>Educação Pública</t>
         </is>
       </c>
-      <c r="F16" s="32" t="inlineStr">
+      <c r="F18" s="33" t="inlineStr">
         <is>
           <t>Rodada seed liderada pelo Fundo GovTech (KPTL+Cedro), com DOMO.VC, Criabiz Ventures e Rosey Ventures (Grupo Marista). 90% dos alunos em escolas públicas. Meta: 10M alunos até 2030.</t>
         </is>
@@ -2566,7 +2633,7 @@
       </c>
       <c r="D10" s="15" t="inlineStr">
         <is>
-          <t>São Paulo - SP</t>
+          <t>Salvador - BA</t>
         </is>
       </c>
       <c r="E10" s="15" t="inlineStr">
@@ -2581,12 +2648,12 @@
       </c>
       <c r="G10" s="15" t="inlineStr">
         <is>
-          <t>R$ 3,4M aporte</t>
+          <t>R$ 3,4M aporte (Fundo GovTech)</t>
         </is>
       </c>
       <c r="H10" s="15" t="inlineStr">
         <is>
-          <t>Ecossistema SaaS de digitalização de RTS: gestão de CCTs, IA 'Norma' para análise de cláusulas, assembleias virtuais e data intelligence. Integração com HCM via parceria LG. Prêmio inovação RH 2025. R$3,4M Fundo GovTech KPTL.</t>
+          <t>Ecossistema SaaS de digitalização de RTS: gestão de CCTs, IA 'Norma' para análise de cláusulas, assembleias virtuais e data intelligence. Integração com HCM via parceria LG. Prêmio inovação RH 2025. R$3,4M Fundo GovTech KPTL (jun/2025). Lançou GRTS Contábil (12 contratos nas primeiras 3 semanas). Co-investidor Aleve Legal Tech. Meta: R$25M faturamento até 2027. CEO Uirá Menezes, sede Salvador BA.</t>
         </is>
       </c>
       <c r="I10" s="16" t="inlineStr">
@@ -2677,12 +2744,12 @@
       </c>
       <c r="G12" s="15" t="inlineStr">
         <is>
-          <t>R$3-7M (Fundo GovTech)</t>
+          <t>~R$25M total (MDIF+Luminate+EDP+KPTL)</t>
         </is>
       </c>
       <c r="H12" s="15" t="inlineStr">
         <is>
-          <t>Plataforma multicanal (web, app, WhatsApp) de gestão de serviços digitais, participação cidadã e CRM governamental. IA digitaliza qualquer serviço público em minutos. Em 2025 viabilizou OP Digital do Piauí (273k participantes) com validação via Receita Federal e blockchain. Portfólio KPTL+Cedro. Co-invest EDP.</t>
+          <t>Plataforma multicanal (web, app, WhatsApp) de gestão de serviços digitais, participação cidadã e CRM governamental. IA digitaliza qualquer serviço público em minutos. Em 2025 viabilizou OP Digital do Piauí (273k participantes) com validação via Receita Federal e blockchain. Lançou Colab Gov.AI (AWS Bedrock, out/2025): 94% de aceleração na criação de serviços digitais, 500+ prompts em 14 dias. Novos clientes: TCU, Diadema, Rio das Ostras, Duque de Caxias. Rodada US$10M+ em curso para 2026. Portfólio KPTL+Cedro. Co-invest EDP Ventures + Luminate + MDIF.</t>
         </is>
       </c>
       <c r="I12" s="16" t="inlineStr">
@@ -3634,7 +3701,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:J10"/>
+  <dimension ref="A1:J11"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="28" customWidth="1" min="1" max="1"/>
@@ -4071,6 +4138,58 @@
         </is>
       </c>
       <c r="J10" s="15" t="inlineStr"/>
+    </row>
+    <row r="11" ht="48" customHeight="1">
+      <c r="A11" s="12" t="inlineStr">
+        <is>
+          <t>Proesc</t>
+        </is>
+      </c>
+      <c r="B11" s="13" t="inlineStr">
+        <is>
+          <t>Gestão Escolar com IA + Vertical Pública (Proesc Gov)</t>
+        </is>
+      </c>
+      <c r="C11" s="13" t="inlineStr">
+        <is>
+          <t>Scale-up</t>
+        </is>
+      </c>
+      <c r="D11" s="13" t="inlineStr">
+        <is>
+          <t>Macapá - AP</t>
+        </is>
+      </c>
+      <c r="E11" s="13" t="inlineStr">
+        <is>
+          <t>N/D</t>
+        </is>
+      </c>
+      <c r="F11" s="13" t="inlineStr">
+        <is>
+          <t>3.000–3.500+ escolas | 5 países | 35+ redes parceiras BR | Prefeitura de Macapá (105 escolas)</t>
+        </is>
+      </c>
+      <c r="G11" s="13" t="inlineStr">
+        <is>
+          <t>Maior rodada de invest. na Amazônia (Exame)</t>
+        </is>
+      </c>
+      <c r="H11" s="13" t="inlineStr">
+        <is>
+          <t>Edtech amapaense fundada às margens do Rio Amazonas. Vertical pública Proesc Gov já implantada na Secretaria de Educação de Macapá: diário eletrônico com app offline, matrículas digitais, IDEB/VAAR e gestão da secretaria. Diferencial: Botão Alerta Escolar conecta as 105 escolas municipais à Guarda Civil Municipal. IA 'LIA' para decisões estratégicas nas secretarias. 3.000–3.500+ escolas parceiras (privadas + públicas), 5 países, 35+ redes pelo Brasil. Captou a maior rodada de investimento já realizada na Amazônia (Exame).</t>
+        </is>
+      </c>
+      <c r="I11" s="17" t="inlineStr">
+        <is>
+          <t>Watch — pública + Amazônia</t>
+        </is>
+      </c>
+      <c r="J11" s="21" t="inlineStr">
+        <is>
+          <t>✓</t>
+        </is>
+      </c>
     </row>
   </sheetData>
   <mergeCells count="1">
@@ -4102,7 +4221,7 @@
   </cols>
   <sheetData>
     <row r="1" ht="28" customHeight="1">
-      <c r="A1" s="21" t="inlineStr">
+      <c r="A1" s="22" t="inlineStr">
         <is>
           <t>🤖 IA Horizontal &amp; Automação — Radar GovTech Brasil 2025/2026</t>
         </is>
@@ -4442,7 +4561,7 @@
           <t>M&amp;A Watch — portfólio Cedro</t>
         </is>
       </c>
-      <c r="J8" s="22" t="inlineStr">
+      <c r="J8" s="23" t="inlineStr">
         <is>
           <t>✓</t>
         </is>
@@ -4526,7 +4645,7 @@
   </cols>
   <sheetData>
     <row r="1" ht="28" customHeight="1">
-      <c r="A1" s="23" t="inlineStr">
+      <c r="A1" s="24" t="inlineStr">
         <is>
           <t>⚖️ Procuradorias &amp; Jurídico — Radar GovTech Brasil 2025/2026</t>
         </is>
@@ -4922,7 +5041,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:J8"/>
+  <dimension ref="A1:J10"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="28" customWidth="1" min="1" max="1"/>
@@ -4938,7 +5057,7 @@
   </cols>
   <sheetData>
     <row r="1" ht="28" customHeight="1">
-      <c r="A1" s="24" t="inlineStr">
+      <c r="A1" s="25" t="inlineStr">
         <is>
           <t>📋 Licitações &amp; Compras Públicas — Radar GovTech Brasil 2025/2026</t>
         </is>
@@ -5275,6 +5394,110 @@
         </is>
       </c>
       <c r="J8" s="15" t="inlineStr"/>
+    </row>
+    <row r="9" ht="48" customHeight="1">
+      <c r="A9" s="12" t="inlineStr">
+        <is>
+          <t>Licitagram</t>
+        </is>
+      </c>
+      <c r="B9" s="13" t="inlineStr">
+        <is>
+          <t>SO de IA Multi-Agente para Licitações (Sell-side + Buy-side)</t>
+        </is>
+      </c>
+      <c r="C9" s="13" t="inlineStr">
+        <is>
+          <t>Startup</t>
+        </is>
+      </c>
+      <c r="D9" s="13" t="inlineStr">
+        <is>
+          <t>Brasil</t>
+        </is>
+      </c>
+      <c r="E9" s="13" t="inlineStr">
+        <is>
+          <t>N/D</t>
+        </is>
+      </c>
+      <c r="F9" s="13" t="inlineStr">
+        <is>
+          <t>200k+ licitações/mês | R$1T+ oportunidades | 67M+ CNPJs cruzados</t>
+        </is>
+      </c>
+      <c r="G9" s="13" t="inlineStr">
+        <is>
+          <t>N/D</t>
+        </is>
+      </c>
+      <c r="H9" s="13" t="inlineStr">
+        <is>
+          <t>1º Sistema Operacional de IA Multi-Agente para Licitações da América Latina. 14 módulos IA: AI Matching score 0–100, robô de lances IA, inteligência competitiva (5 módulos), pesquisa de preços IN 65/2021, grafo societário, detecção de anomalias, compliance checker e forensic replay. Cobre sell-side (fornecedores) + buy-side (entes públicos) + compliance (TCUs). Integração PNCP. Planos: R$297–R$1.497/mês.</t>
+        </is>
+      </c>
+      <c r="I9" s="17" t="inlineStr">
+        <is>
+          <t>Watch — IA licitações multi-agente</t>
+        </is>
+      </c>
+      <c r="J9" s="21" t="inlineStr">
+        <is>
+          <t>✓</t>
+        </is>
+      </c>
+    </row>
+    <row r="10" ht="48" customHeight="1">
+      <c r="A10" s="14" t="inlineStr">
+        <is>
+          <t>Licitei</t>
+        </is>
+      </c>
+      <c r="B10" s="15" t="inlineStr">
+        <is>
+          <t>Licitações Sell-side para PMEs</t>
+        </is>
+      </c>
+      <c r="C10" s="15" t="inlineStr">
+        <is>
+          <t>Startup</t>
+        </is>
+      </c>
+      <c r="D10" s="15" t="inlineStr">
+        <is>
+          <t>Belo Horizonte - MG</t>
+        </is>
+      </c>
+      <c r="E10" s="15" t="inlineStr">
+        <is>
+          <t>N/D</t>
+        </is>
+      </c>
+      <c r="F10" s="15" t="inlineStr">
+        <is>
+          <t>4.000+ usuários | 206k+ editais | PNCP integrado</t>
+        </is>
+      </c>
+      <c r="G10" s="15" t="inlineStr">
+        <is>
+          <t>R$3,5M (Thompson Participações, jun/2024)</t>
+        </is>
+      </c>
+      <c r="H10" s="15" t="inlineStr">
+        <is>
+          <t>Plataforma sell-side focada em PMEs que vendem para governo: robô de lances IA, análise de editais com IA, monitoramento de oportunidades e integração PNCP. Aporte de R$3,5M da Thompson Participações (jun/2024). CEO: Felipe Nardes. 4.000+ usuários ativos, 206k+ editais monitorados. Diferencia-se da StartGi por foco em PMEs e preço acessível.</t>
+        </is>
+      </c>
+      <c r="I10" s="16" t="inlineStr">
+        <is>
+          <t>Watch — sell-side PME</t>
+        </is>
+      </c>
+      <c r="J10" s="23" t="inlineStr">
+        <is>
+          <t>✓</t>
+        </is>
+      </c>
     </row>
   </sheetData>
   <mergeCells count="1">
@@ -5306,7 +5529,7 @@
   </cols>
   <sheetData>
     <row r="1" ht="28" customHeight="1">
-      <c r="A1" s="25" t="inlineStr">
+      <c r="A1" s="26" t="inlineStr">
         <is>
           <t>🏘️ Habitação &amp; Regularização Fundiária — Radar GovTech Brasil 2025/2026</t>
         </is>

</xml_diff>

<commit_message>
v14: iBridge adicionada + senha de acesso removida (radar público)
- iBridge Technology (gestao): plataforma de Contact Center / PABX IP para centrais municipais (156 e ouvidorias), 5.000+ posições, 50M+ chamadas/mês, Florianópolis SC, 17 anos
- Login overlay e CSS de autenticação removidos do template HTML — radar agora público e aberto

Co-Authored-By: Claude Sonnet 4.6 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/Radar_GovTechs_Brasil_2026.xlsx
+++ b/Radar_GovTechs_Brasil_2026.xlsx
@@ -221,6 +221,9 @@
     <xf numFmtId="0" fontId="5" fillId="6" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment vertical="top" wrapText="1"/>
     </xf>
+    <xf numFmtId="0" fontId="6" fillId="6" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment vertical="top" wrapText="1"/>
+    </xf>
     <xf numFmtId="0" fontId="5" fillId="5" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment vertical="top" wrapText="1"/>
     </xf>
@@ -238,9 +241,6 @@
     </xf>
     <xf numFmtId="0" fontId="4" fillId="9" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="6" fillId="6" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment vertical="top" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="4" fillId="10" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center"/>
@@ -647,7 +647,7 @@
     <row r="1" ht="32" customHeight="1">
       <c r="A1" s="1" t="inlineStr">
         <is>
-          <t>🇧🇷 Radar GovTech Brasil 2025/2026 — DLG · Maio 2026 · v13</t>
+          <t>🇧🇷 Radar GovTech Brasil 2025/2026 — DLG · Maio 2026 · v14</t>
         </is>
       </c>
     </row>
@@ -670,7 +670,7 @@
         </is>
       </c>
       <c r="B4" s="4" t="n">
-        <v>12</v>
+        <v>13</v>
       </c>
     </row>
     <row r="5">
@@ -780,7 +780,7 @@
         </is>
       </c>
       <c r="B15" s="6" t="n">
-        <v>73</v>
+        <v>74</v>
       </c>
     </row>
     <row r="16">
@@ -790,7 +790,7 @@
         </is>
       </c>
       <c r="B16" s="8" t="n">
-        <v>71</v>
+        <v>72</v>
       </c>
     </row>
     <row r="18">
@@ -932,7 +932,7 @@
           <t>Sistema de Gestão Ambiental Compartilhada (eGAC): SaaS de licenciamento ambiental municipal 100% digital. Integra SINAFLOR, GEOBAHIA, SEMA-BA e CEPRAM. Cobrança automática de taxa ambiental via Pix/boleto. 70% redução de custos declarada, onboarding em 30 dias. Nasceu da pandemia de 2021 em colaboração com gestores municipais baianos. Conformidade CEPRAM 4.327/13.</t>
         </is>
       </c>
-      <c r="I3" s="17" t="inlineStr">
+      <c r="I3" s="18" t="inlineStr">
         <is>
           <t>Watch — lic. ambiental nicho virgem</t>
         </is>
@@ -1028,7 +1028,7 @@
           <t>Plataforma + hardware IoT proprietário (H-SAT) para rastreabilidade de resíduos sólidos do ponto de coleta ao destino final. Gera documentos auditáveis com fotos georreferenciadas, telemetria e carimbos de tempo. Conformidade PNRS. Modelo híbrido: software + presença onsite. PIT-SJC. Fundada jun/2024.</t>
         </is>
       </c>
-      <c r="I5" s="17" t="inlineStr">
+      <c r="I5" s="18" t="inlineStr">
         <is>
           <t>Watch — PNRS compliance IoT</t>
         </is>
@@ -1164,7 +1164,7 @@
           <t>Plataforma baseada em FIWARE para cidades inteligentes: data spaces interoperáveis, IoT, mobilidade, segurança e clima. Smart Mafra: 1ª cidade BR com lei municipal FIWARE (centraliza tributação, alvarás e todos os serviços públicos em sistema único). Amurel Conectada: integra 18 municípios Região de Laguna/SC — 1º espaço de dados regional BR em operação. SC aprovou Lei 19.494 adotando FIWARE como padrão estadual. CEO: Gilsoni Lunardi Albino. Prêmio Smart City Expo Curitiba 2025 + Barcelona 2025.</t>
         </is>
       </c>
-      <c r="I3" s="17" t="inlineStr">
+      <c r="I3" s="18" t="inlineStr">
         <is>
           <t>Watch — padrão FIWARE em SC</t>
         </is>
@@ -1348,7 +1348,7 @@
           <t>IA para previsão antecipada de desastres naturais com dados NASA e bases nacionais. Alerta SMS via Defesa Civil municipal. Selecionada COP26. Foco em mitigação de riscos climáticos e resiliência urbana.</t>
         </is>
       </c>
-      <c r="I3" s="17" t="inlineStr">
+      <c r="I3" s="18" t="inlineStr">
         <is>
           <t>Watch — clima/risco</t>
         </is>
@@ -1532,7 +1532,7 @@
           <t>ClimaTech com plataforma SPEHC (SaaS) para previsões hidroclimáticas: antecipação de enchentes, gestão de barragens e operação de usinas. Integra múltiplos modelos, radares e dados em tempo real. Referência nacional na Defesa Civil de SC. Escritório também em Bauru/SP. Portfólio KPTL 2019.</t>
         </is>
       </c>
-      <c r="I7" s="17" t="inlineStr">
+      <c r="I7" s="18" t="inlineStr">
         <is>
           <t>Portfólio KPTL</t>
         </is>
@@ -1953,7 +1953,7 @@
           <t>Augen — Biosolvit (exit)</t>
         </is>
       </c>
-      <c r="B11" s="17" t="inlineStr">
+      <c r="B11" s="18" t="inlineStr">
         <is>
           <t>Exit estratégico</t>
         </is>
@@ -2217,7 +2217,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:J14"/>
+  <dimension ref="A1:J15"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="28" customWidth="1" min="1" max="1"/>
@@ -2338,32 +2338,32 @@
     <row r="4" ht="48" customHeight="1">
       <c r="A4" s="14" t="inlineStr">
         <is>
-          <t>GovDigital</t>
+          <t>iBridge Technology</t>
         </is>
       </c>
       <c r="B4" s="15" t="inlineStr">
         <is>
-          <t>App Municipal SaaS / Relacionamento Cidadão-Governo</t>
+          <t>Contact Center / PABX IP para Centrais Municipais (156 e Ouvidorias)</t>
         </is>
       </c>
       <c r="C4" s="15" t="inlineStr">
         <is>
-          <t>Startup / Scale-up</t>
+          <t>PME Estabelecida</t>
         </is>
       </c>
       <c r="D4" s="15" t="inlineStr">
         <is>
-          <t>Jaraguá do Sul - SC</t>
+          <t>Florianópolis - SC</t>
         </is>
       </c>
       <c r="E4" s="15" t="inlineStr">
         <is>
-          <t>~2020</t>
+          <t>2008</t>
         </is>
       </c>
       <c r="F4" s="15" t="inlineStr">
         <is>
-          <t>Múltiplos municípios SC e outros estados</t>
+          <t>5.000+ posições de atendimento | 50M+ chamadas/mês | 250k+ vendas/mês</t>
         </is>
       </c>
       <c r="G4" s="15" t="inlineStr">
@@ -2373,69 +2373,77 @@
       </c>
       <c r="H4" s="15" t="inlineStr">
         <is>
-          <t>App oficial white-label de prefeituras reunindo zeladoria, agendamento, formulários online, notícias e comunicação direta cidadão-prefeitura. Integrações com IPTU, protocolo e ouvidoria. CEO: Elias Raasch. Expansão nacional sem VC.</t>
+          <t>Plataforma completa de gestão de contact center e PABX IP em nuvem para operações ativas, receptivas e mistas. Callcenter Manager: controle em tempo real, discador preditivo, gravação de ramais, fila de atendimento com URA, dashboards de performance e integrações com CRM (Salesforce, Dynamics 365, RD Station, Zendesk). PABX IP compatível com redes VoIP e PSTN (analógico, digital, IP ou híbrido). Aplicável a centrais 156 e ouvidorias municipais para modernização do atendimento ao cidadão. CEO: Vinicius Bossle Fagundes. 17 anos de atuação.</t>
         </is>
       </c>
       <c r="I4" s="16" t="inlineStr">
         <is>
-          <t>Watch — expansão nacional</t>
-        </is>
-      </c>
-      <c r="J4" s="15" t="inlineStr"/>
+          <t>Watch — canal 156 municipal</t>
+        </is>
+      </c>
+      <c r="J4" s="17" t="inlineStr">
+        <is>
+          <t>✓</t>
+        </is>
+      </c>
     </row>
     <row r="5" ht="48" customHeight="1">
       <c r="A5" s="12" t="inlineStr">
         <is>
-          <t>Desenvolve Cidade</t>
+          <t>GovDigital</t>
         </is>
       </c>
       <c r="B5" s="13" t="inlineStr">
         <is>
-          <t>Licenciamento e Tributação Municipal Digital</t>
+          <t>App Municipal SaaS / Relacionamento Cidadão-Governo</t>
         </is>
       </c>
       <c r="C5" s="13" t="inlineStr">
         <is>
-          <t>Startup</t>
+          <t>Startup / Scale-up</t>
         </is>
       </c>
       <c r="D5" s="13" t="inlineStr">
         <is>
-          <t>Campinas - SP</t>
+          <t>Jaraguá do Sul - SC</t>
         </is>
       </c>
       <c r="E5" s="13" t="inlineStr">
         <is>
-          <t>~2014</t>
+          <t>~2020</t>
         </is>
       </c>
       <c r="F5" s="13" t="inlineStr">
         <is>
-          <t>Municípios Norte e outras regiões | Scale-Up Endeavor 2021</t>
+          <t>Múltiplos municípios SC e outros estados</t>
         </is>
       </c>
       <c r="G5" s="13" t="inlineStr">
         <is>
-          <t>N/D</t>
+          <t>N/D (bootstrap)</t>
         </is>
       </c>
       <c r="H5" s="13" t="inlineStr">
         <is>
-          <t>Plataforma integrada de licenciamento digital (urbanístico, ambiental, sanitário, obras), abertura/baixa de empresas, IPTU e ISS digitais integrada à REDESIM federal. Foco em desburocratização e aumento de receita própria municipal. TOP2 Open Startups 2024.</t>
-        </is>
-      </c>
-      <c r="I5" s="13" t="inlineStr"/>
+          <t>App oficial white-label de prefeituras reunindo zeladoria, agendamento, formulários online, notícias e comunicação direta cidadão-prefeitura. Integrações com IPTU, protocolo e ouvidoria. CEO: Elias Raasch. Expansão nacional sem VC.</t>
+        </is>
+      </c>
+      <c r="I5" s="18" t="inlineStr">
+        <is>
+          <t>Watch — expansão nacional</t>
+        </is>
+      </c>
       <c r="J5" s="13" t="inlineStr"/>
     </row>
     <row r="6" ht="48" customHeight="1">
       <c r="A6" s="14" t="inlineStr">
         <is>
-          <t>IP Inovação</t>
+          <t>Desenvolve Cidade</t>
         </is>
       </c>
       <c r="B6" s="15" t="inlineStr">
         <is>
-          <t>Capacitação e Consultoria em Gestão Pública</t>
+          <t>Licenciamento e Tributação Municipal Digital</t>
         </is>
       </c>
       <c r="C6" s="15" t="inlineStr">
@@ -2445,17 +2453,17 @@
       </c>
       <c r="D6" s="15" t="inlineStr">
         <is>
-          <t>Belém - PA</t>
+          <t>Campinas - SP</t>
         </is>
       </c>
       <c r="E6" s="15" t="inlineStr">
         <is>
-          <t>2014</t>
+          <t>~2014</t>
         </is>
       </c>
       <c r="F6" s="15" t="inlineStr">
         <is>
-          <t>Ecossistema Norte do Brasil</t>
+          <t>Municípios Norte e outras regiões | Scale-Up Endeavor 2021</t>
         </is>
       </c>
       <c r="G6" s="15" t="inlineStr">
@@ -2465,45 +2473,41 @@
       </c>
       <c r="H6" s="15" t="inlineStr">
         <is>
-          <t>Empresa de capacitação e consultoria para gestão pública municipal na região Norte. TOP 3 Open Startups 2024. Não foram identificados produtos SaaS com identidade digital clara — oportunidade de due diligence.</t>
-        </is>
-      </c>
-      <c r="I6" s="16" t="inlineStr">
-        <is>
-          <t>Watch — due diligence necessário</t>
-        </is>
-      </c>
+          <t>Plataforma integrada de licenciamento digital (urbanístico, ambiental, sanitário, obras), abertura/baixa de empresas, IPTU e ISS digitais integrada à REDESIM federal. Foco em desburocratização e aumento de receita própria municipal. TOP2 Open Startups 2024.</t>
+        </is>
+      </c>
+      <c r="I6" s="15" t="inlineStr"/>
       <c r="J6" s="15" t="inlineStr"/>
     </row>
     <row r="7" ht="48" customHeight="1">
       <c r="A7" s="12" t="inlineStr">
         <is>
-          <t>GESUAS</t>
+          <t>IP Inovação</t>
         </is>
       </c>
       <c r="B7" s="13" t="inlineStr">
         <is>
-          <t>Gestão do SUAS / Assistência Social</t>
+          <t>Capacitação e Consultoria em Gestão Pública</t>
         </is>
       </c>
       <c r="C7" s="13" t="inlineStr">
         <is>
-          <t>Startup / PME</t>
+          <t>Startup</t>
         </is>
       </c>
       <c r="D7" s="13" t="inlineStr">
         <is>
-          <t>Viçosa - MG</t>
+          <t>Belém - PA</t>
         </is>
       </c>
       <c r="E7" s="13" t="inlineStr">
         <is>
-          <t>2008</t>
+          <t>2014</t>
         </is>
       </c>
       <c r="F7" s="13" t="inlineStr">
         <is>
-          <t>Centenas de municípios | CRASs e CREASs</t>
+          <t>Ecossistema Norte do Brasil</t>
         </is>
       </c>
       <c r="G7" s="13" t="inlineStr">
@@ -2513,12 +2517,12 @@
       </c>
       <c r="H7" s="13" t="inlineStr">
         <is>
-          <t>SaaS de gestão do SUAS com Prontuário Digital integrado ao CadÚnico, planos PAIF/PAEFI/PIA, vigilância socioassistencial georreferenciada e relatórios MDS. 56 colaboradores. Líder IE GovTech 2020. Vertical exclusivo sem concorrente direto.</t>
-        </is>
-      </c>
-      <c r="I7" s="17" t="inlineStr">
-        <is>
-          <t>Vertical exclusivo mapeado</t>
+          <t>Empresa de capacitação e consultoria para gestão pública municipal na região Norte. TOP 3 Open Startups 2024. Não foram identificados produtos SaaS com identidade digital clara — oportunidade de due diligence.</t>
+        </is>
+      </c>
+      <c r="I7" s="18" t="inlineStr">
+        <is>
+          <t>Watch — due diligence necessário</t>
         </is>
       </c>
       <c r="J7" s="13" t="inlineStr"/>
@@ -2526,47 +2530,47 @@
     <row r="8" ht="48" customHeight="1">
       <c r="A8" s="14" t="inlineStr">
         <is>
-          <t>Prosas</t>
+          <t>GESUAS</t>
         </is>
       </c>
       <c r="B8" s="15" t="inlineStr">
         <is>
-          <t>Gestão de Editais e Investimento Social</t>
+          <t>Gestão do SUAS / Assistência Social</t>
         </is>
       </c>
       <c r="C8" s="15" t="inlineStr">
         <is>
-          <t>Startup</t>
+          <t>Startup / PME</t>
         </is>
       </c>
       <c r="D8" s="15" t="inlineStr">
         <is>
-          <t>Belo Horizonte - MG</t>
+          <t>Viçosa - MG</t>
         </is>
       </c>
       <c r="E8" s="15" t="inlineStr">
         <is>
-          <t>2014</t>
+          <t>2008</t>
         </is>
       </c>
       <c r="F8" s="15" t="inlineStr">
         <is>
-          <t>13k+ editais | institutos e fundações corporativas</t>
+          <t>Centenas de municípios | CRASs e CREASs</t>
         </is>
       </c>
       <c r="G8" s="15" t="inlineStr">
         <is>
-          <t>R$4M (KPTL)</t>
+          <t>N/D</t>
         </is>
       </c>
       <c r="H8" s="15" t="inlineStr">
         <is>
-          <t>Maior base de editais do terceiro setor no Brasil. Plataforma para criação de editais, inscrições online, pareceristas e monitoramento de projetos. Venture Round out/2024. Portfólio Fundo GovTech KPTL. 51 funcionários.</t>
+          <t>SaaS de gestão do SUAS com Prontuário Digital integrado ao CadÚnico, planos PAIF/PAEFI/PIA, vigilância socioassistencial georreferenciada e relatórios MDS. 56 colaboradores. Líder IE GovTech 2020. Vertical exclusivo sem concorrente direto.</t>
         </is>
       </c>
       <c r="I8" s="16" t="inlineStr">
         <is>
-          <t>Portfólio KPTL</t>
+          <t>Vertical exclusivo mapeado</t>
         </is>
       </c>
       <c r="J8" s="15" t="inlineStr"/>
@@ -2574,12 +2578,12 @@
     <row r="9" ht="48" customHeight="1">
       <c r="A9" s="12" t="inlineStr">
         <is>
-          <t>Lemobs</t>
+          <t>Prosas</t>
         </is>
       </c>
       <c r="B9" s="13" t="inlineStr">
         <is>
-          <t>Gestão Urbana Integrada / Smart Cities</t>
+          <t>Gestão de Editais e Investimento Social</t>
         </is>
       </c>
       <c r="C9" s="13" t="inlineStr">
@@ -2589,41 +2593,45 @@
       </c>
       <c r="D9" s="13" t="inlineStr">
         <is>
-          <t>Rio de Janeiro - RJ</t>
+          <t>Belo Horizonte - MG</t>
         </is>
       </c>
       <c r="E9" s="13" t="inlineStr">
         <is>
-          <t>2015</t>
+          <t>2014</t>
         </is>
       </c>
       <c r="F9" s="13" t="inlineStr">
         <is>
-          <t>79k+ pontos monitorados | prefeituras e Petrobras</t>
+          <t>13k+ editais | institutos e fundações corporativas</t>
         </is>
       </c>
       <c r="G9" s="13" t="inlineStr">
         <is>
-          <t>N/D</t>
+          <t>R$4M (KPTL)</t>
         </is>
       </c>
       <c r="H9" s="13" t="inlineStr">
         <is>
-          <t>GovTech de cidades inteligentes com SIGELU (limpeza urbana), fiscalização móvel, gestão nutricional escolar e saúde. Primeiro contrato pelo Marco Legal das Startups. Origem COPPE/UFRJ. Selo GovTech BrazilLAB.</t>
-        </is>
-      </c>
-      <c r="I9" s="13" t="inlineStr"/>
+          <t>Maior base de editais do terceiro setor no Brasil. Plataforma para criação de editais, inscrições online, pareceristas e monitoramento de projetos. Venture Round out/2024. Portfólio Fundo GovTech KPTL. 51 funcionários.</t>
+        </is>
+      </c>
+      <c r="I9" s="18" t="inlineStr">
+        <is>
+          <t>Portfólio KPTL</t>
+        </is>
+      </c>
       <c r="J9" s="13" t="inlineStr"/>
     </row>
     <row r="10" ht="48" customHeight="1">
       <c r="A10" s="14" t="inlineStr">
         <is>
-          <t>GRTS Digital</t>
+          <t>Lemobs</t>
         </is>
       </c>
       <c r="B10" s="15" t="inlineStr">
         <is>
-          <t>Gestão de Relações Trabalhistas e Sindicais (RTS)</t>
+          <t>Gestão Urbana Integrada / Smart Cities</t>
         </is>
       </c>
       <c r="C10" s="15" t="inlineStr">
@@ -2633,80 +2641,76 @@
       </c>
       <c r="D10" s="15" t="inlineStr">
         <is>
-          <t>Salvador - BA</t>
+          <t>Rio de Janeiro - RJ</t>
         </is>
       </c>
       <c r="E10" s="15" t="inlineStr">
         <is>
-          <t>2019</t>
+          <t>2015</t>
         </is>
       </c>
       <c r="F10" s="15" t="inlineStr">
         <is>
-          <t>Unilever, Coca-Cola, Vivo, Burger King, C&amp;A | 29 colaboradores</t>
+          <t>79k+ pontos monitorados | prefeituras e Petrobras</t>
         </is>
       </c>
       <c r="G10" s="15" t="inlineStr">
         <is>
-          <t>R$ 3,4M aporte (Fundo GovTech)</t>
+          <t>N/D</t>
         </is>
       </c>
       <c r="H10" s="15" t="inlineStr">
         <is>
-          <t>Ecossistema SaaS de digitalização de RTS: gestão de CCTs, IA 'Norma' para análise de cláusulas, assembleias virtuais e data intelligence. Integração com HCM via parceria LG. Prêmio inovação RH 2025. R$3,4M Fundo GovTech KPTL (jun/2025). Lançou GRTS Contábil (12 contratos nas primeiras 3 semanas). Co-investidor Aleve Legal Tech. Meta: R$25M faturamento até 2027. CEO Uirá Menezes, sede Salvador BA.</t>
-        </is>
-      </c>
-      <c r="I10" s="16" t="inlineStr">
-        <is>
-          <t>Portfólio KPTL</t>
-        </is>
-      </c>
+          <t>GovTech de cidades inteligentes com SIGELU (limpeza urbana), fiscalização móvel, gestão nutricional escolar e saúde. Primeiro contrato pelo Marco Legal das Startups. Origem COPPE/UFRJ. Selo GovTech BrazilLAB.</t>
+        </is>
+      </c>
+      <c r="I10" s="15" t="inlineStr"/>
       <c r="J10" s="15" t="inlineStr"/>
     </row>
     <row r="11" ht="48" customHeight="1">
       <c r="A11" s="12" t="inlineStr">
         <is>
-          <t>Governar</t>
+          <t>GRTS Digital</t>
         </is>
       </c>
       <c r="B11" s="13" t="inlineStr">
         <is>
-          <t>ERP Municipal Integrado / SIAFIC Cloud</t>
+          <t>Gestão de Relações Trabalhistas e Sindicais (RTS)</t>
         </is>
       </c>
       <c r="C11" s="13" t="inlineStr">
         <is>
-          <t>Startup / Scale-up</t>
+          <t>Startup</t>
         </is>
       </c>
       <c r="D11" s="13" t="inlineStr">
         <is>
-          <t>Brasil</t>
+          <t>Salvador - BA</t>
         </is>
       </c>
       <c r="E11" s="13" t="inlineStr">
         <is>
-          <t>N/D</t>
+          <t>2019</t>
         </is>
       </c>
       <c r="F11" s="13" t="inlineStr">
         <is>
-          <t>Municípios de qualquer porte | SIAFIC + SIEDUC disponíveis</t>
+          <t>Unilever, Coca-Cola, Vivo, Burger King, C&amp;A | 29 colaboradores</t>
         </is>
       </c>
       <c r="G11" s="13" t="inlineStr">
         <is>
-          <t>N/D</t>
+          <t>R$ 3,4M aporte (Fundo GovTech)</t>
         </is>
       </c>
       <c r="H11" s="13" t="inlineStr">
         <is>
-          <t>Suite ERP municipal integrada em nuvem com base de dados única: SIAFIC (financeiro/tributário), SIEDUC (educação), SISAÚDE e SIASOC. Conformidade SICONFI, SIOPE, e-Social, eSUS. Produto novo no mercado com proposta de stack completo integrado.</t>
-        </is>
-      </c>
-      <c r="I11" s="17" t="inlineStr">
-        <is>
-          <t>Watch — SIAFIC driver</t>
+          <t>Ecossistema SaaS de digitalização de RTS: gestão de CCTs, IA 'Norma' para análise de cláusulas, assembleias virtuais e data intelligence. Integração com HCM via parceria LG. Prêmio inovação RH 2025. R$3,4M Fundo GovTech KPTL (jun/2025). Lançou GRTS Contábil (12 contratos nas primeiras 3 semanas). Co-investidor Aleve Legal Tech. Meta: R$25M faturamento até 2027. CEO Uirá Menezes, sede Salvador BA.</t>
+        </is>
+      </c>
+      <c r="I11" s="18" t="inlineStr">
+        <is>
+          <t>Portfólio KPTL</t>
         </is>
       </c>
       <c r="J11" s="13" t="inlineStr"/>
@@ -2714,47 +2718,47 @@
     <row r="12" ht="48" customHeight="1">
       <c r="A12" s="14" t="inlineStr">
         <is>
-          <t>Colab</t>
+          <t>Governar</t>
         </is>
       </c>
       <c r="B12" s="15" t="inlineStr">
         <is>
-          <t>Participação Cidadã e Serviços Digitais Municipais</t>
+          <t>ERP Municipal Integrado / SIAFIC Cloud</t>
         </is>
       </c>
       <c r="C12" s="15" t="inlineStr">
         <is>
-          <t>Scale-up</t>
+          <t>Startup / Scale-up</t>
         </is>
       </c>
       <c r="D12" s="15" t="inlineStr">
         <is>
-          <t>São Paulo - SP</t>
+          <t>Brasil</t>
         </is>
       </c>
       <c r="E12" s="15" t="inlineStr">
         <is>
-          <t>2013</t>
+          <t>N/D</t>
         </is>
       </c>
       <c r="F12" s="15" t="inlineStr">
         <is>
-          <t>5 países | 1M+ cidadãos | Piauí, São Gonçalo, Santo André | Parceiro ONU-Habitat</t>
+          <t>Municípios de qualquer porte | SIAFIC + SIEDUC disponíveis</t>
         </is>
       </c>
       <c r="G12" s="15" t="inlineStr">
         <is>
-          <t>~R$25M total (MDIF+Luminate+EDP+KPTL)</t>
+          <t>N/D</t>
         </is>
       </c>
       <c r="H12" s="15" t="inlineStr">
         <is>
-          <t>Plataforma multicanal (web, app, WhatsApp) de gestão de serviços digitais, participação cidadã e CRM governamental. IA digitaliza qualquer serviço público em minutos. Em 2025 viabilizou OP Digital do Piauí (273k participantes) com validação via Receita Federal e blockchain. Lançou Colab Gov.AI (AWS Bedrock, out/2025): 94% de aceleração na criação de serviços digitais, 500+ prompts em 14 dias. Novos clientes: TCU, Diadema, Rio das Ostras, Duque de Caxias. Rodada US$10M+ em curso para 2026. Portfólio KPTL+Cedro. Co-invest EDP Ventures + Luminate + MDIF.</t>
+          <t>Suite ERP municipal integrada em nuvem com base de dados única: SIAFIC (financeiro/tributário), SIEDUC (educação), SISAÚDE e SIASOC. Conformidade SICONFI, SIOPE, e-Social, eSUS. Produto novo no mercado com proposta de stack completo integrado.</t>
         </is>
       </c>
       <c r="I12" s="16" t="inlineStr">
         <is>
-          <t>Portfólio KPTL+Cedro</t>
+          <t>Watch — SIAFIC driver</t>
         </is>
       </c>
       <c r="J12" s="15" t="inlineStr"/>
@@ -2762,47 +2766,47 @@
     <row r="13" ht="48" customHeight="1">
       <c r="A13" s="12" t="inlineStr">
         <is>
-          <t>Pública Tecnologia</t>
+          <t>Colab</t>
         </is>
       </c>
       <c r="B13" s="13" t="inlineStr">
         <is>
-          <t>ERP Municipal Full Suite</t>
+          <t>Participação Cidadã e Serviços Digitais Municipais</t>
         </is>
       </c>
       <c r="C13" s="13" t="inlineStr">
         <is>
-          <t>PME Estabelecida</t>
+          <t>Scale-up</t>
         </is>
       </c>
       <c r="D13" s="13" t="inlineStr">
         <is>
-          <t>Blumenau - SC</t>
+          <t>São Paulo - SP</t>
         </is>
       </c>
       <c r="E13" s="13" t="inlineStr">
         <is>
-          <t>1993</t>
+          <t>2013</t>
         </is>
       </c>
       <c r="F13" s="13" t="inlineStr">
         <is>
-          <t>Municípios BR + Portugal + Venezuela</t>
+          <t>5 países | 1M+ cidadãos | Piauí, São Gonçalo, Santo André | Parceiro ONU-Habitat</t>
         </is>
       </c>
       <c r="G13" s="13" t="inlineStr">
         <is>
-          <t>N/D</t>
+          <t>~R$25M total (MDIF+Luminate+EDP+KPTL)</t>
         </is>
       </c>
       <c r="H13" s="13" t="inlineStr">
         <is>
-          <t>ERP municipal full suite com 9 áreas: Financeira (contabilidade pública, NF-e), Tributária (ISS, IPTU), Gestão de Pessoas (RH, eSocial, ponto eletrônico), Saúde, Escolar, Assistência Social (SUAS), Administrativa (compras, frotas, patrimônio), Atendimento ao Cidadão (portal transparência, app Cidade Pública) e Gestão (BI, GED, PPA). 33 anos de atuação, 98 funcionários. Great Place to Work. Presença internacional: Portugal e Venezuela. Sede Blumenau/SC.</t>
-        </is>
-      </c>
-      <c r="I13" s="17" t="inlineStr">
-        <is>
-          <t>Target roll-up</t>
+          <t>Plataforma multicanal (web, app, WhatsApp) de gestão de serviços digitais, participação cidadã e CRM governamental. IA digitaliza qualquer serviço público em minutos. Em 2025 viabilizou OP Digital do Piauí (273k participantes) com validação via Receita Federal e blockchain. Lançou Colab Gov.AI (AWS Bedrock, out/2025): 94% de aceleração na criação de serviços digitais, 500+ prompts em 14 dias. Novos clientes: TCU, Diadema, Rio das Ostras, Duque de Caxias. Rodada US$10M+ em curso para 2026. Portfólio KPTL+Cedro. Co-invest EDP Ventures + Luminate + MDIF.</t>
+        </is>
+      </c>
+      <c r="I13" s="18" t="inlineStr">
+        <is>
+          <t>Portfólio KPTL+Cedro</t>
         </is>
       </c>
       <c r="J13" s="13" t="inlineStr"/>
@@ -2810,50 +2814,98 @@
     <row r="14" ht="48" customHeight="1">
       <c r="A14" s="14" t="inlineStr">
         <is>
+          <t>Pública Tecnologia</t>
+        </is>
+      </c>
+      <c r="B14" s="15" t="inlineStr">
+        <is>
+          <t>ERP Municipal Full Suite</t>
+        </is>
+      </c>
+      <c r="C14" s="15" t="inlineStr">
+        <is>
+          <t>PME Estabelecida</t>
+        </is>
+      </c>
+      <c r="D14" s="15" t="inlineStr">
+        <is>
+          <t>Blumenau - SC</t>
+        </is>
+      </c>
+      <c r="E14" s="15" t="inlineStr">
+        <is>
+          <t>1993</t>
+        </is>
+      </c>
+      <c r="F14" s="15" t="inlineStr">
+        <is>
+          <t>Municípios BR + Portugal + Venezuela</t>
+        </is>
+      </c>
+      <c r="G14" s="15" t="inlineStr">
+        <is>
+          <t>N/D</t>
+        </is>
+      </c>
+      <c r="H14" s="15" t="inlineStr">
+        <is>
+          <t>ERP municipal full suite com 9 áreas: Financeira (contabilidade pública, NF-e), Tributária (ISS, IPTU), Gestão de Pessoas (RH, eSocial, ponto eletrônico), Saúde, Escolar, Assistência Social (SUAS), Administrativa (compras, frotas, patrimônio), Atendimento ao Cidadão (portal transparência, app Cidade Pública) e Gestão (BI, GED, PPA). 33 anos de atuação, 98 funcionários. Great Place to Work. Presença internacional: Portugal e Venezuela. Sede Blumenau/SC.</t>
+        </is>
+      </c>
+      <c r="I14" s="16" t="inlineStr">
+        <is>
+          <t>Target roll-up</t>
+        </is>
+      </c>
+      <c r="J14" s="15" t="inlineStr"/>
+    </row>
+    <row r="15" ht="48" customHeight="1">
+      <c r="A15" s="12" t="inlineStr">
+        <is>
           <t>PLACE</t>
         </is>
       </c>
-      <c r="B14" s="15" t="inlineStr">
+      <c r="B15" s="13" t="inlineStr">
         <is>
           <t>Planejamento Urbano e Geointeligência / Urban Twin</t>
         </is>
       </c>
-      <c r="C14" s="15" t="inlineStr">
+      <c r="C15" s="13" t="inlineStr">
         <is>
           <t>Startup</t>
         </is>
       </c>
-      <c r="D14" s="15" t="inlineStr">
+      <c r="D15" s="13" t="inlineStr">
         <is>
           <t>Brasil</t>
         </is>
       </c>
-      <c r="E14" s="15" t="inlineStr">
-        <is>
-          <t>N/D</t>
-        </is>
-      </c>
-      <c r="F14" s="15" t="inlineStr">
+      <c r="E15" s="13" t="inlineStr">
+        <is>
+          <t>N/D</t>
+        </is>
+      </c>
+      <c r="F15" s="13" t="inlineStr">
         <is>
           <t>Prefeituras e mercado imobiliário privado</t>
         </is>
       </c>
-      <c r="G14" s="15" t="inlineStr">
-        <is>
-          <t>N/D</t>
-        </is>
-      </c>
-      <c r="H14" s="15" t="inlineStr">
+      <c r="G15" s="13" t="inlineStr">
+        <is>
+          <t>N/D</t>
+        </is>
+      </c>
+      <c r="H15" s="13" t="inlineStr">
         <is>
           <t>Plataforma dual (govtech + proptech) de inteligência territorial com Gêmeo Digital: integra bases públicas, rotinas urbanísticas, pré-aprovação de projetos e visualização 2D/3D com IA aplicada à legislação urbanística. Para o setor privado: viabilidade e gestão de portfólio imobiliário. Certificada BrazilLAB.</t>
         </is>
       </c>
-      <c r="I14" s="16" t="inlineStr">
+      <c r="I15" s="18" t="inlineStr">
         <is>
           <t>Watch — urbanismo digital</t>
         </is>
       </c>
-      <c r="J14" s="15" t="inlineStr"/>
+      <c r="J15" s="13" t="inlineStr"/>
     </row>
   </sheetData>
   <mergeCells count="1">
@@ -2885,7 +2937,7 @@
   </cols>
   <sheetData>
     <row r="1" ht="28" customHeight="1">
-      <c r="A1" s="18" t="inlineStr">
+      <c r="A1" s="19" t="inlineStr">
         <is>
           <t>📊 Fiscal &amp; Convênios Municipais — Radar GovTech Brasil 2025/2026</t>
         </is>
@@ -3076,7 +3128,7 @@
           <t>Primeiro sistema inteligente de gestão de convênios para prefeituras: unifica automaticamente TransfereGov, Simec, Sismob, FNS e Sigcon em painel único com IA. Kanban automático de diligências, alertas de prazo, monitoramento de certidões, previsão de repasses e elaboração de propostas com IA baseadas em cotações federais. Diferencial: deixa a IA captar e monitorar enquanto a prefeitura foca na execução.</t>
         </is>
       </c>
-      <c r="I5" s="17" t="inlineStr">
+      <c r="I5" s="18" t="inlineStr">
         <is>
           <t>Watch — convênios nicho virgem</t>
         </is>
@@ -3172,7 +3224,7 @@
           <t>18 anos como líder em geointeligência para prefeituras. Plataforma Geopixel Cidades integra geoprocessamento com IA para IPTU, ITBI, ISS e alvarás (digital e por QR Code). Módulos: SIG municipal integrado, monitoramento por satélite de alterações, mobilidade de campo e eventos ambientais. Reforma Tributária (LC 214/2025) cria janela de demanda direta e imediata.</t>
         </is>
       </c>
-      <c r="I7" s="17" t="inlineStr">
+      <c r="I7" s="18" t="inlineStr">
         <is>
           <t>Oportunidade fiscal 2025</t>
         </is>
@@ -3268,7 +3320,7 @@
           <t>Plataforma de IA para gestão pública com metodologia exclusiva 3P: Preditiva (projeta receitas, saúde e matrículas), Preventiva (alertas automáticos de anomalias e contratos) e Prescritiva (sugere onde cortar custos, otimizar frota e compras). Dashboards interativos para todas as secretarias. Chat inteligente para consultas sobre dados oficiais da cidade. Marketplace de soluções parceiras integradas nativamente.</t>
         </is>
       </c>
-      <c r="I9" s="17" t="inlineStr">
+      <c r="I9" s="18" t="inlineStr">
         <is>
           <t>Watch</t>
         </is>
@@ -3305,7 +3357,7 @@
   </cols>
   <sheetData>
     <row r="1" ht="28" customHeight="1">
-      <c r="A1" s="19" t="inlineStr">
+      <c r="A1" s="20" t="inlineStr">
         <is>
           <t>🏥 Saúde Pública — Radar GovTech Brasil 2025/2026</t>
         </is>
@@ -3404,7 +3456,7 @@
           <t>Suite modular de soluções estratégicas para gestão pública: Saúde Simples (prontuário, telemedicina, IA transcrevendo consultas), Educação Simples (gestão escolar), DadosGov Simples (BI exclusivo setor público), Mob Simples (gestão de frotas), Doc+ Simples (gestão documental), Outsourcing Simples (impressão) e Mentor Público (IEG-M com IA). 1º prontuário transcrito por IA da saúde pública do Brasil. Crescimento 40% na pandemia.</t>
         </is>
       </c>
-      <c r="I3" s="17" t="inlineStr">
+      <c r="I3" s="18" t="inlineStr">
         <is>
           <t>Target roll-up</t>
         </is>
@@ -3500,7 +3552,7 @@
           <t>26 anos de operação em saúde pública e gestão municipal. Selos Ouro/Prata Bora Vacinar (mar/2025). Cliente Sorocaba SP avançou C+ → B no IEGM 2025. Foco saúde pública + educação municipal integradas.</t>
         </is>
       </c>
-      <c r="I5" s="17" t="inlineStr">
+      <c r="I5" s="18" t="inlineStr">
         <is>
           <t>Target roll-up</t>
         </is>
@@ -3680,7 +3732,7 @@
           <t>Aplicativo para gestão de escala médica em um só lugar: elimina planilhas, automatiza escalas de plantão e reduz glosas e fraudes administrativas. 50+ organizações economizando milhões. Top 30 Sebrae 2024. Acelerada GovTech Pará.</t>
         </is>
       </c>
-      <c r="I9" s="17" t="inlineStr">
+      <c r="I9" s="18" t="inlineStr">
         <is>
           <t>Watch — anti-fraude saúde</t>
         </is>
@@ -3717,7 +3769,7 @@
   </cols>
   <sheetData>
     <row r="1" ht="28" customHeight="1">
-      <c r="A1" s="20" t="inlineStr">
+      <c r="A1" s="21" t="inlineStr">
         <is>
           <t>📚 Educação Pública — Radar GovTech Brasil 2025/2026</t>
         </is>
@@ -3816,7 +3868,7 @@
           <t>Mantenedora do i-Educar (software público federal MEC). Abriu o código-fonte do Pré-Matrícula Digital (PMD) em parceria com MEC, Fundação Lemann e MP-SC. Também atua em assistência social (SUAS): 50+ municípios, 200k+ famílias. Meta: 1,5M alunos até 2027. Parceria Portábilis+Educa Rios expandindo para AM.</t>
         </is>
       </c>
-      <c r="I3" s="17" t="inlineStr">
+      <c r="I3" s="18" t="inlineStr">
         <is>
           <t>Target / impacto</t>
         </is>
@@ -4084,7 +4136,7 @@
           <t>Software público federal mantido pela Portabilis. Pré-Matrícula Digital PMD aberto ao público em 2025 (código no GitHub). Monte Alegre (RN) economizou R$2,4M. Parceria MEC + Fundação Lemann + MP-SC. Canoas RS referência em implementação.</t>
         </is>
       </c>
-      <c r="I9" s="17" t="inlineStr">
+      <c r="I9" s="18" t="inlineStr">
         <is>
           <t>Referência pública</t>
         </is>
@@ -4180,12 +4232,12 @@
           <t>Edtech amapaense fundada às margens do Rio Amazonas. Vertical pública Proesc Gov já implantada na Secretaria de Educação de Macapá: diário eletrônico com app offline, matrículas digitais, IDEB/VAAR e gestão da secretaria. Diferencial: Botão Alerta Escolar conecta as 105 escolas municipais à Guarda Civil Municipal. IA 'LIA' para decisões estratégicas nas secretarias. 3.000–3.500+ escolas parceiras (privadas + públicas), 5 países, 35+ redes pelo Brasil. Captou a maior rodada de investimento já realizada na Amazônia (Exame).</t>
         </is>
       </c>
-      <c r="I11" s="17" t="inlineStr">
+      <c r="I11" s="18" t="inlineStr">
         <is>
           <t>Watch — pública + Amazônia</t>
         </is>
       </c>
-      <c r="J11" s="21" t="inlineStr">
+      <c r="J11" s="22" t="inlineStr">
         <is>
           <t>✓</t>
         </is>
@@ -4221,7 +4273,7 @@
   </cols>
   <sheetData>
     <row r="1" ht="28" customHeight="1">
-      <c r="A1" s="22" t="inlineStr">
+      <c r="A1" s="23" t="inlineStr">
         <is>
           <t>🤖 IA Horizontal &amp; Automação — Radar GovTech Brasil 2025/2026</t>
         </is>
@@ -4320,7 +4372,7 @@
           <t>Agentes IA via WhatsApp que operam sistemas municipais sem integração tradicional. 200+ municípios em menos de 12 meses. Modelo viral de adoção. Potencial alvo de aquisição.</t>
         </is>
       </c>
-      <c r="I3" s="17" t="inlineStr">
+      <c r="I3" s="18" t="inlineStr">
         <is>
           <t>M&amp;A Watch</t>
         </is>
@@ -4412,7 +4464,7 @@
           <t>Instituto de P&amp;D referência em telecomunicações e tecnologias convergentes. Projeto INSPIRE com MGI (R$390M, 4 anos): IA personalizada para serviços de governo digital — assistentes virtuais de voz, recomendação e acessibilidade. Portfólio inclui IoT, Blockchain, IA, Conectividade Inteligente, OSS/BSS. Mais de 30 soluções comerciais.</t>
         </is>
       </c>
-      <c r="I5" s="17" t="inlineStr">
+      <c r="I5" s="18" t="inlineStr">
         <is>
           <t>Parceria estratégica MGI</t>
         </is>
@@ -4508,7 +4560,7 @@
           <t>Pioneira em monitoramento automatizado de dados governamentais (Legislativo, Executivo, Judiciário). 4M+ proposições monitoradas, +700 fontes incluindo Diários Oficiais. IA com termômetro de aprovação de PLs (&gt;98% acurácia). Única com 100% de cobertura das Assembleias Estaduais. Plataforma de Stakeholders para gestão de contatos e RIG. Ranking 100 Open Startups, Mapa GovTech. Cubo Itaú, Inovabra, Distrito.</t>
         </is>
       </c>
-      <c r="I7" s="17" t="inlineStr">
+      <c r="I7" s="18" t="inlineStr">
         <is>
           <t>Watch — inteligência regulatória</t>
         </is>
@@ -4561,7 +4613,7 @@
           <t>M&amp;A Watch — portfólio Cedro</t>
         </is>
       </c>
-      <c r="J8" s="23" t="inlineStr">
+      <c r="J8" s="17" t="inlineStr">
         <is>
           <t>✓</t>
         </is>
@@ -4608,7 +4660,7 @@
           <t>IA + visão computacional para análises ergonômicas e psicossociais automatizadas: reconhecimento de movimentos, quantificação de riscos biomecânicos e cronoanálise (Indústria 4.0). Resultados: -38% FAP, -30% afastamentos por DORT, análises 5x mais rápidas. Clientes: Marfrig, CNH Industrial, P&amp;G, Electrolux, Vibra. 8º investimento Fundo GovTech (KPTL+Cedro), R$3M fev/2026. Campus da Indústria FIEP. 29 países.</t>
         </is>
       </c>
-      <c r="I9" s="17" t="inlineStr">
+      <c r="I9" s="18" t="inlineStr">
         <is>
           <t>Portfólio KPTL+Cedro</t>
         </is>
@@ -4744,7 +4796,7 @@
           <t>10M+ minutas geradas. TJRS, STM, TRE-PB/BA, Tocantins. CNJ Resolução 615/2025. Exportou para a Argentina.</t>
         </is>
       </c>
-      <c r="I3" s="17" t="inlineStr">
+      <c r="I3" s="18" t="inlineStr">
         <is>
           <t>Watch — tração judicial</t>
         </is>
@@ -4928,7 +4980,7 @@
           <t>Prisma: detecção de irregularidades em contratos públicos e lavagem de dinheiro. Cruzamento de bases abertas por IA. Selecionada CPSI MPRJ.</t>
         </is>
       </c>
-      <c r="I7" s="17" t="inlineStr">
+      <c r="I7" s="18" t="inlineStr">
         <is>
           <t>Contrato CPSI</t>
         </is>
@@ -5156,7 +5208,7 @@
           <t>Maior marketplace de licitações do Brasil. 40%+ dos municípios. Fundadores: Leonardo + Bruno Ladeira (Ecustomize). Certificações ISO 9001, 27001, 27701, 20000-1. Integrado ao PNCP. 35% crescimento anual. Portfólio Cedro Capital (FIP Venture Brasil Central) — disponível para M&amp;A, sem mandatada.</t>
         </is>
       </c>
-      <c r="I3" s="17" t="inlineStr">
+      <c r="I3" s="18" t="inlineStr">
         <is>
           <t>M&amp;A Watch — portfólio Cedro</t>
         </is>
@@ -5248,7 +5300,7 @@
           <t>Suite SaaS para fornecedores que vendem para governo: i-Ganhei (captação com IA, workflow, propostas automáticas, gestão de contratos), i-Pesquisei (inteligência de mercado B2G), i-Documentei (gestão de certidões), BPO de Licitações e i-One (projetos IA sob medida). Portfólio Fundo GovTech KPTL. 300% mais eficiência declarada.</t>
         </is>
       </c>
-      <c r="I5" s="17" t="inlineStr">
+      <c r="I5" s="18" t="inlineStr">
         <is>
           <t>Portfólio KPTL</t>
         </is>
@@ -5340,7 +5392,7 @@
           <t>Plataforma SaaS 100% flexível de gestão de compras corporativas com IA: cotação, disputas (aberta/fechada/leilão reverso), gestão de contratos, portal do fornecedor e BI de saving. Conformidade 14.133, 13.303 e Pregão Eletrônico. IA Pesquisa de Mercado premiada (Desafio TREM). Parte do Grupo Squadra (venture builder + data intelligence + cybersec). Integra Totvs, SAP, Oracle, Dynamics.</t>
         </is>
       </c>
-      <c r="I7" s="17" t="inlineStr">
+      <c r="I7" s="18" t="inlineStr">
         <is>
           <t>Watch — compras gov</t>
         </is>
@@ -5436,12 +5488,12 @@
           <t>1º Sistema Operacional de IA Multi-Agente para Licitações da América Latina. 14 módulos IA: AI Matching score 0–100, robô de lances IA, inteligência competitiva (5 módulos), pesquisa de preços IN 65/2021, grafo societário, detecção de anomalias, compliance checker e forensic replay. Cobre sell-side (fornecedores) + buy-side (entes públicos) + compliance (TCUs). Integração PNCP. Planos: R$297–R$1.497/mês.</t>
         </is>
       </c>
-      <c r="I9" s="17" t="inlineStr">
+      <c r="I9" s="18" t="inlineStr">
         <is>
           <t>Watch — IA licitações multi-agente</t>
         </is>
       </c>
-      <c r="J9" s="21" t="inlineStr">
+      <c r="J9" s="22" t="inlineStr">
         <is>
           <t>✓</t>
         </is>
@@ -5493,7 +5545,7 @@
           <t>Watch — sell-side PME</t>
         </is>
       </c>
-      <c r="J10" s="23" t="inlineStr">
+      <c r="J10" s="17" t="inlineStr">
         <is>
           <t>✓</t>
         </is>
@@ -5628,7 +5680,7 @@
           <t>Plataforma SaaS para regularização fundiária urbana (REURB) ponta a ponta. App offline para coleta de campo. Emissão automática de relatórios técnicos, Títulos de Legitimação e Posse (TLP) e CRF. Integração com cartórios. Reduz 180 dias para 60 dias no processo. Municípios atendidos: Vitória ES, Vila Velha ES, Aracruz ES, Itabuna BA, Parnamirim RN, entre outros. ESG: 100% digital, zero papel.</t>
         </is>
       </c>
-      <c r="I3" s="17" t="inlineStr">
+      <c r="I3" s="18" t="inlineStr">
         <is>
           <t>Watch — REURB nicho virgem</t>
         </is>
@@ -5724,7 +5776,7 @@
           <t>Plataforma corporativa para REURB: diagnóstico, mapeamento geoespacial, emissão automática de CRF e integração com cartórios. 30k+ matrículas abertas em 12 meses. Contratos com Governo do Piauí (PROURBE) e Tribunal de Justiça.</t>
         </is>
       </c>
-      <c r="I5" s="17" t="inlineStr">
+      <c r="I5" s="18" t="inlineStr">
         <is>
           <t>Watch — tração judicial</t>
         </is>

</xml_diff>

<commit_message>
v15: adiciona 8 govtechs da varredura de mercado
SentinelX, Camerite, Monuv (segpub), Zaelo, Licito.guru (lic),
Munitax (fiscal), Leme, Layers (educ). Aporte Layers R$21M incluído
nos APORTES. Total: 80 empresas únicas, 82 aparições, 17 aportes.

Co-Authored-By: Claude Sonnet 4.6 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/Radar_GovTechs_Brasil_2026.xlsx
+++ b/Radar_GovTechs_Brasil_2026.xlsx
@@ -230,14 +230,14 @@
     <xf numFmtId="0" fontId="4" fillId="7" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center"/>
     </xf>
+    <xf numFmtId="0" fontId="6" fillId="5" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment vertical="top" wrapText="1"/>
+    </xf>
     <xf numFmtId="0" fontId="4" fillId="8" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="4" fillId="3" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="6" fillId="5" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment vertical="top" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="4" fillId="9" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center"/>
@@ -647,7 +647,7 @@
     <row r="1" ht="32" customHeight="1">
       <c r="A1" s="1" t="inlineStr">
         <is>
-          <t>🇧🇷 Radar GovTech Brasil 2025/2026 — DLG · Maio 2026 · v14</t>
+          <t>🇧🇷 Radar GovTech Brasil 2025/2026 — DLG · Maio 2026 · v15</t>
         </is>
       </c>
     </row>
@@ -680,7 +680,7 @@
         </is>
       </c>
       <c r="B5" s="4" t="n">
-        <v>7</v>
+        <v>8</v>
       </c>
     </row>
     <row r="6">
@@ -700,7 +700,7 @@
         </is>
       </c>
       <c r="B7" s="4" t="n">
-        <v>9</v>
+        <v>11</v>
       </c>
     </row>
     <row r="8">
@@ -730,7 +730,7 @@
         </is>
       </c>
       <c r="B10" s="4" t="n">
-        <v>8</v>
+        <v>10</v>
       </c>
     </row>
     <row r="11">
@@ -770,7 +770,7 @@
         </is>
       </c>
       <c r="B14" s="4" t="n">
-        <v>7</v>
+        <v>10</v>
       </c>
     </row>
     <row r="15">
@@ -780,7 +780,7 @@
         </is>
       </c>
       <c r="B15" s="6" t="n">
-        <v>74</v>
+        <v>82</v>
       </c>
     </row>
     <row r="16">
@@ -790,7 +790,7 @@
         </is>
       </c>
       <c r="B16" s="8" t="n">
-        <v>72</v>
+        <v>80</v>
       </c>
     </row>
     <row r="18">
@@ -800,7 +800,7 @@
         </is>
       </c>
       <c r="B18" s="9" t="n">
-        <v>16</v>
+        <v>17</v>
       </c>
     </row>
   </sheetData>
@@ -1233,7 +1233,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:J9"/>
+  <dimension ref="A1:J12"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="28" customWidth="1" min="1" max="1"/>
@@ -1310,128 +1310,136 @@
     <row r="3" ht="48" customHeight="1">
       <c r="A3" s="12" t="inlineStr">
         <is>
-          <t>Sipremo</t>
+          <t>SentinelX</t>
         </is>
       </c>
       <c r="B3" s="13" t="inlineStr">
         <is>
-          <t>Previsão de Desastres / ClimateTech</t>
+          <t>Reconhecimento Facial com IA / Segurança Pública Urbana</t>
         </is>
       </c>
       <c r="C3" s="13" t="inlineStr">
         <is>
-          <t>Startup</t>
+          <t>Scale-up</t>
         </is>
       </c>
       <c r="D3" s="13" t="inlineStr">
         <is>
-          <t>Ribeirão Preto - SP</t>
+          <t>São Paulo - SP</t>
         </is>
       </c>
       <c r="E3" s="13" t="inlineStr">
         <is>
-          <t>~2018</t>
+          <t>N/D</t>
         </is>
       </c>
       <c r="F3" s="13" t="inlineStr">
         <is>
-          <t>Defesa Civil + seguros</t>
+          <t>40K+ câmeras | 2.718+ foragidos capturados | 3.650+ presos em flagrante (2025) | 48+ projetos em andamento</t>
         </is>
       </c>
       <c r="G3" s="13" t="inlineStr">
         <is>
-          <t>R$200k (2022)</t>
+          <t>N/D</t>
         </is>
       </c>
       <c r="H3" s="13" t="inlineStr">
         <is>
-          <t>IA para previsão antecipada de desastres naturais com dados NASA e bases nacionais. Alerta SMS via Defesa Civil municipal. Selecionada COP26. Foco em mitigação de riscos climáticos e resiliência urbana.</t>
+          <t>Maior plataforma de reconhecimento facial com IA da América Latina. Motor tecnológico por trás do Smart Sampa (SP): sistema de videomonitoramento integrado da cidade de São Paulo. 2.718+ criminosos foragidos capturados e 3.650+ pessoas presas em flagrante em 2025. R$40M de investimento em novas tecnologias planejado. 48+ projetos em andamento no Brasil. CEO: Cristian Aquino. Reconhecimento facial em tempo real em escala urbana.</t>
         </is>
       </c>
       <c r="I3" s="18" t="inlineStr">
         <is>
-          <t>Watch — clima/risco</t>
-        </is>
-      </c>
-      <c r="J3" s="13" t="inlineStr"/>
+          <t>🔥 Deal — Smart Sampa</t>
+        </is>
+      </c>
+      <c r="J3" s="20" t="inlineStr">
+        <is>
+          <t>✓</t>
+        </is>
+      </c>
     </row>
     <row r="4" ht="48" customHeight="1">
       <c r="A4" s="14" t="inlineStr">
         <is>
-          <t>i4Sea</t>
+          <t>Camerite</t>
         </is>
       </c>
       <c r="B4" s="15" t="inlineStr">
         <is>
-          <t>Previsões Microclimáticas / Portos e Energia</t>
+          <t>IA para Videomonitoramento Multimarcas (Facial + Placas)</t>
         </is>
       </c>
       <c r="C4" s="15" t="inlineStr">
         <is>
-          <t>Startup</t>
+          <t>Startup / Scale-up</t>
         </is>
       </c>
       <c r="D4" s="15" t="inlineStr">
         <is>
-          <t>Santos - SP</t>
+          <t>Brasil</t>
         </is>
       </c>
       <c r="E4" s="15" t="inlineStr">
         <is>
-          <t>~2018</t>
+          <t>N/D</t>
         </is>
       </c>
       <c r="F4" s="15" t="inlineStr">
         <is>
-          <t>Portos, setor elétrico e renovável | Porto do Açu, Wilson Sons, Santos Brasil</t>
+          <t>Sete Lagoas MG (Guardião 7L) | Smart Sampa SP | modelo franquia nacional</t>
         </is>
       </c>
       <c r="G4" s="15" t="inlineStr">
         <is>
-          <t>R$ 7,5M (Fundo GovTech)</t>
+          <t>N/D</t>
         </is>
       </c>
       <c r="H4" s="15" t="inlineStr">
         <is>
-          <t>Plataforma i4cast® de decisão baseada em inteligência climática: previsões hiperlocais de mar e clima para operações portuárias, logística marítima e geração de energia renovável. Precisão 2x superior a previsões genéricas (94% acurácia no Porto do Açu). Captou R$7,5M do Fundo GovTech KPTL.</t>
+          <t>Plataforma de IA para videomonitoramento compatível com câmeras de qualquer fabricante. Plataforma Cortex com IA 'Hórus': reconhecimento facial, leitura de placas, detecção de comportamentos suspeitos e rede colaborativa entre câmeras de diferentes entes. Modelo de franquia para expansão nacional. Cases: Sete Lagoas MG (Projeto Guardião 7L) e integração ao Smart Sampa (SP). Reduz custo de implantação por não exigir troca de hardware existente.</t>
         </is>
       </c>
       <c r="I4" s="16" t="inlineStr">
         <is>
-          <t>Portfólio KPTL</t>
-        </is>
-      </c>
-      <c r="J4" s="15" t="inlineStr"/>
+          <t>Watch — expansão franquias</t>
+        </is>
+      </c>
+      <c r="J4" s="17" t="inlineStr">
+        <is>
+          <t>✓</t>
+        </is>
+      </c>
     </row>
     <row r="5" ht="48" customHeight="1">
       <c r="A5" s="12" t="inlineStr">
         <is>
-          <t>IPQ Tecnologia</t>
+          <t>Monuv</t>
         </is>
       </c>
       <c r="B5" s="13" t="inlineStr">
         <is>
-          <t>Segurança Pública / TIC para Ambientes Críticos</t>
+          <t>VMS em Nuvem + IA / Videomonitoramento Urbano</t>
         </is>
       </c>
       <c r="C5" s="13" t="inlineStr">
         <is>
-          <t>PME / Scale-up</t>
+          <t>Startup / Scale-up</t>
         </is>
       </c>
       <c r="D5" s="13" t="inlineStr">
         <is>
-          <t>Porto Alegre - RS</t>
+          <t>Brasil</t>
         </is>
       </c>
       <c r="E5" s="13" t="inlineStr">
         <is>
-          <t>~2001</t>
+          <t>N/D</t>
         </is>
       </c>
       <c r="F5" s="13" t="inlineStr">
         <is>
-          <t>Nacional e internacional | órgãos públicos, presídios, hospitais, rodovias</t>
+          <t>14.000+ câmeras no Smart Sampa SP (principal provedor) | planos a partir de R$900/mês</t>
         </is>
       </c>
       <c r="G5" s="13" t="inlineStr">
@@ -1441,95 +1449,107 @@
       </c>
       <c r="H5" s="13" t="inlineStr">
         <is>
-          <t>25+ anos desenvolvendo e integrando soluções de TIC com IA e Analytics para segurança pública e ambientes críticos. Portfólio: videomonitoramento, controle de acesso, redes de dados públicas/privadas, infraestrutura para Defesa e Segurança. Atuação descentralizada com cobertura nacional.</t>
-        </is>
-      </c>
-      <c r="I5" s="13" t="inlineStr"/>
-      <c r="J5" s="13" t="inlineStr"/>
+          <t>VMS (Video Management System) 100% em nuvem com IA embarcada. Principal fornecedor do Smart Sampa: 14.000+ câmeras integradas ao sistema de videomonitoramento da cidade de São Paulo. Detecção de pessoas por IA lançada abr/2026 (98%+ acurácia, reduz 100x falsos alarmes). Plataforma agnóstica de hardware — integra câmeras de qualquer fabricante. Modelo SaaS acessível com planos a partir de R$900/mês, escalável do pequeno município à metrópole. Obs.: Monuv faz detecção de objetos/faces mas não reconhecimento facial biométrico (diferente da SentinelX).</t>
+        </is>
+      </c>
+      <c r="I5" s="18" t="inlineStr">
+        <is>
+          <t>🔥 Deal — Smart Sampa</t>
+        </is>
+      </c>
+      <c r="J5" s="20" t="inlineStr">
+        <is>
+          <t>✓</t>
+        </is>
+      </c>
     </row>
     <row r="6" ht="48" customHeight="1">
       <c r="A6" s="14" t="inlineStr">
         <is>
-          <t>Atech</t>
+          <t>Sipremo</t>
         </is>
       </c>
       <c r="B6" s="15" t="inlineStr">
         <is>
-          <t>Comando &amp; Controle / Defesa e Segurança Pública</t>
+          <t>Previsão de Desastres / ClimateTech</t>
         </is>
       </c>
       <c r="C6" s="15" t="inlineStr">
         <is>
-          <t>Médio Porte</t>
+          <t>Startup</t>
         </is>
       </c>
       <c r="D6" s="15" t="inlineStr">
         <is>
-          <t>São Paulo - SP</t>
+          <t>Ribeirão Preto - SP</t>
         </is>
       </c>
       <c r="E6" s="15" t="inlineStr">
         <is>
-          <t>1999</t>
+          <t>~2018</t>
         </is>
       </c>
       <c r="F6" s="15" t="inlineStr">
         <is>
-          <t>Nacional / Defesa, ATM, Segurança</t>
+          <t>Defesa Civil + seguros</t>
         </is>
       </c>
       <c r="G6" s="15" t="inlineStr">
         <is>
-          <t>N/D</t>
+          <t>R$200k (2022)</t>
         </is>
       </c>
       <c r="H6" s="15" t="inlineStr">
         <is>
-          <t>Empresa do Grupo Embraer e Empresa Estratégica de Defesa (EED). Especialista em sistemas de missão crítica: Gerenciamento de Tráfego Aéreo (ATM), Comando &amp; Controle (C4I), Gestão de UTM (drones), Segurança Pública, Sistemas Navais, Cibersegurança e Sistemas Embarcados. Certificações ISO internacionais.</t>
-        </is>
-      </c>
-      <c r="I6" s="15" t="inlineStr"/>
+          <t>IA para previsão antecipada de desastres naturais com dados NASA e bases nacionais. Alerta SMS via Defesa Civil municipal. Selecionada COP26. Foco em mitigação de riscos climáticos e resiliência urbana.</t>
+        </is>
+      </c>
+      <c r="I6" s="16" t="inlineStr">
+        <is>
+          <t>Watch — clima/risco</t>
+        </is>
+      </c>
       <c r="J6" s="15" t="inlineStr"/>
     </row>
     <row r="7" ht="48" customHeight="1">
       <c r="A7" s="12" t="inlineStr">
         <is>
-          <t>Fractal</t>
+          <t>i4Sea</t>
         </is>
       </c>
       <c r="B7" s="13" t="inlineStr">
         <is>
-          <t>Previsão Hidroclimática / ClimateTech</t>
+          <t>Previsões Microclimáticas / Portos e Energia</t>
         </is>
       </c>
       <c r="C7" s="13" t="inlineStr">
         <is>
-          <t>Startup / Scale-up</t>
+          <t>Startup</t>
         </is>
       </c>
       <c r="D7" s="13" t="inlineStr">
         <is>
-          <t>Florianópolis - SC</t>
+          <t>Santos - SP</t>
         </is>
       </c>
       <c r="E7" s="13" t="inlineStr">
         <is>
-          <t>2010</t>
+          <t>~2018</t>
         </is>
       </c>
       <c r="F7" s="13" t="inlineStr">
         <is>
-          <t>Defesa Civil SC | usinas hidrelétricas | Clientes: CPFL, Statkraft</t>
+          <t>Portos, setor elétrico e renovável | Porto do Açu, Wilson Sons, Santos Brasil</t>
         </is>
       </c>
       <c r="G7" s="13" t="inlineStr">
         <is>
-          <t>N/D (KPTL 2019)</t>
+          <t>R$ 7,5M (Fundo GovTech)</t>
         </is>
       </c>
       <c r="H7" s="13" t="inlineStr">
         <is>
-          <t>ClimaTech com plataforma SPEHC (SaaS) para previsões hidroclimáticas: antecipação de enchentes, gestão de barragens e operação de usinas. Integra múltiplos modelos, radares e dados em tempo real. Referência nacional na Defesa Civil de SC. Escritório também em Bauru/SP. Portfólio KPTL 2019.</t>
+          <t>Plataforma i4cast® de decisão baseada em inteligência climática: previsões hiperlocais de mar e clima para operações portuárias, logística marítima e geração de energia renovável. Precisão 2x superior a previsões genéricas (94% acurácia no Porto do Açu). Captou R$7,5M do Fundo GovTech KPTL.</t>
         </is>
       </c>
       <c r="I7" s="18" t="inlineStr">
@@ -1542,32 +1562,32 @@
     <row r="8" ht="48" customHeight="1">
       <c r="A8" s="14" t="inlineStr">
         <is>
-          <t>Horus Smart Det.</t>
+          <t>IPQ Tecnologia</t>
         </is>
       </c>
       <c r="B8" s="15" t="inlineStr">
         <is>
-          <t>Monitoramento Aéreo / Fiscalização com IA</t>
+          <t>Segurança Pública / TIC para Ambientes Críticos</t>
         </is>
       </c>
       <c r="C8" s="15" t="inlineStr">
         <is>
-          <t>Scale-up</t>
+          <t>PME / Scale-up</t>
         </is>
       </c>
       <c r="D8" s="15" t="inlineStr">
         <is>
-          <t>Florianópolis - SC</t>
+          <t>Porto Alegre - RS</t>
         </is>
       </c>
       <c r="E8" s="15" t="inlineStr">
         <is>
-          <t>2014</t>
+          <t>~2001</t>
         </is>
       </c>
       <c r="F8" s="15" t="inlineStr">
         <is>
-          <t>100+ clientes gov e privado | Florianópolis (Monitora Floripa), telco, energia</t>
+          <t>Nacional e internacional | órgãos públicos, presídios, hospitais, rodovias</t>
         </is>
       </c>
       <c r="G8" s="15" t="inlineStr">
@@ -1577,7 +1597,7 @@
       </c>
       <c r="H8" s="15" t="inlineStr">
         <is>
-          <t>Plataforma de análise de imagens com IA para decisões inteligentes: sistema Monitora detecta obras irregulares e desmatamento via satélite + drones (identificação automática, 50% mais eficácia de fiscalização). Prêmio Connected Smart Cities 2021. Também atua em inspeção solar e telecom (Vivo, ENEL). CEO: Fabrício Hertz. Sede Parque Tecnológico ALFA Florianópolis.</t>
+          <t>25+ anos desenvolvendo e integrando soluções de TIC com IA e Analytics para segurança pública e ambientes críticos. Portfólio: videomonitoramento, controle de acesso, redes de dados públicas/privadas, infraestrutura para Defesa e Segurança. Atuação descentralizada com cobertura nacional.</t>
         </is>
       </c>
       <c r="I8" s="15" t="inlineStr"/>
@@ -1586,17 +1606,17 @@
     <row r="9" ht="48" customHeight="1">
       <c r="A9" s="12" t="inlineStr">
         <is>
-          <t>Intelicity</t>
+          <t>Atech</t>
         </is>
       </c>
       <c r="B9" s="13" t="inlineStr">
         <is>
-          <t>Gestão Urbana Preditiva / Pavimento e Zeladoria com IA</t>
+          <t>Comando &amp; Controle / Defesa e Segurança Pública</t>
         </is>
       </c>
       <c r="C9" s="13" t="inlineStr">
         <is>
-          <t>Startup / Scale-up</t>
+          <t>Médio Porte</t>
         </is>
       </c>
       <c r="D9" s="13" t="inlineStr">
@@ -1606,12 +1626,12 @@
       </c>
       <c r="E9" s="13" t="inlineStr">
         <is>
-          <t>~2019</t>
+          <t>1999</t>
         </is>
       </c>
       <c r="F9" s="13" t="inlineStr">
         <is>
-          <t>15M+ cidadãos | 8+ estados | São Paulo, Porto Alegre, Gravatá</t>
+          <t>Nacional / Defesa, ATM, Segurança</t>
         </is>
       </c>
       <c r="G9" s="13" t="inlineStr">
@@ -1621,11 +1641,147 @@
       </c>
       <c r="H9" s="13" t="inlineStr">
         <is>
-          <t>Plataforma de gestão urbana inteligente com visão computacional embarcada em veículos: mapeia qualidade de pavimento, iluminação, encostas e ativos urbanos georreferenciados. Sistema Gaia (SP) apoia programa de recape. Dashboard preditivo com Machine Learning. Também gerencia zeladoria (OS) e intervenções de concessionárias. Integra portal do cidadão. 40+ tipos de ativos monitorados.</t>
+          <t>Empresa do Grupo Embraer e Empresa Estratégica de Defesa (EED). Especialista em sistemas de missão crítica: Gerenciamento de Tráfego Aéreo (ATM), Comando &amp; Controle (C4I), Gestão de UTM (drones), Segurança Pública, Sistemas Navais, Cibersegurança e Sistemas Embarcados. Certificações ISO internacionais.</t>
         </is>
       </c>
       <c r="I9" s="13" t="inlineStr"/>
       <c r="J9" s="13" t="inlineStr"/>
+    </row>
+    <row r="10" ht="48" customHeight="1">
+      <c r="A10" s="14" t="inlineStr">
+        <is>
+          <t>Fractal</t>
+        </is>
+      </c>
+      <c r="B10" s="15" t="inlineStr">
+        <is>
+          <t>Previsão Hidroclimática / ClimateTech</t>
+        </is>
+      </c>
+      <c r="C10" s="15" t="inlineStr">
+        <is>
+          <t>Startup / Scale-up</t>
+        </is>
+      </c>
+      <c r="D10" s="15" t="inlineStr">
+        <is>
+          <t>Florianópolis - SC</t>
+        </is>
+      </c>
+      <c r="E10" s="15" t="inlineStr">
+        <is>
+          <t>2010</t>
+        </is>
+      </c>
+      <c r="F10" s="15" t="inlineStr">
+        <is>
+          <t>Defesa Civil SC | usinas hidrelétricas | Clientes: CPFL, Statkraft</t>
+        </is>
+      </c>
+      <c r="G10" s="15" t="inlineStr">
+        <is>
+          <t>N/D (KPTL 2019)</t>
+        </is>
+      </c>
+      <c r="H10" s="15" t="inlineStr">
+        <is>
+          <t>ClimaTech com plataforma SPEHC (SaaS) para previsões hidroclimáticas: antecipação de enchentes, gestão de barragens e operação de usinas. Integra múltiplos modelos, radares e dados em tempo real. Referência nacional na Defesa Civil de SC. Escritório também em Bauru/SP. Portfólio KPTL 2019.</t>
+        </is>
+      </c>
+      <c r="I10" s="16" t="inlineStr">
+        <is>
+          <t>Portfólio KPTL</t>
+        </is>
+      </c>
+      <c r="J10" s="15" t="inlineStr"/>
+    </row>
+    <row r="11" ht="48" customHeight="1">
+      <c r="A11" s="12" t="inlineStr">
+        <is>
+          <t>Horus Smart Det.</t>
+        </is>
+      </c>
+      <c r="B11" s="13" t="inlineStr">
+        <is>
+          <t>Monitoramento Aéreo / Fiscalização com IA</t>
+        </is>
+      </c>
+      <c r="C11" s="13" t="inlineStr">
+        <is>
+          <t>Scale-up</t>
+        </is>
+      </c>
+      <c r="D11" s="13" t="inlineStr">
+        <is>
+          <t>Florianópolis - SC</t>
+        </is>
+      </c>
+      <c r="E11" s="13" t="inlineStr">
+        <is>
+          <t>2014</t>
+        </is>
+      </c>
+      <c r="F11" s="13" t="inlineStr">
+        <is>
+          <t>100+ clientes gov e privado | Florianópolis (Monitora Floripa), telco, energia</t>
+        </is>
+      </c>
+      <c r="G11" s="13" t="inlineStr">
+        <is>
+          <t>N/D</t>
+        </is>
+      </c>
+      <c r="H11" s="13" t="inlineStr">
+        <is>
+          <t>Plataforma de análise de imagens com IA para decisões inteligentes: sistema Monitora detecta obras irregulares e desmatamento via satélite + drones (identificação automática, 50% mais eficácia de fiscalização). Prêmio Connected Smart Cities 2021. Também atua em inspeção solar e telecom (Vivo, ENEL). CEO: Fabrício Hertz. Sede Parque Tecnológico ALFA Florianópolis.</t>
+        </is>
+      </c>
+      <c r="I11" s="13" t="inlineStr"/>
+      <c r="J11" s="13" t="inlineStr"/>
+    </row>
+    <row r="12" ht="48" customHeight="1">
+      <c r="A12" s="14" t="inlineStr">
+        <is>
+          <t>Intelicity</t>
+        </is>
+      </c>
+      <c r="B12" s="15" t="inlineStr">
+        <is>
+          <t>Gestão Urbana Preditiva / Pavimento e Zeladoria com IA</t>
+        </is>
+      </c>
+      <c r="C12" s="15" t="inlineStr">
+        <is>
+          <t>Startup / Scale-up</t>
+        </is>
+      </c>
+      <c r="D12" s="15" t="inlineStr">
+        <is>
+          <t>São Paulo - SP</t>
+        </is>
+      </c>
+      <c r="E12" s="15" t="inlineStr">
+        <is>
+          <t>~2019</t>
+        </is>
+      </c>
+      <c r="F12" s="15" t="inlineStr">
+        <is>
+          <t>15M+ cidadãos | 8+ estados | São Paulo, Porto Alegre, Gravatá</t>
+        </is>
+      </c>
+      <c r="G12" s="15" t="inlineStr">
+        <is>
+          <t>N/D</t>
+        </is>
+      </c>
+      <c r="H12" s="15" t="inlineStr">
+        <is>
+          <t>Plataforma de gestão urbana inteligente com visão computacional embarcada em veículos: mapeia qualidade de pavimento, iluminação, encostas e ativos urbanos georreferenciados. Sistema Gaia (SP) apoia programa de recape. Dashboard preditivo com Machine Learning. Também gerencia zeladoria (OS) e intervenções de concessionárias. Integra portal do cidadão. 40+ tipos de ativos monitorados.</t>
+        </is>
+      </c>
+      <c r="I12" s="15" t="inlineStr"/>
+      <c r="J12" s="15" t="inlineStr"/>
     </row>
   </sheetData>
   <mergeCells count="1">
@@ -1641,7 +1797,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:F18"/>
+  <dimension ref="A1:F19"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="32" customWidth="1" min="1" max="1"/>
@@ -2110,94 +2266,126 @@
     <row r="16" ht="48" customHeight="1">
       <c r="A16" s="32" t="inlineStr">
         <is>
-          <t>MITRA — Valid (51%)</t>
+          <t>Layers — fundo canadense (pré-série A)</t>
         </is>
       </c>
       <c r="B16" s="33" t="inlineStr">
         <is>
-          <t>Aquisição (M&amp;A)</t>
+          <t>Aporte Pré-Série A</t>
         </is>
       </c>
       <c r="C16" s="33" t="inlineStr">
         <is>
-          <t>N/D</t>
+          <t>R$ 21M</t>
         </is>
       </c>
       <c r="D16" s="33" t="inlineStr">
         <is>
-          <t>2025</t>
+          <t>set/2025</t>
         </is>
       </c>
       <c r="E16" s="33" t="inlineStr">
         <is>
-          <t>Gestão Municipal Integrada</t>
+          <t>Educação Pública / EdTech</t>
         </is>
       </c>
       <c r="F16" s="33" t="inlineStr">
         <is>
-          <t>Valid adquire 51% da MITRA, plataforma de gestão municipal integrada com proposta 'Governo Único para um Cidadão Único'. Cidades atendidas: São Caetano do Sul SP, Santo André SP, Vinhedo SP, Araraquara SP, Campos dos Goytacazes RJ. 1,7M+ cidadãos impactados.</t>
+          <t>SuperApp escolar capta R$21M em pré-série A liderado por fundo canadense. Valuation R$120M. 7.600 escolas públicas (gratuito) + 1.800 privadas. R$1Bi+ transacionado. CEO Danilo Yoneshige. São Caetano do Sul SP.</t>
         </is>
       </c>
     </row>
     <row r="17" ht="48" customHeight="1">
       <c r="A17" s="12" t="inlineStr">
         <is>
-          <t>Kinebot — Fundo GovTech (KPTL+Cedro)</t>
+          <t>MITRA — Valid (51%)</t>
         </is>
       </c>
       <c r="B17" s="13" t="inlineStr">
         <is>
-          <t>Aporte</t>
+          <t>Aquisição (M&amp;A)</t>
         </is>
       </c>
       <c r="C17" s="13" t="inlineStr">
         <is>
-          <t>R$ 3M</t>
+          <t>N/D</t>
         </is>
       </c>
       <c r="D17" s="13" t="inlineStr">
         <is>
-          <t>fev/2026</t>
+          <t>2025</t>
         </is>
       </c>
       <c r="E17" s="13" t="inlineStr">
         <is>
-          <t>IA Ergonomia / Saúde Gov</t>
+          <t>Gestão Municipal Integrada</t>
         </is>
       </c>
       <c r="F17" s="13" t="inlineStr">
         <is>
-          <t>8º investimento do Fundo GovTech. IA para análises ergonômicas e psicossociais. Clientes: Marfrig, P&amp;G, Electrolux. Expansão global planejada para 2026.</t>
+          <t>Valid adquire 51% da MITRA, plataforma de gestão municipal integrada com proposta 'Governo Único para um Cidadão Único'. Cidades atendidas: São Caetano do Sul SP, Santo André SP, Vinhedo SP, Araraquara SP, Campos dos Goytacazes RJ. 1,7M+ cidadãos impactados.</t>
         </is>
       </c>
     </row>
     <row r="18" ht="48" customHeight="1">
       <c r="A18" s="32" t="inlineStr">
         <is>
+          <t>Kinebot — Fundo GovTech (KPTL+Cedro)</t>
+        </is>
+      </c>
+      <c r="B18" s="33" t="inlineStr">
+        <is>
+          <t>Aporte</t>
+        </is>
+      </c>
+      <c r="C18" s="33" t="inlineStr">
+        <is>
+          <t>R$ 3M</t>
+        </is>
+      </c>
+      <c r="D18" s="33" t="inlineStr">
+        <is>
+          <t>fev/2026</t>
+        </is>
+      </c>
+      <c r="E18" s="33" t="inlineStr">
+        <is>
+          <t>IA Ergonomia / Saúde Gov</t>
+        </is>
+      </c>
+      <c r="F18" s="33" t="inlineStr">
+        <is>
+          <t>8º investimento do Fundo GovTech. IA para análises ergonômicas e psicossociais. Clientes: Marfrig, P&amp;G, Electrolux. Expansão global planejada para 2026.</t>
+        </is>
+      </c>
+    </row>
+    <row r="19" ht="48" customHeight="1">
+      <c r="A19" s="12" t="inlineStr">
+        <is>
           <t>Jovens Gênios — Fundo GovTech+DOMO</t>
         </is>
       </c>
-      <c r="B18" s="33" t="inlineStr">
+      <c r="B19" s="13" t="inlineStr">
         <is>
           <t>Aporte Seed</t>
         </is>
       </c>
-      <c r="C18" s="33" t="inlineStr">
+      <c r="C19" s="13" t="inlineStr">
         <is>
           <t>R$ 11,8M</t>
         </is>
       </c>
-      <c r="D18" s="33" t="inlineStr">
+      <c r="D19" s="13" t="inlineStr">
         <is>
           <t>mar/2026</t>
         </is>
       </c>
-      <c r="E18" s="33" t="inlineStr">
+      <c r="E19" s="13" t="inlineStr">
         <is>
           <t>Educação Pública</t>
         </is>
       </c>
-      <c r="F18" s="33" t="inlineStr">
+      <c r="F19" s="13" t="inlineStr">
         <is>
           <t>Rodada seed liderada pelo Fundo GovTech (KPTL+Cedro), com DOMO.VC, Criabiz Ventures e Rosey Ventures (Grupo Marista). 90% dos alunos em escolas públicas. Meta: 10M alunos até 2030.</t>
         </is>
@@ -2921,7 +3109,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:J9"/>
+  <dimension ref="A1:J10"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="28" customWidth="1" min="1" max="1"/>
@@ -2998,32 +3186,32 @@
     <row r="3" ht="48" customHeight="1">
       <c r="A3" s="12" t="inlineStr">
         <is>
-          <t>LICI GovTech</t>
+          <t>Munitax</t>
         </is>
       </c>
       <c r="B3" s="13" t="inlineStr">
         <is>
-          <t>Governança Municipal Baseada em Dados / ODS</t>
+          <t>Inteligência Tributária Municipal Completa</t>
         </is>
       </c>
       <c r="C3" s="13" t="inlineStr">
         <is>
-          <t>Startup</t>
+          <t>Startup / Scale-up</t>
         </is>
       </c>
       <c r="D3" s="13" t="inlineStr">
         <is>
-          <t>Belo Horizonte - MG</t>
+          <t>Brasil</t>
         </is>
       </c>
       <c r="E3" s="13" t="inlineStr">
         <is>
-          <t>2018</t>
+          <t>N/D</t>
         </is>
       </c>
       <c r="F3" s="13" t="inlineStr">
         <is>
-          <t>1.000+ gestores formados | SEDE-MG, FINEP, PNUD, UNESCO, ALMG</t>
+          <t>Municípios de qualquer porte | cobertura IPTU, ISS, ITBI, dívida ativa</t>
         </is>
       </c>
       <c r="G3" s="13" t="inlineStr">
@@ -3033,21 +3221,29 @@
       </c>
       <c r="H3" s="13" t="inlineStr">
         <is>
-          <t>GovTech de governança orientada a dados com metodologia CHESI (registrada no INPI): 160+ indicadores ODS monitorados em tempo real, conectando projetos a financiamento público. Produz Relatórios Locais Voluntários para Agenda 2030. Coordena GT Cidades Inteligentes da ALMG.</t>
-        </is>
-      </c>
-      <c r="I3" s="13" t="inlineStr"/>
-      <c r="J3" s="13" t="inlineStr"/>
+          <t>Plataforma completa de inteligência tributária para municípios: IPTU, ISS, ITBI, dívida ativa, notificações automatizadas e processos administrativos fiscais end-to-end. Cruzamento automático com bases da Receita Federal e juntas comerciais para enriquecimento cadastral e detecção de inconsistências tributárias. MuniAcademy: maior plataforma de capacitação em tributação municipal do Brasil com 320+ publicações e 140h de conteúdo. CEO: Harrison Leite (doutor em Direito Tributário, autor de 30+ livros). Combinação rara de tecnologia + doutrina jurídica tributária.</t>
+        </is>
+      </c>
+      <c r="I3" s="18" t="inlineStr">
+        <is>
+          <t>Watch — fiscal municipal</t>
+        </is>
+      </c>
+      <c r="J3" s="20" t="inlineStr">
+        <is>
+          <t>✓</t>
+        </is>
+      </c>
     </row>
     <row r="4" ht="48" customHeight="1">
       <c r="A4" s="14" t="inlineStr">
         <is>
-          <t>Quasar</t>
+          <t>LICI GovTech</t>
         </is>
       </c>
       <c r="B4" s="15" t="inlineStr">
         <is>
-          <t>Alvará Digital e Licenciamento de Empresas Municipal</t>
+          <t>Governança Municipal Baseada em Dados / ODS</t>
         </is>
       </c>
       <c r="C4" s="15" t="inlineStr">
@@ -3062,12 +3258,12 @@
       </c>
       <c r="E4" s="15" t="inlineStr">
         <is>
-          <t>2019</t>
+          <t>2018</t>
         </is>
       </c>
       <c r="F4" s="15" t="inlineStr">
         <is>
-          <t>MG, RO, PE, MT | 480+ municípios via Jucemg/SINAL</t>
+          <t>1.000+ gestores formados | SEDE-MG, FINEP, PNUD, UNESCO, ALMG</t>
         </is>
       </c>
       <c r="G4" s="15" t="inlineStr">
@@ -3077,25 +3273,21 @@
       </c>
       <c r="H4" s="15" t="inlineStr">
         <is>
-          <t>Sistema de gestão de licenciamento e abertura de empresas, com alvarás digitais via QR Code e integração REDESIM. Parceiro estadual da Jucemg para o sistema SINAL (480+ municípios de MG). Apoio Seed-MG e AWS. Reduz prazo de emissão de alvarás em 90%. BrazilLAB 2023.</t>
-        </is>
-      </c>
-      <c r="I4" s="16" t="inlineStr">
-        <is>
-          <t>Watch — expansão estadual Jucemg</t>
-        </is>
-      </c>
+          <t>GovTech de governança orientada a dados com metodologia CHESI (registrada no INPI): 160+ indicadores ODS monitorados em tempo real, conectando projetos a financiamento público. Produz Relatórios Locais Voluntários para Agenda 2030. Coordena GT Cidades Inteligentes da ALMG.</t>
+        </is>
+      </c>
+      <c r="I4" s="15" t="inlineStr"/>
       <c r="J4" s="15" t="inlineStr"/>
     </row>
     <row r="5" ht="48" customHeight="1">
       <c r="A5" s="12" t="inlineStr">
         <is>
-          <t>Qiatech</t>
+          <t>Quasar</t>
         </is>
       </c>
       <c r="B5" s="13" t="inlineStr">
         <is>
-          <t>Gestão de Convênios e Transferências Federais com IA</t>
+          <t>Alvará Digital e Licenciamento de Empresas Municipal</t>
         </is>
       </c>
       <c r="C5" s="13" t="inlineStr">
@@ -3105,17 +3297,17 @@
       </c>
       <c r="D5" s="13" t="inlineStr">
         <is>
-          <t>Brasil</t>
+          <t>Belo Horizonte - MG</t>
         </is>
       </c>
       <c r="E5" s="13" t="inlineStr">
         <is>
-          <t>N/D</t>
+          <t>2019</t>
         </is>
       </c>
       <c r="F5" s="13" t="inlineStr">
         <is>
-          <t>Municípios de qualquer porte | integra TransfereGov, Simec, Sismob, FNS, Sigcon</t>
+          <t>MG, RO, PE, MT | 480+ municípios via Jucemg/SINAL</t>
         </is>
       </c>
       <c r="G5" s="13" t="inlineStr">
@@ -3125,12 +3317,12 @@
       </c>
       <c r="H5" s="13" t="inlineStr">
         <is>
-          <t>Primeiro sistema inteligente de gestão de convênios para prefeituras: unifica automaticamente TransfereGov, Simec, Sismob, FNS e Sigcon em painel único com IA. Kanban automático de diligências, alertas de prazo, monitoramento de certidões, previsão de repasses e elaboração de propostas com IA baseadas em cotações federais. Diferencial: deixa a IA captar e monitorar enquanto a prefeitura foca na execução.</t>
+          <t>Sistema de gestão de licenciamento e abertura de empresas, com alvarás digitais via QR Code e integração REDESIM. Parceiro estadual da Jucemg para o sistema SINAL (480+ municípios de MG). Apoio Seed-MG e AWS. Reduz prazo de emissão de alvarás em 90%. BrazilLAB 2023.</t>
         </is>
       </c>
       <c r="I5" s="18" t="inlineStr">
         <is>
-          <t>Watch — convênios nicho virgem</t>
+          <t>Watch — expansão estadual Jucemg</t>
         </is>
       </c>
       <c r="J5" s="13" t="inlineStr"/>
@@ -3138,12 +3330,12 @@
     <row r="6" ht="48" customHeight="1">
       <c r="A6" s="14" t="inlineStr">
         <is>
-          <t>MuniScore</t>
+          <t>Qiatech</t>
         </is>
       </c>
       <c r="B6" s="15" t="inlineStr">
         <is>
-          <t>Score Fiscal e Inteligência de Risco Municipal</t>
+          <t>Gestão de Convênios e Transferências Federais com IA</t>
         </is>
       </c>
       <c r="C6" s="15" t="inlineStr">
@@ -3153,17 +3345,17 @@
       </c>
       <c r="D6" s="15" t="inlineStr">
         <is>
-          <t>Belo Horizonte - MG</t>
+          <t>Brasil</t>
         </is>
       </c>
       <c r="E6" s="15" t="inlineStr">
         <is>
-          <t>2026</t>
+          <t>N/D</t>
         </is>
       </c>
       <c r="F6" s="15" t="inlineStr">
         <is>
-          <t>100% dos 5.570 municípios brasileiros (dados) | B2B: fornecedores, bancos, seguradoras</t>
+          <t>Municípios de qualquer porte | integra TransfereGov, Simec, Sismob, FNS, Sigcon</t>
         </is>
       </c>
       <c r="G6" s="15" t="inlineStr">
@@ -3173,12 +3365,12 @@
       </c>
       <c r="H6" s="15" t="inlineStr">
         <is>
-          <t>Plataforma SaaS de score fiscal para municípios: nota de 0 a 1000 cruzando receita, despesa, endividamento e CAPAG (STN). Integra PNCP, TransfereGov, emendas parlamentares e PCA para identificar oportunidades de fornecimento. Assistente de IA com 4 perspectivas analíticas. Fundadores: Diego Barros (CEO) e Antonio Firmino (Chairman / Grupo Triasa). Planos a partir de R$97/mês.</t>
+          <t>Primeiro sistema inteligente de gestão de convênios para prefeituras: unifica automaticamente TransfereGov, Simec, Sismob, FNS e Sigcon em painel único com IA. Kanban automático de diligências, alertas de prazo, monitoramento de certidões, previsão de repasses e elaboração de propostas com IA baseadas em cotações federais. Diferencial: deixa a IA captar e monitorar enquanto a prefeitura foca na execução.</t>
         </is>
       </c>
       <c r="I6" s="16" t="inlineStr">
         <is>
-          <t>Watch — dado fiscal municipal</t>
+          <t>Watch — convênios nicho virgem</t>
         </is>
       </c>
       <c r="J6" s="15" t="inlineStr"/>
@@ -3186,32 +3378,32 @@
     <row r="7" ht="48" customHeight="1">
       <c r="A7" s="12" t="inlineStr">
         <is>
-          <t>Geopixel</t>
+          <t>MuniScore</t>
         </is>
       </c>
       <c r="B7" s="13" t="inlineStr">
         <is>
-          <t>GeoInteligência Fiscal / Cadastro Imobiliário</t>
+          <t>Score Fiscal e Inteligência de Risco Municipal</t>
         </is>
       </c>
       <c r="C7" s="13" t="inlineStr">
         <is>
-          <t>PME</t>
+          <t>Startup</t>
         </is>
       </c>
       <c r="D7" s="13" t="inlineStr">
         <is>
-          <t>São José dos Campos - SP</t>
+          <t>Belo Horizonte - MG</t>
         </is>
       </c>
       <c r="E7" s="13" t="inlineStr">
         <is>
-          <t>~2008</t>
+          <t>2026</t>
         </is>
       </c>
       <c r="F7" s="13" t="inlineStr">
         <is>
-          <t>100+ municípios | clientes: Amparo SP, Teresópolis RJ, Guaratinguetá SP</t>
+          <t>100% dos 5.570 municípios brasileiros (dados) | B2B: fornecedores, bancos, seguradoras</t>
         </is>
       </c>
       <c r="G7" s="13" t="inlineStr">
@@ -3221,12 +3413,12 @@
       </c>
       <c r="H7" s="13" t="inlineStr">
         <is>
-          <t>18 anos como líder em geointeligência para prefeituras. Plataforma Geopixel Cidades integra geoprocessamento com IA para IPTU, ITBI, ISS e alvarás (digital e por QR Code). Módulos: SIG municipal integrado, monitoramento por satélite de alterações, mobilidade de campo e eventos ambientais. Reforma Tributária (LC 214/2025) cria janela de demanda direta e imediata.</t>
+          <t>Plataforma SaaS de score fiscal para municípios: nota de 0 a 1000 cruzando receita, despesa, endividamento e CAPAG (STN). Integra PNCP, TransfereGov, emendas parlamentares e PCA para identificar oportunidades de fornecimento. Assistente de IA com 4 perspectivas analíticas. Fundadores: Diego Barros (CEO) e Antonio Firmino (Chairman / Grupo Triasa). Planos a partir de R$97/mês.</t>
         </is>
       </c>
       <c r="I7" s="18" t="inlineStr">
         <is>
-          <t>Oportunidade fiscal 2025</t>
+          <t>Watch — dado fiscal municipal</t>
         </is>
       </c>
       <c r="J7" s="13" t="inlineStr"/>
@@ -3234,47 +3426,47 @@
     <row r="8" ht="48" customHeight="1">
       <c r="A8" s="14" t="inlineStr">
         <is>
-          <t>Gove</t>
+          <t>Geopixel</t>
         </is>
       </c>
       <c r="B8" s="15" t="inlineStr">
         <is>
-          <t>CRM Municipal / Cobrança &amp; Automação via IA</t>
+          <t>GeoInteligência Fiscal / Cadastro Imobiliário</t>
         </is>
       </c>
       <c r="C8" s="15" t="inlineStr">
         <is>
-          <t>Startup / Scale-up</t>
+          <t>PME</t>
         </is>
       </c>
       <c r="D8" s="15" t="inlineStr">
         <is>
-          <t>São Paulo - SP</t>
+          <t>São José dos Campos - SP</t>
         </is>
       </c>
       <c r="E8" s="15" t="inlineStr">
         <is>
-          <t>2018</t>
+          <t>~2008</t>
         </is>
       </c>
       <c r="F8" s="15" t="inlineStr">
         <is>
-          <t>SP, MG, AM, BA, RJ, TO+</t>
+          <t>100+ municípios | clientes: Amparo SP, Teresópolis RJ, Guaratinguetá SP</t>
         </is>
       </c>
       <c r="G8" s="15" t="inlineStr">
         <is>
-          <t>R$ 8M (Astella)</t>
+          <t>N/D</t>
         </is>
       </c>
       <c r="H8" s="15" t="inlineStr">
         <is>
-          <t>Único CRM para setor público com chatbot WhatsApp verificado (login Gov.br), automação de serviços via IA e enriquecimento cadastral contínuo. Foco em arrecadação: cobrança ativa por WhatsApp/SMS/email/Domicílio Eletrônico, cruzamento com Receita Federal. CEO: Rodolfo Fiori (MIT). CTO: Dayanne Ramos. Cases: Salvador BA (R$29M recuperação crédito tributário), Araguaína TO (ROI 32x — R$300k→R$9,6M, 1º CPSI do país), Areal RJ (+135% arrecadação dívida ativa), Manaus AM, Pindamonhangaba SP. Prêmio InovaCidade 2023. Aporte Astella Series A (R$8M, 2020). BrazilLAB Turma 7.</t>
+          <t>18 anos como líder em geointeligência para prefeituras. Plataforma Geopixel Cidades integra geoprocessamento com IA para IPTU, ITBI, ISS e alvarás (digital e por QR Code). Módulos: SIG municipal integrado, monitoramento por satélite de alterações, mobilidade de campo e eventos ambientais. Reforma Tributária (LC 214/2025) cria janela de demanda direta e imediata.</t>
         </is>
       </c>
       <c r="I8" s="16" t="inlineStr">
         <is>
-          <t>M&amp;A Watch — tração comprovada</t>
+          <t>Oportunidade fiscal 2025</t>
         </is>
       </c>
       <c r="J8" s="15" t="inlineStr"/>
@@ -3282,50 +3474,98 @@
     <row r="9" ht="48" customHeight="1">
       <c r="A9" s="12" t="inlineStr">
         <is>
+          <t>Gove</t>
+        </is>
+      </c>
+      <c r="B9" s="13" t="inlineStr">
+        <is>
+          <t>CRM Municipal / Cobrança &amp; Automação via IA</t>
+        </is>
+      </c>
+      <c r="C9" s="13" t="inlineStr">
+        <is>
+          <t>Startup / Scale-up</t>
+        </is>
+      </c>
+      <c r="D9" s="13" t="inlineStr">
+        <is>
+          <t>São Paulo - SP</t>
+        </is>
+      </c>
+      <c r="E9" s="13" t="inlineStr">
+        <is>
+          <t>2018</t>
+        </is>
+      </c>
+      <c r="F9" s="13" t="inlineStr">
+        <is>
+          <t>SP, MG, AM, BA, RJ, TO+</t>
+        </is>
+      </c>
+      <c r="G9" s="13" t="inlineStr">
+        <is>
+          <t>R$ 8M (Astella)</t>
+        </is>
+      </c>
+      <c r="H9" s="13" t="inlineStr">
+        <is>
+          <t>Único CRM para setor público com chatbot WhatsApp verificado (login Gov.br), automação de serviços via IA e enriquecimento cadastral contínuo. Foco em arrecadação: cobrança ativa por WhatsApp/SMS/email/Domicílio Eletrônico, cruzamento com Receita Federal. CEO: Rodolfo Fiori (MIT). CTO: Dayanne Ramos. Cases: Salvador BA (R$29M recuperação crédito tributário), Araguaína TO (ROI 32x — R$300k→R$9,6M, 1º CPSI do país), Areal RJ (+135% arrecadação dívida ativa), Manaus AM, Pindamonhangaba SP. Prêmio InovaCidade 2023. Aporte Astella Series A (R$8M, 2020). BrazilLAB Turma 7.</t>
+        </is>
+      </c>
+      <c r="I9" s="18" t="inlineStr">
+        <is>
+          <t>M&amp;A Watch — tração comprovada</t>
+        </is>
+      </c>
+      <c r="J9" s="13" t="inlineStr"/>
+    </row>
+    <row r="10" ht="48" customHeight="1">
+      <c r="A10" s="14" t="inlineStr">
+        <is>
           <t>Hub Esfera</t>
         </is>
       </c>
-      <c r="B9" s="13" t="inlineStr">
+      <c r="B10" s="15" t="inlineStr">
         <is>
           <t>IA 3P para Gestão Municipal / Dashboard Analítico</t>
         </is>
       </c>
-      <c r="C9" s="13" t="inlineStr">
+      <c r="C10" s="15" t="inlineStr">
         <is>
           <t>Startup</t>
         </is>
       </c>
-      <c r="D9" s="13" t="inlineStr">
+      <c r="D10" s="15" t="inlineStr">
         <is>
           <t>Porto Alegre - RS</t>
         </is>
       </c>
-      <c r="E9" s="13" t="inlineStr">
-        <is>
-          <t>N/D</t>
-        </is>
-      </c>
-      <c r="F9" s="13" t="inlineStr">
+      <c r="E10" s="15" t="inlineStr">
+        <is>
+          <t>N/D</t>
+        </is>
+      </c>
+      <c r="F10" s="15" t="inlineStr">
         <is>
           <t>50+ municípios | 8 áreas da gestão pública</t>
         </is>
       </c>
-      <c r="G9" s="13" t="inlineStr">
-        <is>
-          <t>N/D</t>
-        </is>
-      </c>
-      <c r="H9" s="13" t="inlineStr">
+      <c r="G10" s="15" t="inlineStr">
+        <is>
+          <t>N/D</t>
+        </is>
+      </c>
+      <c r="H10" s="15" t="inlineStr">
         <is>
           <t>Plataforma de IA para gestão pública com metodologia exclusiva 3P: Preditiva (projeta receitas, saúde e matrículas), Preventiva (alertas automáticos de anomalias e contratos) e Prescritiva (sugere onde cortar custos, otimizar frota e compras). Dashboards interativos para todas as secretarias. Chat inteligente para consultas sobre dados oficiais da cidade. Marketplace de soluções parceiras integradas nativamente.</t>
         </is>
       </c>
-      <c r="I9" s="18" t="inlineStr">
+      <c r="I10" s="16" t="inlineStr">
         <is>
           <t>Watch</t>
         </is>
       </c>
-      <c r="J9" s="13" t="inlineStr"/>
+      <c r="J10" s="15" t="inlineStr"/>
     </row>
   </sheetData>
   <mergeCells count="1">
@@ -3357,7 +3597,7 @@
   </cols>
   <sheetData>
     <row r="1" ht="28" customHeight="1">
-      <c r="A1" s="20" t="inlineStr">
+      <c r="A1" s="21" t="inlineStr">
         <is>
           <t>🏥 Saúde Pública — Radar GovTech Brasil 2025/2026</t>
         </is>
@@ -3753,7 +3993,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:J11"/>
+  <dimension ref="A1:J13"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="28" customWidth="1" min="1" max="1"/>
@@ -3769,7 +4009,7 @@
   </cols>
   <sheetData>
     <row r="1" ht="28" customHeight="1">
-      <c r="A1" s="21" t="inlineStr">
+      <c r="A1" s="22" t="inlineStr">
         <is>
           <t>📚 Educação Pública — Radar GovTech Brasil 2025/2026</t>
         </is>
@@ -4194,50 +4434,154 @@
     <row r="11" ht="48" customHeight="1">
       <c r="A11" s="12" t="inlineStr">
         <is>
+          <t>Leme</t>
+        </is>
+      </c>
+      <c r="B11" s="13" t="inlineStr">
+        <is>
+          <t>Gestão Educacional Orientada por Dados / VAAR para Secretarias</t>
+        </is>
+      </c>
+      <c r="C11" s="13" t="inlineStr">
+        <is>
+          <t>Startup</t>
+        </is>
+      </c>
+      <c r="D11" s="13" t="inlineStr">
+        <is>
+          <t>Brasil</t>
+        </is>
+      </c>
+      <c r="E11" s="13" t="inlineStr">
+        <is>
+          <t>N/D</t>
+        </is>
+      </c>
+      <c r="F11" s="13" t="inlineStr">
+        <is>
+          <t>15+ municípios | 100K+ alunos | Mogi das Cruzes SP | São Vicente SP | Teresópolis RJ | Propriá SE</t>
+        </is>
+      </c>
+      <c r="G11" s="13" t="inlineStr">
+        <is>
+          <t>N/D</t>
+        </is>
+      </c>
+      <c r="H11" s="13" t="inlineStr">
+        <is>
+          <t>Plataforma de gestão educacional orientada por dados com metodologia MAPA (4 fases) e indicador VAAR (Valor Agregado com Ajuste de Risco). Foco em equidade racial e inclusão de alunos PPIs (Pretos, Pardos e Indígenas). +26% de desempenho médio em apenas 4 meses de implementação. 15+ municípios atendidos, 100K+ alunos impactados. Clientes de referência: Mogi das Cruzes SP, São Vicente SP, Teresópolis RJ, Propriá SE. Dispensa de licitação disponível para contratação simplificada.</t>
+        </is>
+      </c>
+      <c r="I11" s="18" t="inlineStr">
+        <is>
+          <t>Watch — municipal</t>
+        </is>
+      </c>
+      <c r="J11" s="20" t="inlineStr">
+        <is>
+          <t>✓</t>
+        </is>
+      </c>
+    </row>
+    <row r="12" ht="48" customHeight="1">
+      <c r="A12" s="14" t="inlineStr">
+        <is>
+          <t>Layers</t>
+        </is>
+      </c>
+      <c r="B12" s="15" t="inlineStr">
+        <is>
+          <t>SuperApp Escolar / Plataforma Educacional Unificada</t>
+        </is>
+      </c>
+      <c r="C12" s="15" t="inlineStr">
+        <is>
+          <t>Scale-up</t>
+        </is>
+      </c>
+      <c r="D12" s="15" t="inlineStr">
+        <is>
+          <t>São Caetano do Sul - SP</t>
+        </is>
+      </c>
+      <c r="E12" s="15" t="inlineStr">
+        <is>
+          <t>N/D</t>
+        </is>
+      </c>
+      <c r="F12" s="15" t="inlineStr">
+        <is>
+          <t>7.600 escolas públicas (gratuito) | 1.800 escolas privadas | R$1Bi+ transacionado | 20+ ERPs integrados | 50+ soluções edtech parceiras</t>
+        </is>
+      </c>
+      <c r="G12" s="15" t="inlineStr">
+        <is>
+          <t>R$21M (pré-série A, set/2025) | valuation R$120M</t>
+        </is>
+      </c>
+      <c r="H12" s="15" t="inlineStr">
+        <is>
+          <t>SuperApp escolar que unifica comunicação, gestão e pagamentos em uma só plataforma. Para escolas públicas: totalmente gratuito (7.600 escolas). Para privadas: modelo SaaS premium (1.800 escolas). Ecossistema robusto: integra 20+ ERPs e 50+ soluções edtech parceiras. R$1Bi+ transacionado na plataforma. Aporte pré-série A de R$21M liderado por fundo canadense (set/2025), valuation R$120M. CEO: Danilo Yoneshige. Sede São Caetano do Sul SP. Diferencial: cobertura do setor público + privado com uma única plataforma.</t>
+        </is>
+      </c>
+      <c r="I12" s="16" t="inlineStr">
+        <is>
+          <t>🔥 Deal — aporte recente</t>
+        </is>
+      </c>
+      <c r="J12" s="17" t="inlineStr">
+        <is>
+          <t>✓</t>
+        </is>
+      </c>
+    </row>
+    <row r="13" ht="48" customHeight="1">
+      <c r="A13" s="12" t="inlineStr">
+        <is>
           <t>Proesc</t>
         </is>
       </c>
-      <c r="B11" s="13" t="inlineStr">
+      <c r="B13" s="13" t="inlineStr">
         <is>
           <t>Gestão Escolar com IA + Vertical Pública (Proesc Gov)</t>
         </is>
       </c>
-      <c r="C11" s="13" t="inlineStr">
+      <c r="C13" s="13" t="inlineStr">
         <is>
           <t>Scale-up</t>
         </is>
       </c>
-      <c r="D11" s="13" t="inlineStr">
+      <c r="D13" s="13" t="inlineStr">
         <is>
           <t>Macapá - AP</t>
         </is>
       </c>
-      <c r="E11" s="13" t="inlineStr">
-        <is>
-          <t>N/D</t>
-        </is>
-      </c>
-      <c r="F11" s="13" t="inlineStr">
+      <c r="E13" s="13" t="inlineStr">
+        <is>
+          <t>N/D</t>
+        </is>
+      </c>
+      <c r="F13" s="13" t="inlineStr">
         <is>
           <t>3.000–3.500+ escolas | 5 países | 35+ redes parceiras BR | Prefeitura de Macapá (105 escolas)</t>
         </is>
       </c>
-      <c r="G11" s="13" t="inlineStr">
+      <c r="G13" s="13" t="inlineStr">
         <is>
           <t>Maior rodada de invest. na Amazônia (Exame)</t>
         </is>
       </c>
-      <c r="H11" s="13" t="inlineStr">
+      <c r="H13" s="13" t="inlineStr">
         <is>
           <t>Edtech amapaense fundada às margens do Rio Amazonas. Vertical pública Proesc Gov já implantada na Secretaria de Educação de Macapá: diário eletrônico com app offline, matrículas digitais, IDEB/VAAR e gestão da secretaria. Diferencial: Botão Alerta Escolar conecta as 105 escolas municipais à Guarda Civil Municipal. IA 'LIA' para decisões estratégicas nas secretarias. 3.000–3.500+ escolas parceiras (privadas + públicas), 5 países, 35+ redes pelo Brasil. Captou a maior rodada de investimento já realizada na Amazônia (Exame).</t>
         </is>
       </c>
-      <c r="I11" s="18" t="inlineStr">
+      <c r="I13" s="18" t="inlineStr">
         <is>
           <t>Watch — pública + Amazônia</t>
         </is>
       </c>
-      <c r="J11" s="22" t="inlineStr">
+      <c r="J13" s="20" t="inlineStr">
         <is>
           <t>✓</t>
         </is>
@@ -5093,7 +5437,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:J10"/>
+  <dimension ref="A1:J12"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="28" customWidth="1" min="1" max="1"/>
@@ -5450,50 +5794,50 @@
     <row r="9" ht="48" customHeight="1">
       <c r="A9" s="12" t="inlineStr">
         <is>
-          <t>Licitagram</t>
+          <t>Zaelo</t>
         </is>
       </c>
       <c r="B9" s="13" t="inlineStr">
         <is>
-          <t>SO de IA Multi-Agente para Licitações (Sell-side + Buy-side)</t>
+          <t>Compras Públicas Buy-side (Órgãos) + Auditoria IA</t>
         </is>
       </c>
       <c r="C9" s="13" t="inlineStr">
         <is>
-          <t>Startup</t>
+          <t>Scale-up</t>
         </is>
       </c>
       <c r="D9" s="13" t="inlineStr">
         <is>
-          <t>Brasil</t>
+          <t>Itajaí - SC</t>
         </is>
       </c>
       <c r="E9" s="13" t="inlineStr">
         <is>
-          <t>N/D</t>
+          <t>2016</t>
         </is>
       </c>
       <c r="F9" s="13" t="inlineStr">
         <is>
-          <t>200k+ licitações/mês | R$1T+ oportunidades | 67M+ CNPJs cruzados</t>
+          <t>170+ órgãos públicos | 10K+ servidores públicos</t>
         </is>
       </c>
       <c r="G9" s="13" t="inlineStr">
         <is>
-          <t>N/D</t>
+          <t>N/D (bootstrap)</t>
         </is>
       </c>
       <c r="H9" s="13" t="inlineStr">
         <is>
-          <t>1º Sistema Operacional de IA Multi-Agente para Licitações da América Latina. 14 módulos IA: AI Matching score 0–100, robô de lances IA, inteligência competitiva (5 módulos), pesquisa de preços IN 65/2021, grafo societário, detecção de anomalias, compliance checker e forensic replay. Cobre sell-side (fornecedores) + buy-side (entes públicos) + compliance (TCUs). Integração PNCP. Planos: R$297–R$1.497/mês.</t>
+          <t>GovTech de compras públicas focada no lado dos órgãos (buy-side). Dois produtos principais: Loja Pública Gestor — cobrindo todo o ciclo (planejamento → execução) com conformidade Lei 14.133/2021; e Sentinela — auditoria inteligente de contratos com IA, detecta anomalias e superfaturamento automaticamente. Até 45% de economia declarada em processos de compras. 170+ órgãos atendidos, 10K+ servidores capacitados. Fundada em 2016, 10 anos de mercado, bootstrap. Sede Itajaí SC.</t>
         </is>
       </c>
       <c r="I9" s="18" t="inlineStr">
         <is>
-          <t>Watch — IA licitações multi-agente</t>
-        </is>
-      </c>
-      <c r="J9" s="22" t="inlineStr">
+          <t>Watch — buy-side maduro</t>
+        </is>
+      </c>
+      <c r="J9" s="20" t="inlineStr">
         <is>
           <t>✓</t>
         </is>
@@ -5502,50 +5846,154 @@
     <row r="10" ht="48" customHeight="1">
       <c r="A10" s="14" t="inlineStr">
         <is>
+          <t>Licito.guru</t>
+        </is>
+      </c>
+      <c r="B10" s="15" t="inlineStr">
+        <is>
+          <t>IA Buy-side para Licitações em Órgãos Públicos</t>
+        </is>
+      </c>
+      <c r="C10" s="15" t="inlineStr">
+        <is>
+          <t>Startup</t>
+        </is>
+      </c>
+      <c r="D10" s="15" t="inlineStr">
+        <is>
+          <t>Florianópolis - SC</t>
+        </is>
+      </c>
+      <c r="E10" s="15" t="inlineStr">
+        <is>
+          <t>N/D</t>
+        </is>
+      </c>
+      <c r="F10" s="15" t="inlineStr">
+        <is>
+          <t>Pref. São Paulo SP | Gov. Paraná | Gov. Santa Catarina | MP | TJ | Pref. Curitiba PR</t>
+        </is>
+      </c>
+      <c r="G10" s="15" t="inlineStr">
+        <is>
+          <t>N/D</t>
+        </is>
+      </c>
+      <c r="H10" s="15" t="inlineStr">
+        <is>
+          <t>Plataforma de IA para o lado dos órgãos na contratação pública. Gera automaticamente os principais documentos obrigatórios: ETP (Estudo Técnico Preliminar), DFD (Documento de Formalização de Demanda), TR (Termo de Referência), Mapa de Risco, Edital, Contrato e mais. IA customizável por órgão — aprende os padrões e histórico de cada cliente. Treinada e supervisionada pelo Prof. Gustavo Schiefler (referência nacional em licitações públicas). Carteira com órgãos de alto perfil: Prefeitura de SP, Governos do PR e SC, MP, TJ, Prefeitura de Curitiba. Florianópolis SC.</t>
+        </is>
+      </c>
+      <c r="I10" s="16" t="inlineStr">
+        <is>
+          <t>🔥 Deal — carteira premium</t>
+        </is>
+      </c>
+      <c r="J10" s="17" t="inlineStr">
+        <is>
+          <t>✓</t>
+        </is>
+      </c>
+    </row>
+    <row r="11" ht="48" customHeight="1">
+      <c r="A11" s="12" t="inlineStr">
+        <is>
+          <t>Licitagram</t>
+        </is>
+      </c>
+      <c r="B11" s="13" t="inlineStr">
+        <is>
+          <t>SO de IA Multi-Agente para Licitações (Sell-side + Buy-side)</t>
+        </is>
+      </c>
+      <c r="C11" s="13" t="inlineStr">
+        <is>
+          <t>Startup</t>
+        </is>
+      </c>
+      <c r="D11" s="13" t="inlineStr">
+        <is>
+          <t>Brasil</t>
+        </is>
+      </c>
+      <c r="E11" s="13" t="inlineStr">
+        <is>
+          <t>N/D</t>
+        </is>
+      </c>
+      <c r="F11" s="13" t="inlineStr">
+        <is>
+          <t>200k+ licitações/mês | R$1T+ oportunidades | 67M+ CNPJs cruzados</t>
+        </is>
+      </c>
+      <c r="G11" s="13" t="inlineStr">
+        <is>
+          <t>N/D</t>
+        </is>
+      </c>
+      <c r="H11" s="13" t="inlineStr">
+        <is>
+          <t>1º Sistema Operacional de IA Multi-Agente para Licitações da América Latina. 14 módulos IA: AI Matching score 0–100, robô de lances IA, inteligência competitiva (5 módulos), pesquisa de preços IN 65/2021, grafo societário, detecção de anomalias, compliance checker e forensic replay. Cobre sell-side (fornecedores) + buy-side (entes públicos) + compliance (TCUs). Integração PNCP. Planos: R$297–R$1.497/mês.</t>
+        </is>
+      </c>
+      <c r="I11" s="18" t="inlineStr">
+        <is>
+          <t>Watch — IA licitações multi-agente</t>
+        </is>
+      </c>
+      <c r="J11" s="20" t="inlineStr">
+        <is>
+          <t>✓</t>
+        </is>
+      </c>
+    </row>
+    <row r="12" ht="48" customHeight="1">
+      <c r="A12" s="14" t="inlineStr">
+        <is>
           <t>Licitei</t>
         </is>
       </c>
-      <c r="B10" s="15" t="inlineStr">
+      <c r="B12" s="15" t="inlineStr">
         <is>
           <t>Licitações Sell-side para PMEs</t>
         </is>
       </c>
-      <c r="C10" s="15" t="inlineStr">
+      <c r="C12" s="15" t="inlineStr">
         <is>
           <t>Startup</t>
         </is>
       </c>
-      <c r="D10" s="15" t="inlineStr">
+      <c r="D12" s="15" t="inlineStr">
         <is>
           <t>Belo Horizonte - MG</t>
         </is>
       </c>
-      <c r="E10" s="15" t="inlineStr">
-        <is>
-          <t>N/D</t>
-        </is>
-      </c>
-      <c r="F10" s="15" t="inlineStr">
+      <c r="E12" s="15" t="inlineStr">
+        <is>
+          <t>N/D</t>
+        </is>
+      </c>
+      <c r="F12" s="15" t="inlineStr">
         <is>
           <t>4.000+ usuários | 206k+ editais | PNCP integrado</t>
         </is>
       </c>
-      <c r="G10" s="15" t="inlineStr">
+      <c r="G12" s="15" t="inlineStr">
         <is>
           <t>R$3,5M (Thompson Participações, jun/2024)</t>
         </is>
       </c>
-      <c r="H10" s="15" t="inlineStr">
+      <c r="H12" s="15" t="inlineStr">
         <is>
           <t>Plataforma sell-side focada em PMEs que vendem para governo: robô de lances IA, análise de editais com IA, monitoramento de oportunidades e integração PNCP. Aporte de R$3,5M da Thompson Participações (jun/2024). CEO: Felipe Nardes. 4.000+ usuários ativos, 206k+ editais monitorados. Diferencia-se da StartGi por foco em PMEs e preço acessível.</t>
         </is>
       </c>
-      <c r="I10" s="16" t="inlineStr">
+      <c r="I12" s="16" t="inlineStr">
         <is>
           <t>Watch — sell-side PME</t>
         </is>
       </c>
-      <c r="J10" s="17" t="inlineStr">
+      <c r="J12" s="17" t="inlineStr">
         <is>
           <t>✓</t>
         </is>

</xml_diff>

<commit_message>
v16: adiciona Kodefy (gestao) — metas e projetos municipais
Plataforma de gerenciamento de projetos/metas para prefeituras.
App 4.8★, Tapejara RS. Total: 81 empresas únicas, 83 aparições.

Co-Authored-By: Claude Sonnet 4.6 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/Radar_GovTechs_Brasil_2026.xlsx
+++ b/Radar_GovTechs_Brasil_2026.xlsx
@@ -227,11 +227,11 @@
     <xf numFmtId="0" fontId="5" fillId="5" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment vertical="top" wrapText="1"/>
     </xf>
+    <xf numFmtId="0" fontId="6" fillId="5" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment vertical="top" wrapText="1"/>
+    </xf>
     <xf numFmtId="0" fontId="4" fillId="7" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="6" fillId="5" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment vertical="top" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="4" fillId="8" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center"/>
@@ -647,7 +647,7 @@
     <row r="1" ht="32" customHeight="1">
       <c r="A1" s="1" t="inlineStr">
         <is>
-          <t>🇧🇷 Radar GovTech Brasil 2025/2026 — DLG · Maio 2026 · v15</t>
+          <t>🇧🇷 Radar GovTech Brasil 2025/2026 — DLG · Maio 2026 · v16</t>
         </is>
       </c>
     </row>
@@ -670,7 +670,7 @@
         </is>
       </c>
       <c r="B4" s="4" t="n">
-        <v>13</v>
+        <v>14</v>
       </c>
     </row>
     <row r="5">
@@ -780,7 +780,7 @@
         </is>
       </c>
       <c r="B15" s="6" t="n">
-        <v>82</v>
+        <v>83</v>
       </c>
     </row>
     <row r="16">
@@ -790,7 +790,7 @@
         </is>
       </c>
       <c r="B16" s="8" t="n">
-        <v>80</v>
+        <v>81</v>
       </c>
     </row>
     <row r="18">
@@ -1353,7 +1353,7 @@
           <t>🔥 Deal — Smart Sampa</t>
         </is>
       </c>
-      <c r="J3" s="20" t="inlineStr">
+      <c r="J3" s="19" t="inlineStr">
         <is>
           <t>✓</t>
         </is>
@@ -1457,7 +1457,7 @@
           <t>🔥 Deal — Smart Sampa</t>
         </is>
       </c>
-      <c r="J5" s="20" t="inlineStr">
+      <c r="J5" s="19" t="inlineStr">
         <is>
           <t>✓</t>
         </is>
@@ -2405,7 +2405,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:J15"/>
+  <dimension ref="A1:J16"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="28" customWidth="1" min="1" max="1"/>
@@ -2578,32 +2578,32 @@
     <row r="5" ht="48" customHeight="1">
       <c r="A5" s="12" t="inlineStr">
         <is>
-          <t>GovDigital</t>
+          <t>Kodefy</t>
         </is>
       </c>
       <c r="B5" s="13" t="inlineStr">
         <is>
-          <t>App Municipal SaaS / Relacionamento Cidadão-Governo</t>
+          <t>Gerenciamento de Projetos e Metas Municipais / App de Prefeitura</t>
         </is>
       </c>
       <c r="C5" s="13" t="inlineStr">
         <is>
-          <t>Startup / Scale-up</t>
+          <t>Startup</t>
         </is>
       </c>
       <c r="D5" s="13" t="inlineStr">
         <is>
-          <t>Jaraguá do Sul - SC</t>
+          <t>Tapejara - RS</t>
         </is>
       </c>
       <c r="E5" s="13" t="inlineStr">
         <is>
-          <t>~2020</t>
+          <t>N/D</t>
         </is>
       </c>
       <c r="F5" s="13" t="inlineStr">
         <is>
-          <t>Múltiplos municípios SC e outros estados</t>
+          <t>Municípios RS e outros estados | contratada por inexigibilidade (art. 74 IV Lei 14.133/2021)</t>
         </is>
       </c>
       <c r="G5" s="13" t="inlineStr">
@@ -2613,69 +2613,77 @@
       </c>
       <c r="H5" s="13" t="inlineStr">
         <is>
-          <t>App oficial white-label de prefeituras reunindo zeladoria, agendamento, formulários online, notícias e comunicação direta cidadão-prefeitura. Integrações com IPTU, protocolo e ouvidoria. CEO: Elias Raasch. Expansão nacional sem VC.</t>
+          <t>Plataforma dual: (1) Gov — cadastramento e gerenciamento de projetos e metas da administração pública municipal: gestores acompanham objetivos da gestão em tempo real, com dashboards e relatórios de execução; contratada via inexigibilidade de licitação (ex: Selbach-RS, 2026). (2) Fidelizec — plataforma B2C de programas de fidelidade para comércio local, com R$7,7M movimentados em uma única Black Friday. Apps com média 4.8★ (de 5.0) nas lojas. CNPJ: 41.426.978/0001-05. Sede: Tapejara RS.</t>
         </is>
       </c>
       <c r="I5" s="18" t="inlineStr">
         <is>
-          <t>Watch — expansão nacional</t>
-        </is>
-      </c>
-      <c r="J5" s="13" t="inlineStr"/>
+          <t>Watch — metas municipais</t>
+        </is>
+      </c>
+      <c r="J5" s="19" t="inlineStr">
+        <is>
+          <t>✓</t>
+        </is>
+      </c>
     </row>
     <row r="6" ht="48" customHeight="1">
       <c r="A6" s="14" t="inlineStr">
         <is>
-          <t>Desenvolve Cidade</t>
+          <t>GovDigital</t>
         </is>
       </c>
       <c r="B6" s="15" t="inlineStr">
         <is>
-          <t>Licenciamento e Tributação Municipal Digital</t>
+          <t>App Municipal SaaS / Relacionamento Cidadão-Governo</t>
         </is>
       </c>
       <c r="C6" s="15" t="inlineStr">
         <is>
-          <t>Startup</t>
+          <t>Startup / Scale-up</t>
         </is>
       </c>
       <c r="D6" s="15" t="inlineStr">
         <is>
-          <t>Campinas - SP</t>
+          <t>Jaraguá do Sul - SC</t>
         </is>
       </c>
       <c r="E6" s="15" t="inlineStr">
         <is>
-          <t>~2014</t>
+          <t>~2020</t>
         </is>
       </c>
       <c r="F6" s="15" t="inlineStr">
         <is>
-          <t>Municípios Norte e outras regiões | Scale-Up Endeavor 2021</t>
+          <t>Múltiplos municípios SC e outros estados</t>
         </is>
       </c>
       <c r="G6" s="15" t="inlineStr">
         <is>
-          <t>N/D</t>
+          <t>N/D (bootstrap)</t>
         </is>
       </c>
       <c r="H6" s="15" t="inlineStr">
         <is>
-          <t>Plataforma integrada de licenciamento digital (urbanístico, ambiental, sanitário, obras), abertura/baixa de empresas, IPTU e ISS digitais integrada à REDESIM federal. Foco em desburocratização e aumento de receita própria municipal. TOP2 Open Startups 2024.</t>
-        </is>
-      </c>
-      <c r="I6" s="15" t="inlineStr"/>
+          <t>App oficial white-label de prefeituras reunindo zeladoria, agendamento, formulários online, notícias e comunicação direta cidadão-prefeitura. Integrações com IPTU, protocolo e ouvidoria. CEO: Elias Raasch. Expansão nacional sem VC.</t>
+        </is>
+      </c>
+      <c r="I6" s="16" t="inlineStr">
+        <is>
+          <t>Watch — expansão nacional</t>
+        </is>
+      </c>
       <c r="J6" s="15" t="inlineStr"/>
     </row>
     <row r="7" ht="48" customHeight="1">
       <c r="A7" s="12" t="inlineStr">
         <is>
-          <t>IP Inovação</t>
+          <t>Desenvolve Cidade</t>
         </is>
       </c>
       <c r="B7" s="13" t="inlineStr">
         <is>
-          <t>Capacitação e Consultoria em Gestão Pública</t>
+          <t>Licenciamento e Tributação Municipal Digital</t>
         </is>
       </c>
       <c r="C7" s="13" t="inlineStr">
@@ -2685,17 +2693,17 @@
       </c>
       <c r="D7" s="13" t="inlineStr">
         <is>
-          <t>Belém - PA</t>
+          <t>Campinas - SP</t>
         </is>
       </c>
       <c r="E7" s="13" t="inlineStr">
         <is>
-          <t>2014</t>
+          <t>~2014</t>
         </is>
       </c>
       <c r="F7" s="13" t="inlineStr">
         <is>
-          <t>Ecossistema Norte do Brasil</t>
+          <t>Municípios Norte e outras regiões | Scale-Up Endeavor 2021</t>
         </is>
       </c>
       <c r="G7" s="13" t="inlineStr">
@@ -2705,45 +2713,41 @@
       </c>
       <c r="H7" s="13" t="inlineStr">
         <is>
-          <t>Empresa de capacitação e consultoria para gestão pública municipal na região Norte. TOP 3 Open Startups 2024. Não foram identificados produtos SaaS com identidade digital clara — oportunidade de due diligence.</t>
-        </is>
-      </c>
-      <c r="I7" s="18" t="inlineStr">
-        <is>
-          <t>Watch — due diligence necessário</t>
-        </is>
-      </c>
+          <t>Plataforma integrada de licenciamento digital (urbanístico, ambiental, sanitário, obras), abertura/baixa de empresas, IPTU e ISS digitais integrada à REDESIM federal. Foco em desburocratização e aumento de receita própria municipal. TOP2 Open Startups 2024.</t>
+        </is>
+      </c>
+      <c r="I7" s="13" t="inlineStr"/>
       <c r="J7" s="13" t="inlineStr"/>
     </row>
     <row r="8" ht="48" customHeight="1">
       <c r="A8" s="14" t="inlineStr">
         <is>
-          <t>GESUAS</t>
+          <t>IP Inovação</t>
         </is>
       </c>
       <c r="B8" s="15" t="inlineStr">
         <is>
-          <t>Gestão do SUAS / Assistência Social</t>
+          <t>Capacitação e Consultoria em Gestão Pública</t>
         </is>
       </c>
       <c r="C8" s="15" t="inlineStr">
         <is>
-          <t>Startup / PME</t>
+          <t>Startup</t>
         </is>
       </c>
       <c r="D8" s="15" t="inlineStr">
         <is>
-          <t>Viçosa - MG</t>
+          <t>Belém - PA</t>
         </is>
       </c>
       <c r="E8" s="15" t="inlineStr">
         <is>
-          <t>2008</t>
+          <t>2014</t>
         </is>
       </c>
       <c r="F8" s="15" t="inlineStr">
         <is>
-          <t>Centenas de municípios | CRASs e CREASs</t>
+          <t>Ecossistema Norte do Brasil</t>
         </is>
       </c>
       <c r="G8" s="15" t="inlineStr">
@@ -2753,12 +2757,12 @@
       </c>
       <c r="H8" s="15" t="inlineStr">
         <is>
-          <t>SaaS de gestão do SUAS com Prontuário Digital integrado ao CadÚnico, planos PAIF/PAEFI/PIA, vigilância socioassistencial georreferenciada e relatórios MDS. 56 colaboradores. Líder IE GovTech 2020. Vertical exclusivo sem concorrente direto.</t>
+          <t>Empresa de capacitação e consultoria para gestão pública municipal na região Norte. TOP 3 Open Startups 2024. Não foram identificados produtos SaaS com identidade digital clara — oportunidade de due diligence.</t>
         </is>
       </c>
       <c r="I8" s="16" t="inlineStr">
         <is>
-          <t>Vertical exclusivo mapeado</t>
+          <t>Watch — due diligence necessário</t>
         </is>
       </c>
       <c r="J8" s="15" t="inlineStr"/>
@@ -2766,47 +2770,47 @@
     <row r="9" ht="48" customHeight="1">
       <c r="A9" s="12" t="inlineStr">
         <is>
-          <t>Prosas</t>
+          <t>GESUAS</t>
         </is>
       </c>
       <c r="B9" s="13" t="inlineStr">
         <is>
-          <t>Gestão de Editais e Investimento Social</t>
+          <t>Gestão do SUAS / Assistência Social</t>
         </is>
       </c>
       <c r="C9" s="13" t="inlineStr">
         <is>
-          <t>Startup</t>
+          <t>Startup / PME</t>
         </is>
       </c>
       <c r="D9" s="13" t="inlineStr">
         <is>
-          <t>Belo Horizonte - MG</t>
+          <t>Viçosa - MG</t>
         </is>
       </c>
       <c r="E9" s="13" t="inlineStr">
         <is>
-          <t>2014</t>
+          <t>2008</t>
         </is>
       </c>
       <c r="F9" s="13" t="inlineStr">
         <is>
-          <t>13k+ editais | institutos e fundações corporativas</t>
+          <t>Centenas de municípios | CRASs e CREASs</t>
         </is>
       </c>
       <c r="G9" s="13" t="inlineStr">
         <is>
-          <t>R$4M (KPTL)</t>
+          <t>N/D</t>
         </is>
       </c>
       <c r="H9" s="13" t="inlineStr">
         <is>
-          <t>Maior base de editais do terceiro setor no Brasil. Plataforma para criação de editais, inscrições online, pareceristas e monitoramento de projetos. Venture Round out/2024. Portfólio Fundo GovTech KPTL. 51 funcionários.</t>
+          <t>SaaS de gestão do SUAS com Prontuário Digital integrado ao CadÚnico, planos PAIF/PAEFI/PIA, vigilância socioassistencial georreferenciada e relatórios MDS. 56 colaboradores. Líder IE GovTech 2020. Vertical exclusivo sem concorrente direto.</t>
         </is>
       </c>
       <c r="I9" s="18" t="inlineStr">
         <is>
-          <t>Portfólio KPTL</t>
+          <t>Vertical exclusivo mapeado</t>
         </is>
       </c>
       <c r="J9" s="13" t="inlineStr"/>
@@ -2814,12 +2818,12 @@
     <row r="10" ht="48" customHeight="1">
       <c r="A10" s="14" t="inlineStr">
         <is>
-          <t>Lemobs</t>
+          <t>Prosas</t>
         </is>
       </c>
       <c r="B10" s="15" t="inlineStr">
         <is>
-          <t>Gestão Urbana Integrada / Smart Cities</t>
+          <t>Gestão de Editais e Investimento Social</t>
         </is>
       </c>
       <c r="C10" s="15" t="inlineStr">
@@ -2829,41 +2833,45 @@
       </c>
       <c r="D10" s="15" t="inlineStr">
         <is>
-          <t>Rio de Janeiro - RJ</t>
+          <t>Belo Horizonte - MG</t>
         </is>
       </c>
       <c r="E10" s="15" t="inlineStr">
         <is>
-          <t>2015</t>
+          <t>2014</t>
         </is>
       </c>
       <c r="F10" s="15" t="inlineStr">
         <is>
-          <t>79k+ pontos monitorados | prefeituras e Petrobras</t>
+          <t>13k+ editais | institutos e fundações corporativas</t>
         </is>
       </c>
       <c r="G10" s="15" t="inlineStr">
         <is>
-          <t>N/D</t>
+          <t>R$4M (KPTL)</t>
         </is>
       </c>
       <c r="H10" s="15" t="inlineStr">
         <is>
-          <t>GovTech de cidades inteligentes com SIGELU (limpeza urbana), fiscalização móvel, gestão nutricional escolar e saúde. Primeiro contrato pelo Marco Legal das Startups. Origem COPPE/UFRJ. Selo GovTech BrazilLAB.</t>
-        </is>
-      </c>
-      <c r="I10" s="15" t="inlineStr"/>
+          <t>Maior base de editais do terceiro setor no Brasil. Plataforma para criação de editais, inscrições online, pareceristas e monitoramento de projetos. Venture Round out/2024. Portfólio Fundo GovTech KPTL. 51 funcionários.</t>
+        </is>
+      </c>
+      <c r="I10" s="16" t="inlineStr">
+        <is>
+          <t>Portfólio KPTL</t>
+        </is>
+      </c>
       <c r="J10" s="15" t="inlineStr"/>
     </row>
     <row r="11" ht="48" customHeight="1">
       <c r="A11" s="12" t="inlineStr">
         <is>
-          <t>GRTS Digital</t>
+          <t>Lemobs</t>
         </is>
       </c>
       <c r="B11" s="13" t="inlineStr">
         <is>
-          <t>Gestão de Relações Trabalhistas e Sindicais (RTS)</t>
+          <t>Gestão Urbana Integrada / Smart Cities</t>
         </is>
       </c>
       <c r="C11" s="13" t="inlineStr">
@@ -2873,80 +2881,76 @@
       </c>
       <c r="D11" s="13" t="inlineStr">
         <is>
-          <t>Salvador - BA</t>
+          <t>Rio de Janeiro - RJ</t>
         </is>
       </c>
       <c r="E11" s="13" t="inlineStr">
         <is>
-          <t>2019</t>
+          <t>2015</t>
         </is>
       </c>
       <c r="F11" s="13" t="inlineStr">
         <is>
-          <t>Unilever, Coca-Cola, Vivo, Burger King, C&amp;A | 29 colaboradores</t>
+          <t>79k+ pontos monitorados | prefeituras e Petrobras</t>
         </is>
       </c>
       <c r="G11" s="13" t="inlineStr">
         <is>
-          <t>R$ 3,4M aporte (Fundo GovTech)</t>
+          <t>N/D</t>
         </is>
       </c>
       <c r="H11" s="13" t="inlineStr">
         <is>
-          <t>Ecossistema SaaS de digitalização de RTS: gestão de CCTs, IA 'Norma' para análise de cláusulas, assembleias virtuais e data intelligence. Integração com HCM via parceria LG. Prêmio inovação RH 2025. R$3,4M Fundo GovTech KPTL (jun/2025). Lançou GRTS Contábil (12 contratos nas primeiras 3 semanas). Co-investidor Aleve Legal Tech. Meta: R$25M faturamento até 2027. CEO Uirá Menezes, sede Salvador BA.</t>
-        </is>
-      </c>
-      <c r="I11" s="18" t="inlineStr">
-        <is>
-          <t>Portfólio KPTL</t>
-        </is>
-      </c>
+          <t>GovTech de cidades inteligentes com SIGELU (limpeza urbana), fiscalização móvel, gestão nutricional escolar e saúde. Primeiro contrato pelo Marco Legal das Startups. Origem COPPE/UFRJ. Selo GovTech BrazilLAB.</t>
+        </is>
+      </c>
+      <c r="I11" s="13" t="inlineStr"/>
       <c r="J11" s="13" t="inlineStr"/>
     </row>
     <row r="12" ht="48" customHeight="1">
       <c r="A12" s="14" t="inlineStr">
         <is>
-          <t>Governar</t>
+          <t>GRTS Digital</t>
         </is>
       </c>
       <c r="B12" s="15" t="inlineStr">
         <is>
-          <t>ERP Municipal Integrado / SIAFIC Cloud</t>
+          <t>Gestão de Relações Trabalhistas e Sindicais (RTS)</t>
         </is>
       </c>
       <c r="C12" s="15" t="inlineStr">
         <is>
-          <t>Startup / Scale-up</t>
+          <t>Startup</t>
         </is>
       </c>
       <c r="D12" s="15" t="inlineStr">
         <is>
-          <t>Brasil</t>
+          <t>Salvador - BA</t>
         </is>
       </c>
       <c r="E12" s="15" t="inlineStr">
         <is>
-          <t>N/D</t>
+          <t>2019</t>
         </is>
       </c>
       <c r="F12" s="15" t="inlineStr">
         <is>
-          <t>Municípios de qualquer porte | SIAFIC + SIEDUC disponíveis</t>
+          <t>Unilever, Coca-Cola, Vivo, Burger King, C&amp;A | 29 colaboradores</t>
         </is>
       </c>
       <c r="G12" s="15" t="inlineStr">
         <is>
-          <t>N/D</t>
+          <t>R$ 3,4M aporte (Fundo GovTech)</t>
         </is>
       </c>
       <c r="H12" s="15" t="inlineStr">
         <is>
-          <t>Suite ERP municipal integrada em nuvem com base de dados única: SIAFIC (financeiro/tributário), SIEDUC (educação), SISAÚDE e SIASOC. Conformidade SICONFI, SIOPE, e-Social, eSUS. Produto novo no mercado com proposta de stack completo integrado.</t>
+          <t>Ecossistema SaaS de digitalização de RTS: gestão de CCTs, IA 'Norma' para análise de cláusulas, assembleias virtuais e data intelligence. Integração com HCM via parceria LG. Prêmio inovação RH 2025. R$3,4M Fundo GovTech KPTL (jun/2025). Lançou GRTS Contábil (12 contratos nas primeiras 3 semanas). Co-investidor Aleve Legal Tech. Meta: R$25M faturamento até 2027. CEO Uirá Menezes, sede Salvador BA.</t>
         </is>
       </c>
       <c r="I12" s="16" t="inlineStr">
         <is>
-          <t>Watch — SIAFIC driver</t>
+          <t>Portfólio KPTL</t>
         </is>
       </c>
       <c r="J12" s="15" t="inlineStr"/>
@@ -2954,47 +2958,47 @@
     <row r="13" ht="48" customHeight="1">
       <c r="A13" s="12" t="inlineStr">
         <is>
-          <t>Colab</t>
+          <t>Governar</t>
         </is>
       </c>
       <c r="B13" s="13" t="inlineStr">
         <is>
-          <t>Participação Cidadã e Serviços Digitais Municipais</t>
+          <t>ERP Municipal Integrado / SIAFIC Cloud</t>
         </is>
       </c>
       <c r="C13" s="13" t="inlineStr">
         <is>
-          <t>Scale-up</t>
+          <t>Startup / Scale-up</t>
         </is>
       </c>
       <c r="D13" s="13" t="inlineStr">
         <is>
-          <t>São Paulo - SP</t>
+          <t>Brasil</t>
         </is>
       </c>
       <c r="E13" s="13" t="inlineStr">
         <is>
-          <t>2013</t>
+          <t>N/D</t>
         </is>
       </c>
       <c r="F13" s="13" t="inlineStr">
         <is>
-          <t>5 países | 1M+ cidadãos | Piauí, São Gonçalo, Santo André | Parceiro ONU-Habitat</t>
+          <t>Municípios de qualquer porte | SIAFIC + SIEDUC disponíveis</t>
         </is>
       </c>
       <c r="G13" s="13" t="inlineStr">
         <is>
-          <t>~R$25M total (MDIF+Luminate+EDP+KPTL)</t>
+          <t>N/D</t>
         </is>
       </c>
       <c r="H13" s="13" t="inlineStr">
         <is>
-          <t>Plataforma multicanal (web, app, WhatsApp) de gestão de serviços digitais, participação cidadã e CRM governamental. IA digitaliza qualquer serviço público em minutos. Em 2025 viabilizou OP Digital do Piauí (273k participantes) com validação via Receita Federal e blockchain. Lançou Colab Gov.AI (AWS Bedrock, out/2025): 94% de aceleração na criação de serviços digitais, 500+ prompts em 14 dias. Novos clientes: TCU, Diadema, Rio das Ostras, Duque de Caxias. Rodada US$10M+ em curso para 2026. Portfólio KPTL+Cedro. Co-invest EDP Ventures + Luminate + MDIF.</t>
+          <t>Suite ERP municipal integrada em nuvem com base de dados única: SIAFIC (financeiro/tributário), SIEDUC (educação), SISAÚDE e SIASOC. Conformidade SICONFI, SIOPE, e-Social, eSUS. Produto novo no mercado com proposta de stack completo integrado.</t>
         </is>
       </c>
       <c r="I13" s="18" t="inlineStr">
         <is>
-          <t>Portfólio KPTL+Cedro</t>
+          <t>Watch — SIAFIC driver</t>
         </is>
       </c>
       <c r="J13" s="13" t="inlineStr"/>
@@ -3002,47 +3006,47 @@
     <row r="14" ht="48" customHeight="1">
       <c r="A14" s="14" t="inlineStr">
         <is>
-          <t>Pública Tecnologia</t>
+          <t>Colab</t>
         </is>
       </c>
       <c r="B14" s="15" t="inlineStr">
         <is>
-          <t>ERP Municipal Full Suite</t>
+          <t>Participação Cidadã e Serviços Digitais Municipais</t>
         </is>
       </c>
       <c r="C14" s="15" t="inlineStr">
         <is>
-          <t>PME Estabelecida</t>
+          <t>Scale-up</t>
         </is>
       </c>
       <c r="D14" s="15" t="inlineStr">
         <is>
-          <t>Blumenau - SC</t>
+          <t>São Paulo - SP</t>
         </is>
       </c>
       <c r="E14" s="15" t="inlineStr">
         <is>
-          <t>1993</t>
+          <t>2013</t>
         </is>
       </c>
       <c r="F14" s="15" t="inlineStr">
         <is>
-          <t>Municípios BR + Portugal + Venezuela</t>
+          <t>5 países | 1M+ cidadãos | Piauí, São Gonçalo, Santo André | Parceiro ONU-Habitat</t>
         </is>
       </c>
       <c r="G14" s="15" t="inlineStr">
         <is>
-          <t>N/D</t>
+          <t>~R$25M total (MDIF+Luminate+EDP+KPTL)</t>
         </is>
       </c>
       <c r="H14" s="15" t="inlineStr">
         <is>
-          <t>ERP municipal full suite com 9 áreas: Financeira (contabilidade pública, NF-e), Tributária (ISS, IPTU), Gestão de Pessoas (RH, eSocial, ponto eletrônico), Saúde, Escolar, Assistência Social (SUAS), Administrativa (compras, frotas, patrimônio), Atendimento ao Cidadão (portal transparência, app Cidade Pública) e Gestão (BI, GED, PPA). 33 anos de atuação, 98 funcionários. Great Place to Work. Presença internacional: Portugal e Venezuela. Sede Blumenau/SC.</t>
+          <t>Plataforma multicanal (web, app, WhatsApp) de gestão de serviços digitais, participação cidadã e CRM governamental. IA digitaliza qualquer serviço público em minutos. Em 2025 viabilizou OP Digital do Piauí (273k participantes) com validação via Receita Federal e blockchain. Lançou Colab Gov.AI (AWS Bedrock, out/2025): 94% de aceleração na criação de serviços digitais, 500+ prompts em 14 dias. Novos clientes: TCU, Diadema, Rio das Ostras, Duque de Caxias. Rodada US$10M+ em curso para 2026. Portfólio KPTL+Cedro. Co-invest EDP Ventures + Luminate + MDIF.</t>
         </is>
       </c>
       <c r="I14" s="16" t="inlineStr">
         <is>
-          <t>Target roll-up</t>
+          <t>Portfólio KPTL+Cedro</t>
         </is>
       </c>
       <c r="J14" s="15" t="inlineStr"/>
@@ -3050,50 +3054,98 @@
     <row r="15" ht="48" customHeight="1">
       <c r="A15" s="12" t="inlineStr">
         <is>
+          <t>Pública Tecnologia</t>
+        </is>
+      </c>
+      <c r="B15" s="13" t="inlineStr">
+        <is>
+          <t>ERP Municipal Full Suite</t>
+        </is>
+      </c>
+      <c r="C15" s="13" t="inlineStr">
+        <is>
+          <t>PME Estabelecida</t>
+        </is>
+      </c>
+      <c r="D15" s="13" t="inlineStr">
+        <is>
+          <t>Blumenau - SC</t>
+        </is>
+      </c>
+      <c r="E15" s="13" t="inlineStr">
+        <is>
+          <t>1993</t>
+        </is>
+      </c>
+      <c r="F15" s="13" t="inlineStr">
+        <is>
+          <t>Municípios BR + Portugal + Venezuela</t>
+        </is>
+      </c>
+      <c r="G15" s="13" t="inlineStr">
+        <is>
+          <t>N/D</t>
+        </is>
+      </c>
+      <c r="H15" s="13" t="inlineStr">
+        <is>
+          <t>ERP municipal full suite com 9 áreas: Financeira (contabilidade pública, NF-e), Tributária (ISS, IPTU), Gestão de Pessoas (RH, eSocial, ponto eletrônico), Saúde, Escolar, Assistência Social (SUAS), Administrativa (compras, frotas, patrimônio), Atendimento ao Cidadão (portal transparência, app Cidade Pública) e Gestão (BI, GED, PPA). 33 anos de atuação, 98 funcionários. Great Place to Work. Presença internacional: Portugal e Venezuela. Sede Blumenau/SC.</t>
+        </is>
+      </c>
+      <c r="I15" s="18" t="inlineStr">
+        <is>
+          <t>Target roll-up</t>
+        </is>
+      </c>
+      <c r="J15" s="13" t="inlineStr"/>
+    </row>
+    <row r="16" ht="48" customHeight="1">
+      <c r="A16" s="14" t="inlineStr">
+        <is>
           <t>PLACE</t>
         </is>
       </c>
-      <c r="B15" s="13" t="inlineStr">
+      <c r="B16" s="15" t="inlineStr">
         <is>
           <t>Planejamento Urbano e Geointeligência / Urban Twin</t>
         </is>
       </c>
-      <c r="C15" s="13" t="inlineStr">
+      <c r="C16" s="15" t="inlineStr">
         <is>
           <t>Startup</t>
         </is>
       </c>
-      <c r="D15" s="13" t="inlineStr">
+      <c r="D16" s="15" t="inlineStr">
         <is>
           <t>Brasil</t>
         </is>
       </c>
-      <c r="E15" s="13" t="inlineStr">
-        <is>
-          <t>N/D</t>
-        </is>
-      </c>
-      <c r="F15" s="13" t="inlineStr">
+      <c r="E16" s="15" t="inlineStr">
+        <is>
+          <t>N/D</t>
+        </is>
+      </c>
+      <c r="F16" s="15" t="inlineStr">
         <is>
           <t>Prefeituras e mercado imobiliário privado</t>
         </is>
       </c>
-      <c r="G15" s="13" t="inlineStr">
-        <is>
-          <t>N/D</t>
-        </is>
-      </c>
-      <c r="H15" s="13" t="inlineStr">
+      <c r="G16" s="15" t="inlineStr">
+        <is>
+          <t>N/D</t>
+        </is>
+      </c>
+      <c r="H16" s="15" t="inlineStr">
         <is>
           <t>Plataforma dual (govtech + proptech) de inteligência territorial com Gêmeo Digital: integra bases públicas, rotinas urbanísticas, pré-aprovação de projetos e visualização 2D/3D com IA aplicada à legislação urbanística. Para o setor privado: viabilidade e gestão de portfólio imobiliário. Certificada BrazilLAB.</t>
         </is>
       </c>
-      <c r="I15" s="18" t="inlineStr">
+      <c r="I16" s="16" t="inlineStr">
         <is>
           <t>Watch — urbanismo digital</t>
         </is>
       </c>
-      <c r="J15" s="13" t="inlineStr"/>
+      <c r="J16" s="15" t="inlineStr"/>
     </row>
   </sheetData>
   <mergeCells count="1">
@@ -3125,7 +3177,7 @@
   </cols>
   <sheetData>
     <row r="1" ht="28" customHeight="1">
-      <c r="A1" s="19" t="inlineStr">
+      <c r="A1" s="20" t="inlineStr">
         <is>
           <t>📊 Fiscal &amp; Convênios Municipais — Radar GovTech Brasil 2025/2026</t>
         </is>
@@ -3229,7 +3281,7 @@
           <t>Watch — fiscal municipal</t>
         </is>
       </c>
-      <c r="J3" s="20" t="inlineStr">
+      <c r="J3" s="19" t="inlineStr">
         <is>
           <t>✓</t>
         </is>
@@ -4477,7 +4529,7 @@
           <t>Watch — municipal</t>
         </is>
       </c>
-      <c r="J11" s="20" t="inlineStr">
+      <c r="J11" s="19" t="inlineStr">
         <is>
           <t>✓</t>
         </is>
@@ -4581,7 +4633,7 @@
           <t>Watch — pública + Amazônia</t>
         </is>
       </c>
-      <c r="J13" s="20" t="inlineStr">
+      <c r="J13" s="19" t="inlineStr">
         <is>
           <t>✓</t>
         </is>
@@ -5837,7 +5889,7 @@
           <t>Watch — buy-side maduro</t>
         </is>
       </c>
-      <c r="J9" s="20" t="inlineStr">
+      <c r="J9" s="19" t="inlineStr">
         <is>
           <t>✓</t>
         </is>
@@ -5941,7 +5993,7 @@
           <t>Watch — IA licitações multi-agente</t>
         </is>
       </c>
-      <c r="J11" s="20" t="inlineStr">
+      <c r="J11" s="19" t="inlineStr">
         <is>
           <t>✓</t>
         </is>

</xml_diff>

<commit_message>
v17: adiciona Assesi (gestao) — portais e transparência municipal
Suíte SaaS: aSiteGov, aLegislativo, aCidadão, aDiário, aOuvidoria,
CarteirinhaGov. 600+ municípios, 27 estados, 14 anos, Fortaleza CE.
Total: 82 empresas únicas, 84 aparições.

Co-Authored-By: Claude Sonnet 4.6 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/Radar_GovTechs_Brasil_2026.xlsx
+++ b/Radar_GovTechs_Brasil_2026.xlsx
@@ -647,7 +647,7 @@
     <row r="1" ht="32" customHeight="1">
       <c r="A1" s="1" t="inlineStr">
         <is>
-          <t>🇧🇷 Radar GovTech Brasil 2025/2026 — DLG · Maio 2026 · v16</t>
+          <t>🇧🇷 Radar GovTech Brasil 2025/2026 — DLG · Maio 2026 · v17</t>
         </is>
       </c>
     </row>
@@ -670,7 +670,7 @@
         </is>
       </c>
       <c r="B4" s="4" t="n">
-        <v>14</v>
+        <v>15</v>
       </c>
     </row>
     <row r="5">
@@ -780,7 +780,7 @@
         </is>
       </c>
       <c r="B15" s="6" t="n">
-        <v>83</v>
+        <v>84</v>
       </c>
     </row>
     <row r="16">
@@ -790,7 +790,7 @@
         </is>
       </c>
       <c r="B16" s="8" t="n">
-        <v>81</v>
+        <v>82</v>
       </c>
     </row>
     <row r="18">
@@ -2405,7 +2405,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:J16"/>
+  <dimension ref="A1:J17"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="28" customWidth="1" min="1" max="1"/>
@@ -2578,32 +2578,32 @@
     <row r="5" ht="48" customHeight="1">
       <c r="A5" s="12" t="inlineStr">
         <is>
-          <t>Kodefy</t>
+          <t>Assesi</t>
         </is>
       </c>
       <c r="B5" s="13" t="inlineStr">
         <is>
-          <t>Gerenciamento de Projetos e Metas Municipais / App de Prefeitura</t>
+          <t>Portais Governamentais e Transparência Municipal (LAI / LGPD / e-PING)</t>
         </is>
       </c>
       <c r="C5" s="13" t="inlineStr">
         <is>
-          <t>Startup</t>
+          <t>PME Estabelecida</t>
         </is>
       </c>
       <c r="D5" s="13" t="inlineStr">
         <is>
-          <t>Tapejara - RS</t>
+          <t>Fortaleza - CE</t>
         </is>
       </c>
       <c r="E5" s="13" t="inlineStr">
         <is>
-          <t>N/D</t>
+          <t>2011</t>
         </is>
       </c>
       <c r="F5" s="13" t="inlineStr">
         <is>
-          <t>Municípios RS e outros estados | contratada por inexigibilidade (art. 74 IV Lei 14.133/2021)</t>
+          <t>600+ municípios | 27 estados | prefeituras, câmaras, SAAEs, autarquias e consórcios</t>
         </is>
       </c>
       <c r="G5" s="13" t="inlineStr">
@@ -2613,12 +2613,12 @@
       </c>
       <c r="H5" s="13" t="inlineStr">
         <is>
-          <t>Plataforma dual: (1) Gov — cadastramento e gerenciamento de projetos e metas da administração pública municipal: gestores acompanham objetivos da gestão em tempo real, com dashboards e relatórios de execução; contratada via inexigibilidade de licitação (ex: Selbach-RS, 2026). (2) Fidelizec — plataforma B2C de programas de fidelidade para comércio local, com R$7,7M movimentados em uma única Black Friday. Apps com média 4.8★ (de 5.0) nas lojas. CNPJ: 41.426.978/0001-05. Sede: Tapejara RS.</t>
+          <t>Suíte SaaS de portais governamentais e transparência para o setor público: aSiteGov (CMS white-label para sites de prefeituras e câmaras — LAI, LGPD, e-PING e acessibilidade W3C, 99,97% uptime, atualização sem código), aLegislativo (gestão de processos e transparência para câmaras de vereadores — sessões, votações, propostas), aCidadão (portal do cidadão), aCartaServiços (carta de serviços públicos digital), aDiário (diário oficial eletrônico), aOuvidoria (ouvidoria digital) e CarteirinhaGov. Clientes: Prefeitura de Tauá CE, Prefeitura de Caucaia CE, Câmara de Senador Elói de Souza RN, entre 600+ outros. 25 colaboradores. 14 anos de mercado. Contato: +55 85 3025-2726.</t>
         </is>
       </c>
       <c r="I5" s="18" t="inlineStr">
         <is>
-          <t>Watch — metas municipais</t>
+          <t>Watch — transparência municipal</t>
         </is>
       </c>
       <c r="J5" s="19" t="inlineStr">
@@ -2630,32 +2630,32 @@
     <row r="6" ht="48" customHeight="1">
       <c r="A6" s="14" t="inlineStr">
         <is>
-          <t>GovDigital</t>
+          <t>Kodefy</t>
         </is>
       </c>
       <c r="B6" s="15" t="inlineStr">
         <is>
-          <t>App Municipal SaaS / Relacionamento Cidadão-Governo</t>
+          <t>Gerenciamento de Projetos e Metas Municipais / App de Prefeitura</t>
         </is>
       </c>
       <c r="C6" s="15" t="inlineStr">
         <is>
-          <t>Startup / Scale-up</t>
+          <t>Startup</t>
         </is>
       </c>
       <c r="D6" s="15" t="inlineStr">
         <is>
-          <t>Jaraguá do Sul - SC</t>
+          <t>Tapejara - RS</t>
         </is>
       </c>
       <c r="E6" s="15" t="inlineStr">
         <is>
-          <t>~2020</t>
+          <t>N/D</t>
         </is>
       </c>
       <c r="F6" s="15" t="inlineStr">
         <is>
-          <t>Múltiplos municípios SC e outros estados</t>
+          <t>Municípios RS e outros estados | contratada por inexigibilidade (art. 74 IV Lei 14.133/2021)</t>
         </is>
       </c>
       <c r="G6" s="15" t="inlineStr">
@@ -2665,69 +2665,77 @@
       </c>
       <c r="H6" s="15" t="inlineStr">
         <is>
-          <t>App oficial white-label de prefeituras reunindo zeladoria, agendamento, formulários online, notícias e comunicação direta cidadão-prefeitura. Integrações com IPTU, protocolo e ouvidoria. CEO: Elias Raasch. Expansão nacional sem VC.</t>
+          <t>Plataforma dual: (1) Gov — cadastramento e gerenciamento de projetos e metas da administração pública municipal: gestores acompanham objetivos da gestão em tempo real, com dashboards e relatórios de execução; contratada via inexigibilidade de licitação (ex: Selbach-RS, 2026). (2) Fidelizec — plataforma B2C de programas de fidelidade para comércio local, com R$7,7M movimentados em uma única Black Friday. Apps com média 4.8★ (de 5.0) nas lojas. CNPJ: 41.426.978/0001-05. Sede: Tapejara RS.</t>
         </is>
       </c>
       <c r="I6" s="16" t="inlineStr">
         <is>
-          <t>Watch — expansão nacional</t>
-        </is>
-      </c>
-      <c r="J6" s="15" t="inlineStr"/>
+          <t>Watch — metas municipais</t>
+        </is>
+      </c>
+      <c r="J6" s="17" t="inlineStr">
+        <is>
+          <t>✓</t>
+        </is>
+      </c>
     </row>
     <row r="7" ht="48" customHeight="1">
       <c r="A7" s="12" t="inlineStr">
         <is>
-          <t>Desenvolve Cidade</t>
+          <t>GovDigital</t>
         </is>
       </c>
       <c r="B7" s="13" t="inlineStr">
         <is>
-          <t>Licenciamento e Tributação Municipal Digital</t>
+          <t>App Municipal SaaS / Relacionamento Cidadão-Governo</t>
         </is>
       </c>
       <c r="C7" s="13" t="inlineStr">
         <is>
-          <t>Startup</t>
+          <t>Startup / Scale-up</t>
         </is>
       </c>
       <c r="D7" s="13" t="inlineStr">
         <is>
-          <t>Campinas - SP</t>
+          <t>Jaraguá do Sul - SC</t>
         </is>
       </c>
       <c r="E7" s="13" t="inlineStr">
         <is>
-          <t>~2014</t>
+          <t>~2020</t>
         </is>
       </c>
       <c r="F7" s="13" t="inlineStr">
         <is>
-          <t>Municípios Norte e outras regiões | Scale-Up Endeavor 2021</t>
+          <t>Múltiplos municípios SC e outros estados</t>
         </is>
       </c>
       <c r="G7" s="13" t="inlineStr">
         <is>
-          <t>N/D</t>
+          <t>N/D (bootstrap)</t>
         </is>
       </c>
       <c r="H7" s="13" t="inlineStr">
         <is>
-          <t>Plataforma integrada de licenciamento digital (urbanístico, ambiental, sanitário, obras), abertura/baixa de empresas, IPTU e ISS digitais integrada à REDESIM federal. Foco em desburocratização e aumento de receita própria municipal. TOP2 Open Startups 2024.</t>
-        </is>
-      </c>
-      <c r="I7" s="13" t="inlineStr"/>
+          <t>App oficial white-label de prefeituras reunindo zeladoria, agendamento, formulários online, notícias e comunicação direta cidadão-prefeitura. Integrações com IPTU, protocolo e ouvidoria. CEO: Elias Raasch. Expansão nacional sem VC.</t>
+        </is>
+      </c>
+      <c r="I7" s="18" t="inlineStr">
+        <is>
+          <t>Watch — expansão nacional</t>
+        </is>
+      </c>
       <c r="J7" s="13" t="inlineStr"/>
     </row>
     <row r="8" ht="48" customHeight="1">
       <c r="A8" s="14" t="inlineStr">
         <is>
-          <t>IP Inovação</t>
+          <t>Desenvolve Cidade</t>
         </is>
       </c>
       <c r="B8" s="15" t="inlineStr">
         <is>
-          <t>Capacitação e Consultoria em Gestão Pública</t>
+          <t>Licenciamento e Tributação Municipal Digital</t>
         </is>
       </c>
       <c r="C8" s="15" t="inlineStr">
@@ -2737,17 +2745,17 @@
       </c>
       <c r="D8" s="15" t="inlineStr">
         <is>
-          <t>Belém - PA</t>
+          <t>Campinas - SP</t>
         </is>
       </c>
       <c r="E8" s="15" t="inlineStr">
         <is>
-          <t>2014</t>
+          <t>~2014</t>
         </is>
       </c>
       <c r="F8" s="15" t="inlineStr">
         <is>
-          <t>Ecossistema Norte do Brasil</t>
+          <t>Municípios Norte e outras regiões | Scale-Up Endeavor 2021</t>
         </is>
       </c>
       <c r="G8" s="15" t="inlineStr">
@@ -2757,45 +2765,41 @@
       </c>
       <c r="H8" s="15" t="inlineStr">
         <is>
-          <t>Empresa de capacitação e consultoria para gestão pública municipal na região Norte. TOP 3 Open Startups 2024. Não foram identificados produtos SaaS com identidade digital clara — oportunidade de due diligence.</t>
-        </is>
-      </c>
-      <c r="I8" s="16" t="inlineStr">
-        <is>
-          <t>Watch — due diligence necessário</t>
-        </is>
-      </c>
+          <t>Plataforma integrada de licenciamento digital (urbanístico, ambiental, sanitário, obras), abertura/baixa de empresas, IPTU e ISS digitais integrada à REDESIM federal. Foco em desburocratização e aumento de receita própria municipal. TOP2 Open Startups 2024.</t>
+        </is>
+      </c>
+      <c r="I8" s="15" t="inlineStr"/>
       <c r="J8" s="15" t="inlineStr"/>
     </row>
     <row r="9" ht="48" customHeight="1">
       <c r="A9" s="12" t="inlineStr">
         <is>
-          <t>GESUAS</t>
+          <t>IP Inovação</t>
         </is>
       </c>
       <c r="B9" s="13" t="inlineStr">
         <is>
-          <t>Gestão do SUAS / Assistência Social</t>
+          <t>Capacitação e Consultoria em Gestão Pública</t>
         </is>
       </c>
       <c r="C9" s="13" t="inlineStr">
         <is>
-          <t>Startup / PME</t>
+          <t>Startup</t>
         </is>
       </c>
       <c r="D9" s="13" t="inlineStr">
         <is>
-          <t>Viçosa - MG</t>
+          <t>Belém - PA</t>
         </is>
       </c>
       <c r="E9" s="13" t="inlineStr">
         <is>
-          <t>2008</t>
+          <t>2014</t>
         </is>
       </c>
       <c r="F9" s="13" t="inlineStr">
         <is>
-          <t>Centenas de municípios | CRASs e CREASs</t>
+          <t>Ecossistema Norte do Brasil</t>
         </is>
       </c>
       <c r="G9" s="13" t="inlineStr">
@@ -2805,12 +2809,12 @@
       </c>
       <c r="H9" s="13" t="inlineStr">
         <is>
-          <t>SaaS de gestão do SUAS com Prontuário Digital integrado ao CadÚnico, planos PAIF/PAEFI/PIA, vigilância socioassistencial georreferenciada e relatórios MDS. 56 colaboradores. Líder IE GovTech 2020. Vertical exclusivo sem concorrente direto.</t>
+          <t>Empresa de capacitação e consultoria para gestão pública municipal na região Norte. TOP 3 Open Startups 2024. Não foram identificados produtos SaaS com identidade digital clara — oportunidade de due diligence.</t>
         </is>
       </c>
       <c r="I9" s="18" t="inlineStr">
         <is>
-          <t>Vertical exclusivo mapeado</t>
+          <t>Watch — due diligence necessário</t>
         </is>
       </c>
       <c r="J9" s="13" t="inlineStr"/>
@@ -2818,47 +2822,47 @@
     <row r="10" ht="48" customHeight="1">
       <c r="A10" s="14" t="inlineStr">
         <is>
-          <t>Prosas</t>
+          <t>GESUAS</t>
         </is>
       </c>
       <c r="B10" s="15" t="inlineStr">
         <is>
-          <t>Gestão de Editais e Investimento Social</t>
+          <t>Gestão do SUAS / Assistência Social</t>
         </is>
       </c>
       <c r="C10" s="15" t="inlineStr">
         <is>
-          <t>Startup</t>
+          <t>Startup / PME</t>
         </is>
       </c>
       <c r="D10" s="15" t="inlineStr">
         <is>
-          <t>Belo Horizonte - MG</t>
+          <t>Viçosa - MG</t>
         </is>
       </c>
       <c r="E10" s="15" t="inlineStr">
         <is>
-          <t>2014</t>
+          <t>2008</t>
         </is>
       </c>
       <c r="F10" s="15" t="inlineStr">
         <is>
-          <t>13k+ editais | institutos e fundações corporativas</t>
+          <t>Centenas de municípios | CRASs e CREASs</t>
         </is>
       </c>
       <c r="G10" s="15" t="inlineStr">
         <is>
-          <t>R$4M (KPTL)</t>
+          <t>N/D</t>
         </is>
       </c>
       <c r="H10" s="15" t="inlineStr">
         <is>
-          <t>Maior base de editais do terceiro setor no Brasil. Plataforma para criação de editais, inscrições online, pareceristas e monitoramento de projetos. Venture Round out/2024. Portfólio Fundo GovTech KPTL. 51 funcionários.</t>
+          <t>SaaS de gestão do SUAS com Prontuário Digital integrado ao CadÚnico, planos PAIF/PAEFI/PIA, vigilância socioassistencial georreferenciada e relatórios MDS. 56 colaboradores. Líder IE GovTech 2020. Vertical exclusivo sem concorrente direto.</t>
         </is>
       </c>
       <c r="I10" s="16" t="inlineStr">
         <is>
-          <t>Portfólio KPTL</t>
+          <t>Vertical exclusivo mapeado</t>
         </is>
       </c>
       <c r="J10" s="15" t="inlineStr"/>
@@ -2866,12 +2870,12 @@
     <row r="11" ht="48" customHeight="1">
       <c r="A11" s="12" t="inlineStr">
         <is>
-          <t>Lemobs</t>
+          <t>Prosas</t>
         </is>
       </c>
       <c r="B11" s="13" t="inlineStr">
         <is>
-          <t>Gestão Urbana Integrada / Smart Cities</t>
+          <t>Gestão de Editais e Investimento Social</t>
         </is>
       </c>
       <c r="C11" s="13" t="inlineStr">
@@ -2881,41 +2885,45 @@
       </c>
       <c r="D11" s="13" t="inlineStr">
         <is>
-          <t>Rio de Janeiro - RJ</t>
+          <t>Belo Horizonte - MG</t>
         </is>
       </c>
       <c r="E11" s="13" t="inlineStr">
         <is>
-          <t>2015</t>
+          <t>2014</t>
         </is>
       </c>
       <c r="F11" s="13" t="inlineStr">
         <is>
-          <t>79k+ pontos monitorados | prefeituras e Petrobras</t>
+          <t>13k+ editais | institutos e fundações corporativas</t>
         </is>
       </c>
       <c r="G11" s="13" t="inlineStr">
         <is>
-          <t>N/D</t>
+          <t>R$4M (KPTL)</t>
         </is>
       </c>
       <c r="H11" s="13" t="inlineStr">
         <is>
-          <t>GovTech de cidades inteligentes com SIGELU (limpeza urbana), fiscalização móvel, gestão nutricional escolar e saúde. Primeiro contrato pelo Marco Legal das Startups. Origem COPPE/UFRJ. Selo GovTech BrazilLAB.</t>
-        </is>
-      </c>
-      <c r="I11" s="13" t="inlineStr"/>
+          <t>Maior base de editais do terceiro setor no Brasil. Plataforma para criação de editais, inscrições online, pareceristas e monitoramento de projetos. Venture Round out/2024. Portfólio Fundo GovTech KPTL. 51 funcionários.</t>
+        </is>
+      </c>
+      <c r="I11" s="18" t="inlineStr">
+        <is>
+          <t>Portfólio KPTL</t>
+        </is>
+      </c>
       <c r="J11" s="13" t="inlineStr"/>
     </row>
     <row r="12" ht="48" customHeight="1">
       <c r="A12" s="14" t="inlineStr">
         <is>
-          <t>GRTS Digital</t>
+          <t>Lemobs</t>
         </is>
       </c>
       <c r="B12" s="15" t="inlineStr">
         <is>
-          <t>Gestão de Relações Trabalhistas e Sindicais (RTS)</t>
+          <t>Gestão Urbana Integrada / Smart Cities</t>
         </is>
       </c>
       <c r="C12" s="15" t="inlineStr">
@@ -2925,80 +2933,76 @@
       </c>
       <c r="D12" s="15" t="inlineStr">
         <is>
-          <t>Salvador - BA</t>
+          <t>Rio de Janeiro - RJ</t>
         </is>
       </c>
       <c r="E12" s="15" t="inlineStr">
         <is>
-          <t>2019</t>
+          <t>2015</t>
         </is>
       </c>
       <c r="F12" s="15" t="inlineStr">
         <is>
-          <t>Unilever, Coca-Cola, Vivo, Burger King, C&amp;A | 29 colaboradores</t>
+          <t>79k+ pontos monitorados | prefeituras e Petrobras</t>
         </is>
       </c>
       <c r="G12" s="15" t="inlineStr">
         <is>
-          <t>R$ 3,4M aporte (Fundo GovTech)</t>
+          <t>N/D</t>
         </is>
       </c>
       <c r="H12" s="15" t="inlineStr">
         <is>
-          <t>Ecossistema SaaS de digitalização de RTS: gestão de CCTs, IA 'Norma' para análise de cláusulas, assembleias virtuais e data intelligence. Integração com HCM via parceria LG. Prêmio inovação RH 2025. R$3,4M Fundo GovTech KPTL (jun/2025). Lançou GRTS Contábil (12 contratos nas primeiras 3 semanas). Co-investidor Aleve Legal Tech. Meta: R$25M faturamento até 2027. CEO Uirá Menezes, sede Salvador BA.</t>
-        </is>
-      </c>
-      <c r="I12" s="16" t="inlineStr">
-        <is>
-          <t>Portfólio KPTL</t>
-        </is>
-      </c>
+          <t>GovTech de cidades inteligentes com SIGELU (limpeza urbana), fiscalização móvel, gestão nutricional escolar e saúde. Primeiro contrato pelo Marco Legal das Startups. Origem COPPE/UFRJ. Selo GovTech BrazilLAB.</t>
+        </is>
+      </c>
+      <c r="I12" s="15" t="inlineStr"/>
       <c r="J12" s="15" t="inlineStr"/>
     </row>
     <row r="13" ht="48" customHeight="1">
       <c r="A13" s="12" t="inlineStr">
         <is>
-          <t>Governar</t>
+          <t>GRTS Digital</t>
         </is>
       </c>
       <c r="B13" s="13" t="inlineStr">
         <is>
-          <t>ERP Municipal Integrado / SIAFIC Cloud</t>
+          <t>Gestão de Relações Trabalhistas e Sindicais (RTS)</t>
         </is>
       </c>
       <c r="C13" s="13" t="inlineStr">
         <is>
-          <t>Startup / Scale-up</t>
+          <t>Startup</t>
         </is>
       </c>
       <c r="D13" s="13" t="inlineStr">
         <is>
-          <t>Brasil</t>
+          <t>Salvador - BA</t>
         </is>
       </c>
       <c r="E13" s="13" t="inlineStr">
         <is>
-          <t>N/D</t>
+          <t>2019</t>
         </is>
       </c>
       <c r="F13" s="13" t="inlineStr">
         <is>
-          <t>Municípios de qualquer porte | SIAFIC + SIEDUC disponíveis</t>
+          <t>Unilever, Coca-Cola, Vivo, Burger King, C&amp;A | 29 colaboradores</t>
         </is>
       </c>
       <c r="G13" s="13" t="inlineStr">
         <is>
-          <t>N/D</t>
+          <t>R$ 3,4M aporte (Fundo GovTech)</t>
         </is>
       </c>
       <c r="H13" s="13" t="inlineStr">
         <is>
-          <t>Suite ERP municipal integrada em nuvem com base de dados única: SIAFIC (financeiro/tributário), SIEDUC (educação), SISAÚDE e SIASOC. Conformidade SICONFI, SIOPE, e-Social, eSUS. Produto novo no mercado com proposta de stack completo integrado.</t>
+          <t>Ecossistema SaaS de digitalização de RTS: gestão de CCTs, IA 'Norma' para análise de cláusulas, assembleias virtuais e data intelligence. Integração com HCM via parceria LG. Prêmio inovação RH 2025. R$3,4M Fundo GovTech KPTL (jun/2025). Lançou GRTS Contábil (12 contratos nas primeiras 3 semanas). Co-investidor Aleve Legal Tech. Meta: R$25M faturamento até 2027. CEO Uirá Menezes, sede Salvador BA.</t>
         </is>
       </c>
       <c r="I13" s="18" t="inlineStr">
         <is>
-          <t>Watch — SIAFIC driver</t>
+          <t>Portfólio KPTL</t>
         </is>
       </c>
       <c r="J13" s="13" t="inlineStr"/>
@@ -3006,47 +3010,47 @@
     <row r="14" ht="48" customHeight="1">
       <c r="A14" s="14" t="inlineStr">
         <is>
-          <t>Colab</t>
+          <t>Governar</t>
         </is>
       </c>
       <c r="B14" s="15" t="inlineStr">
         <is>
-          <t>Participação Cidadã e Serviços Digitais Municipais</t>
+          <t>ERP Municipal Integrado / SIAFIC Cloud</t>
         </is>
       </c>
       <c r="C14" s="15" t="inlineStr">
         <is>
-          <t>Scale-up</t>
+          <t>Startup / Scale-up</t>
         </is>
       </c>
       <c r="D14" s="15" t="inlineStr">
         <is>
-          <t>São Paulo - SP</t>
+          <t>Brasil</t>
         </is>
       </c>
       <c r="E14" s="15" t="inlineStr">
         <is>
-          <t>2013</t>
+          <t>N/D</t>
         </is>
       </c>
       <c r="F14" s="15" t="inlineStr">
         <is>
-          <t>5 países | 1M+ cidadãos | Piauí, São Gonçalo, Santo André | Parceiro ONU-Habitat</t>
+          <t>Municípios de qualquer porte | SIAFIC + SIEDUC disponíveis</t>
         </is>
       </c>
       <c r="G14" s="15" t="inlineStr">
         <is>
-          <t>~R$25M total (MDIF+Luminate+EDP+KPTL)</t>
+          <t>N/D</t>
         </is>
       </c>
       <c r="H14" s="15" t="inlineStr">
         <is>
-          <t>Plataforma multicanal (web, app, WhatsApp) de gestão de serviços digitais, participação cidadã e CRM governamental. IA digitaliza qualquer serviço público em minutos. Em 2025 viabilizou OP Digital do Piauí (273k participantes) com validação via Receita Federal e blockchain. Lançou Colab Gov.AI (AWS Bedrock, out/2025): 94% de aceleração na criação de serviços digitais, 500+ prompts em 14 dias. Novos clientes: TCU, Diadema, Rio das Ostras, Duque de Caxias. Rodada US$10M+ em curso para 2026. Portfólio KPTL+Cedro. Co-invest EDP Ventures + Luminate + MDIF.</t>
+          <t>Suite ERP municipal integrada em nuvem com base de dados única: SIAFIC (financeiro/tributário), SIEDUC (educação), SISAÚDE e SIASOC. Conformidade SICONFI, SIOPE, e-Social, eSUS. Produto novo no mercado com proposta de stack completo integrado.</t>
         </is>
       </c>
       <c r="I14" s="16" t="inlineStr">
         <is>
-          <t>Portfólio KPTL+Cedro</t>
+          <t>Watch — SIAFIC driver</t>
         </is>
       </c>
       <c r="J14" s="15" t="inlineStr"/>
@@ -3054,47 +3058,47 @@
     <row r="15" ht="48" customHeight="1">
       <c r="A15" s="12" t="inlineStr">
         <is>
-          <t>Pública Tecnologia</t>
+          <t>Colab</t>
         </is>
       </c>
       <c r="B15" s="13" t="inlineStr">
         <is>
-          <t>ERP Municipal Full Suite</t>
+          <t>Participação Cidadã e Serviços Digitais Municipais</t>
         </is>
       </c>
       <c r="C15" s="13" t="inlineStr">
         <is>
-          <t>PME Estabelecida</t>
+          <t>Scale-up</t>
         </is>
       </c>
       <c r="D15" s="13" t="inlineStr">
         <is>
-          <t>Blumenau - SC</t>
+          <t>São Paulo - SP</t>
         </is>
       </c>
       <c r="E15" s="13" t="inlineStr">
         <is>
-          <t>1993</t>
+          <t>2013</t>
         </is>
       </c>
       <c r="F15" s="13" t="inlineStr">
         <is>
-          <t>Municípios BR + Portugal + Venezuela</t>
+          <t>5 países | 1M+ cidadãos | Piauí, São Gonçalo, Santo André | Parceiro ONU-Habitat</t>
         </is>
       </c>
       <c r="G15" s="13" t="inlineStr">
         <is>
-          <t>N/D</t>
+          <t>~R$25M total (MDIF+Luminate+EDP+KPTL)</t>
         </is>
       </c>
       <c r="H15" s="13" t="inlineStr">
         <is>
-          <t>ERP municipal full suite com 9 áreas: Financeira (contabilidade pública, NF-e), Tributária (ISS, IPTU), Gestão de Pessoas (RH, eSocial, ponto eletrônico), Saúde, Escolar, Assistência Social (SUAS), Administrativa (compras, frotas, patrimônio), Atendimento ao Cidadão (portal transparência, app Cidade Pública) e Gestão (BI, GED, PPA). 33 anos de atuação, 98 funcionários. Great Place to Work. Presença internacional: Portugal e Venezuela. Sede Blumenau/SC.</t>
+          <t>Plataforma multicanal (web, app, WhatsApp) de gestão de serviços digitais, participação cidadã e CRM governamental. IA digitaliza qualquer serviço público em minutos. Em 2025 viabilizou OP Digital do Piauí (273k participantes) com validação via Receita Federal e blockchain. Lançou Colab Gov.AI (AWS Bedrock, out/2025): 94% de aceleração na criação de serviços digitais, 500+ prompts em 14 dias. Novos clientes: TCU, Diadema, Rio das Ostras, Duque de Caxias. Rodada US$10M+ em curso para 2026. Portfólio KPTL+Cedro. Co-invest EDP Ventures + Luminate + MDIF.</t>
         </is>
       </c>
       <c r="I15" s="18" t="inlineStr">
         <is>
-          <t>Target roll-up</t>
+          <t>Portfólio KPTL+Cedro</t>
         </is>
       </c>
       <c r="J15" s="13" t="inlineStr"/>
@@ -3102,50 +3106,98 @@
     <row r="16" ht="48" customHeight="1">
       <c r="A16" s="14" t="inlineStr">
         <is>
+          <t>Pública Tecnologia</t>
+        </is>
+      </c>
+      <c r="B16" s="15" t="inlineStr">
+        <is>
+          <t>ERP Municipal Full Suite</t>
+        </is>
+      </c>
+      <c r="C16" s="15" t="inlineStr">
+        <is>
+          <t>PME Estabelecida</t>
+        </is>
+      </c>
+      <c r="D16" s="15" t="inlineStr">
+        <is>
+          <t>Blumenau - SC</t>
+        </is>
+      </c>
+      <c r="E16" s="15" t="inlineStr">
+        <is>
+          <t>1993</t>
+        </is>
+      </c>
+      <c r="F16" s="15" t="inlineStr">
+        <is>
+          <t>Municípios BR + Portugal + Venezuela</t>
+        </is>
+      </c>
+      <c r="G16" s="15" t="inlineStr">
+        <is>
+          <t>N/D</t>
+        </is>
+      </c>
+      <c r="H16" s="15" t="inlineStr">
+        <is>
+          <t>ERP municipal full suite com 9 áreas: Financeira (contabilidade pública, NF-e), Tributária (ISS, IPTU), Gestão de Pessoas (RH, eSocial, ponto eletrônico), Saúde, Escolar, Assistência Social (SUAS), Administrativa (compras, frotas, patrimônio), Atendimento ao Cidadão (portal transparência, app Cidade Pública) e Gestão (BI, GED, PPA). 33 anos de atuação, 98 funcionários. Great Place to Work. Presença internacional: Portugal e Venezuela. Sede Blumenau/SC.</t>
+        </is>
+      </c>
+      <c r="I16" s="16" t="inlineStr">
+        <is>
+          <t>Target roll-up</t>
+        </is>
+      </c>
+      <c r="J16" s="15" t="inlineStr"/>
+    </row>
+    <row r="17" ht="48" customHeight="1">
+      <c r="A17" s="12" t="inlineStr">
+        <is>
           <t>PLACE</t>
         </is>
       </c>
-      <c r="B16" s="15" t="inlineStr">
+      <c r="B17" s="13" t="inlineStr">
         <is>
           <t>Planejamento Urbano e Geointeligência / Urban Twin</t>
         </is>
       </c>
-      <c r="C16" s="15" t="inlineStr">
+      <c r="C17" s="13" t="inlineStr">
         <is>
           <t>Startup</t>
         </is>
       </c>
-      <c r="D16" s="15" t="inlineStr">
+      <c r="D17" s="13" t="inlineStr">
         <is>
           <t>Brasil</t>
         </is>
       </c>
-      <c r="E16" s="15" t="inlineStr">
-        <is>
-          <t>N/D</t>
-        </is>
-      </c>
-      <c r="F16" s="15" t="inlineStr">
+      <c r="E17" s="13" t="inlineStr">
+        <is>
+          <t>N/D</t>
+        </is>
+      </c>
+      <c r="F17" s="13" t="inlineStr">
         <is>
           <t>Prefeituras e mercado imobiliário privado</t>
         </is>
       </c>
-      <c r="G16" s="15" t="inlineStr">
-        <is>
-          <t>N/D</t>
-        </is>
-      </c>
-      <c r="H16" s="15" t="inlineStr">
+      <c r="G17" s="13" t="inlineStr">
+        <is>
+          <t>N/D</t>
+        </is>
+      </c>
+      <c r="H17" s="13" t="inlineStr">
         <is>
           <t>Plataforma dual (govtech + proptech) de inteligência territorial com Gêmeo Digital: integra bases públicas, rotinas urbanísticas, pré-aprovação de projetos e visualização 2D/3D com IA aplicada à legislação urbanística. Para o setor privado: viabilidade e gestão de portfólio imobiliário. Certificada BrazilLAB.</t>
         </is>
       </c>
-      <c r="I16" s="16" t="inlineStr">
+      <c r="I17" s="18" t="inlineStr">
         <is>
           <t>Watch — urbanismo digital</t>
         </is>
       </c>
-      <c r="J16" s="15" t="inlineStr"/>
+      <c r="J17" s="13" t="inlineStr"/>
     </row>
   </sheetData>
   <mergeCells count="1">

</xml_diff>

<commit_message>
v18: adiciona Minuta.Tech (proc) — IA jurídica setor público
Minutas para PGE/PGM, TCs, MP e Judiciário. Base RAGJUR 22M+
decisões, API Local, especialidade LGPD pública. Concorre com
MinutaIA/jAI. Total: 83 empresas únicas, 85 aparições.

Co-Authored-By: Claude Sonnet 4.6 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/Radar_GovTechs_Brasil_2026.xlsx
+++ b/Radar_GovTechs_Brasil_2026.xlsx
@@ -647,7 +647,7 @@
     <row r="1" ht="32" customHeight="1">
       <c r="A1" s="1" t="inlineStr">
         <is>
-          <t>🇧🇷 Radar GovTech Brasil 2025/2026 — DLG · Maio 2026 · v17</t>
+          <t>🇧🇷 Radar GovTech Brasil 2025/2026 — DLG · Maio 2026 · v18</t>
         </is>
       </c>
     </row>
@@ -720,7 +720,7 @@
         </is>
       </c>
       <c r="B9" s="4" t="n">
-        <v>7</v>
+        <v>8</v>
       </c>
     </row>
     <row r="10">
@@ -780,7 +780,7 @@
         </is>
       </c>
       <c r="B15" s="6" t="n">
-        <v>84</v>
+        <v>85</v>
       </c>
     </row>
     <row r="16">
@@ -790,7 +790,7 @@
         </is>
       </c>
       <c r="B16" s="8" t="n">
-        <v>82</v>
+        <v>83</v>
       </c>
     </row>
     <row r="18">
@@ -5129,7 +5129,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:J9"/>
+  <dimension ref="A1:J10"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="28" customWidth="1" min="1" max="1"/>
@@ -5206,12 +5206,12 @@
     <row r="3" ht="48" customHeight="1">
       <c r="A3" s="12" t="inlineStr">
         <is>
-          <t>MinutaIA (jAI)</t>
+          <t>Minuta.Tech</t>
         </is>
       </c>
       <c r="B3" s="13" t="inlineStr">
         <is>
-          <t>IA Jurídica / Judicial</t>
+          <t>IA Jurídica para Setor Público — Minutas, Pareceres e LGPD</t>
         </is>
       </c>
       <c r="C3" s="13" t="inlineStr">
@@ -5221,17 +5221,17 @@
       </c>
       <c r="D3" s="13" t="inlineStr">
         <is>
-          <t>Belo Horizonte - MG</t>
+          <t>Brasil</t>
         </is>
       </c>
       <c r="E3" s="13" t="inlineStr">
         <is>
-          <t>fev/2024</t>
+          <t>N/D</t>
         </is>
       </c>
       <c r="F3" s="13" t="inlineStr">
         <is>
-          <t>7 tribunais | 100k+ usr</t>
+          <t>Procuradorias (PGE/PGM) | Defensorias | Tribunais de Contas (TCU, TCEs, TCMs) | MP | Judiciário</t>
         </is>
       </c>
       <c r="G3" s="13" t="inlineStr">
@@ -5241,60 +5241,64 @@
       </c>
       <c r="H3" s="13" t="inlineStr">
         <is>
-          <t>10M+ minutas geradas. TJRS, STM, TRE-PB/BA, Tocantins. CNJ Resolução 615/2025. Exportou para a Argentina.</t>
+          <t>Plataforma de IA de minutas jurídicas desenvolvida exclusivamente para o setor público. 5 modelos de IA combinados: Claude Opus + Gemini 3.1 Pro para o corpo das minutas; Gemini Deep Research + RAGJUR (base própria com 22M+ decisões do STF, STJ e TCs) para citações verificadas. Verticais: Procuradorias (PGE/PGM — pareceres, informações em mandados de segurança, contestações), Tribunais de Contas (relatórios, votos, pareceres, instruções), Judiciário (minutas de decisões, sentenças, acórdãos), Defensorias e MP. Especialidade em LGPD pública: pareceres, RIPD, políticas de privacidade e termos de uso para órgãos. API Local disponível (documentos nunca saem da rede interna). Planos institucionais com até 15 usuários. Contratável via licitação ou dispensa. Concorre diretamente com MinutaIA/jAI, com diferencial de foco exclusivo em setor público e base RAGJUR proprietária.</t>
         </is>
       </c>
       <c r="I3" s="18" t="inlineStr">
         <is>
-          <t>Watch — tração judicial</t>
-        </is>
-      </c>
-      <c r="J3" s="13" t="inlineStr"/>
+          <t>Watch — concorre com MinutaIA</t>
+        </is>
+      </c>
+      <c r="J3" s="19" t="inlineStr">
+        <is>
+          <t>✓</t>
+        </is>
+      </c>
     </row>
     <row r="4" ht="48" customHeight="1">
       <c r="A4" s="14" t="inlineStr">
         <is>
-          <t>Attus</t>
+          <t>MinutaIA (jAI)</t>
         </is>
       </c>
       <c r="B4" s="15" t="inlineStr">
         <is>
-          <t>IA Generativa + Automações para Procuradorias (PGE/PGM)</t>
+          <t>IA Jurídica / Judicial</t>
         </is>
       </c>
       <c r="C4" s="15" t="inlineStr">
         <is>
-          <t>Scale-up</t>
+          <t>Startup</t>
         </is>
       </c>
       <c r="D4" s="15" t="inlineStr">
         <is>
-          <t>São Ludgero - SC (Grupo Eloware)</t>
+          <t>Belo Horizonte - MG</t>
         </is>
       </c>
       <c r="E4" s="15" t="inlineStr">
         <is>
-          <t>~2018</t>
+          <t>fev/2024</t>
         </is>
       </c>
       <c r="F4" s="15" t="inlineStr">
         <is>
-          <t>PGE-SP, PGE-BA, PGE-PA, PGM-Palmas</t>
+          <t>7 tribunais | 100k+ usr</t>
         </is>
       </c>
       <c r="G4" s="15" t="inlineStr">
         <is>
-          <t>SaaS Oracle Cloud</t>
+          <t>N/D</t>
         </is>
       </c>
       <c r="H4" s="15" t="inlineStr">
         <is>
-          <t>Rebrand de Attornatus (dez/2023) para Attus. IA generativa treinada exclusivamente na realidade de cada procuradoria: sínteses inteligentes de processos, geração de minutas, agente jurídico interativo. Centenas de automações em bastidores. Recuperação inteligente de Dívida Ativa com enriquecimento cadastral via Receita Federal. 4,3M+ processos analisados. 73% classificados automaticamente (98,5% acurácia). 642k+ peças geradas por IA. Referência nacional pós PGE-SP.</t>
+          <t>10M+ minutas geradas. TJRS, STM, TRE-PB/BA, Tocantins. CNJ Resolução 615/2025. Exportou para a Argentina.</t>
         </is>
       </c>
       <c r="I4" s="16" t="inlineStr">
         <is>
-          <t>M&amp;A Watch — líder do segmento</t>
+          <t>Watch — tração judicial</t>
         </is>
       </c>
       <c r="J4" s="15" t="inlineStr"/>
@@ -5302,56 +5306,60 @@
     <row r="5" ht="48" customHeight="1">
       <c r="A5" s="12" t="inlineStr">
         <is>
-          <t>Eicon / Giex</t>
+          <t>Attus</t>
         </is>
       </c>
       <c r="B5" s="13" t="inlineStr">
         <is>
-          <t>Dívida Ativa / Execução Fiscal</t>
+          <t>IA Generativa + Automações para Procuradorias (PGE/PGM)</t>
         </is>
       </c>
       <c r="C5" s="13" t="inlineStr">
         <is>
-          <t>PME</t>
+          <t>Scale-up</t>
         </is>
       </c>
       <c r="D5" s="13" t="inlineStr">
         <is>
-          <t>Brasil</t>
+          <t>São Ludgero - SC (Grupo Eloware)</t>
         </is>
       </c>
       <c r="E5" s="13" t="inlineStr">
         <is>
-          <t>N/D</t>
+          <t>~2018</t>
         </is>
       </c>
       <c r="F5" s="13" t="inlineStr">
         <is>
-          <t>PGE e PGM — múltiplos estados</t>
+          <t>PGE-SP, PGE-BA, PGE-PA, PGM-Palmas</t>
         </is>
       </c>
       <c r="G5" s="13" t="inlineStr">
         <is>
-          <t>N/D</t>
+          <t>SaaS Oracle Cloud</t>
         </is>
       </c>
       <c r="H5" s="13" t="inlineStr">
         <is>
-          <t>Giex: perfil completo do devedor. Integração direta com TJs. Automação de CDA, penhoras e prazos. iCad: alvarás e licenças digitais (concorrente da Quasar). +15 produtos para governo.</t>
-        </is>
-      </c>
-      <c r="I5" s="13" t="inlineStr"/>
+          <t>Rebrand de Attornatus (dez/2023) para Attus. IA generativa treinada exclusivamente na realidade de cada procuradoria: sínteses inteligentes de processos, geração de minutas, agente jurídico interativo. Centenas de automações em bastidores. Recuperação inteligente de Dívida Ativa com enriquecimento cadastral via Receita Federal. 4,3M+ processos analisados. 73% classificados automaticamente (98,5% acurácia). 642k+ peças geradas por IA. Referência nacional pós PGE-SP.</t>
+        </is>
+      </c>
+      <c r="I5" s="18" t="inlineStr">
+        <is>
+          <t>M&amp;A Watch — líder do segmento</t>
+        </is>
+      </c>
       <c r="J5" s="13" t="inlineStr"/>
     </row>
     <row r="6" ht="48" customHeight="1">
       <c r="A6" s="14" t="inlineStr">
         <is>
-          <t>PGMNET</t>
+          <t>Eicon / Giex</t>
         </is>
       </c>
       <c r="B6" s="15" t="inlineStr">
         <is>
-          <t>Gestão Jurídica Municipal + RPA</t>
+          <t>Dívida Ativa / Execução Fiscal</t>
         </is>
       </c>
       <c r="C6" s="15" t="inlineStr">
@@ -5361,7 +5369,7 @@
       </c>
       <c r="D6" s="15" t="inlineStr">
         <is>
-          <t>Campos dos Goytacazes - RJ</t>
+          <t>Brasil</t>
         </is>
       </c>
       <c r="E6" s="15" t="inlineStr">
@@ -5371,7 +5379,7 @@
       </c>
       <c r="F6" s="15" t="inlineStr">
         <is>
-          <t>Procuradorias municipais RJ e outros estados</t>
+          <t>PGE e PGM — múltiplos estados</t>
         </is>
       </c>
       <c r="G6" s="15" t="inlineStr">
@@ -5381,7 +5389,7 @@
       </c>
       <c r="H6" s="15" t="inlineStr">
         <is>
-          <t>Software jurídico SaaS para procuradorias municipais com automação RPA: peticionamento automático em qualquer TJ do país, captura de publicações e intimações 24/7, gestão de prazos e processos judiciais e administrativos. IA integrada. Desenvolvido co-criação com procuradores. Cases: PGM Campos dos Goytacazes RJ, São Francisco de Itabopoana RJ, São Pedro da Aldeia RJ, COMSERCAF Cabo Frio RJ.</t>
+          <t>Giex: perfil completo do devedor. Integração direta com TJs. Automação de CDA, penhoras e prazos. iCad: alvarás e licenças digitais (concorrente da Quasar). +15 produtos para governo.</t>
         </is>
       </c>
       <c r="I6" s="15" t="inlineStr"/>
@@ -5390,22 +5398,22 @@
     <row r="7" ht="48" customHeight="1">
       <c r="A7" s="12" t="inlineStr">
         <is>
-          <t>Aetos Tech</t>
+          <t>PGMNET</t>
         </is>
       </c>
       <c r="B7" s="13" t="inlineStr">
         <is>
-          <t>IA Anti-fraude Contratos (Prisma)</t>
+          <t>Gestão Jurídica Municipal + RPA</t>
         </is>
       </c>
       <c r="C7" s="13" t="inlineStr">
         <is>
-          <t>Startup</t>
+          <t>PME</t>
         </is>
       </c>
       <c r="D7" s="13" t="inlineStr">
         <is>
-          <t>Brasil</t>
+          <t>Campos dos Goytacazes - RJ</t>
         </is>
       </c>
       <c r="E7" s="13" t="inlineStr">
@@ -5415,35 +5423,31 @@
       </c>
       <c r="F7" s="13" t="inlineStr">
         <is>
-          <t>MPRJ (CPSI 2024)</t>
+          <t>Procuradorias municipais RJ e outros estados</t>
         </is>
       </c>
       <c r="G7" s="13" t="inlineStr">
         <is>
-          <t>Contrato CPSI</t>
+          <t>N/D</t>
         </is>
       </c>
       <c r="H7" s="13" t="inlineStr">
         <is>
-          <t>Prisma: detecção de irregularidades em contratos públicos e lavagem de dinheiro. Cruzamento de bases abertas por IA. Selecionada CPSI MPRJ.</t>
-        </is>
-      </c>
-      <c r="I7" s="18" t="inlineStr">
-        <is>
-          <t>Contrato CPSI</t>
-        </is>
-      </c>
+          <t>Software jurídico SaaS para procuradorias municipais com automação RPA: peticionamento automático em qualquer TJ do país, captura de publicações e intimações 24/7, gestão de prazos e processos judiciais e administrativos. IA integrada. Desenvolvido co-criação com procuradores. Cases: PGM Campos dos Goytacazes RJ, São Francisco de Itabopoana RJ, São Pedro da Aldeia RJ, COMSERCAF Cabo Frio RJ.</t>
+        </is>
+      </c>
+      <c r="I7" s="13" t="inlineStr"/>
       <c r="J7" s="13" t="inlineStr"/>
     </row>
     <row r="8" ht="48" customHeight="1">
       <c r="A8" s="14" t="inlineStr">
         <is>
-          <t>Sumé Tecnologia</t>
+          <t>Aetos Tech</t>
         </is>
       </c>
       <c r="B8" s="15" t="inlineStr">
         <is>
-          <t>Monitoramento Políticas Públicas (Sonar)</t>
+          <t>IA Anti-fraude Contratos (Prisma)</t>
         </is>
       </c>
       <c r="C8" s="15" t="inlineStr">
@@ -5473,7 +5477,7 @@
       </c>
       <c r="H8" s="15" t="inlineStr">
         <is>
-          <t>Sonar: controle externo automatizado do executivo municipal. Monitora 92 municípios do RJ via MPRJ. Selecionada CPSI MPRJ.</t>
+          <t>Prisma: detecção de irregularidades em contratos públicos e lavagem de dinheiro. Cruzamento de bases abertas por IA. Selecionada CPSI MPRJ.</t>
         </is>
       </c>
       <c r="I8" s="16" t="inlineStr">
@@ -5486,46 +5490,94 @@
     <row r="9" ht="48" customHeight="1">
       <c r="A9" s="12" t="inlineStr">
         <is>
+          <t>Sumé Tecnologia</t>
+        </is>
+      </c>
+      <c r="B9" s="13" t="inlineStr">
+        <is>
+          <t>Monitoramento Políticas Públicas (Sonar)</t>
+        </is>
+      </c>
+      <c r="C9" s="13" t="inlineStr">
+        <is>
+          <t>Startup</t>
+        </is>
+      </c>
+      <c r="D9" s="13" t="inlineStr">
+        <is>
+          <t>Brasil</t>
+        </is>
+      </c>
+      <c r="E9" s="13" t="inlineStr">
+        <is>
+          <t>N/D</t>
+        </is>
+      </c>
+      <c r="F9" s="13" t="inlineStr">
+        <is>
+          <t>MPRJ (CPSI 2024)</t>
+        </is>
+      </c>
+      <c r="G9" s="13" t="inlineStr">
+        <is>
+          <t>Contrato CPSI</t>
+        </is>
+      </c>
+      <c r="H9" s="13" t="inlineStr">
+        <is>
+          <t>Sonar: controle externo automatizado do executivo municipal. Monitora 92 municípios do RJ via MPRJ. Selecionada CPSI MPRJ.</t>
+        </is>
+      </c>
+      <c r="I9" s="18" t="inlineStr">
+        <is>
+          <t>Contrato CPSI</t>
+        </is>
+      </c>
+      <c r="J9" s="13" t="inlineStr"/>
+    </row>
+    <row r="10" ht="48" customHeight="1">
+      <c r="A10" s="14" t="inlineStr">
+        <is>
           <t>Prodata Gestão Estratégica</t>
         </is>
       </c>
-      <c r="B9" s="13" t="inlineStr">
+      <c r="B10" s="15" t="inlineStr">
         <is>
           <t>Módulo Procuradoria / ERP Municipal</t>
         </is>
       </c>
-      <c r="C9" s="13" t="inlineStr">
+      <c r="C10" s="15" t="inlineStr">
         <is>
           <t>PME</t>
         </is>
       </c>
-      <c r="D9" s="13" t="inlineStr">
+      <c r="D10" s="15" t="inlineStr">
         <is>
           <t>Goiânia - GO</t>
         </is>
       </c>
-      <c r="E9" s="13" t="inlineStr">
-        <is>
-          <t>N/D</t>
-        </is>
-      </c>
-      <c r="F9" s="13" t="inlineStr">
+      <c r="E10" s="15" t="inlineStr">
+        <is>
+          <t>N/D</t>
+        </is>
+      </c>
+      <c r="F10" s="15" t="inlineStr">
         <is>
           <t>Municípios Centro-Oeste</t>
         </is>
       </c>
-      <c r="G9" s="13" t="inlineStr">
-        <is>
-          <t>N/D</t>
-        </is>
-      </c>
-      <c r="H9" s="13" t="inlineStr">
+      <c r="G10" s="15" t="inlineStr">
+        <is>
+          <t>N/D</t>
+        </is>
+      </c>
+      <c r="H10" s="15" t="inlineStr">
         <is>
           <t>Módulo procuradoria integrado ao ERP municipal Prodata. Gestão de contencioso, consultivo e execução fiscal para prefeituras de pequeno e médio porte.</t>
         </is>
       </c>
-      <c r="I9" s="13" t="inlineStr"/>
-      <c r="J9" s="13" t="inlineStr"/>
+      <c r="I10" s="15" t="inlineStr"/>
+      <c r="J10" s="15" t="inlineStr"/>
     </row>
   </sheetData>
   <mergeCells count="1">

</xml_diff>